<commit_message>
Perbarui data SE2026 17/08/2026 17:14:52,32
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="169">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 17 Agu 2026, 06.16 | Dicetak: 17 Agu 2026, 08.20</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 17 Agu 2026, 12.30 | Dicetak: 17 Agu 2026, 17.14</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,22 +123,22 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>62,36</t>
-  </si>
-  <si>
-    <t>1,74</t>
+    <t>62,57</t>
+  </si>
+  <si>
+    <t>1,75</t>
   </si>
   <si>
     <t>0,05</t>
   </si>
   <si>
-    <t>20,29</t>
+    <t>20,35</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>73,37</t>
+    <t>73,61</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>78,06</t>
+    <t>78,18</t>
   </si>
   <si>
     <t>1,12</t>
@@ -156,13 +156,13 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>17,89</t>
+    <t>17,91</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>90,77</t>
+    <t>90,92</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,16 +171,16 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>65,3</t>
+    <t>65,46</t>
   </si>
   <si>
     <t>0,96</t>
   </si>
   <si>
-    <t>16,02</t>
-  </si>
-  <si>
-    <t>79,49</t>
+    <t>16,05</t>
+  </si>
+  <si>
+    <t>79,69</t>
   </si>
   <si>
     <t>1803</t>
@@ -189,19 +189,19 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>57,01</t>
+    <t>57,17</t>
   </si>
   <si>
     <t>1,15</t>
   </si>
   <si>
-    <t>18,89</t>
+    <t>18,94</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>68,64</t>
+    <t>68,83</t>
   </si>
   <si>
     <t>1804</t>
@@ -210,19 +210,19 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>64,12</t>
+    <t>64,32</t>
   </si>
   <si>
     <t>1,84</t>
   </si>
   <si>
-    <t>17,72</t>
+    <t>17,76</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>72,68</t>
+    <t>72,9</t>
   </si>
   <si>
     <t>1805</t>
@@ -231,19 +231,19 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>63,48</t>
-  </si>
-  <si>
-    <t>2,63</t>
-  </si>
-  <si>
-    <t>17,59</t>
+    <t>63,72</t>
+  </si>
+  <si>
+    <t>2,64</t>
+  </si>
+  <si>
+    <t>17,68</t>
   </si>
   <si>
     <t>0,21</t>
   </si>
   <si>
-    <t>71,96</t>
+    <t>72,22</t>
   </si>
   <si>
     <t>1806</t>
@@ -252,22 +252,22 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>63,14</t>
-  </si>
-  <si>
-    <t>1,91</t>
+    <t>63,4</t>
+  </si>
+  <si>
+    <t>1,92</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>24,82</t>
+    <t>24,91</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>74,15</t>
+    <t>74,45</t>
   </si>
   <si>
     <t>1807</t>
@@ -276,13 +276,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>63,31</t>
+    <t>63,62</t>
   </si>
   <si>
     <t>1,65</t>
   </si>
   <si>
-    <t>17,94</t>
+    <t>18,03</t>
+  </si>
+  <si>
+    <t>74,51</t>
   </si>
   <si>
     <t>1808</t>
@@ -291,19 +294,19 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>55,36</t>
+    <t>55,59</t>
   </si>
   <si>
     <t>2,21</t>
   </si>
   <si>
-    <t>24,83</t>
+    <t>24,89</t>
   </si>
   <si>
     <t>0,01</t>
   </si>
   <si>
-    <t>66,35</t>
+    <t>66,63</t>
   </si>
   <si>
     <t>1809</t>
@@ -312,19 +315,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>69,22</t>
+    <t>69,37</t>
   </si>
   <si>
     <t>2,94</t>
   </si>
   <si>
-    <t>20,48</t>
+    <t>20,51</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>82,35</t>
+    <t>82,52</t>
   </si>
   <si>
     <t>1810</t>
@@ -333,19 +336,19 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>68,49</t>
-  </si>
-  <si>
-    <t>1,42</t>
-  </si>
-  <si>
-    <t>15,44</t>
+    <t>68,75</t>
+  </si>
+  <si>
+    <t>1,43</t>
+  </si>
+  <si>
+    <t>15,49</t>
   </si>
   <si>
     <t>0,03</t>
   </si>
   <si>
-    <t>77,24</t>
+    <t>77,54</t>
   </si>
   <si>
     <t>1811</t>
@@ -354,7 +357,7 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>73,25</t>
+    <t>73,32</t>
   </si>
   <si>
     <t>1,58</t>
@@ -363,13 +366,10 @@
     <t>0,11</t>
   </si>
   <si>
-    <t>24,91</t>
-  </si>
-  <si>
     <t>0,15</t>
   </si>
   <si>
-    <t>89,09</t>
+    <t>89,21</t>
   </si>
   <si>
     <t>1812</t>
@@ -378,19 +378,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>71,28</t>
+    <t>71,47</t>
   </si>
   <si>
     <t>2,41</t>
   </si>
   <si>
-    <t>22,82</t>
+    <t>22,87</t>
   </si>
   <si>
     <t>0,22</t>
   </si>
   <si>
-    <t>83,59</t>
+    <t>83,83</t>
   </si>
   <si>
     <t>1813</t>
@@ -399,16 +399,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>80,13</t>
+    <t>80,24</t>
   </si>
   <si>
     <t>0,83</t>
   </si>
   <si>
-    <t>17,43</t>
-  </si>
-  <si>
-    <t>97,45</t>
+    <t>17,46</t>
+  </si>
+  <si>
+    <t>97,61</t>
   </si>
   <si>
     <t>1871</t>
@@ -417,16 +417,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>45,48</t>
+    <t>45,68</t>
   </si>
   <si>
     <t>0,82</t>
   </si>
   <si>
-    <t>29,32</t>
-  </si>
-  <si>
-    <t>58,21</t>
+    <t>29,4</t>
+  </si>
+  <si>
+    <t>58,45</t>
   </si>
   <si>
     <t>1872</t>
@@ -435,16 +435,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>60,55</t>
+    <t>60,74</t>
   </si>
   <si>
     <t>1,33</t>
   </si>
   <si>
-    <t>20,84</t>
-  </si>
-  <si>
-    <t>69,42</t>
+    <t>20,91</t>
+  </si>
+  <si>
+    <t>69,63</t>
   </si>
   <si>
     <t/>
@@ -489,7 +489,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>7</t>
+    <t>7,18</t>
   </si>
   <si>
     <t>0</t>
@@ -498,10 +498,7 @@
     <t>4,35</t>
   </si>
   <si>
-    <t>3,26</t>
-  </si>
-  <si>
-    <t>2,58</t>
+    <t>2,56</t>
   </si>
   <si>
     <t>10</t>
@@ -513,10 +510,10 @@
     <t>2,86</t>
   </si>
   <si>
-    <t>3,45</t>
-  </si>
-  <si>
-    <t>8,06</t>
+    <t>6,9</t>
+  </si>
+  <si>
+    <t>7,69</t>
   </si>
   <si>
     <t>1,71</t>
@@ -1183,28 +1180,28 @@
         <v>2730931</v>
       </c>
       <c r="D6" s="6">
-        <v>1703096</v>
+        <v>1708608</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>300586</v>
+        <v>301518</v>
       </c>
       <c r="G6" s="6">
-        <v>47604</v>
+        <v>47673</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1365</v>
+        <v>1367</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>554142</v>
+        <v>555780</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1216,7 +1213,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2003682</v>
+        <v>2010126</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1233,16 +1230,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>66462</v>
+        <v>66566</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10828</v>
+        <v>10850</v>
       </c>
       <c r="G7" s="9">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1254,7 +1251,7 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15236</v>
+        <v>15251</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1266,7 +1263,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>77290</v>
+        <v>77416</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1283,16 +1280,16 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>112944</v>
+        <v>113226</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>24534</v>
+        <v>24600</v>
       </c>
       <c r="G8" s="9">
-        <v>1652</v>
+        <v>1654</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
@@ -1304,7 +1301,7 @@
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>27709</v>
+        <v>27755</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1316,7 +1313,7 @@
         <v>48</v>
       </c>
       <c r="O8" s="9">
-        <v>137478</v>
+        <v>137826</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>55</v>
@@ -1333,16 +1330,16 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>195399</v>
+        <v>195928</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>58</v>
       </c>
       <c r="F9" s="9">
-        <v>39864</v>
+        <v>39970</v>
       </c>
       <c r="G9" s="9">
-        <v>3943</v>
+        <v>3954</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>59</v>
@@ -1354,7 +1351,7 @@
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>64747</v>
+        <v>64927</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>60</v>
@@ -1366,7 +1363,7 @@
         <v>61</v>
       </c>
       <c r="O9" s="9">
-        <v>235263</v>
+        <v>235898</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>62</v>
@@ -1383,16 +1380,16 @@
         <v>362837</v>
       </c>
       <c r="D10" s="9">
-        <v>232633</v>
+        <v>233373</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>65</v>
       </c>
       <c r="F10" s="9">
-        <v>31067</v>
+        <v>31148</v>
       </c>
       <c r="G10" s="9">
-        <v>6676</v>
+        <v>6687</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>66</v>
@@ -1404,7 +1401,7 @@
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>64282</v>
+        <v>64437</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>67</v>
@@ -1416,7 +1413,7 @@
         <v>68</v>
       </c>
       <c r="O10" s="9">
-        <v>263700</v>
+        <v>264521</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>69</v>
@@ -1433,28 +1430,28 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>285404</v>
+        <v>286466</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>72</v>
       </c>
       <c r="F11" s="9">
-        <v>38117</v>
+        <v>38225</v>
       </c>
       <c r="G11" s="9">
-        <v>11837</v>
+        <v>11858</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I11" s="9">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="K11" s="9">
-        <v>79059</v>
+        <v>79470</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>74</v>
@@ -1466,7 +1463,7 @@
         <v>75</v>
       </c>
       <c r="O11" s="9">
-        <v>323521</v>
+        <v>324691</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>76</v>
@@ -1483,16 +1480,16 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>125903</v>
+        <v>126420</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>79</v>
       </c>
       <c r="F12" s="9">
-        <v>21940</v>
+        <v>22027</v>
       </c>
       <c r="G12" s="9">
-        <v>3817</v>
+        <v>3829</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>80</v>
@@ -1504,7 +1501,7 @@
         <v>81</v>
       </c>
       <c r="K12" s="9">
-        <v>49489</v>
+        <v>49672</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>82</v>
@@ -1516,7 +1513,7 @@
         <v>83</v>
       </c>
       <c r="O12" s="9">
-        <v>147843</v>
+        <v>148447</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>84</v>
@@ -1533,16 +1530,16 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>92485</v>
+        <v>92942</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>87</v>
       </c>
       <c r="F13" s="9">
-        <v>15845</v>
+        <v>15911</v>
       </c>
       <c r="G13" s="9">
-        <v>2411</v>
+        <v>2412</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>88</v>
@@ -1554,7 +1551,7 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>26209</v>
+        <v>26343</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>89</v>
@@ -1566,36 +1563,36 @@
         <v>61</v>
       </c>
       <c r="O13" s="9">
-        <v>108330</v>
+        <v>108853</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" s="9">
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>74872</v>
+        <v>75190</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F14" s="9">
-        <v>14868</v>
+        <v>14934</v>
       </c>
       <c r="G14" s="9">
         <v>2990</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I14" s="9">
         <v>32</v>
@@ -1604,48 +1601,48 @@
         <v>81</v>
       </c>
       <c r="K14" s="9">
-        <v>33582</v>
+        <v>33666</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M14" s="9">
         <v>20</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="O14" s="9">
-        <v>89740</v>
+        <v>90124</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C15" s="9">
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>105329</v>
+        <v>105545</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F15" s="9">
-        <v>19973</v>
+        <v>20021</v>
       </c>
       <c r="G15" s="9">
-        <v>4468</v>
+        <v>4470</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I15" s="9">
         <v>55</v>
@@ -1654,110 +1651,110 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>31158</v>
+        <v>31200</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M15" s="9">
         <v>178</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="O15" s="9">
-        <v>125302</v>
+        <v>125566</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C16" s="9">
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>92971</v>
+        <v>93320</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F16" s="9">
-        <v>11880</v>
+        <v>11937</v>
       </c>
       <c r="G16" s="9">
-        <v>1931</v>
+        <v>1935</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I16" s="9">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>48</v>
       </c>
       <c r="K16" s="9">
-        <v>20962</v>
+        <v>21029</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="M16" s="9">
         <v>45</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="O16" s="9">
-        <v>104851</v>
+        <v>105257</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" s="9">
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55020</v>
+        <v>55076</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F17" s="9">
-        <v>11898</v>
+        <v>11931</v>
       </c>
       <c r="G17" s="9">
         <v>1186</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I17" s="9">
         <v>80</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K17" s="9">
-        <v>18710</v>
+        <v>18708</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>116</v>
+        <v>82</v>
       </c>
       <c r="M17" s="9">
         <v>110</v>
@@ -1766,7 +1763,7 @@
         <v>117</v>
       </c>
       <c r="O17" s="9">
-        <v>66918</v>
+        <v>67007</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>118</v>
@@ -1783,13 +1780,13 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>70688</v>
+        <v>70878</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>121</v>
       </c>
       <c r="F18" s="9">
-        <v>12211</v>
+        <v>12258</v>
       </c>
       <c r="G18" s="9">
         <v>2392</v>
@@ -1804,7 +1801,7 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22627</v>
+        <v>22678</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>123</v>
@@ -1816,7 +1813,7 @@
         <v>124</v>
       </c>
       <c r="O18" s="9">
-        <v>82899</v>
+        <v>83136</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>125</v>
@@ -1833,13 +1830,13 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33471</v>
+        <v>33516</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F19" s="9">
-        <v>7237</v>
+        <v>7256</v>
       </c>
       <c r="G19" s="9">
         <v>346</v>
@@ -1854,7 +1851,7 @@
         <v>48</v>
       </c>
       <c r="K19" s="9">
-        <v>7281</v>
+        <v>7293</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>130</v>
@@ -1866,7 +1863,7 @@
         <v>48</v>
       </c>
       <c r="O19" s="9">
-        <v>40708</v>
+        <v>40772</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>131</v>
@@ -1883,28 +1880,28 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>127115</v>
+        <v>127663</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>134</v>
       </c>
       <c r="F20" s="9">
-        <v>35581</v>
+        <v>35691</v>
       </c>
       <c r="G20" s="9">
-        <v>2291</v>
+        <v>2295</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>135</v>
       </c>
       <c r="I20" s="9">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>81941</v>
+        <v>82163</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>136</v>
@@ -1913,10 +1910,10 @@
         <v>90</v>
       </c>
       <c r="N20" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="O20" s="9">
-        <v>162696</v>
+        <v>163354</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>137</v>
@@ -1933,13 +1930,13 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>32400</v>
+        <v>32499</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>140</v>
       </c>
       <c r="F21" s="9">
-        <v>4743</v>
+        <v>4759</v>
       </c>
       <c r="G21" s="9">
         <v>712</v>
@@ -1948,13 +1945,13 @@
         <v>141</v>
       </c>
       <c r="I21" s="9">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J21" s="10" t="s">
         <v>68</v>
       </c>
       <c r="K21" s="9">
-        <v>11150</v>
+        <v>11188</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>142</v>
@@ -1966,7 +1963,7 @@
         <v>81</v>
       </c>
       <c r="O21" s="9">
-        <v>37143</v>
+        <v>37258</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>143</v>
@@ -1983,28 +1980,28 @@
         <v>2730931</v>
       </c>
       <c r="D22" s="12">
-        <v>1703096</v>
+        <v>1708608</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>300586</v>
+        <v>301518</v>
       </c>
       <c r="G22" s="12">
-        <v>47604</v>
+        <v>47673</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1365</v>
+        <v>1367</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>554142</v>
+        <v>555780</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2016,7 +2013,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2003682</v>
+        <v>2010126</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2143,28 +2140,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6015101</v>
+        <v>6035822</v>
       </c>
       <c r="D6" s="6">
-        <v>103984</v>
+        <v>104237</v>
       </c>
       <c r="E6" s="6">
-        <v>65263</v>
+        <v>65470</v>
       </c>
       <c r="F6" s="6">
-        <v>326697</v>
+        <v>327703</v>
       </c>
       <c r="G6" s="6">
-        <v>52981</v>
+        <v>53153</v>
       </c>
       <c r="H6" s="6">
-        <v>9034</v>
+        <v>9051</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6119085</v>
+        <v>6140059</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2175,19 +2172,19 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>242541</v>
+        <v>242953</v>
       </c>
       <c r="D7" s="9">
-        <v>2834</v>
+        <v>2844</v>
       </c>
       <c r="E7" s="9">
-        <v>2073</v>
+        <v>2074</v>
       </c>
       <c r="F7" s="9">
-        <v>12853</v>
+        <v>12872</v>
       </c>
       <c r="G7" s="9">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H7" s="9">
         <v>396</v>
@@ -2196,7 +2193,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>245375</v>
+        <v>245797</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2207,19 +2204,19 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>419893</v>
+        <v>421054</v>
       </c>
       <c r="D8" s="9">
-        <v>5585</v>
+        <v>5593</v>
       </c>
       <c r="E8" s="9">
-        <v>4144</v>
+        <v>4153</v>
       </c>
       <c r="F8" s="9">
-        <v>32265</v>
+        <v>32343</v>
       </c>
       <c r="G8" s="9">
-        <v>3836</v>
+        <v>3846</v>
       </c>
       <c r="H8" s="9">
         <v>552</v>
@@ -2228,7 +2225,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>425478</v>
+        <v>426647</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2239,28 +2236,28 @@
         <v>57</v>
       </c>
       <c r="C9" s="9">
-        <v>715827</v>
+        <v>717862</v>
       </c>
       <c r="D9" s="9">
-        <v>12539</v>
+        <v>12556</v>
       </c>
       <c r="E9" s="9">
-        <v>8163</v>
+        <v>8176</v>
       </c>
       <c r="F9" s="9">
-        <v>35720</v>
+        <v>35821</v>
       </c>
       <c r="G9" s="9">
-        <v>4393</v>
+        <v>4405</v>
       </c>
       <c r="H9" s="9">
-        <v>965</v>
+        <v>967</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>728366</v>
+        <v>730418</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2271,28 +2268,28 @@
         <v>64</v>
       </c>
       <c r="C10" s="9">
-        <v>746174</v>
+        <v>748602</v>
       </c>
       <c r="D10" s="9">
-        <v>14632</v>
+        <v>14661</v>
       </c>
       <c r="E10" s="9">
-        <v>8783</v>
+        <v>8807</v>
       </c>
       <c r="F10" s="9">
-        <v>37101</v>
+        <v>37214</v>
       </c>
       <c r="G10" s="9">
-        <v>18507</v>
+        <v>18574</v>
       </c>
       <c r="H10" s="9">
-        <v>1032</v>
+        <v>1035</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>760806</v>
+        <v>763263</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2303,28 +2300,28 @@
         <v>71</v>
       </c>
       <c r="C11" s="9">
-        <v>945209</v>
+        <v>948845</v>
       </c>
       <c r="D11" s="9">
-        <v>19366</v>
+        <v>19431</v>
       </c>
       <c r="E11" s="9">
-        <v>11352</v>
+        <v>11394</v>
       </c>
       <c r="F11" s="9">
-        <v>42952</v>
+        <v>43084</v>
       </c>
       <c r="G11" s="9">
-        <v>7771</v>
+        <v>7789</v>
       </c>
       <c r="H11" s="9">
-        <v>1667</v>
+        <v>1668</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>964575</v>
+        <v>968276</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2335,19 +2332,19 @@
         <v>78</v>
       </c>
       <c r="C12" s="9">
-        <v>457229</v>
+        <v>459311</v>
       </c>
       <c r="D12" s="9">
-        <v>5956</v>
+        <v>5962</v>
       </c>
       <c r="E12" s="9">
-        <v>5527</v>
+        <v>5557</v>
       </c>
       <c r="F12" s="9">
-        <v>26258</v>
+        <v>26355</v>
       </c>
       <c r="G12" s="9">
-        <v>1870</v>
+        <v>1881</v>
       </c>
       <c r="H12" s="9">
         <v>496</v>
@@ -2356,7 +2353,7 @@
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>463185</v>
+        <v>465273</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2367,19 +2364,19 @@
         <v>86</v>
       </c>
       <c r="C13" s="9">
-        <v>324858</v>
+        <v>326535</v>
       </c>
       <c r="D13" s="9">
-        <v>4168</v>
+        <v>4194</v>
       </c>
       <c r="E13" s="9">
-        <v>3685</v>
+        <v>3710</v>
       </c>
       <c r="F13" s="9">
-        <v>23435</v>
+        <v>23568</v>
       </c>
       <c r="G13" s="9">
-        <v>1285</v>
+        <v>1291</v>
       </c>
       <c r="H13" s="9">
         <v>454</v>
@@ -2388,135 +2385,135 @@
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>329026</v>
+        <v>330729</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" s="9">
-        <v>265243</v>
+        <v>266487</v>
       </c>
       <c r="D14" s="9">
-        <v>7652</v>
+        <v>7680</v>
       </c>
       <c r="E14" s="9">
-        <v>2971</v>
+        <v>2986</v>
       </c>
       <c r="F14" s="9">
-        <v>18089</v>
+        <v>18169</v>
       </c>
       <c r="G14" s="9">
-        <v>1823</v>
+        <v>1827</v>
       </c>
       <c r="H14" s="9">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>272895</v>
+        <v>274167</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C15" s="9">
-        <v>377374</v>
+        <v>378234</v>
       </c>
       <c r="D15" s="9">
-        <v>7361</v>
+        <v>7375</v>
       </c>
       <c r="E15" s="9">
-        <v>6176</v>
+        <v>6188</v>
       </c>
       <c r="F15" s="9">
-        <v>25709</v>
+        <v>25750</v>
       </c>
       <c r="G15" s="9">
-        <v>3704</v>
+        <v>3711</v>
       </c>
       <c r="H15" s="9">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>384735</v>
+        <v>385609</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C16" s="9">
-        <v>309790</v>
+        <v>311074</v>
       </c>
       <c r="D16" s="9">
-        <v>4527</v>
+        <v>4536</v>
       </c>
       <c r="E16" s="9">
-        <v>2685</v>
+        <v>2693</v>
       </c>
       <c r="F16" s="9">
-        <v>18030</v>
+        <v>18106</v>
       </c>
       <c r="G16" s="9">
-        <v>3617</v>
+        <v>3637</v>
       </c>
       <c r="H16" s="9">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>314317</v>
+        <v>315610</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" s="9">
-        <v>193950</v>
+        <v>194224</v>
       </c>
       <c r="D17" s="9">
-        <v>4765</v>
+        <v>4766</v>
       </c>
       <c r="E17" s="9">
-        <v>2152</v>
+        <v>2155</v>
       </c>
       <c r="F17" s="9">
-        <v>10125</v>
+        <v>10135</v>
       </c>
       <c r="G17" s="9">
         <v>1696</v>
       </c>
       <c r="H17" s="9">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="I17" s="9">
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>198715</v>
+        <v>198990</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2527,28 +2524,28 @@
         <v>120</v>
       </c>
       <c r="C18" s="9">
-        <v>238637</v>
+        <v>239401</v>
       </c>
       <c r="D18" s="9">
-        <v>5259</v>
+        <v>5266</v>
       </c>
       <c r="E18" s="9">
-        <v>2550</v>
+        <v>2558</v>
       </c>
       <c r="F18" s="9">
-        <v>13730</v>
+        <v>13757</v>
       </c>
       <c r="G18" s="9">
-        <v>2308</v>
+        <v>2314</v>
       </c>
       <c r="H18" s="9">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>243896</v>
+        <v>244667</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2559,16 +2556,16 @@
         <v>127</v>
       </c>
       <c r="C19" s="9">
-        <v>134266</v>
+        <v>134517</v>
       </c>
       <c r="D19" s="9">
-        <v>1726</v>
+        <v>1728</v>
       </c>
       <c r="E19" s="9">
         <v>1025</v>
       </c>
       <c r="F19" s="9">
-        <v>10244</v>
+        <v>10258</v>
       </c>
       <c r="G19" s="9">
         <v>219</v>
@@ -2580,7 +2577,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>135992</v>
+        <v>136245</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2591,28 +2588,28 @@
         <v>133</v>
       </c>
       <c r="C20" s="9">
-        <v>532818</v>
+        <v>535112</v>
       </c>
       <c r="D20" s="9">
-        <v>6560</v>
+        <v>6589</v>
       </c>
       <c r="E20" s="9">
-        <v>3177</v>
+        <v>3192</v>
       </c>
       <c r="F20" s="9">
-        <v>15395</v>
+        <v>15467</v>
       </c>
       <c r="G20" s="9">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="H20" s="9">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>539378</v>
+        <v>541701</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2623,28 +2620,28 @@
         <v>139</v>
       </c>
       <c r="C21" s="9">
-        <v>111292</v>
+        <v>111611</v>
       </c>
       <c r="D21" s="9">
-        <v>1054</v>
+        <v>1056</v>
       </c>
       <c r="E21" s="9">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="F21" s="9">
-        <v>4791</v>
+        <v>4804</v>
       </c>
       <c r="G21" s="9">
-        <v>714</v>
+        <v>721</v>
       </c>
       <c r="H21" s="9">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>112346</v>
+        <v>112667</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2655,28 +2652,28 @@
         <v>145</v>
       </c>
       <c r="C22" s="12">
-        <v>6015101</v>
+        <v>6035822</v>
       </c>
       <c r="D22" s="12">
-        <v>103984</v>
+        <v>104237</v>
       </c>
       <c r="E22" s="12">
-        <v>65263</v>
+        <v>65470</v>
       </c>
       <c r="F22" s="12">
-        <v>326697</v>
+        <v>327703</v>
       </c>
       <c r="G22" s="12">
-        <v>52981</v>
+        <v>53153</v>
       </c>
       <c r="H22" s="12">
-        <v>9034</v>
+        <v>9051</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6119085</v>
+        <v>6140059</v>
       </c>
     </row>
   </sheetData>
@@ -2770,10 +2767,10 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="D7" s="6">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>158</v>
@@ -2824,10 +2821,10 @@
         <v>92</v>
       </c>
       <c r="D10" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2855,13 +2852,13 @@
         <v>71</v>
       </c>
       <c r="C12" s="9">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D12" s="9">
         <v>4</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2878,7 +2875,7 @@
         <v>2</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2900,10 +2897,10 @@
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C15" s="9">
         <v>94</v>
@@ -2917,10 +2914,10 @@
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C16" s="9">
         <v>151</v>
@@ -2929,15 +2926,15 @@
         <v>36</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C17" s="9">
         <v>35</v>
@@ -2946,24 +2943,24 @@
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C18" s="9">
         <v>29</v>
       </c>
       <c r="D18" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2974,13 +2971,13 @@
         <v>120</v>
       </c>
       <c r="C19" s="9">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D19" s="9">
         <v>5</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3014,7 +3011,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3031,7 +3028,7 @@
         <v>12</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3042,10 +3039,10 @@
         <v>145</v>
       </c>
       <c r="C23" s="12">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="D23" s="12">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>158</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 18/08/2026  6:17:16,24
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="168">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 17 Agu 2026, 12.30 | Dicetak: 17 Agu 2026, 17.14</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 17 Agu 2026, 18.16 | Dicetak: 18 Agu 2026, 06.16</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,7 +123,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>62,57</t>
+    <t>62,84</t>
   </si>
   <si>
     <t>1,75</t>
@@ -132,13 +132,13 @@
     <t>0,05</t>
   </si>
   <si>
-    <t>20,35</t>
+    <t>20,42</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>73,61</t>
+    <t>73,92</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>78,18</t>
+    <t>78,28</t>
   </si>
   <si>
     <t>1,12</t>
@@ -156,31 +156,34 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>17,91</t>
+    <t>17,98</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>91,04</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>65,72</t>
+  </si>
+  <si>
+    <t>0,96</t>
+  </si>
+  <si>
+    <t>16,09</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>90,92</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>65,46</t>
-  </si>
-  <si>
-    <t>0,96</t>
-  </si>
-  <si>
-    <t>16,05</t>
-  </si>
-  <si>
-    <t>79,69</t>
+    <t>79,99</t>
   </si>
   <si>
     <t>1803</t>
@@ -189,19 +192,16 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>57,17</t>
-  </si>
-  <si>
-    <t>1,15</t>
-  </si>
-  <si>
-    <t>18,94</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>68,83</t>
+    <t>57,39</t>
+  </si>
+  <si>
+    <t>1,16</t>
+  </si>
+  <si>
+    <t>18,99</t>
+  </si>
+  <si>
+    <t>69,09</t>
   </si>
   <si>
     <t>1804</t>
@@ -210,223 +210,220 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>64,32</t>
-  </si>
-  <si>
-    <t>1,84</t>
-  </si>
-  <si>
-    <t>17,76</t>
+    <t>64,58</t>
+  </si>
+  <si>
+    <t>1,85</t>
+  </si>
+  <si>
+    <t>17,8</t>
+  </si>
+  <si>
+    <t>73,2</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>64,05</t>
+  </si>
+  <si>
+    <t>2,65</t>
+  </si>
+  <si>
+    <t>17,78</t>
+  </si>
+  <si>
+    <t>0,22</t>
+  </si>
+  <si>
+    <t>72,59</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>63,74</t>
+  </si>
+  <si>
+    <t>1,92</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>25,02</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>74,84</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>63,89</t>
+  </si>
+  <si>
+    <t>1,65</t>
+  </si>
+  <si>
+    <t>18,09</t>
+  </si>
+  <si>
+    <t>74,82</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>55,94</t>
+  </si>
+  <si>
+    <t>2,21</t>
+  </si>
+  <si>
+    <t>24,97</t>
+  </si>
+  <si>
+    <t>67,06</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>69,55</t>
+  </si>
+  <si>
+    <t>2,94</t>
+  </si>
+  <si>
+    <t>20,54</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>82,74</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>69,06</t>
+  </si>
+  <si>
+    <t>1,43</t>
+  </si>
+  <si>
+    <t>15,55</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>72,9</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>63,72</t>
-  </si>
-  <si>
-    <t>2,64</t>
-  </si>
-  <si>
-    <t>17,68</t>
-  </si>
-  <si>
-    <t>0,21</t>
-  </si>
-  <si>
-    <t>72,22</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>63,4</t>
-  </si>
-  <si>
-    <t>1,92</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>24,91</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>74,45</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>63,62</t>
-  </si>
-  <si>
-    <t>1,65</t>
-  </si>
-  <si>
-    <t>18,03</t>
-  </si>
-  <si>
-    <t>74,51</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>55,59</t>
-  </si>
-  <si>
-    <t>2,21</t>
-  </si>
-  <si>
-    <t>24,89</t>
-  </si>
-  <si>
-    <t>0,01</t>
-  </si>
-  <si>
-    <t>66,63</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>69,37</t>
-  </si>
-  <si>
-    <t>2,94</t>
-  </si>
-  <si>
-    <t>20,51</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>82,52</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>68,75</t>
-  </si>
-  <si>
-    <t>1,43</t>
-  </si>
-  <si>
-    <t>15,49</t>
+    <t>77,88</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>73,48</t>
+  </si>
+  <si>
+    <t>1,58</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>89,4</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>71,76</t>
+  </si>
+  <si>
+    <t>2,42</t>
+  </si>
+  <si>
+    <t>22,93</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>84,15</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>80,4</t>
+  </si>
+  <si>
+    <t>0,83</t>
+  </si>
+  <si>
+    <t>17,51</t>
+  </si>
+  <si>
+    <t>97,81</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>46,01</t>
+  </si>
+  <si>
+    <t>0,82</t>
+  </si>
+  <si>
+    <t>29,48</t>
   </si>
   <si>
     <t>0,03</t>
   </si>
   <si>
-    <t>77,54</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>73,32</t>
-  </si>
-  <si>
-    <t>1,58</t>
-  </si>
-  <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>89,21</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>71,47</t>
-  </si>
-  <si>
-    <t>2,41</t>
-  </si>
-  <si>
-    <t>22,87</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>83,83</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>80,24</t>
-  </si>
-  <si>
-    <t>0,83</t>
-  </si>
-  <si>
-    <t>17,46</t>
-  </si>
-  <si>
-    <t>97,61</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>45,68</t>
-  </si>
-  <si>
-    <t>0,82</t>
-  </si>
-  <si>
-    <t>29,4</t>
-  </si>
-  <si>
-    <t>58,45</t>
+    <t>58,85</t>
   </si>
   <si>
     <t>1872</t>
@@ -435,16 +432,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>60,74</t>
+    <t>60,94</t>
   </si>
   <si>
     <t>1,33</t>
   </si>
   <si>
-    <t>20,91</t>
-  </si>
-  <si>
-    <t>69,63</t>
+    <t>21,01</t>
+  </si>
+  <si>
+    <t>69,86</t>
   </si>
   <si>
     <t/>
@@ -489,7 +486,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>7,18</t>
+    <t>7,17</t>
   </si>
   <si>
     <t>0</t>
@@ -498,7 +495,7 @@
     <t>4,35</t>
   </si>
   <si>
-    <t>2,56</t>
+    <t>2,55</t>
   </si>
   <si>
     <t>10</t>
@@ -510,7 +507,7 @@
     <t>2,86</t>
   </si>
   <si>
-    <t>6,9</t>
+    <t>7,14</t>
   </si>
   <si>
     <t>7,69</t>
@@ -1177,43 +1174,43 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>2730931</v>
+        <v>2730932</v>
       </c>
       <c r="D6" s="6">
-        <v>1708608</v>
+        <v>1716087</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>301518</v>
+        <v>302692</v>
       </c>
       <c r="G6" s="6">
-        <v>47673</v>
+        <v>47773</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1367</v>
+        <v>1372</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>555780</v>
+        <v>557603</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
       </c>
       <c r="M6" s="6">
-        <v>2646</v>
+        <v>2761</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2010126</v>
+        <v>2018779</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1230,16 +1227,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>66566</v>
+        <v>66650</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10850</v>
+        <v>10868</v>
       </c>
       <c r="G7" s="9">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1251,19 +1248,19 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15251</v>
+        <v>15306</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
       </c>
       <c r="M7" s="9">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="N7" s="10" t="s">
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>77416</v>
+        <v>77518</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1280,16 +1277,16 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>113226</v>
+        <v>113669</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>24600</v>
+        <v>24683</v>
       </c>
       <c r="G8" s="9">
-        <v>1654</v>
+        <v>1655</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
@@ -1301,69 +1298,69 @@
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>27755</v>
+        <v>27827</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
       </c>
       <c r="M8" s="9">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>137826</v>
+        <v>138352</v>
       </c>
       <c r="P8" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" s="9">
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>195928</v>
+        <v>196694</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>39970</v>
+        <v>40092</v>
       </c>
       <c r="G9" s="9">
-        <v>3954</v>
+        <v>3966</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>64927</v>
+        <v>65074</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="M9" s="9">
         <v>288</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="O9" s="9">
-        <v>235898</v>
+        <v>236786</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>62</v>
@@ -1377,172 +1374,172 @@
         <v>64</v>
       </c>
       <c r="C10" s="9">
-        <v>362837</v>
+        <v>362838</v>
       </c>
       <c r="D10" s="9">
-        <v>233373</v>
+        <v>234319</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>65</v>
       </c>
       <c r="F10" s="9">
-        <v>31148</v>
+        <v>31280</v>
       </c>
       <c r="G10" s="9">
-        <v>6687</v>
+        <v>6701</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I10" s="9">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>64437</v>
+        <v>64574</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>67</v>
       </c>
       <c r="M10" s="9">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="N10" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O10" s="9">
+        <v>265599</v>
+      </c>
+      <c r="P10" s="10" t="s">
         <v>68</v>
-      </c>
-      <c r="O10" s="9">
-        <v>264521</v>
-      </c>
-      <c r="P10" s="10" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>71</v>
       </c>
       <c r="C11" s="9">
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>286466</v>
+        <v>287956</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="9">
+        <v>38403</v>
+      </c>
+      <c r="G11" s="9">
+        <v>11896</v>
+      </c>
+      <c r="H11" s="10" t="s">
         <v>72</v>
-      </c>
-      <c r="F11" s="9">
-        <v>38225</v>
-      </c>
-      <c r="G11" s="9">
-        <v>11858</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>73</v>
       </c>
       <c r="I11" s="9">
         <v>293</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>79470</v>
+        <v>79927</v>
       </c>
       <c r="L11" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="M11" s="9">
+        <v>988</v>
+      </c>
+      <c r="N11" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="M11" s="9">
-        <v>950</v>
-      </c>
-      <c r="N11" s="10" t="s">
+      <c r="O11" s="9">
+        <v>326359</v>
+      </c>
+      <c r="P11" s="10" t="s">
         <v>75</v>
-      </c>
-      <c r="O11" s="9">
-        <v>324691</v>
-      </c>
-      <c r="P11" s="10" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>77</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>78</v>
       </c>
       <c r="C12" s="9">
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>126420</v>
+        <v>127086</v>
       </c>
       <c r="E12" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F12" s="9">
+        <v>22132</v>
+      </c>
+      <c r="G12" s="9">
+        <v>3837</v>
+      </c>
+      <c r="H12" s="10" t="s">
         <v>79</v>
-      </c>
-      <c r="F12" s="9">
-        <v>22027</v>
-      </c>
-      <c r="G12" s="9">
-        <v>3829</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>80</v>
       </c>
       <c r="I12" s="9">
         <v>44</v>
       </c>
       <c r="J12" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="K12" s="9">
+        <v>49898</v>
+      </c>
+      <c r="L12" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="K12" s="9">
-        <v>49672</v>
-      </c>
-      <c r="L12" s="10" t="s">
+      <c r="M12" s="9">
+        <v>180</v>
+      </c>
+      <c r="N12" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="M12" s="9">
-        <v>175</v>
-      </c>
-      <c r="N12" s="10" t="s">
+      <c r="O12" s="9">
+        <v>149218</v>
+      </c>
+      <c r="P12" s="10" t="s">
         <v>83</v>
-      </c>
-      <c r="O12" s="9">
-        <v>148447</v>
-      </c>
-      <c r="P12" s="10" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>85</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>86</v>
       </c>
       <c r="C13" s="9">
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>92942</v>
+        <v>93338</v>
       </c>
       <c r="E13" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F13" s="9">
+        <v>15969</v>
+      </c>
+      <c r="G13" s="9">
+        <v>2413</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>87</v>
-      </c>
-      <c r="F13" s="9">
-        <v>15911</v>
-      </c>
-      <c r="G13" s="9">
-        <v>2412</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>88</v>
       </c>
       <c r="I13" s="9">
         <v>75</v>
@@ -1551,98 +1548,98 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>26343</v>
+        <v>26430</v>
       </c>
       <c r="L13" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="M13" s="9">
+        <v>124</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="O13" s="9">
+        <v>109307</v>
+      </c>
+      <c r="P13" s="10" t="s">
         <v>89</v>
-      </c>
-      <c r="M13" s="9">
-        <v>118</v>
-      </c>
-      <c r="N13" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="O13" s="9">
-        <v>108853</v>
-      </c>
-      <c r="P13" s="10" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>91</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>92</v>
       </c>
       <c r="C14" s="9">
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>75190</v>
+        <v>75664</v>
       </c>
       <c r="E14" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" s="9">
+        <v>15036</v>
+      </c>
+      <c r="G14" s="9">
+        <v>2993</v>
+      </c>
+      <c r="H14" s="10" t="s">
         <v>93</v>
-      </c>
-      <c r="F14" s="9">
-        <v>14934</v>
-      </c>
-      <c r="G14" s="9">
-        <v>2990</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>94</v>
       </c>
       <c r="I14" s="9">
         <v>32</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K14" s="9">
-        <v>33666</v>
+        <v>33777</v>
       </c>
       <c r="L14" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="M14" s="9">
+        <v>21</v>
+      </c>
+      <c r="N14" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="O14" s="9">
+        <v>90700</v>
+      </c>
+      <c r="P14" s="10" t="s">
         <v>95</v>
-      </c>
-      <c r="M14" s="9">
-        <v>20</v>
-      </c>
-      <c r="N14" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="O14" s="9">
-        <v>90124</v>
-      </c>
-      <c r="P14" s="10" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C15" s="9">
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>105545</v>
+        <v>105831</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F15" s="9">
-        <v>20021</v>
+        <v>20071</v>
       </c>
       <c r="G15" s="9">
-        <v>4470</v>
+        <v>4471</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I15" s="9">
         <v>55</v>
@@ -1651,248 +1648,248 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>31200</v>
+        <v>31253</v>
       </c>
       <c r="L15" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="M15" s="9">
+        <v>180</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="O15" s="9">
+        <v>125902</v>
+      </c>
+      <c r="P15" s="10" t="s">
         <v>102</v>
-      </c>
-      <c r="M15" s="9">
-        <v>178</v>
-      </c>
-      <c r="N15" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="O15" s="9">
-        <v>125566</v>
-      </c>
-      <c r="P15" s="10" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C16" s="9">
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>93320</v>
+        <v>93739</v>
       </c>
       <c r="E16" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="F16" s="9">
+        <v>11979</v>
+      </c>
+      <c r="G16" s="9">
+        <v>1940</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="I16" s="9">
+        <v>97</v>
+      </c>
+      <c r="J16" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="K16" s="9">
+        <v>21106</v>
+      </c>
+      <c r="L16" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="F16" s="9">
-        <v>11937</v>
-      </c>
-      <c r="G16" s="9">
-        <v>1935</v>
-      </c>
-      <c r="H16" s="10" t="s">
+      <c r="M16" s="9">
+        <v>83</v>
+      </c>
+      <c r="N16" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="I16" s="9">
-        <v>96</v>
-      </c>
-      <c r="J16" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="K16" s="9">
-        <v>21029</v>
-      </c>
-      <c r="L16" s="10" t="s">
+      <c r="O16" s="9">
+        <v>105718</v>
+      </c>
+      <c r="P16" s="10" t="s">
         <v>109</v>
-      </c>
-      <c r="M16" s="9">
-        <v>45</v>
-      </c>
-      <c r="N16" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="O16" s="9">
-        <v>105257</v>
-      </c>
-      <c r="P16" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C17" s="9">
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55076</v>
+        <v>55194</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F17" s="9">
-        <v>11931</v>
+        <v>11961</v>
       </c>
       <c r="G17" s="9">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I17" s="9">
         <v>80</v>
       </c>
       <c r="J17" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="K17" s="9">
+        <v>18757</v>
+      </c>
+      <c r="L17" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="M17" s="9">
+        <v>114</v>
+      </c>
+      <c r="N17" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="O17" s="9">
+        <v>67155</v>
+      </c>
+      <c r="P17" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="K17" s="9">
-        <v>18708</v>
-      </c>
-      <c r="L17" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="M17" s="9">
-        <v>110</v>
-      </c>
-      <c r="N17" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="O17" s="9">
-        <v>67007</v>
-      </c>
-      <c r="P17" s="10" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C18" s="9">
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>70878</v>
+        <v>71166</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F18" s="9">
-        <v>12258</v>
+        <v>12282</v>
       </c>
       <c r="G18" s="9">
-        <v>2392</v>
+        <v>2398</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="I18" s="9">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J18" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22678</v>
+        <v>22737</v>
       </c>
       <c r="L18" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="M18" s="9">
+        <v>227</v>
+      </c>
+      <c r="N18" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="O18" s="9">
+        <v>83448</v>
+      </c>
+      <c r="P18" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="M18" s="9">
-        <v>222</v>
-      </c>
-      <c r="N18" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="O18" s="9">
-        <v>83136</v>
-      </c>
-      <c r="P18" s="10" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C19" s="9">
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33516</v>
+        <v>33585</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F19" s="9">
-        <v>7256</v>
+        <v>7271</v>
       </c>
       <c r="G19" s="9">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I19" s="9">
         <v>28</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="K19" s="9">
-        <v>7293</v>
+        <v>7313</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="M19" s="9">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="O19" s="9">
-        <v>40772</v>
+        <v>40856</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C20" s="9">
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>127663</v>
+        <v>128591</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F20" s="9">
-        <v>35691</v>
+        <v>35893</v>
       </c>
       <c r="G20" s="9">
-        <v>2295</v>
+        <v>2302</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I20" s="9">
         <v>127</v>
@@ -1901,119 +1898,119 @@
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>82163</v>
+        <v>82385</v>
       </c>
       <c r="L20" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="M20" s="9">
+        <v>91</v>
+      </c>
+      <c r="N20" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="O20" s="9">
+        <v>164484</v>
+      </c>
+      <c r="P20" s="10" t="s">
         <v>136</v>
-      </c>
-      <c r="M20" s="9">
-        <v>90</v>
-      </c>
-      <c r="N20" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="O20" s="9">
-        <v>163354</v>
-      </c>
-      <c r="P20" s="10" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>138</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>139</v>
       </c>
       <c r="C21" s="9">
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>32499</v>
+        <v>32605</v>
       </c>
       <c r="E21" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="F21" s="9">
+        <v>4772</v>
+      </c>
+      <c r="G21" s="9">
+        <v>713</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>140</v>
-      </c>
-      <c r="F21" s="9">
-        <v>4759</v>
-      </c>
-      <c r="G21" s="9">
-        <v>712</v>
-      </c>
-      <c r="H21" s="10" t="s">
-        <v>141</v>
       </c>
       <c r="I21" s="9">
         <v>33</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="K21" s="9">
-        <v>11188</v>
+        <v>11239</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="M21" s="9">
         <v>11</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O21" s="9">
-        <v>37258</v>
+        <v>37377</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>145</v>
-      </c>
       <c r="C22" s="12">
-        <v>2730931</v>
+        <v>2730932</v>
       </c>
       <c r="D22" s="12">
-        <v>1708608</v>
+        <v>1716087</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>301518</v>
+        <v>302692</v>
       </c>
       <c r="G22" s="12">
-        <v>47673</v>
+        <v>47773</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1367</v>
+        <v>1372</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>555780</v>
+        <v>557603</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
       </c>
       <c r="M22" s="12">
-        <v>2646</v>
+        <v>2761</v>
       </c>
       <c r="N22" s="13" t="s">
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2010126</v>
+        <v>2018779</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2042,7 +2039,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2076,28 +2073,28 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>147</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>148</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>150</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>151</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2140,28 +2137,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6035822</v>
+        <v>6061355</v>
       </c>
       <c r="D6" s="6">
-        <v>104237</v>
+        <v>104542</v>
       </c>
       <c r="E6" s="6">
-        <v>65470</v>
+        <v>65706</v>
       </c>
       <c r="F6" s="6">
-        <v>327703</v>
+        <v>328895</v>
       </c>
       <c r="G6" s="6">
-        <v>53153</v>
+        <v>53361</v>
       </c>
       <c r="H6" s="6">
-        <v>9051</v>
+        <v>9068</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6140059</v>
+        <v>6165897</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2172,19 +2169,19 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>242953</v>
+        <v>243234</v>
       </c>
       <c r="D7" s="9">
-        <v>2844</v>
+        <v>2845</v>
       </c>
       <c r="E7" s="9">
-        <v>2074</v>
+        <v>2075</v>
       </c>
       <c r="F7" s="9">
-        <v>12872</v>
+        <v>12884</v>
       </c>
       <c r="G7" s="9">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="H7" s="9">
         <v>396</v>
@@ -2193,7 +2190,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>245797</v>
+        <v>246079</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2204,60 +2201,60 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>421054</v>
+        <v>422614</v>
       </c>
       <c r="D8" s="9">
-        <v>5593</v>
+        <v>5600</v>
       </c>
       <c r="E8" s="9">
-        <v>4153</v>
+        <v>4167</v>
       </c>
       <c r="F8" s="9">
-        <v>32343</v>
+        <v>32434</v>
       </c>
       <c r="G8" s="9">
-        <v>3846</v>
+        <v>3857</v>
       </c>
       <c r="H8" s="9">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="I8" s="9">
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>426647</v>
+        <v>428214</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>717862</v>
+        <v>720462</v>
       </c>
       <c r="D9" s="9">
-        <v>12556</v>
+        <v>12585</v>
       </c>
       <c r="E9" s="9">
-        <v>8176</v>
+        <v>8205</v>
       </c>
       <c r="F9" s="9">
-        <v>35821</v>
+        <v>35975</v>
       </c>
       <c r="G9" s="9">
-        <v>4405</v>
+        <v>4420</v>
       </c>
       <c r="H9" s="9">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>730418</v>
+        <v>733047</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2268,83 +2265,83 @@
         <v>64</v>
       </c>
       <c r="C10" s="9">
-        <v>748602</v>
+        <v>751702</v>
       </c>
       <c r="D10" s="9">
-        <v>14661</v>
+        <v>14693</v>
       </c>
       <c r="E10" s="9">
-        <v>8807</v>
+        <v>8839</v>
       </c>
       <c r="F10" s="9">
-        <v>37214</v>
+        <v>37318</v>
       </c>
       <c r="G10" s="9">
-        <v>18574</v>
+        <v>18652</v>
       </c>
       <c r="H10" s="9">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>763263</v>
+        <v>766395</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>71</v>
-      </c>
       <c r="C11" s="9">
-        <v>948845</v>
+        <v>953668</v>
       </c>
       <c r="D11" s="9">
-        <v>19431</v>
+        <v>19496</v>
       </c>
       <c r="E11" s="9">
-        <v>11394</v>
+        <v>11455</v>
       </c>
       <c r="F11" s="9">
-        <v>43084</v>
+        <v>43280</v>
       </c>
       <c r="G11" s="9">
-        <v>7789</v>
+        <v>7832</v>
       </c>
       <c r="H11" s="9">
-        <v>1668</v>
+        <v>1670</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>968276</v>
+        <v>973164</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>78</v>
-      </c>
       <c r="C12" s="9">
-        <v>459311</v>
+        <v>461578</v>
       </c>
       <c r="D12" s="9">
-        <v>5962</v>
+        <v>5983</v>
       </c>
       <c r="E12" s="9">
-        <v>5557</v>
+        <v>5576</v>
       </c>
       <c r="F12" s="9">
-        <v>26355</v>
+        <v>26487</v>
       </c>
       <c r="G12" s="9">
-        <v>1881</v>
+        <v>1888</v>
       </c>
       <c r="H12" s="9">
         <v>496</v>
@@ -2353,30 +2350,30 @@
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>465273</v>
+        <v>467561</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>86</v>
-      </c>
       <c r="C13" s="9">
-        <v>326535</v>
+        <v>327888</v>
       </c>
       <c r="D13" s="9">
-        <v>4194</v>
+        <v>4210</v>
       </c>
       <c r="E13" s="9">
-        <v>3710</v>
+        <v>3727</v>
       </c>
       <c r="F13" s="9">
-        <v>23568</v>
+        <v>23663</v>
       </c>
       <c r="G13" s="9">
-        <v>1291</v>
+        <v>1295</v>
       </c>
       <c r="H13" s="9">
         <v>454</v>
@@ -2385,94 +2382,94 @@
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>330729</v>
+        <v>332098</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>92</v>
-      </c>
       <c r="C14" s="9">
-        <v>266487</v>
+        <v>268164</v>
       </c>
       <c r="D14" s="9">
-        <v>7680</v>
+        <v>7714</v>
       </c>
       <c r="E14" s="9">
-        <v>2986</v>
+        <v>2995</v>
       </c>
       <c r="F14" s="9">
-        <v>18169</v>
+        <v>18250</v>
       </c>
       <c r="G14" s="9">
-        <v>1827</v>
+        <v>1838</v>
       </c>
       <c r="H14" s="9">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>274167</v>
+        <v>275878</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C15" s="9">
-        <v>378234</v>
+        <v>379236</v>
       </c>
       <c r="D15" s="9">
-        <v>7375</v>
+        <v>7390</v>
       </c>
       <c r="E15" s="9">
-        <v>6188</v>
+        <v>6199</v>
       </c>
       <c r="F15" s="9">
-        <v>25750</v>
+        <v>25805</v>
       </c>
       <c r="G15" s="9">
-        <v>3711</v>
+        <v>3717</v>
       </c>
       <c r="H15" s="9">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>385609</v>
+        <v>386626</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C16" s="9">
-        <v>311074</v>
+        <v>312362</v>
       </c>
       <c r="D16" s="9">
-        <v>4536</v>
+        <v>4562</v>
       </c>
       <c r="E16" s="9">
-        <v>2693</v>
+        <v>2697</v>
       </c>
       <c r="F16" s="9">
-        <v>18106</v>
+        <v>18197</v>
       </c>
       <c r="G16" s="9">
-        <v>3637</v>
+        <v>3649</v>
       </c>
       <c r="H16" s="9">
         <v>245</v>
@@ -2481,62 +2478,62 @@
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>315610</v>
+        <v>316924</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C17" s="9">
-        <v>194224</v>
+        <v>194633</v>
       </c>
       <c r="D17" s="9">
-        <v>4766</v>
+        <v>4781</v>
       </c>
       <c r="E17" s="9">
-        <v>2155</v>
+        <v>2160</v>
       </c>
       <c r="F17" s="9">
-        <v>10135</v>
+        <v>10160</v>
       </c>
       <c r="G17" s="9">
-        <v>1696</v>
+        <v>1698</v>
       </c>
       <c r="H17" s="9">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I17" s="9">
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>198990</v>
+        <v>199414</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C18" s="9">
-        <v>239401</v>
+        <v>240308</v>
       </c>
       <c r="D18" s="9">
-        <v>5266</v>
+        <v>5281</v>
       </c>
       <c r="E18" s="9">
-        <v>2558</v>
+        <v>2565</v>
       </c>
       <c r="F18" s="9">
-        <v>13757</v>
+        <v>13792</v>
       </c>
       <c r="G18" s="9">
-        <v>2314</v>
+        <v>2321</v>
       </c>
       <c r="H18" s="9">
         <v>482</v>
@@ -2545,30 +2542,30 @@
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>244667</v>
+        <v>245589</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C19" s="9">
-        <v>134517</v>
+        <v>134806</v>
       </c>
       <c r="D19" s="9">
-        <v>1728</v>
+        <v>1730</v>
       </c>
       <c r="E19" s="9">
-        <v>1025</v>
+        <v>1027</v>
       </c>
       <c r="F19" s="9">
-        <v>10258</v>
+        <v>10274</v>
       </c>
       <c r="G19" s="9">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H19" s="9">
         <v>231</v>
@@ -2577,103 +2574,103 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>136245</v>
+        <v>136536</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C20" s="9">
-        <v>535112</v>
+        <v>538707</v>
       </c>
       <c r="D20" s="9">
-        <v>6589</v>
+        <v>6612</v>
       </c>
       <c r="E20" s="9">
-        <v>3192</v>
+        <v>3213</v>
       </c>
       <c r="F20" s="9">
-        <v>15467</v>
+        <v>15554</v>
       </c>
       <c r="G20" s="9">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="H20" s="9">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>541701</v>
+        <v>545319</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>139</v>
-      </c>
       <c r="C21" s="9">
-        <v>111611</v>
+        <v>111993</v>
       </c>
       <c r="D21" s="9">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="E21" s="9">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="F21" s="9">
-        <v>4804</v>
+        <v>4822</v>
       </c>
       <c r="G21" s="9">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="H21" s="9">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>112667</v>
+        <v>113053</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>145</v>
-      </c>
       <c r="C22" s="12">
-        <v>6035822</v>
+        <v>6061355</v>
       </c>
       <c r="D22" s="12">
-        <v>104237</v>
+        <v>104542</v>
       </c>
       <c r="E22" s="12">
-        <v>65470</v>
+        <v>65706</v>
       </c>
       <c r="F22" s="12">
-        <v>327703</v>
+        <v>328895</v>
       </c>
       <c r="G22" s="12">
-        <v>53153</v>
+        <v>53361</v>
       </c>
       <c r="H22" s="12">
-        <v>9051</v>
+        <v>9068</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6140059</v>
+        <v>6165897</v>
       </c>
     </row>
   </sheetData>
@@ -2700,7 +2697,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2724,7 +2721,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2733,13 +2730,13 @@
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2767,13 +2764,13 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="D7" s="6">
         <v>69</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2790,7 +2787,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2807,15 +2804,15 @@
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" s="9">
         <v>92</v>
@@ -2824,7 +2821,7 @@
         <v>4</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2835,38 +2832,38 @@
         <v>64</v>
       </c>
       <c r="C11" s="9">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D11" s="9">
         <v>0</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>71</v>
-      </c>
       <c r="C12" s="9">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D12" s="9">
         <v>4</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>77</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>78</v>
       </c>
       <c r="C13" s="9">
         <v>20</v>
@@ -2875,32 +2872,32 @@
         <v>2</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>86</v>
-      </c>
       <c r="C14" s="9">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>91</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>92</v>
       </c>
       <c r="C15" s="9">
         <v>94</v>
@@ -2909,15 +2906,15 @@
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C16" s="9">
         <v>151</v>
@@ -2926,15 +2923,15 @@
         <v>36</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C17" s="9">
         <v>35</v>
@@ -2943,32 +2940,32 @@
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C18" s="9">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D18" s="9">
         <v>2</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C19" s="9">
         <v>65</v>
@@ -2977,15 +2974,15 @@
         <v>5</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C20" s="9">
         <v>13</v>
@@ -2994,15 +2991,15 @@
         <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C21" s="9">
         <v>117</v>
@@ -3011,15 +3008,15 @@
         <v>2</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>138</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>139</v>
       </c>
       <c r="C22" s="9">
         <v>60</v>
@@ -3028,24 +3025,24 @@
         <v>12</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>145</v>
-      </c>
       <c r="C23" s="12">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="D23" s="12">
         <v>69</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 18/08/2026  7:20:58,80
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="166">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 17 Agu 2026, 18.16 | Dicetak: 18 Agu 2026, 06.16</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 18 Agu 2026, 06.16 | Dicetak: 18 Agu 2026, 07.20</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,7 +123,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>62,84</t>
+    <t>63,27</t>
   </si>
   <si>
     <t>1,75</t>
@@ -132,13 +132,13 @@
     <t>0,05</t>
   </si>
   <si>
-    <t>20,42</t>
+    <t>20,5</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>73,92</t>
+    <t>74,42</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>78,28</t>
+    <t>78,52</t>
   </si>
   <si>
     <t>1,12</t>
@@ -156,13 +156,13 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>17,98</t>
+    <t>18,08</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>91,04</t>
+    <t>91,33</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>65,72</t>
+    <t>66,09</t>
   </si>
   <si>
     <t>0,96</t>
   </si>
   <si>
-    <t>16,09</t>
+    <t>16,18</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>79,99</t>
+    <t>80,46</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,16 +192,16 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>57,39</t>
+    <t>57,76</t>
   </si>
   <si>
     <t>1,16</t>
   </si>
   <si>
-    <t>18,99</t>
-  </si>
-  <si>
-    <t>69,09</t>
+    <t>19,05</t>
+  </si>
+  <si>
+    <t>69,53</t>
   </si>
   <si>
     <t>1804</t>
@@ -210,16 +210,16 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>64,58</t>
+    <t>65,01</t>
   </si>
   <si>
     <t>1,85</t>
   </si>
   <si>
-    <t>17,8</t>
-  </si>
-  <si>
-    <t>73,2</t>
+    <t>17,89</t>
+  </si>
+  <si>
+    <t>73,69</t>
   </si>
   <si>
     <t>1805</t>
@@ -228,19 +228,19 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>64,05</t>
-  </si>
-  <si>
-    <t>2,65</t>
-  </si>
-  <si>
-    <t>17,78</t>
+    <t>64,51</t>
+  </si>
+  <si>
+    <t>2,66</t>
+  </si>
+  <si>
+    <t>17,87</t>
   </si>
   <si>
     <t>0,22</t>
   </si>
   <si>
-    <t>72,59</t>
+    <t>73,11</t>
   </si>
   <si>
     <t>1806</t>
@@ -249,22 +249,22 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>63,74</t>
-  </si>
-  <si>
-    <t>1,92</t>
+    <t>64,23</t>
+  </si>
+  <si>
+    <t>1,93</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>25,02</t>
+    <t>25,12</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>74,84</t>
+    <t>75,42</t>
   </si>
   <si>
     <t>1807</t>
@@ -273,16 +273,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>63,89</t>
-  </si>
-  <si>
-    <t>1,65</t>
-  </si>
-  <si>
-    <t>18,09</t>
-  </si>
-  <si>
-    <t>74,82</t>
+    <t>64,3</t>
+  </si>
+  <si>
+    <t>1,66</t>
+  </si>
+  <si>
+    <t>18,15</t>
+  </si>
+  <si>
+    <t>75,3</t>
   </si>
   <si>
     <t>1808</t>
@@ -291,16 +291,16 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>55,94</t>
-  </si>
-  <si>
-    <t>2,21</t>
-  </si>
-  <si>
-    <t>24,97</t>
-  </si>
-  <si>
-    <t>67,06</t>
+    <t>56,58</t>
+  </si>
+  <si>
+    <t>2,22</t>
+  </si>
+  <si>
+    <t>25,07</t>
+  </si>
+  <si>
+    <t>67,82</t>
   </si>
   <si>
     <t>1809</t>
@@ -309,19 +309,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>69,55</t>
+    <t>69,93</t>
   </si>
   <si>
     <t>2,94</t>
   </si>
   <si>
-    <t>20,54</t>
+    <t>20,6</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>82,74</t>
+    <t>83,19</t>
   </si>
   <si>
     <t>1810</t>
@@ -330,19 +330,19 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>69,06</t>
+    <t>69,49</t>
   </si>
   <si>
     <t>1,43</t>
   </si>
   <si>
-    <t>15,55</t>
+    <t>15,61</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>77,88</t>
+    <t>78,37</t>
   </si>
   <si>
     <t>1811</t>
@@ -351,19 +351,19 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>73,48</t>
-  </si>
-  <si>
     <t>1,58</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
+    <t>25</t>
+  </si>
+  <si>
     <t>0,15</t>
   </si>
   <si>
-    <t>89,4</t>
+    <t>89,7</t>
   </si>
   <si>
     <t>1812</t>
@@ -372,19 +372,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>71,76</t>
+    <t>72,14</t>
   </si>
   <si>
     <t>2,42</t>
   </si>
   <si>
-    <t>22,93</t>
+    <t>22,98</t>
   </si>
   <si>
     <t>0,23</t>
   </si>
   <si>
-    <t>84,15</t>
+    <t>84,6</t>
   </si>
   <si>
     <t>1813</t>
@@ -393,16 +393,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>80,4</t>
+    <t>80,64</t>
   </si>
   <si>
     <t>0,83</t>
   </si>
   <si>
-    <t>17,51</t>
-  </si>
-  <si>
-    <t>97,81</t>
+    <t>17,53</t>
+  </si>
+  <si>
+    <t>98,11</t>
   </si>
   <si>
     <t>1871</t>
@@ -411,19 +411,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>46,01</t>
-  </si>
-  <si>
-    <t>0,82</t>
-  </si>
-  <si>
-    <t>29,48</t>
+    <t>46,53</t>
+  </si>
+  <si>
+    <t>29,62</t>
   </si>
   <si>
     <t>0,03</t>
   </si>
   <si>
-    <t>58,85</t>
+    <t>59,49</t>
   </si>
   <si>
     <t>1872</t>
@@ -432,16 +429,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>60,94</t>
+    <t>61,43</t>
   </si>
   <si>
     <t>1,33</t>
   </si>
   <si>
-    <t>21,01</t>
-  </si>
-  <si>
-    <t>69,86</t>
+    <t>21,15</t>
+  </si>
+  <si>
+    <t>70,39</t>
   </si>
   <si>
     <t/>
@@ -486,7 +483,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>7,17</t>
+    <t>7,14</t>
   </si>
   <si>
     <t>0</t>
@@ -495,22 +492,19 @@
     <t>4,35</t>
   </si>
   <si>
-    <t>2,55</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>23,84</t>
-  </si>
-  <si>
-    <t>2,86</t>
-  </si>
-  <si>
-    <t>7,14</t>
-  </si>
-  <si>
-    <t>7,69</t>
+    <t>2,53</t>
+  </si>
+  <si>
+    <t>9,52</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>2,78</t>
+  </si>
+  <si>
+    <t>7,58</t>
   </si>
   <si>
     <t>1,71</t>
@@ -1177,28 +1171,28 @@
         <v>2730932</v>
       </c>
       <c r="D6" s="6">
-        <v>1716087</v>
+        <v>1727736</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>302692</v>
+        <v>304756</v>
       </c>
       <c r="G6" s="6">
-        <v>47773</v>
+        <v>47884</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1372</v>
+        <v>1383</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>557603</v>
+        <v>559929</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1210,7 +1204,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2018779</v>
+        <v>2032492</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1227,13 +1221,13 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>66650</v>
+        <v>66855</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10868</v>
+        <v>10905</v>
       </c>
       <c r="G7" s="9">
         <v>954</v>
@@ -1248,7 +1242,7 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15306</v>
+        <v>15391</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1260,7 +1254,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>77518</v>
+        <v>77760</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1277,28 +1271,28 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>113669</v>
+        <v>114306</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>24683</v>
+        <v>24849</v>
       </c>
       <c r="G8" s="9">
-        <v>1655</v>
+        <v>1661</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="9">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>27827</v>
+        <v>27977</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1310,7 +1304,7 @@
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>138352</v>
+        <v>139155</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1327,28 +1321,28 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>196694</v>
+        <v>197976</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>40092</v>
+        <v>40323</v>
       </c>
       <c r="G9" s="9">
-        <v>3966</v>
+        <v>3986</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>65074</v>
+        <v>65281</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
@@ -1360,7 +1354,7 @@
         <v>48</v>
       </c>
       <c r="O9" s="9">
-        <v>236786</v>
+        <v>238299</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>62</v>
@@ -1377,28 +1371,28 @@
         <v>362838</v>
       </c>
       <c r="D10" s="9">
-        <v>234319</v>
+        <v>235868</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>65</v>
       </c>
       <c r="F10" s="9">
-        <v>31280</v>
+        <v>31490</v>
       </c>
       <c r="G10" s="9">
-        <v>6701</v>
+        <v>6715</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I10" s="9">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>64574</v>
+        <v>64896</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>67</v>
@@ -1410,7 +1404,7 @@
         <v>55</v>
       </c>
       <c r="O10" s="9">
-        <v>265599</v>
+        <v>267358</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>68</v>
@@ -1427,16 +1421,16 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>287956</v>
+        <v>289999</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="9">
-        <v>38403</v>
+        <v>38672</v>
       </c>
       <c r="G11" s="9">
-        <v>11896</v>
+        <v>11937</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>72</v>
@@ -1448,7 +1442,7 @@
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>79927</v>
+        <v>80340</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>73</v>
@@ -1460,7 +1454,7 @@
         <v>74</v>
       </c>
       <c r="O11" s="9">
-        <v>326359</v>
+        <v>328671</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>75</v>
@@ -1477,16 +1471,16 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>127086</v>
+        <v>128065</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>78</v>
       </c>
       <c r="F12" s="9">
-        <v>22132</v>
+        <v>22315</v>
       </c>
       <c r="G12" s="9">
-        <v>3837</v>
+        <v>3840</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>79</v>
@@ -1498,7 +1492,7 @@
         <v>80</v>
       </c>
       <c r="K12" s="9">
-        <v>49898</v>
+        <v>50091</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>81</v>
@@ -1510,7 +1504,7 @@
         <v>82</v>
       </c>
       <c r="O12" s="9">
-        <v>149218</v>
+        <v>150380</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>83</v>
@@ -1527,28 +1521,28 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>93338</v>
+        <v>93935</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>86</v>
       </c>
       <c r="F13" s="9">
-        <v>15969</v>
+        <v>16070</v>
       </c>
       <c r="G13" s="9">
-        <v>2413</v>
+        <v>2419</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>87</v>
       </c>
       <c r="I13" s="9">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J13" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>26430</v>
+        <v>26523</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>88</v>
@@ -1560,7 +1554,7 @@
         <v>48</v>
       </c>
       <c r="O13" s="9">
-        <v>109307</v>
+        <v>110005</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>89</v>
@@ -1577,16 +1571,16 @@
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>75664</v>
+        <v>76524</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>92</v>
       </c>
       <c r="F14" s="9">
-        <v>15036</v>
+        <v>15202</v>
       </c>
       <c r="G14" s="9">
-        <v>2993</v>
+        <v>2996</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>93</v>
@@ -1598,7 +1592,7 @@
         <v>80</v>
       </c>
       <c r="K14" s="9">
-        <v>33777</v>
+        <v>33904</v>
       </c>
       <c r="L14" s="10" t="s">
         <v>94</v>
@@ -1610,7 +1604,7 @@
         <v>80</v>
       </c>
       <c r="O14" s="9">
-        <v>90700</v>
+        <v>91726</v>
       </c>
       <c r="P14" s="10" t="s">
         <v>95</v>
@@ -1627,16 +1621,16 @@
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>105831</v>
+        <v>106397</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>98</v>
       </c>
       <c r="F15" s="9">
-        <v>20071</v>
+        <v>20188</v>
       </c>
       <c r="G15" s="9">
-        <v>4471</v>
+        <v>4475</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>99</v>
@@ -1648,7 +1642,7 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>31253</v>
+        <v>31348</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>100</v>
@@ -1660,7 +1654,7 @@
         <v>101</v>
       </c>
       <c r="O15" s="9">
-        <v>125902</v>
+        <v>126585</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>102</v>
@@ -1677,16 +1671,16 @@
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>93739</v>
+        <v>94327</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>105</v>
       </c>
       <c r="F16" s="9">
-        <v>11979</v>
+        <v>12057</v>
       </c>
       <c r="G16" s="9">
-        <v>1940</v>
+        <v>1941</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>106</v>
@@ -1698,7 +1692,7 @@
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>21106</v>
+        <v>21192</v>
       </c>
       <c r="L16" s="10" t="s">
         <v>107</v>
@@ -1710,7 +1704,7 @@
         <v>108</v>
       </c>
       <c r="O16" s="9">
-        <v>105718</v>
+        <v>106384</v>
       </c>
       <c r="P16" s="10" t="s">
         <v>109</v>
@@ -1727,31 +1721,31 @@
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55194</v>
+        <v>55355</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>112</v>
+        <v>68</v>
       </c>
       <c r="F17" s="9">
-        <v>11961</v>
+        <v>12022</v>
       </c>
       <c r="G17" s="9">
         <v>1187</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I17" s="9">
         <v>80</v>
       </c>
       <c r="J17" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="K17" s="9">
+        <v>18782</v>
+      </c>
+      <c r="L17" s="10" t="s">
         <v>114</v>
-      </c>
-      <c r="K17" s="9">
-        <v>18757</v>
-      </c>
-      <c r="L17" s="10" t="s">
-        <v>94</v>
       </c>
       <c r="M17" s="9">
         <v>114</v>
@@ -1760,7 +1754,7 @@
         <v>115</v>
       </c>
       <c r="O17" s="9">
-        <v>67155</v>
+        <v>67377</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>116</v>
@@ -1777,16 +1771,16 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>71166</v>
+        <v>71537</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>119</v>
       </c>
       <c r="F18" s="9">
-        <v>12282</v>
+        <v>12356</v>
       </c>
       <c r="G18" s="9">
-        <v>2398</v>
+        <v>2400</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>120</v>
@@ -1798,7 +1792,7 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22737</v>
+        <v>22785</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>121</v>
@@ -1810,7 +1804,7 @@
         <v>122</v>
       </c>
       <c r="O18" s="9">
-        <v>83448</v>
+        <v>83893</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>123</v>
@@ -1827,13 +1821,13 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33585</v>
+        <v>33685</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>126</v>
       </c>
       <c r="F19" s="9">
-        <v>7271</v>
+        <v>7299</v>
       </c>
       <c r="G19" s="9">
         <v>347</v>
@@ -1848,7 +1842,7 @@
         <v>55</v>
       </c>
       <c r="K19" s="9">
-        <v>7313</v>
+        <v>7322</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>128</v>
@@ -1860,7 +1854,7 @@
         <v>55</v>
       </c>
       <c r="O19" s="9">
-        <v>40856</v>
+        <v>40984</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>129</v>
@@ -1877,81 +1871,81 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>128591</v>
+        <v>130038</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>132</v>
       </c>
       <c r="F20" s="9">
-        <v>35893</v>
+        <v>36214</v>
       </c>
       <c r="G20" s="9">
-        <v>2302</v>
+        <v>2312</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="I20" s="9">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>82385</v>
+        <v>82783</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="M20" s="9">
         <v>91</v>
       </c>
       <c r="N20" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="O20" s="9">
+        <v>166252</v>
+      </c>
+      <c r="P20" s="10" t="s">
         <v>135</v>
-      </c>
-      <c r="O20" s="9">
-        <v>164484</v>
-      </c>
-      <c r="P20" s="10" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>138</v>
       </c>
       <c r="C21" s="9">
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>32605</v>
+        <v>32869</v>
       </c>
       <c r="E21" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="F21" s="9">
+        <v>4794</v>
+      </c>
+      <c r="G21" s="9">
+        <v>714</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="F21" s="9">
-        <v>4772</v>
-      </c>
-      <c r="G21" s="9">
-        <v>713</v>
-      </c>
-      <c r="H21" s="10" t="s">
-        <v>140</v>
-      </c>
       <c r="I21" s="9">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J21" s="10" t="s">
         <v>108</v>
       </c>
       <c r="K21" s="9">
-        <v>11239</v>
+        <v>11314</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="M21" s="9">
         <v>11</v>
@@ -1960,45 +1954,45 @@
         <v>80</v>
       </c>
       <c r="O21" s="9">
-        <v>37377</v>
+        <v>37663</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>143</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>144</v>
       </c>
       <c r="C22" s="12">
         <v>2730932</v>
       </c>
       <c r="D22" s="12">
-        <v>1716087</v>
+        <v>1727736</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>302692</v>
+        <v>304756</v>
       </c>
       <c r="G22" s="12">
-        <v>47773</v>
+        <v>47884</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1372</v>
+        <v>1383</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>557603</v>
+        <v>559929</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2010,7 +2004,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2018779</v>
+        <v>2032492</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2039,7 +2033,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2073,28 +2067,28 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>146</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>147</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>148</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>149</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>150</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2137,28 +2131,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6061355</v>
+        <v>6103234</v>
       </c>
       <c r="D6" s="6">
-        <v>104542</v>
+        <v>105126</v>
       </c>
       <c r="E6" s="6">
-        <v>65706</v>
+        <v>66118</v>
       </c>
       <c r="F6" s="6">
-        <v>328895</v>
+        <v>330952</v>
       </c>
       <c r="G6" s="6">
-        <v>53361</v>
+        <v>53694</v>
       </c>
       <c r="H6" s="6">
-        <v>9068</v>
+        <v>9116</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6165897</v>
+        <v>6208360</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2169,28 +2163,28 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>243234</v>
+        <v>243969</v>
       </c>
       <c r="D7" s="9">
-        <v>2845</v>
+        <v>2859</v>
       </c>
       <c r="E7" s="9">
-        <v>2075</v>
+        <v>2079</v>
       </c>
       <c r="F7" s="9">
-        <v>12884</v>
+        <v>12930</v>
       </c>
       <c r="G7" s="9">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="H7" s="9">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="I7" s="9">
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>246079</v>
+        <v>246828</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2201,19 +2195,19 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>422614</v>
+        <v>425093</v>
       </c>
       <c r="D8" s="9">
-        <v>5600</v>
+        <v>5630</v>
       </c>
       <c r="E8" s="9">
-        <v>4167</v>
+        <v>4185</v>
       </c>
       <c r="F8" s="9">
-        <v>32434</v>
+        <v>32643</v>
       </c>
       <c r="G8" s="9">
-        <v>3857</v>
+        <v>3878</v>
       </c>
       <c r="H8" s="9">
         <v>554</v>
@@ -2222,7 +2216,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>428214</v>
+        <v>430723</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2233,28 +2227,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>720462</v>
+        <v>725218</v>
       </c>
       <c r="D9" s="9">
-        <v>12585</v>
+        <v>12651</v>
       </c>
       <c r="E9" s="9">
-        <v>8205</v>
+        <v>8254</v>
       </c>
       <c r="F9" s="9">
-        <v>35975</v>
+        <v>36179</v>
       </c>
       <c r="G9" s="9">
-        <v>4420</v>
+        <v>4440</v>
       </c>
       <c r="H9" s="9">
-        <v>968</v>
+        <v>971</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>733047</v>
+        <v>737869</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2265,28 +2259,28 @@
         <v>64</v>
       </c>
       <c r="C10" s="9">
-        <v>751702</v>
+        <v>756703</v>
       </c>
       <c r="D10" s="9">
-        <v>14693</v>
+        <v>14760</v>
       </c>
       <c r="E10" s="9">
-        <v>8839</v>
+        <v>8896</v>
       </c>
       <c r="F10" s="9">
-        <v>37318</v>
+        <v>37522</v>
       </c>
       <c r="G10" s="9">
-        <v>18652</v>
+        <v>18777</v>
       </c>
       <c r="H10" s="9">
-        <v>1036</v>
+        <v>1042</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>766395</v>
+        <v>771463</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2297,28 +2291,28 @@
         <v>70</v>
       </c>
       <c r="C11" s="9">
-        <v>953668</v>
+        <v>960431</v>
       </c>
       <c r="D11" s="9">
-        <v>19496</v>
+        <v>19605</v>
       </c>
       <c r="E11" s="9">
-        <v>11455</v>
+        <v>11529</v>
       </c>
       <c r="F11" s="9">
-        <v>43280</v>
+        <v>43509</v>
       </c>
       <c r="G11" s="9">
-        <v>7832</v>
+        <v>7902</v>
       </c>
       <c r="H11" s="9">
-        <v>1670</v>
+        <v>1682</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>973164</v>
+        <v>980036</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2329,28 +2323,28 @@
         <v>77</v>
       </c>
       <c r="C12" s="9">
-        <v>461578</v>
+        <v>465302</v>
       </c>
       <c r="D12" s="9">
-        <v>5983</v>
+        <v>6016</v>
       </c>
       <c r="E12" s="9">
-        <v>5576</v>
+        <v>5611</v>
       </c>
       <c r="F12" s="9">
-        <v>26487</v>
+        <v>26682</v>
       </c>
       <c r="G12" s="9">
-        <v>1888</v>
+        <v>1901</v>
       </c>
       <c r="H12" s="9">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>467561</v>
+        <v>471318</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2361,28 +2355,28 @@
         <v>85</v>
       </c>
       <c r="C13" s="9">
-        <v>327888</v>
+        <v>330008</v>
       </c>
       <c r="D13" s="9">
-        <v>4210</v>
+        <v>4226</v>
       </c>
       <c r="E13" s="9">
-        <v>3727</v>
+        <v>3741</v>
       </c>
       <c r="F13" s="9">
-        <v>23663</v>
+        <v>23800</v>
       </c>
       <c r="G13" s="9">
-        <v>1295</v>
+        <v>1306</v>
       </c>
       <c r="H13" s="9">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>332098</v>
+        <v>334234</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2393,28 +2387,28 @@
         <v>91</v>
       </c>
       <c r="C14" s="9">
-        <v>268164</v>
+        <v>271273</v>
       </c>
       <c r="D14" s="9">
-        <v>7714</v>
+        <v>7772</v>
       </c>
       <c r="E14" s="9">
-        <v>2995</v>
+        <v>3027</v>
       </c>
       <c r="F14" s="9">
-        <v>18250</v>
+        <v>18477</v>
       </c>
       <c r="G14" s="9">
-        <v>1838</v>
+        <v>1855</v>
       </c>
       <c r="H14" s="9">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>275878</v>
+        <v>279045</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2425,28 +2419,28 @@
         <v>97</v>
       </c>
       <c r="C15" s="9">
-        <v>379236</v>
+        <v>381304</v>
       </c>
       <c r="D15" s="9">
-        <v>7390</v>
+        <v>7442</v>
       </c>
       <c r="E15" s="9">
-        <v>6199</v>
+        <v>6233</v>
       </c>
       <c r="F15" s="9">
-        <v>25805</v>
+        <v>25947</v>
       </c>
       <c r="G15" s="9">
-        <v>3717</v>
+        <v>3732</v>
       </c>
       <c r="H15" s="9">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>386626</v>
+        <v>388746</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2457,28 +2451,28 @@
         <v>104</v>
       </c>
       <c r="C16" s="9">
-        <v>312362</v>
+        <v>314351</v>
       </c>
       <c r="D16" s="9">
-        <v>4562</v>
+        <v>4576</v>
       </c>
       <c r="E16" s="9">
-        <v>2697</v>
+        <v>2723</v>
       </c>
       <c r="F16" s="9">
-        <v>18197</v>
+        <v>18328</v>
       </c>
       <c r="G16" s="9">
-        <v>3649</v>
+        <v>3665</v>
       </c>
       <c r="H16" s="9">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>316924</v>
+        <v>318927</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2489,28 +2483,28 @@
         <v>111</v>
       </c>
       <c r="C17" s="9">
-        <v>194633</v>
+        <v>195292</v>
       </c>
       <c r="D17" s="9">
-        <v>4781</v>
+        <v>4804</v>
       </c>
       <c r="E17" s="9">
-        <v>2160</v>
+        <v>2165</v>
       </c>
       <c r="F17" s="9">
-        <v>10160</v>
+        <v>10193</v>
       </c>
       <c r="G17" s="9">
-        <v>1698</v>
+        <v>1702</v>
       </c>
       <c r="H17" s="9">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="I17" s="9">
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>199414</v>
+        <v>200096</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2521,28 +2515,28 @@
         <v>118</v>
       </c>
       <c r="C18" s="9">
-        <v>240308</v>
+        <v>241678</v>
       </c>
       <c r="D18" s="9">
-        <v>5281</v>
+        <v>5306</v>
       </c>
       <c r="E18" s="9">
-        <v>2565</v>
+        <v>2576</v>
       </c>
       <c r="F18" s="9">
-        <v>13792</v>
+        <v>13866</v>
       </c>
       <c r="G18" s="9">
-        <v>2321</v>
+        <v>2328</v>
       </c>
       <c r="H18" s="9">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>245589</v>
+        <v>246984</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2553,28 +2547,28 @@
         <v>125</v>
       </c>
       <c r="C19" s="9">
-        <v>134806</v>
+        <v>135234</v>
       </c>
       <c r="D19" s="9">
-        <v>1730</v>
+        <v>1736</v>
       </c>
       <c r="E19" s="9">
-        <v>1027</v>
+        <v>1032</v>
       </c>
       <c r="F19" s="9">
-        <v>10274</v>
+        <v>10305</v>
       </c>
       <c r="G19" s="9">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H19" s="9">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="I19" s="9">
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>136536</v>
+        <v>136970</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2585,92 +2579,92 @@
         <v>131</v>
       </c>
       <c r="C20" s="9">
-        <v>538707</v>
+        <v>544484</v>
       </c>
       <c r="D20" s="9">
-        <v>6612</v>
+        <v>6673</v>
       </c>
       <c r="E20" s="9">
-        <v>3213</v>
+        <v>3257</v>
       </c>
       <c r="F20" s="9">
-        <v>15554</v>
+        <v>15708</v>
       </c>
       <c r="G20" s="9">
-        <v>949</v>
+        <v>956</v>
       </c>
       <c r="H20" s="9">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>545319</v>
+        <v>551157</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>138</v>
-      </c>
       <c r="C21" s="9">
-        <v>111993</v>
+        <v>112894</v>
       </c>
       <c r="D21" s="9">
-        <v>1060</v>
+        <v>1070</v>
       </c>
       <c r="E21" s="9">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="F21" s="9">
-        <v>4822</v>
+        <v>4863</v>
       </c>
       <c r="G21" s="9">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="H21" s="9">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>113053</v>
+        <v>113964</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>144</v>
-      </c>
       <c r="C22" s="12">
-        <v>6061355</v>
+        <v>6103234</v>
       </c>
       <c r="D22" s="12">
-        <v>104542</v>
+        <v>105126</v>
       </c>
       <c r="E22" s="12">
-        <v>65706</v>
+        <v>66118</v>
       </c>
       <c r="F22" s="12">
-        <v>328895</v>
+        <v>330952</v>
       </c>
       <c r="G22" s="12">
-        <v>53361</v>
+        <v>53694</v>
       </c>
       <c r="H22" s="12">
-        <v>9068</v>
+        <v>9116</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6165897</v>
+        <v>6208360</v>
       </c>
     </row>
   </sheetData>
@@ -2697,7 +2691,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2721,7 +2715,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2730,13 +2724,13 @@
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2764,13 +2758,13 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>963</v>
+        <v>967</v>
       </c>
       <c r="D7" s="6">
         <v>69</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2787,7 +2781,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2804,7 +2798,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2821,7 +2815,7 @@
         <v>4</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2838,7 +2832,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2849,13 +2843,13 @@
         <v>70</v>
       </c>
       <c r="C12" s="9">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D12" s="9">
         <v>4</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2866,13 +2860,13 @@
         <v>77</v>
       </c>
       <c r="C13" s="9">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D13" s="9">
         <v>2</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2883,13 +2877,13 @@
         <v>85</v>
       </c>
       <c r="C14" s="9">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2906,7 +2900,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2917,13 +2911,13 @@
         <v>97</v>
       </c>
       <c r="C16" s="9">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D16" s="9">
         <v>36</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2934,13 +2928,13 @@
         <v>104</v>
       </c>
       <c r="C17" s="9">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D17" s="9">
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2957,7 +2951,7 @@
         <v>2</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2968,13 +2962,13 @@
         <v>118</v>
       </c>
       <c r="C19" s="9">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D19" s="9">
         <v>5</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2991,7 +2985,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3008,15 +3002,15 @@
         <v>2</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>138</v>
       </c>
       <c r="C22" s="9">
         <v>60</v>
@@ -3025,24 +3019,24 @@
         <v>12</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>144</v>
-      </c>
       <c r="C23" s="12">
-        <v>963</v>
+        <v>967</v>
       </c>
       <c r="D23" s="12">
         <v>69</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 18/08/2026 20:53:33,45
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="170">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 18 Agu 2026, 06.16 | Dicetak: 18 Agu 2026, 07.20</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 18 Agu 2026, 18.16 | Dicetak: 18 Agu 2026, 20.52</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,22 +123,22 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>63,27</t>
-  </si>
-  <si>
-    <t>1,75</t>
+    <t>63,76</t>
+  </si>
+  <si>
+    <t>1,76</t>
   </si>
   <si>
     <t>0,05</t>
   </si>
   <si>
-    <t>20,5</t>
+    <t>20,64</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>74,42</t>
+    <t>75</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>78,52</t>
+    <t>78,68</t>
   </si>
   <si>
     <t>1,12</t>
@@ -156,13 +156,13 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>18,08</t>
+    <t>18,16</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>91,33</t>
+    <t>91,5</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>66,09</t>
-  </si>
-  <si>
-    <t>0,96</t>
-  </si>
-  <si>
-    <t>16,18</t>
+    <t>66,62</t>
+  </si>
+  <si>
+    <t>0,97</t>
+  </si>
+  <si>
+    <t>16,41</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>80,46</t>
+    <t>81,1</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,16 +192,16 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>57,76</t>
-  </si>
-  <si>
-    <t>1,16</t>
-  </si>
-  <si>
-    <t>19,05</t>
-  </si>
-  <si>
-    <t>69,53</t>
+    <t>58,36</t>
+  </si>
+  <si>
+    <t>1,17</t>
+  </si>
+  <si>
+    <t>19,19</t>
+  </si>
+  <si>
+    <t>70,24</t>
   </si>
   <si>
     <t>1804</t>
@@ -210,16 +210,16 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>65,01</t>
-  </si>
-  <si>
-    <t>1,85</t>
-  </si>
-  <si>
-    <t>17,89</t>
-  </si>
-  <si>
-    <t>73,69</t>
+    <t>65,53</t>
+  </si>
+  <si>
+    <t>1,86</t>
+  </si>
+  <si>
+    <t>17,98</t>
+  </si>
+  <si>
+    <t>74,27</t>
   </si>
   <si>
     <t>1805</t>
@@ -228,19 +228,16 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>64,51</t>
-  </si>
-  <si>
-    <t>2,66</t>
-  </si>
-  <si>
-    <t>17,87</t>
+    <t>65,06</t>
+  </si>
+  <si>
+    <t>2,67</t>
   </si>
   <si>
     <t>0,22</t>
   </si>
   <si>
-    <t>73,11</t>
+    <t>73,72</t>
   </si>
   <si>
     <t>1806</t>
@@ -249,7 +246,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>64,23</t>
+    <t>64,72</t>
   </si>
   <si>
     <t>1,93</t>
@@ -258,13 +255,13 @@
     <t>0,02</t>
   </si>
   <si>
-    <t>25,12</t>
+    <t>25,26</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>75,42</t>
+    <t>76</t>
   </si>
   <si>
     <t>1807</t>
@@ -273,16 +270,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>64,3</t>
+    <t>64,97</t>
   </si>
   <si>
     <t>1,66</t>
   </si>
   <si>
-    <t>18,15</t>
-  </si>
-  <si>
-    <t>75,3</t>
+    <t>18,26</t>
+  </si>
+  <si>
+    <t>76,1</t>
   </si>
   <si>
     <t>1808</t>
@@ -291,16 +288,16 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>56,58</t>
+    <t>57,22</t>
   </si>
   <si>
     <t>2,22</t>
   </si>
   <si>
-    <t>25,07</t>
-  </si>
-  <si>
-    <t>67,82</t>
+    <t>25,23</t>
+  </si>
+  <si>
+    <t>68,6</t>
   </si>
   <si>
     <t>1809</t>
@@ -309,19 +306,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>69,93</t>
-  </si>
-  <si>
-    <t>2,94</t>
-  </si>
-  <si>
-    <t>20,6</t>
+    <t>70,28</t>
+  </si>
+  <si>
+    <t>2,96</t>
+  </si>
+  <si>
+    <t>20,78</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>83,19</t>
+    <t>83,63</t>
   </si>
   <si>
     <t>1810</t>
@@ -330,19 +327,19 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>69,49</t>
+    <t>70,01</t>
   </si>
   <si>
     <t>1,43</t>
   </si>
   <si>
-    <t>15,61</t>
+    <t>15,73</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>78,37</t>
+    <t>78,95</t>
   </si>
   <si>
     <t>1811</t>
@@ -351,166 +348,181 @@
     <t>MESUJI</t>
   </si>
   <si>
+    <t>73,92</t>
+  </si>
+  <si>
     <t>1,58</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
+    <t>25,02</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>89,98</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>72,52</t>
+  </si>
+  <si>
+    <t>2,42</t>
+  </si>
+  <si>
+    <t>23,02</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>85,02</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>80,83</t>
+  </si>
+  <si>
+    <t>0,83</t>
+  </si>
+  <si>
+    <t>17,54</t>
+  </si>
+  <si>
+    <t>98,33</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>46,92</t>
+  </si>
+  <si>
+    <t>0,84</t>
+  </si>
+  <si>
+    <t>29,84</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>59,97</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>61,96</t>
+  </si>
+  <si>
+    <t>1,34</t>
+  </si>
+  <si>
+    <t>21,32</t>
+  </si>
+  <si>
+    <t>70,99</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>PROGRES PEMUTAKHIRAN KELUARGA - ANGGOTA KELUARGA</t>
+  </si>
+  <si>
+    <t>Tinggal Bersama Keluarga</t>
+  </si>
+  <si>
+    <t>Anggota Keluarga Baru</t>
+  </si>
+  <si>
+    <t>Pindah Dalam Negeri (DN)</t>
+  </si>
+  <si>
+    <t>Pindah Luar Negeri (LN)</t>
+  </si>
+  <si>
+    <t>Anggota Keluarga Khusus</t>
+  </si>
+  <si>
+    <t>Total Anggota Keluarga ((3) + (4))</t>
+  </si>
+  <si>
+    <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA KHUSUS</t>
+  </si>
+  <si>
+    <t>PENDATAAN K1</t>
+  </si>
+  <si>
+    <t>Jumlah Bangunan Keluarga Khusus Hasil Pendataan PPL</t>
+  </si>
+  <si>
+    <t>Jumlah Bangunan Keluarga Khusus Didata</t>
+  </si>
+  <si>
+    <t>Persentase Bangunan Keluarga Khusus Didata</t>
+  </si>
+  <si>
+    <t>8,04</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>4,17</t>
+  </si>
+  <si>
+    <t>4,3</t>
+  </si>
+  <si>
+    <t>2,38</t>
+  </si>
+  <si>
+    <t>2,48</t>
+  </si>
+  <si>
+    <t>9,09</t>
+  </si>
+  <si>
     <t>25</t>
   </si>
   <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>89,7</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>72,14</t>
-  </si>
-  <si>
-    <t>2,42</t>
-  </si>
-  <si>
-    <t>22,98</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>84,6</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>80,64</t>
-  </si>
-  <si>
-    <t>0,83</t>
-  </si>
-  <si>
-    <t>17,53</t>
-  </si>
-  <si>
-    <t>98,11</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>46,53</t>
-  </si>
-  <si>
-    <t>29,62</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>59,49</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>61,43</t>
-  </si>
-  <si>
-    <t>1,33</t>
-  </si>
-  <si>
-    <t>21,15</t>
-  </si>
-  <si>
-    <t>70,39</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>PROGRES PEMUTAKHIRAN KELUARGA - ANGGOTA KELUARGA</t>
-  </si>
-  <si>
-    <t>Tinggal Bersama Keluarga</t>
-  </si>
-  <si>
-    <t>Anggota Keluarga Baru</t>
-  </si>
-  <si>
-    <t>Pindah Dalam Negeri (DN)</t>
-  </si>
-  <si>
-    <t>Pindah Luar Negeri (LN)</t>
-  </si>
-  <si>
-    <t>Anggota Keluarga Khusus</t>
-  </si>
-  <si>
-    <t>Total Anggota Keluarga ((3) + (4))</t>
-  </si>
-  <si>
-    <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA KHUSUS</t>
-  </si>
-  <si>
-    <t>PENDATAAN K1</t>
-  </si>
-  <si>
-    <t>Jumlah Bangunan Keluarga Khusus Hasil Pendataan PPL</t>
-  </si>
-  <si>
-    <t>Jumlah Bangunan Keluarga Khusus Didata</t>
-  </si>
-  <si>
-    <t>Persentase Bangunan Keluarga Khusus Didata</t>
-  </si>
-  <si>
-    <t>7,14</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>4,35</t>
-  </si>
-  <si>
-    <t>2,53</t>
-  </si>
-  <si>
-    <t>9,52</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>2,78</t>
-  </si>
-  <si>
-    <t>7,58</t>
-  </si>
-  <si>
-    <t>1,71</t>
-  </si>
-  <si>
-    <t>20</t>
+    <t>2,7</t>
+  </si>
+  <si>
+    <t>16,67</t>
+  </si>
+  <si>
+    <t>14,49</t>
+  </si>
+  <si>
+    <t>1,68</t>
+  </si>
+  <si>
+    <t>19,67</t>
   </si>
 </sst>
 </file>
@@ -1171,28 +1183,28 @@
         <v>2730932</v>
       </c>
       <c r="D6" s="6">
-        <v>1727736</v>
+        <v>1741282</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>304756</v>
+        <v>307032</v>
       </c>
       <c r="G6" s="6">
-        <v>47884</v>
+        <v>48073</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1383</v>
+        <v>1393</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>559929</v>
+        <v>563599</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1204,7 +1216,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2032492</v>
+        <v>2048314</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1221,28 +1233,28 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>66855</v>
+        <v>66994</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10905</v>
+        <v>10912</v>
       </c>
       <c r="G7" s="9">
-        <v>954</v>
+        <v>956</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
       </c>
       <c r="I7" s="9">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15391</v>
+        <v>15466</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1254,7 +1266,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>77760</v>
+        <v>77906</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1271,28 +1283,28 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>114306</v>
+        <v>115216</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>24849</v>
+        <v>25055</v>
       </c>
       <c r="G8" s="9">
-        <v>1661</v>
+        <v>1671</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="9">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>27977</v>
+        <v>28382</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1304,7 +1316,7 @@
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>139155</v>
+        <v>140271</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1321,28 +1333,28 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>197976</v>
+        <v>200008</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>40323</v>
+        <v>40723</v>
       </c>
       <c r="G9" s="9">
-        <v>3986</v>
+        <v>4006</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>65281</v>
+        <v>65773</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
@@ -1354,7 +1366,7 @@
         <v>48</v>
       </c>
       <c r="O9" s="9">
-        <v>238299</v>
+        <v>240731</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>62</v>
@@ -1371,28 +1383,28 @@
         <v>362838</v>
       </c>
       <c r="D10" s="9">
-        <v>235868</v>
+        <v>237760</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>65</v>
       </c>
       <c r="F10" s="9">
-        <v>31490</v>
+        <v>31724</v>
       </c>
       <c r="G10" s="9">
-        <v>6715</v>
+        <v>6735</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I10" s="9">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>64896</v>
+        <v>65242</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>67</v>
@@ -1404,7 +1416,7 @@
         <v>55</v>
       </c>
       <c r="O10" s="9">
-        <v>267358</v>
+        <v>269484</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>68</v>
@@ -1421,119 +1433,119 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>289999</v>
+        <v>292495</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="9">
-        <v>38672</v>
+        <v>38946</v>
       </c>
       <c r="G11" s="9">
-        <v>11937</v>
+        <v>11988</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>72</v>
       </c>
       <c r="I11" s="9">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>80340</v>
+        <v>80828</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M11" s="9">
         <v>988</v>
       </c>
       <c r="N11" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="O11" s="9">
+        <v>331441</v>
+      </c>
+      <c r="P11" s="10" t="s">
         <v>74</v>
-      </c>
-      <c r="O11" s="9">
-        <v>328671</v>
-      </c>
-      <c r="P11" s="10" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>76</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>77</v>
       </c>
       <c r="C12" s="9">
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>128065</v>
+        <v>129043</v>
       </c>
       <c r="E12" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F12" s="9">
+        <v>22489</v>
+      </c>
+      <c r="G12" s="9">
+        <v>3848</v>
+      </c>
+      <c r="H12" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="9">
-        <v>22315</v>
-      </c>
-      <c r="G12" s="9">
-        <v>3840</v>
-      </c>
-      <c r="H12" s="10" t="s">
+      <c r="I12" s="9">
+        <v>45</v>
+      </c>
+      <c r="J12" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="I12" s="9">
-        <v>44</v>
-      </c>
-      <c r="J12" s="10" t="s">
+      <c r="K12" s="9">
+        <v>50374</v>
+      </c>
+      <c r="L12" s="10" t="s">
         <v>80</v>
-      </c>
-      <c r="K12" s="9">
-        <v>50091</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>81</v>
       </c>
       <c r="M12" s="9">
         <v>180</v>
       </c>
       <c r="N12" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="O12" s="9">
+        <v>151532</v>
+      </c>
+      <c r="P12" s="10" t="s">
         <v>82</v>
-      </c>
-      <c r="O12" s="9">
-        <v>150380</v>
-      </c>
-      <c r="P12" s="10" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>84</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>85</v>
       </c>
       <c r="C13" s="9">
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>93935</v>
+        <v>94912</v>
       </c>
       <c r="E13" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" s="9">
+        <v>16261</v>
+      </c>
+      <c r="G13" s="9">
+        <v>2424</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>86</v>
-      </c>
-      <c r="F13" s="9">
-        <v>16070</v>
-      </c>
-      <c r="G13" s="9">
-        <v>2419</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>87</v>
       </c>
       <c r="I13" s="9">
         <v>78</v>
@@ -1542,10 +1554,10 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>26523</v>
+        <v>26675</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M13" s="9">
         <v>124</v>
@@ -1554,180 +1566,180 @@
         <v>48</v>
       </c>
       <c r="O13" s="9">
-        <v>110005</v>
+        <v>111173</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>90</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>91</v>
       </c>
       <c r="C14" s="9">
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>76524</v>
+        <v>77393</v>
       </c>
       <c r="E14" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F14" s="9">
+        <v>15398</v>
+      </c>
+      <c r="G14" s="9">
+        <v>3008</v>
+      </c>
+      <c r="H14" s="10" t="s">
         <v>92</v>
-      </c>
-      <c r="F14" s="9">
-        <v>15202</v>
-      </c>
-      <c r="G14" s="9">
-        <v>2996</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>93</v>
       </c>
       <c r="I14" s="9">
         <v>32</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K14" s="9">
-        <v>33904</v>
+        <v>34123</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M14" s="9">
         <v>21</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O14" s="9">
-        <v>91726</v>
+        <v>92791</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>96</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>97</v>
       </c>
       <c r="C15" s="9">
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>106397</v>
+        <v>106934</v>
       </c>
       <c r="E15" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F15" s="9">
+        <v>20319</v>
+      </c>
+      <c r="G15" s="9">
+        <v>4498</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="F15" s="9">
-        <v>20188</v>
-      </c>
-      <c r="G15" s="9">
-        <v>4475</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>99</v>
-      </c>
       <c r="I15" s="9">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J15" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>31348</v>
+        <v>31620</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M15" s="9">
         <v>180</v>
       </c>
       <c r="N15" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="O15" s="9">
+        <v>127253</v>
+      </c>
+      <c r="P15" s="10" t="s">
         <v>101</v>
-      </c>
-      <c r="O15" s="9">
-        <v>126585</v>
-      </c>
-      <c r="P15" s="10" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>104</v>
       </c>
       <c r="C16" s="9">
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>94327</v>
+        <v>95036</v>
       </c>
       <c r="E16" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F16" s="9">
+        <v>12137</v>
+      </c>
+      <c r="G16" s="9">
+        <v>1947</v>
+      </c>
+      <c r="H16" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="F16" s="9">
-        <v>12057</v>
-      </c>
-      <c r="G16" s="9">
-        <v>1941</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>106</v>
-      </c>
       <c r="I16" s="9">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>21192</v>
+        <v>21358</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M16" s="9">
         <v>83</v>
       </c>
       <c r="N16" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="O16" s="9">
+        <v>107173</v>
+      </c>
+      <c r="P16" s="10" t="s">
         <v>108</v>
-      </c>
-      <c r="O16" s="9">
-        <v>106384</v>
-      </c>
-      <c r="P16" s="10" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>111</v>
       </c>
       <c r="C17" s="9">
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55355</v>
+        <v>55525</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>68</v>
+        <v>111</v>
       </c>
       <c r="F17" s="9">
-        <v>12022</v>
+        <v>12065</v>
       </c>
       <c r="G17" s="9">
         <v>1187</v>
@@ -1742,7 +1754,7 @@
         <v>113</v>
       </c>
       <c r="K17" s="9">
-        <v>18782</v>
+        <v>18794</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>114</v>
@@ -1754,7 +1766,7 @@
         <v>115</v>
       </c>
       <c r="O17" s="9">
-        <v>67377</v>
+        <v>67590</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>116</v>
@@ -1771,16 +1783,16 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>71537</v>
+        <v>71915</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>119</v>
       </c>
       <c r="F18" s="9">
-        <v>12356</v>
+        <v>12403</v>
       </c>
       <c r="G18" s="9">
-        <v>2400</v>
+        <v>2403</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>120</v>
@@ -1792,7 +1804,7 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22785</v>
+        <v>22833</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>121</v>
@@ -1804,7 +1816,7 @@
         <v>122</v>
       </c>
       <c r="O18" s="9">
-        <v>83893</v>
+        <v>84318</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>123</v>
@@ -1821,13 +1833,13 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33685</v>
+        <v>33763</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>126</v>
       </c>
       <c r="F19" s="9">
-        <v>7299</v>
+        <v>7311</v>
       </c>
       <c r="G19" s="9">
         <v>347</v>
@@ -1836,13 +1848,13 @@
         <v>127</v>
       </c>
       <c r="I19" s="9">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>55</v>
+        <v>107</v>
       </c>
       <c r="K19" s="9">
-        <v>7322</v>
+        <v>7328</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>128</v>
@@ -1854,7 +1866,7 @@
         <v>55</v>
       </c>
       <c r="O19" s="9">
-        <v>40984</v>
+        <v>41074</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>129</v>
@@ -1871,128 +1883,128 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>130038</v>
+        <v>131136</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>132</v>
       </c>
       <c r="F20" s="9">
-        <v>36214</v>
+        <v>36458</v>
       </c>
       <c r="G20" s="9">
-        <v>2312</v>
+        <v>2338</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I20" s="9">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>82783</v>
+        <v>83393</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M20" s="9">
         <v>91</v>
       </c>
       <c r="N20" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O20" s="9">
-        <v>166252</v>
+        <v>167594</v>
       </c>
       <c r="P20" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C21" s="9">
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>32869</v>
+        <v>33152</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F21" s="9">
-        <v>4794</v>
+        <v>4831</v>
       </c>
       <c r="G21" s="9">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I21" s="9">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K21" s="9">
-        <v>11314</v>
+        <v>11410</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M21" s="9">
         <v>11</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O21" s="9">
-        <v>37663</v>
+        <v>37983</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C22" s="12">
         <v>2730932</v>
       </c>
       <c r="D22" s="12">
-        <v>1727736</v>
+        <v>1741282</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>304756</v>
+        <v>307032</v>
       </c>
       <c r="G22" s="12">
-        <v>47884</v>
+        <v>48073</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1383</v>
+        <v>1393</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>559929</v>
+        <v>563599</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2004,7 +2016,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2032492</v>
+        <v>2048314</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2033,7 +2045,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2067,28 +2079,28 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2131,28 +2143,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6103234</v>
+        <v>6151483</v>
       </c>
       <c r="D6" s="6">
-        <v>105126</v>
+        <v>105847</v>
       </c>
       <c r="E6" s="6">
-        <v>66118</v>
+        <v>66621</v>
       </c>
       <c r="F6" s="6">
-        <v>330952</v>
+        <v>333295</v>
       </c>
       <c r="G6" s="6">
-        <v>53694</v>
+        <v>54087</v>
       </c>
       <c r="H6" s="6">
-        <v>9116</v>
+        <v>9174</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6208360</v>
+        <v>6257330</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2163,28 +2175,28 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>243969</v>
+        <v>244430</v>
       </c>
       <c r="D7" s="9">
-        <v>2859</v>
+        <v>2868</v>
       </c>
       <c r="E7" s="9">
-        <v>2079</v>
+        <v>2082</v>
       </c>
       <c r="F7" s="9">
-        <v>12930</v>
+        <v>12954</v>
       </c>
       <c r="G7" s="9">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="H7" s="9">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="I7" s="9">
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>246828</v>
+        <v>247298</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2195,28 +2207,28 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>425093</v>
+        <v>428443</v>
       </c>
       <c r="D8" s="9">
-        <v>5630</v>
+        <v>5685</v>
       </c>
       <c r="E8" s="9">
-        <v>4185</v>
+        <v>4222</v>
       </c>
       <c r="F8" s="9">
-        <v>32643</v>
+        <v>32875</v>
       </c>
       <c r="G8" s="9">
-        <v>3878</v>
+        <v>3902</v>
       </c>
       <c r="H8" s="9">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="I8" s="9">
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>430723</v>
+        <v>434128</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2227,28 +2239,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>725218</v>
+        <v>732700</v>
       </c>
       <c r="D9" s="9">
-        <v>12651</v>
+        <v>12787</v>
       </c>
       <c r="E9" s="9">
-        <v>8254</v>
+        <v>8329</v>
       </c>
       <c r="F9" s="9">
-        <v>36179</v>
+        <v>36475</v>
       </c>
       <c r="G9" s="9">
-        <v>4440</v>
+        <v>4478</v>
       </c>
       <c r="H9" s="9">
-        <v>971</v>
+        <v>979</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>737869</v>
+        <v>745487</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2259,28 +2271,28 @@
         <v>64</v>
       </c>
       <c r="C10" s="9">
-        <v>756703</v>
+        <v>762762</v>
       </c>
       <c r="D10" s="9">
-        <v>14760</v>
+        <v>14864</v>
       </c>
       <c r="E10" s="9">
-        <v>8896</v>
+        <v>8971</v>
       </c>
       <c r="F10" s="9">
-        <v>37522</v>
+        <v>37808</v>
       </c>
       <c r="G10" s="9">
-        <v>18777</v>
+        <v>18936</v>
       </c>
       <c r="H10" s="9">
-        <v>1042</v>
+        <v>1049</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>771463</v>
+        <v>777626</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2291,220 +2303,220 @@
         <v>70</v>
       </c>
       <c r="C11" s="9">
-        <v>960431</v>
+        <v>968701</v>
       </c>
       <c r="D11" s="9">
-        <v>19605</v>
+        <v>19737</v>
       </c>
       <c r="E11" s="9">
-        <v>11529</v>
+        <v>11617</v>
       </c>
       <c r="F11" s="9">
-        <v>43509</v>
+        <v>43828</v>
       </c>
       <c r="G11" s="9">
-        <v>7902</v>
+        <v>7969</v>
       </c>
       <c r="H11" s="9">
-        <v>1682</v>
+        <v>1686</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>980036</v>
+        <v>988438</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>77</v>
-      </c>
       <c r="C12" s="9">
-        <v>465302</v>
+        <v>468989</v>
       </c>
       <c r="D12" s="9">
-        <v>6016</v>
+        <v>6045</v>
       </c>
       <c r="E12" s="9">
-        <v>5611</v>
+        <v>5652</v>
       </c>
       <c r="F12" s="9">
-        <v>26682</v>
+        <v>26902</v>
       </c>
       <c r="G12" s="9">
-        <v>1901</v>
+        <v>1919</v>
       </c>
       <c r="H12" s="9">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>471318</v>
+        <v>475034</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>85</v>
-      </c>
       <c r="C13" s="9">
-        <v>330008</v>
+        <v>333601</v>
       </c>
       <c r="D13" s="9">
-        <v>4226</v>
+        <v>4258</v>
       </c>
       <c r="E13" s="9">
-        <v>3741</v>
+        <v>3774</v>
       </c>
       <c r="F13" s="9">
-        <v>23800</v>
+        <v>24054</v>
       </c>
       <c r="G13" s="9">
-        <v>1306</v>
+        <v>1321</v>
       </c>
       <c r="H13" s="9">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>334234</v>
+        <v>337859</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>91</v>
-      </c>
       <c r="C14" s="9">
-        <v>271273</v>
+        <v>274547</v>
       </c>
       <c r="D14" s="9">
-        <v>7772</v>
+        <v>7844</v>
       </c>
       <c r="E14" s="9">
-        <v>3027</v>
+        <v>3051</v>
       </c>
       <c r="F14" s="9">
-        <v>18477</v>
+        <v>18677</v>
       </c>
       <c r="G14" s="9">
-        <v>1855</v>
+        <v>1865</v>
       </c>
       <c r="H14" s="9">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>279045</v>
+        <v>282391</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>97</v>
-      </c>
       <c r="C15" s="9">
-        <v>381304</v>
+        <v>383343</v>
       </c>
       <c r="D15" s="9">
-        <v>7442</v>
+        <v>7486</v>
       </c>
       <c r="E15" s="9">
-        <v>6233</v>
+        <v>6275</v>
       </c>
       <c r="F15" s="9">
-        <v>25947</v>
+        <v>26065</v>
       </c>
       <c r="G15" s="9">
-        <v>3732</v>
+        <v>3746</v>
       </c>
       <c r="H15" s="9">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>388746</v>
+        <v>390829</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>104</v>
-      </c>
       <c r="C16" s="9">
-        <v>314351</v>
+        <v>316690</v>
       </c>
       <c r="D16" s="9">
-        <v>4576</v>
+        <v>4606</v>
       </c>
       <c r="E16" s="9">
-        <v>2723</v>
+        <v>2747</v>
       </c>
       <c r="F16" s="9">
-        <v>18328</v>
+        <v>18457</v>
       </c>
       <c r="G16" s="9">
-        <v>3665</v>
+        <v>3690</v>
       </c>
       <c r="H16" s="9">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>318927</v>
+        <v>321296</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>111</v>
-      </c>
       <c r="C17" s="9">
-        <v>195292</v>
+        <v>195941</v>
       </c>
       <c r="D17" s="9">
-        <v>4804</v>
+        <v>4813</v>
       </c>
       <c r="E17" s="9">
-        <v>2165</v>
+        <v>2173</v>
       </c>
       <c r="F17" s="9">
-        <v>10193</v>
+        <v>10242</v>
       </c>
       <c r="G17" s="9">
-        <v>1702</v>
+        <v>1705</v>
       </c>
       <c r="H17" s="9">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="I17" s="9">
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>200096</v>
+        <v>200754</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2515,28 +2527,28 @@
         <v>118</v>
       </c>
       <c r="C18" s="9">
-        <v>241678</v>
+        <v>242997</v>
       </c>
       <c r="D18" s="9">
-        <v>5306</v>
+        <v>5330</v>
       </c>
       <c r="E18" s="9">
-        <v>2576</v>
+        <v>2592</v>
       </c>
       <c r="F18" s="9">
-        <v>13866</v>
+        <v>13924</v>
       </c>
       <c r="G18" s="9">
-        <v>2328</v>
+        <v>2338</v>
       </c>
       <c r="H18" s="9">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>246984</v>
+        <v>248327</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2547,16 +2559,16 @@
         <v>125</v>
       </c>
       <c r="C19" s="9">
-        <v>135234</v>
+        <v>135529</v>
       </c>
       <c r="D19" s="9">
         <v>1736</v>
       </c>
       <c r="E19" s="9">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="F19" s="9">
-        <v>10305</v>
+        <v>10331</v>
       </c>
       <c r="G19" s="9">
         <v>221</v>
@@ -2568,7 +2580,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>136970</v>
+        <v>137265</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2579,92 +2591,92 @@
         <v>131</v>
       </c>
       <c r="C20" s="9">
-        <v>544484</v>
+        <v>548956</v>
       </c>
       <c r="D20" s="9">
-        <v>6673</v>
+        <v>6714</v>
       </c>
       <c r="E20" s="9">
-        <v>3257</v>
+        <v>3286</v>
       </c>
       <c r="F20" s="9">
-        <v>15708</v>
+        <v>15809</v>
       </c>
       <c r="G20" s="9">
-        <v>956</v>
+        <v>964</v>
       </c>
       <c r="H20" s="9">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>551157</v>
+        <v>555670</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C21" s="9">
-        <v>112894</v>
+        <v>113854</v>
       </c>
       <c r="D21" s="9">
-        <v>1070</v>
+        <v>1074</v>
       </c>
       <c r="E21" s="9">
-        <v>810</v>
+        <v>817</v>
       </c>
       <c r="F21" s="9">
-        <v>4863</v>
+        <v>4894</v>
       </c>
       <c r="G21" s="9">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="H21" s="9">
-        <v>697</v>
+        <v>714</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>113964</v>
+        <v>114928</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C22" s="12">
-        <v>6103234</v>
+        <v>6151483</v>
       </c>
       <c r="D22" s="12">
-        <v>105126</v>
+        <v>105847</v>
       </c>
       <c r="E22" s="12">
-        <v>66118</v>
+        <v>66621</v>
       </c>
       <c r="F22" s="12">
-        <v>330952</v>
+        <v>333295</v>
       </c>
       <c r="G22" s="12">
-        <v>53694</v>
+        <v>54087</v>
       </c>
       <c r="H22" s="12">
-        <v>9116</v>
+        <v>9174</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6208360</v>
+        <v>6257330</v>
       </c>
     </row>
   </sheetData>
@@ -2691,7 +2703,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2715,7 +2727,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2724,13 +2736,13 @@
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2758,13 +2770,13 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>967</v>
+        <v>1008</v>
       </c>
       <c r="D7" s="6">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2781,7 +2793,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2792,13 +2804,13 @@
         <v>51</v>
       </c>
       <c r="C9" s="9">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" s="9">
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2809,13 +2821,13 @@
         <v>58</v>
       </c>
       <c r="C10" s="9">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D10" s="9">
         <v>4</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2826,13 +2838,13 @@
         <v>64</v>
       </c>
       <c r="C11" s="9">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="D11" s="9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2843,115 +2855,115 @@
         <v>70</v>
       </c>
       <c r="C12" s="9">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D12" s="9">
         <v>4</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>77</v>
-      </c>
       <c r="C13" s="9">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D13" s="9">
         <v>2</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>85</v>
-      </c>
       <c r="C14" s="9">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>91</v>
-      </c>
       <c r="C15" s="9">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>97</v>
-      </c>
       <c r="C16" s="9">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D16" s="9">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>104</v>
-      </c>
       <c r="C17" s="9">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D17" s="9">
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>111</v>
-      </c>
       <c r="C18" s="9">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D18" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2962,13 +2974,13 @@
         <v>118</v>
       </c>
       <c r="C19" s="9">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D19" s="9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2985,7 +2997,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2996,47 +3008,47 @@
         <v>131</v>
       </c>
       <c r="C21" s="9">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D21" s="9">
         <v>2</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C22" s="9">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D22" s="9">
         <v>12</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C23" s="12">
-        <v>967</v>
+        <v>1008</v>
       </c>
       <c r="D23" s="12">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 19/08/2026 14:13:58,26
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -18,7 +18,7 @@
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 18 Agu 2026, 18.16 | Dicetak: 18 Agu 2026, 20.52</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 19 Agu 2026, 06.16 | Dicetak: 19 Agu 2026, 14.11</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,22 +123,22 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>63,76</t>
-  </si>
-  <si>
-    <t>1,76</t>
+    <t>64,21</t>
+  </si>
+  <si>
+    <t>1,77</t>
   </si>
   <si>
     <t>0,05</t>
   </si>
   <si>
-    <t>20,64</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>75</t>
+    <t>20,74</t>
+  </si>
+  <si>
+    <t>0,11</t>
+  </si>
+  <si>
+    <t>75,53</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>78,68</t>
+    <t>78,92</t>
   </si>
   <si>
     <t>1,12</t>
@@ -156,13 +156,13 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>18,16</t>
+    <t>18,21</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>91,5</t>
+    <t>91,75</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>66,62</t>
+    <t>67,05</t>
   </si>
   <si>
     <t>0,97</t>
   </si>
   <si>
-    <t>16,41</t>
+    <t>16,55</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>81,1</t>
+    <t>81,65</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,16 +192,19 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>58,36</t>
+    <t>58,9</t>
   </si>
   <si>
     <t>1,17</t>
   </si>
   <si>
-    <t>19,19</t>
-  </si>
-  <si>
-    <t>70,24</t>
+    <t>19,29</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>70,89</t>
   </si>
   <si>
     <t>1804</t>
@@ -210,16 +213,16 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>65,53</t>
+    <t>65,92</t>
   </si>
   <si>
     <t>1,86</t>
   </si>
   <si>
-    <t>17,98</t>
-  </si>
-  <si>
-    <t>74,27</t>
+    <t>18,05</t>
+  </si>
+  <si>
+    <t>74,71</t>
   </si>
   <si>
     <t>1805</t>
@@ -228,16 +231,19 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>65,06</t>
-  </si>
-  <si>
-    <t>2,67</t>
-  </si>
-  <si>
-    <t>0,22</t>
-  </si>
-  <si>
-    <t>73,72</t>
+    <t>65,58</t>
+  </si>
+  <si>
+    <t>2,68</t>
+  </si>
+  <si>
+    <t>18,09</t>
+  </si>
+  <si>
+    <t>0,23</t>
+  </si>
+  <si>
+    <t>74,3</t>
   </si>
   <si>
     <t>1806</t>
@@ -246,7 +252,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>64,72</t>
+    <t>65,27</t>
   </si>
   <si>
     <t>1,93</t>
@@ -255,13 +261,10 @@
     <t>0,02</t>
   </si>
   <si>
-    <t>25,26</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>76</t>
+    <t>25,39</t>
+  </si>
+  <si>
+    <t>76,63</t>
   </si>
   <si>
     <t>1807</t>
@@ -270,16 +273,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>64,97</t>
-  </si>
-  <si>
-    <t>1,66</t>
-  </si>
-  <si>
-    <t>18,26</t>
-  </si>
-  <si>
-    <t>76,1</t>
+    <t>65,47</t>
+  </si>
+  <si>
+    <t>1,67</t>
+  </si>
+  <si>
+    <t>18,38</t>
+  </si>
+  <si>
+    <t>76,7</t>
   </si>
   <si>
     <t>1808</t>
@@ -288,16 +291,16 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>57,22</t>
-  </si>
-  <si>
-    <t>2,22</t>
-  </si>
-  <si>
-    <t>25,23</t>
-  </si>
-  <si>
-    <t>68,6</t>
+    <t>57,78</t>
+  </si>
+  <si>
+    <t>2,23</t>
+  </si>
+  <si>
+    <t>25,38</t>
+  </si>
+  <si>
+    <t>69,27</t>
   </si>
   <si>
     <t>1809</t>
@@ -306,19 +309,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>70,28</t>
+    <t>70,7</t>
   </si>
   <si>
     <t>2,96</t>
   </si>
   <si>
-    <t>20,78</t>
+    <t>20,86</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>83,63</t>
+    <t>84,13</t>
   </si>
   <si>
     <t>1810</t>
@@ -327,19 +330,19 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>70,01</t>
-  </si>
-  <si>
-    <t>1,43</t>
-  </si>
-  <si>
-    <t>15,73</t>
+    <t>70,55</t>
+  </si>
+  <si>
+    <t>1,44</t>
+  </si>
+  <si>
+    <t>15,84</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>78,95</t>
+    <t>79,56</t>
   </si>
   <si>
     <t>1811</t>
@@ -348,22 +351,19 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>73,92</t>
+    <t>74,07</t>
   </si>
   <si>
     <t>1,58</t>
   </si>
   <si>
-    <t>0,11</t>
-  </si>
-  <si>
-    <t>25,02</t>
-  </si>
-  <si>
-    <t>0,15</t>
-  </si>
-  <si>
-    <t>89,98</t>
+    <t>25,01</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>90,15</t>
   </si>
   <si>
     <t>1812</t>
@@ -372,19 +372,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>72,52</t>
-  </si>
-  <si>
-    <t>2,42</t>
-  </si>
-  <si>
-    <t>23,02</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>85,02</t>
+    <t>72,85</t>
+  </si>
+  <si>
+    <t>2,43</t>
+  </si>
+  <si>
+    <t>23,05</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>85,41</t>
   </si>
   <si>
     <t>1813</t>
@@ -393,16 +393,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>80,83</t>
+    <t>80,96</t>
   </si>
   <si>
     <t>0,83</t>
   </si>
   <si>
-    <t>17,54</t>
-  </si>
-  <si>
-    <t>98,33</t>
+    <t>17,55</t>
+  </si>
+  <si>
+    <t>98,39</t>
   </si>
   <si>
     <t>1871</t>
@@ -411,19 +411,19 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>46,92</t>
+    <t>47,3</t>
   </si>
   <si>
     <t>0,84</t>
   </si>
   <si>
-    <t>29,84</t>
+    <t>30,03</t>
   </si>
   <si>
     <t>0,03</t>
   </si>
   <si>
-    <t>59,97</t>
+    <t>60,43</t>
   </si>
   <si>
     <t>1872</t>
@@ -432,16 +432,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>61,96</t>
+    <t>62,42</t>
   </si>
   <si>
     <t>1,34</t>
   </si>
   <si>
-    <t>21,32</t>
-  </si>
-  <si>
-    <t>70,99</t>
+    <t>21,41</t>
+  </si>
+  <si>
+    <t>71,52</t>
   </si>
   <si>
     <t/>
@@ -486,28 +486,28 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>8,04</t>
+    <t>7,92</t>
   </si>
   <si>
     <t>0</t>
   </si>
   <si>
-    <t>4,17</t>
-  </si>
-  <si>
-    <t>4,3</t>
-  </si>
-  <si>
-    <t>2,38</t>
+    <t>4</t>
+  </si>
+  <si>
+    <t>4,26</t>
+  </si>
+  <si>
+    <t>2,27</t>
   </si>
   <si>
     <t>2,48</t>
   </si>
   <si>
-    <t>9,09</t>
-  </si>
-  <si>
-    <t>25</t>
+    <t>8,33</t>
+  </si>
+  <si>
+    <t>24,84</t>
   </si>
   <si>
     <t>2,7</t>
@@ -516,10 +516,10 @@
     <t>16,67</t>
   </si>
   <si>
-    <t>14,49</t>
-  </si>
-  <si>
-    <t>1,68</t>
+    <t>14,29</t>
+  </si>
+  <si>
+    <t>1,65</t>
   </si>
   <si>
     <t>19,67</t>
@@ -1183,40 +1183,40 @@
         <v>2730932</v>
       </c>
       <c r="D6" s="6">
-        <v>1741282</v>
+        <v>1753600</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>307032</v>
+        <v>309054</v>
       </c>
       <c r="G6" s="6">
-        <v>48073</v>
+        <v>48214</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1393</v>
+        <v>1400</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>563599</v>
+        <v>566466</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
       </c>
       <c r="M6" s="6">
-        <v>2761</v>
+        <v>2868</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2048314</v>
+        <v>2062654</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1233,28 +1233,28 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>66994</v>
+        <v>67194</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10912</v>
+        <v>10929</v>
       </c>
       <c r="G7" s="9">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
       </c>
       <c r="I7" s="9">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15466</v>
+        <v>15502</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1266,7 +1266,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>77906</v>
+        <v>78123</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1283,16 +1283,16 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>115216</v>
+        <v>115968</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>25055</v>
+        <v>25253</v>
       </c>
       <c r="G8" s="9">
-        <v>1671</v>
+        <v>1679</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
@@ -1304,19 +1304,19 @@
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>28382</v>
+        <v>28622</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
       </c>
       <c r="M8" s="9">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="N8" s="10" t="s">
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>140271</v>
+        <v>141221</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1333,219 +1333,219 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>200008</v>
+        <v>201868</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>40723</v>
+        <v>41085</v>
       </c>
       <c r="G9" s="9">
-        <v>4006</v>
+        <v>4016</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>65773</v>
+        <v>66100</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
       </c>
       <c r="M9" s="9">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="N9" s="10" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="O9" s="9">
-        <v>240731</v>
+        <v>242953</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C10" s="9">
         <v>362838</v>
       </c>
       <c r="D10" s="9">
-        <v>237760</v>
+        <v>239183</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F10" s="9">
-        <v>31724</v>
+        <v>31894</v>
       </c>
       <c r="G10" s="9">
-        <v>6735</v>
+        <v>6750</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I10" s="9">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>65242</v>
+        <v>65475</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M10" s="9">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="N10" s="10" t="s">
         <v>55</v>
       </c>
       <c r="O10" s="9">
-        <v>269484</v>
+        <v>271077</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C11" s="9">
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>292495</v>
+        <v>294820</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F11" s="9">
-        <v>38946</v>
+        <v>39231</v>
       </c>
       <c r="G11" s="9">
-        <v>11988</v>
+        <v>12034</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I11" s="9">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>80828</v>
+        <v>81338</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="M11" s="9">
-        <v>988</v>
+        <v>1033</v>
       </c>
       <c r="N11" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O11" s="9">
-        <v>331441</v>
+        <v>334051</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C12" s="9">
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>129043</v>
+        <v>130137</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F12" s="9">
-        <v>22489</v>
+        <v>22667</v>
       </c>
       <c r="G12" s="9">
-        <v>3848</v>
+        <v>3854</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I12" s="9">
         <v>45</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K12" s="9">
-        <v>50374</v>
+        <v>50636</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="M12" s="9">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="N12" s="10" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="O12" s="9">
-        <v>151532</v>
+        <v>152804</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C13" s="9">
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>94912</v>
+        <v>95649</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F13" s="9">
-        <v>16261</v>
+        <v>16397</v>
       </c>
       <c r="G13" s="9">
-        <v>2424</v>
+        <v>2443</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I13" s="9">
         <v>78</v>
@@ -1554,219 +1554,219 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>26675</v>
+        <v>26852</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="M13" s="9">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="O13" s="9">
-        <v>111173</v>
+        <v>112046</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C14" s="9">
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>77393</v>
+        <v>78153</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F14" s="9">
-        <v>15398</v>
+        <v>15536</v>
       </c>
       <c r="G14" s="9">
-        <v>3008</v>
+        <v>3013</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I14" s="9">
         <v>32</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K14" s="9">
-        <v>34123</v>
+        <v>34326</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M14" s="9">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O14" s="9">
-        <v>92791</v>
+        <v>93689</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C15" s="9">
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>106934</v>
+        <v>107570</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F15" s="9">
-        <v>20319</v>
+        <v>20442</v>
       </c>
       <c r="G15" s="9">
-        <v>4498</v>
+        <v>4506</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I15" s="9">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J15" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>31620</v>
+        <v>31745</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M15" s="9">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="O15" s="9">
-        <v>127253</v>
+        <v>128012</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C16" s="9">
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>95036</v>
+        <v>95763</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F16" s="9">
-        <v>12137</v>
+        <v>12228</v>
       </c>
       <c r="G16" s="9">
-        <v>1947</v>
+        <v>1959</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I16" s="9">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>21358</v>
+        <v>21504</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M16" s="9">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="O16" s="9">
-        <v>107173</v>
+        <v>107991</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C17" s="9">
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55525</v>
+        <v>55634</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F17" s="9">
-        <v>12065</v>
+        <v>12085</v>
       </c>
       <c r="G17" s="9">
         <v>1187</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I17" s="9">
         <v>80</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18794</v>
+        <v>18790</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>114</v>
       </c>
       <c r="M17" s="9">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="N17" s="10" t="s">
         <v>115</v>
       </c>
       <c r="O17" s="9">
-        <v>67590</v>
+        <v>67719</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>116</v>
@@ -1783,16 +1783,16 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>71915</v>
+        <v>72242</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>119</v>
       </c>
       <c r="F18" s="9">
-        <v>12403</v>
+        <v>12457</v>
       </c>
       <c r="G18" s="9">
-        <v>2403</v>
+        <v>2405</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>120</v>
@@ -1804,19 +1804,19 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22833</v>
+        <v>22862</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>121</v>
       </c>
       <c r="M18" s="9">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="N18" s="10" t="s">
         <v>122</v>
       </c>
       <c r="O18" s="9">
-        <v>84318</v>
+        <v>84699</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>123</v>
@@ -1833,13 +1833,13 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33763</v>
+        <v>33818</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>126</v>
       </c>
       <c r="F19" s="9">
-        <v>7311</v>
+        <v>7283</v>
       </c>
       <c r="G19" s="9">
         <v>347</v>
@@ -1851,10 +1851,10 @@
         <v>27</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K19" s="9">
-        <v>7328</v>
+        <v>7331</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>128</v>
@@ -1866,7 +1866,7 @@
         <v>55</v>
       </c>
       <c r="O19" s="9">
-        <v>41074</v>
+        <v>41101</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>129</v>
@@ -1883,16 +1883,16 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>131136</v>
+        <v>132202</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>132</v>
       </c>
       <c r="F20" s="9">
-        <v>36458</v>
+        <v>36698</v>
       </c>
       <c r="G20" s="9">
-        <v>2338</v>
+        <v>2345</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>133</v>
@@ -1904,19 +1904,19 @@
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>83393</v>
+        <v>83927</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>134</v>
       </c>
       <c r="M20" s="9">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="N20" s="10" t="s">
         <v>135</v>
       </c>
       <c r="O20" s="9">
-        <v>167594</v>
+        <v>168900</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>136</v>
@@ -1933,16 +1933,16 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>33152</v>
+        <v>33399</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>139</v>
       </c>
       <c r="F21" s="9">
-        <v>4831</v>
+        <v>4869</v>
       </c>
       <c r="G21" s="9">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>140</v>
@@ -1951,10 +1951,10 @@
         <v>33</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K21" s="9">
-        <v>11410</v>
+        <v>11456</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>141</v>
@@ -1963,10 +1963,10 @@
         <v>11</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="O21" s="9">
-        <v>37983</v>
+        <v>38268</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>142</v>
@@ -1983,40 +1983,40 @@
         <v>2730932</v>
       </c>
       <c r="D22" s="12">
-        <v>1741282</v>
+        <v>1753600</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>307032</v>
+        <v>309054</v>
       </c>
       <c r="G22" s="12">
-        <v>48073</v>
+        <v>48214</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1393</v>
+        <v>1400</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>563599</v>
+        <v>566466</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
       </c>
       <c r="M22" s="12">
-        <v>2761</v>
+        <v>2868</v>
       </c>
       <c r="N22" s="13" t="s">
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2048314</v>
+        <v>2062654</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2143,28 +2143,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6151483</v>
+        <v>6194987</v>
       </c>
       <c r="D6" s="6">
-        <v>105847</v>
+        <v>106452</v>
       </c>
       <c r="E6" s="6">
-        <v>66621</v>
+        <v>67110</v>
       </c>
       <c r="F6" s="6">
-        <v>333295</v>
+        <v>335546</v>
       </c>
       <c r="G6" s="6">
-        <v>54087</v>
+        <v>54444</v>
       </c>
       <c r="H6" s="6">
-        <v>9174</v>
+        <v>9212</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6257330</v>
+        <v>6301439</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2175,28 +2175,28 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>244430</v>
+        <v>245076</v>
       </c>
       <c r="D7" s="9">
-        <v>2868</v>
+        <v>2876</v>
       </c>
       <c r="E7" s="9">
-        <v>2082</v>
+        <v>2092</v>
       </c>
       <c r="F7" s="9">
-        <v>12954</v>
+        <v>12992</v>
       </c>
       <c r="G7" s="9">
         <v>303</v>
       </c>
       <c r="H7" s="9">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="I7" s="9">
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>247298</v>
+        <v>247952</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2207,28 +2207,28 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>428443</v>
+        <v>431346</v>
       </c>
       <c r="D8" s="9">
-        <v>5685</v>
+        <v>5718</v>
       </c>
       <c r="E8" s="9">
-        <v>4222</v>
+        <v>4245</v>
       </c>
       <c r="F8" s="9">
-        <v>32875</v>
+        <v>33081</v>
       </c>
       <c r="G8" s="9">
-        <v>3902</v>
+        <v>3920</v>
       </c>
       <c r="H8" s="9">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="I8" s="9">
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>434128</v>
+        <v>437064</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2239,147 +2239,147 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>732700</v>
+        <v>739502</v>
       </c>
       <c r="D9" s="9">
-        <v>12787</v>
+        <v>12865</v>
       </c>
       <c r="E9" s="9">
-        <v>8329</v>
+        <v>8411</v>
       </c>
       <c r="F9" s="9">
-        <v>36475</v>
+        <v>36804</v>
       </c>
       <c r="G9" s="9">
-        <v>4478</v>
+        <v>4511</v>
       </c>
       <c r="H9" s="9">
-        <v>979</v>
+        <v>985</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>745487</v>
+        <v>752367</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>762762</v>
+        <v>767296</v>
       </c>
       <c r="D10" s="9">
-        <v>14864</v>
+        <v>14921</v>
       </c>
       <c r="E10" s="9">
-        <v>8971</v>
+        <v>9030</v>
       </c>
       <c r="F10" s="9">
-        <v>37808</v>
+        <v>38013</v>
       </c>
       <c r="G10" s="9">
-        <v>18936</v>
+        <v>19043</v>
       </c>
       <c r="H10" s="9">
-        <v>1049</v>
+        <v>1051</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>777626</v>
+        <v>782217</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C11" s="9">
-        <v>968701</v>
+        <v>976402</v>
       </c>
       <c r="D11" s="9">
-        <v>19737</v>
+        <v>19857</v>
       </c>
       <c r="E11" s="9">
-        <v>11617</v>
+        <v>11723</v>
       </c>
       <c r="F11" s="9">
-        <v>43828</v>
+        <v>44125</v>
       </c>
       <c r="G11" s="9">
-        <v>7969</v>
+        <v>8030</v>
       </c>
       <c r="H11" s="9">
-        <v>1686</v>
+        <v>1695</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>988438</v>
+        <v>996259</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C12" s="9">
-        <v>468989</v>
+        <v>473023</v>
       </c>
       <c r="D12" s="9">
-        <v>6045</v>
+        <v>6074</v>
       </c>
       <c r="E12" s="9">
-        <v>5652</v>
+        <v>5706</v>
       </c>
       <c r="F12" s="9">
-        <v>26902</v>
+        <v>27137</v>
       </c>
       <c r="G12" s="9">
-        <v>1919</v>
+        <v>1931</v>
       </c>
       <c r="H12" s="9">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>475034</v>
+        <v>479097</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C13" s="9">
-        <v>333601</v>
+        <v>336267</v>
       </c>
       <c r="D13" s="9">
-        <v>4258</v>
+        <v>4275</v>
       </c>
       <c r="E13" s="9">
-        <v>3774</v>
+        <v>3807</v>
       </c>
       <c r="F13" s="9">
-        <v>24054</v>
+        <v>24240</v>
       </c>
       <c r="G13" s="9">
-        <v>1321</v>
+        <v>1331</v>
       </c>
       <c r="H13" s="9">
         <v>458</v>
@@ -2388,62 +2388,62 @@
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>337859</v>
+        <v>340542</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C14" s="9">
-        <v>274547</v>
+        <v>277214</v>
       </c>
       <c r="D14" s="9">
-        <v>7844</v>
+        <v>7956</v>
       </c>
       <c r="E14" s="9">
-        <v>3051</v>
+        <v>3079</v>
       </c>
       <c r="F14" s="9">
-        <v>18677</v>
+        <v>18878</v>
       </c>
       <c r="G14" s="9">
-        <v>1865</v>
+        <v>1878</v>
       </c>
       <c r="H14" s="9">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>282391</v>
+        <v>285170</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C15" s="9">
-        <v>383343</v>
+        <v>385702</v>
       </c>
       <c r="D15" s="9">
-        <v>7486</v>
+        <v>7528</v>
       </c>
       <c r="E15" s="9">
-        <v>6275</v>
+        <v>6312</v>
       </c>
       <c r="F15" s="9">
-        <v>26065</v>
+        <v>26218</v>
       </c>
       <c r="G15" s="9">
-        <v>3746</v>
+        <v>3776</v>
       </c>
       <c r="H15" s="9">
         <v>505</v>
@@ -2452,59 +2452,59 @@
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>390829</v>
+        <v>393230</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C16" s="9">
-        <v>316690</v>
+        <v>319098</v>
       </c>
       <c r="D16" s="9">
-        <v>4606</v>
+        <v>4629</v>
       </c>
       <c r="E16" s="9">
-        <v>2747</v>
+        <v>2766</v>
       </c>
       <c r="F16" s="9">
-        <v>18457</v>
+        <v>18621</v>
       </c>
       <c r="G16" s="9">
-        <v>3690</v>
+        <v>3732</v>
       </c>
       <c r="H16" s="9">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>321296</v>
+        <v>323727</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C17" s="9">
-        <v>195941</v>
+        <v>196353</v>
       </c>
       <c r="D17" s="9">
-        <v>4813</v>
+        <v>4825</v>
       </c>
       <c r="E17" s="9">
-        <v>2173</v>
+        <v>2175</v>
       </c>
       <c r="F17" s="9">
-        <v>10242</v>
+        <v>10264</v>
       </c>
       <c r="G17" s="9">
         <v>1705</v>
@@ -2516,7 +2516,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>200754</v>
+        <v>201178</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2527,28 +2527,28 @@
         <v>118</v>
       </c>
       <c r="C18" s="9">
-        <v>242997</v>
+        <v>244147</v>
       </c>
       <c r="D18" s="9">
-        <v>5330</v>
+        <v>5348</v>
       </c>
       <c r="E18" s="9">
-        <v>2592</v>
+        <v>2603</v>
       </c>
       <c r="F18" s="9">
-        <v>13924</v>
+        <v>13983</v>
       </c>
       <c r="G18" s="9">
-        <v>2338</v>
+        <v>2353</v>
       </c>
       <c r="H18" s="9">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>248327</v>
+        <v>249495</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2559,19 +2559,19 @@
         <v>125</v>
       </c>
       <c r="C19" s="9">
-        <v>135529</v>
+        <v>135612</v>
       </c>
       <c r="D19" s="9">
         <v>1736</v>
       </c>
       <c r="E19" s="9">
-        <v>1033</v>
+        <v>1036</v>
       </c>
       <c r="F19" s="9">
-        <v>10331</v>
+        <v>10342</v>
       </c>
       <c r="G19" s="9">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H19" s="9">
         <v>234</v>
@@ -2580,7 +2580,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>137265</v>
+        <v>137348</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2591,28 +2591,28 @@
         <v>131</v>
       </c>
       <c r="C20" s="9">
-        <v>548956</v>
+        <v>553297</v>
       </c>
       <c r="D20" s="9">
-        <v>6714</v>
+        <v>6760</v>
       </c>
       <c r="E20" s="9">
-        <v>3286</v>
+        <v>3303</v>
       </c>
       <c r="F20" s="9">
-        <v>15809</v>
+        <v>15912</v>
       </c>
       <c r="G20" s="9">
-        <v>964</v>
+        <v>973</v>
       </c>
       <c r="H20" s="9">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>555670</v>
+        <v>560057</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2623,28 +2623,28 @@
         <v>138</v>
       </c>
       <c r="C21" s="9">
-        <v>113854</v>
+        <v>114652</v>
       </c>
       <c r="D21" s="9">
-        <v>1074</v>
+        <v>1084</v>
       </c>
       <c r="E21" s="9">
-        <v>817</v>
+        <v>822</v>
       </c>
       <c r="F21" s="9">
-        <v>4894</v>
+        <v>4936</v>
       </c>
       <c r="G21" s="9">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="H21" s="9">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>114928</v>
+        <v>115736</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2655,28 +2655,28 @@
         <v>144</v>
       </c>
       <c r="C22" s="12">
-        <v>6151483</v>
+        <v>6194987</v>
       </c>
       <c r="D22" s="12">
-        <v>105847</v>
+        <v>106452</v>
       </c>
       <c r="E22" s="12">
-        <v>66621</v>
+        <v>67110</v>
       </c>
       <c r="F22" s="12">
-        <v>333295</v>
+        <v>335546</v>
       </c>
       <c r="G22" s="12">
-        <v>54087</v>
+        <v>54444</v>
       </c>
       <c r="H22" s="12">
-        <v>9174</v>
+        <v>9212</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6257330</v>
+        <v>6301439</v>
       </c>
     </row>
   </sheetData>
@@ -2770,7 +2770,7 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1008</v>
+        <v>1023</v>
       </c>
       <c r="D7" s="6">
         <v>81</v>
@@ -2804,7 +2804,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="9">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D9" s="9">
         <v>1</v>
@@ -2821,7 +2821,7 @@
         <v>58</v>
       </c>
       <c r="C10" s="9">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D10" s="9">
         <v>4</v>
@@ -2832,13 +2832,13 @@
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C11" s="9">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D11" s="9">
         <v>2</v>
@@ -2849,10 +2849,10 @@
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C12" s="9">
         <v>161</v>
@@ -2866,13 +2866,13 @@
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C13" s="9">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D13" s="9">
         <v>2</v>
@@ -2883,13 +2883,13 @@
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C14" s="9">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D14" s="9">
         <v>0</v>
@@ -2900,10 +2900,10 @@
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" s="9">
         <v>93</v>
@@ -2917,13 +2917,13 @@
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C16" s="9">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D16" s="9">
         <v>38</v>
@@ -2934,10 +2934,10 @@
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C17" s="9">
         <v>37</v>
@@ -2951,10 +2951,10 @@
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C18" s="9">
         <v>30</v>
@@ -2974,7 +2974,7 @@
         <v>118</v>
       </c>
       <c r="C19" s="9">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D19" s="9">
         <v>10</v>
@@ -3008,7 +3008,7 @@
         <v>131</v>
       </c>
       <c r="C21" s="9">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D21" s="9">
         <v>2</v>
@@ -3042,7 +3042,7 @@
         <v>144</v>
       </c>
       <c r="C23" s="12">
-        <v>1008</v>
+        <v>1023</v>
       </c>
       <c r="D23" s="12">
         <v>81</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 19/08/2026 20:46:19,19
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="171">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 19 Agu 2026, 06.16 | Dicetak: 19 Agu 2026, 14.11</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 19 Agu 2026, 18.16 | Dicetak: 19 Agu 2026, 20.45</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,7 +123,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>64,21</t>
+    <t>64,66</t>
   </si>
   <si>
     <t>1,77</t>
@@ -132,13 +132,13 @@
     <t>0,05</t>
   </si>
   <si>
-    <t>20,74</t>
+    <t>20,87</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>75,53</t>
+    <t>76,06</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,22 +147,22 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>78,92</t>
-  </si>
-  <si>
-    <t>1,12</t>
+    <t>78,99</t>
+  </si>
+  <si>
+    <t>1,13</t>
   </si>
   <si>
     <t>0,04</t>
   </si>
   <si>
-    <t>18,21</t>
+    <t>18,28</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>91,75</t>
+    <t>91,83</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>67,05</t>
-  </si>
-  <si>
-    <t>0,97</t>
-  </si>
-  <si>
-    <t>16,55</t>
+    <t>67,53</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>16,72</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>81,65</t>
+    <t>82,27</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,19 +192,19 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>58,9</t>
-  </si>
-  <si>
-    <t>1,17</t>
-  </si>
-  <si>
-    <t>19,29</t>
+    <t>59,4</t>
+  </si>
+  <si>
+    <t>1,18</t>
+  </si>
+  <si>
+    <t>19,45</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>70,89</t>
+    <t>71,5</t>
   </si>
   <si>
     <t>1804</t>
@@ -213,16 +213,16 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>65,92</t>
-  </si>
-  <si>
-    <t>1,86</t>
-  </si>
-  <si>
-    <t>18,05</t>
-  </si>
-  <si>
-    <t>74,71</t>
+    <t>66,4</t>
+  </si>
+  <si>
+    <t>1,87</t>
+  </si>
+  <si>
+    <t>18,15</t>
+  </si>
+  <si>
+    <t>75,25</t>
   </si>
   <si>
     <t>1805</t>
@@ -231,19 +231,19 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>65,58</t>
-  </si>
-  <si>
-    <t>2,68</t>
-  </si>
-  <si>
-    <t>18,09</t>
+    <t>66,06</t>
+  </si>
+  <si>
+    <t>2,69</t>
+  </si>
+  <si>
+    <t>18,19</t>
   </si>
   <si>
     <t>0,23</t>
   </si>
   <si>
-    <t>74,3</t>
+    <t>74,84</t>
   </si>
   <si>
     <t>1806</t>
@@ -252,19 +252,19 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>65,27</t>
-  </si>
-  <si>
-    <t>1,93</t>
+    <t>65,73</t>
+  </si>
+  <si>
+    <t>1,94</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>25,39</t>
-  </si>
-  <si>
-    <t>76,63</t>
+    <t>25,55</t>
+  </si>
+  <si>
+    <t>77,18</t>
   </si>
   <si>
     <t>1807</t>
@@ -273,16 +273,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>65,47</t>
-  </si>
-  <si>
-    <t>1,67</t>
-  </si>
-  <si>
-    <t>18,38</t>
-  </si>
-  <si>
-    <t>76,7</t>
+    <t>66,07</t>
+  </si>
+  <si>
+    <t>1,68</t>
+  </si>
+  <si>
+    <t>18,51</t>
+  </si>
+  <si>
+    <t>77,4</t>
   </si>
   <si>
     <t>1808</t>
@@ -291,16 +291,16 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>57,78</t>
-  </si>
-  <si>
-    <t>2,23</t>
-  </si>
-  <si>
-    <t>25,38</t>
-  </si>
-  <si>
-    <t>69,27</t>
+    <t>58,41</t>
+  </si>
+  <si>
+    <t>2,24</t>
+  </si>
+  <si>
+    <t>25,58</t>
+  </si>
+  <si>
+    <t>70,01</t>
   </si>
   <si>
     <t>1809</t>
@@ -309,19 +309,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>70,7</t>
+    <t>71,06</t>
   </si>
   <si>
     <t>2,96</t>
   </si>
   <si>
-    <t>20,86</t>
+    <t>20,95</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>84,13</t>
+    <t>84,58</t>
   </si>
   <si>
     <t>1810</t>
@@ -330,19 +330,19 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>70,55</t>
-  </si>
-  <si>
-    <t>1,44</t>
-  </si>
-  <si>
-    <t>15,84</t>
+    <t>71,09</t>
+  </si>
+  <si>
+    <t>1,45</t>
+  </si>
+  <si>
+    <t>15,99</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>79,56</t>
+    <t>80,16</t>
   </si>
   <si>
     <t>1811</t>
@@ -351,19 +351,19 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>74,07</t>
+    <t>74,18</t>
   </si>
   <si>
     <t>1,58</t>
   </si>
   <si>
-    <t>25,01</t>
+    <t>25,02</t>
   </si>
   <si>
     <t>0,16</t>
   </si>
   <si>
-    <t>90,15</t>
+    <t>90,3</t>
   </si>
   <si>
     <t>1812</t>
@@ -372,19 +372,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>72,85</t>
+    <t>73,17</t>
   </si>
   <si>
     <t>2,43</t>
   </si>
   <si>
-    <t>23,05</t>
+    <t>23,09</t>
   </si>
   <si>
     <t>0,24</t>
   </si>
   <si>
-    <t>85,41</t>
+    <t>85,79</t>
   </si>
   <si>
     <t>1813</t>
@@ -393,7 +393,7 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>80,96</t>
+    <t>81,08</t>
   </si>
   <si>
     <t>0,83</t>
@@ -402,7 +402,7 @@
     <t>17,55</t>
   </si>
   <si>
-    <t>98,39</t>
+    <t>98,55</t>
   </si>
   <si>
     <t>1871</t>
@@ -411,19 +411,19 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>47,3</t>
-  </si>
-  <si>
-    <t>0,84</t>
-  </si>
-  <si>
-    <t>30,03</t>
+    <t>47,73</t>
+  </si>
+  <si>
+    <t>0,85</t>
+  </si>
+  <si>
+    <t>30,25</t>
   </si>
   <si>
     <t>0,03</t>
   </si>
   <si>
-    <t>60,43</t>
+    <t>60,97</t>
   </si>
   <si>
     <t>1872</t>
@@ -432,16 +432,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>62,42</t>
-  </si>
-  <si>
-    <t>1,34</t>
-  </si>
-  <si>
-    <t>21,41</t>
-  </si>
-  <si>
-    <t>71,52</t>
+    <t>62,81</t>
+  </si>
+  <si>
+    <t>1,35</t>
+  </si>
+  <si>
+    <t>21,55</t>
+  </si>
+  <si>
+    <t>71,99</t>
   </si>
   <si>
     <t/>
@@ -486,7 +486,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>7,92</t>
+    <t>9,84</t>
   </si>
   <si>
     <t>0</t>
@@ -495,31 +495,34 @@
     <t>4</t>
   </si>
   <si>
-    <t>4,26</t>
-  </si>
-  <si>
-    <t>2,27</t>
-  </si>
-  <si>
-    <t>2,48</t>
-  </si>
-  <si>
-    <t>8,33</t>
-  </si>
-  <si>
-    <t>24,84</t>
-  </si>
-  <si>
-    <t>2,7</t>
-  </si>
-  <si>
-    <t>16,67</t>
-  </si>
-  <si>
-    <t>14,29</t>
-  </si>
-  <si>
-    <t>1,65</t>
+    <t>4,35</t>
+  </si>
+  <si>
+    <t>2,04</t>
+  </si>
+  <si>
+    <t>7,19</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>2,13</t>
+  </si>
+  <si>
+    <t>26,62</t>
+  </si>
+  <si>
+    <t>2,5</t>
+  </si>
+  <si>
+    <t>28,57</t>
+  </si>
+  <si>
+    <t>22,86</t>
+  </si>
+  <si>
+    <t>2,44</t>
   </si>
   <si>
     <t>19,67</t>
@@ -1183,28 +1186,28 @@
         <v>2730932</v>
       </c>
       <c r="D6" s="6">
-        <v>1753600</v>
+        <v>1765950</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>309054</v>
+        <v>311247</v>
       </c>
       <c r="G6" s="6">
-        <v>48214</v>
+        <v>48446</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1400</v>
+        <v>1406</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>566466</v>
+        <v>570050</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1216,7 +1219,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2062654</v>
+        <v>2077197</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1233,16 +1236,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67194</v>
+        <v>67254</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10929</v>
+        <v>10936</v>
       </c>
       <c r="G7" s="9">
-        <v>957</v>
+        <v>960</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1254,7 +1257,7 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15502</v>
+        <v>15566</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1266,7 +1269,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78123</v>
+        <v>78190</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1283,28 +1286,28 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>115968</v>
+        <v>116805</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>25253</v>
+        <v>25495</v>
       </c>
       <c r="G8" s="9">
-        <v>1679</v>
+        <v>1694</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="9">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>28622</v>
+        <v>28910</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1316,7 +1319,7 @@
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>141221</v>
+        <v>142300</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1333,16 +1336,16 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>201868</v>
+        <v>203601</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>41085</v>
+        <v>41439</v>
       </c>
       <c r="G9" s="9">
-        <v>4016</v>
+        <v>4044</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
@@ -1354,7 +1357,7 @@
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>66100</v>
+        <v>66669</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
@@ -1366,7 +1369,7 @@
         <v>62</v>
       </c>
       <c r="O9" s="9">
-        <v>242953</v>
+        <v>245040</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>63</v>
@@ -1383,28 +1386,28 @@
         <v>362838</v>
       </c>
       <c r="D10" s="9">
-        <v>239183</v>
+        <v>240930</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="9">
-        <v>31894</v>
+        <v>32095</v>
       </c>
       <c r="G10" s="9">
-        <v>6750</v>
+        <v>6780</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>67</v>
       </c>
       <c r="I10" s="9">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>65475</v>
+        <v>65856</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>68</v>
@@ -1416,7 +1419,7 @@
         <v>55</v>
       </c>
       <c r="O10" s="9">
-        <v>271077</v>
+        <v>273025</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>69</v>
@@ -1433,28 +1436,28 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>294820</v>
+        <v>297007</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>72</v>
       </c>
       <c r="F11" s="9">
-        <v>39231</v>
+        <v>39469</v>
       </c>
       <c r="G11" s="9">
-        <v>12034</v>
+        <v>12104</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I11" s="9">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>81338</v>
+        <v>81789</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>74</v>
@@ -1466,7 +1469,7 @@
         <v>75</v>
       </c>
       <c r="O11" s="9">
-        <v>334051</v>
+        <v>336476</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>76</v>
@@ -1483,28 +1486,28 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>130137</v>
+        <v>131066</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>79</v>
       </c>
       <c r="F12" s="9">
-        <v>22667</v>
+        <v>22835</v>
       </c>
       <c r="G12" s="9">
-        <v>3854</v>
+        <v>3870</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>80</v>
       </c>
       <c r="I12" s="9">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="J12" s="10" t="s">
         <v>81</v>
       </c>
       <c r="K12" s="9">
-        <v>50636</v>
+        <v>50944</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>82</v>
@@ -1516,7 +1519,7 @@
         <v>62</v>
       </c>
       <c r="O12" s="9">
-        <v>152804</v>
+        <v>153901</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>83</v>
@@ -1533,16 +1536,16 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>95649</v>
+        <v>96522</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>86</v>
       </c>
       <c r="F13" s="9">
-        <v>16397</v>
+        <v>16553</v>
       </c>
       <c r="G13" s="9">
-        <v>2443</v>
+        <v>2456</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>87</v>
@@ -1554,7 +1557,7 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>26852</v>
+        <v>27041</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>88</v>
@@ -1566,7 +1569,7 @@
         <v>62</v>
       </c>
       <c r="O13" s="9">
-        <v>112046</v>
+        <v>113075</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>89</v>
@@ -1583,28 +1586,28 @@
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>78153</v>
+        <v>78999</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>92</v>
       </c>
       <c r="F14" s="9">
-        <v>15536</v>
+        <v>15693</v>
       </c>
       <c r="G14" s="9">
-        <v>3013</v>
+        <v>3025</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>93</v>
       </c>
       <c r="I14" s="9">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J14" s="10" t="s">
         <v>81</v>
       </c>
       <c r="K14" s="9">
-        <v>34326</v>
+        <v>34602</v>
       </c>
       <c r="L14" s="10" t="s">
         <v>94</v>
@@ -1616,7 +1619,7 @@
         <v>81</v>
       </c>
       <c r="O14" s="9">
-        <v>93689</v>
+        <v>94692</v>
       </c>
       <c r="P14" s="10" t="s">
         <v>95</v>
@@ -1633,16 +1636,16 @@
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>107570</v>
+        <v>108122</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>98</v>
       </c>
       <c r="F15" s="9">
-        <v>20442</v>
+        <v>20567</v>
       </c>
       <c r="G15" s="9">
-        <v>4506</v>
+        <v>4508</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>99</v>
@@ -1654,7 +1657,7 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>31745</v>
+        <v>31883</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>100</v>
@@ -1666,7 +1669,7 @@
         <v>101</v>
       </c>
       <c r="O15" s="9">
-        <v>128012</v>
+        <v>128689</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>102</v>
@@ -1683,16 +1686,16 @@
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>95763</v>
+        <v>96503</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>105</v>
       </c>
       <c r="F16" s="9">
-        <v>12228</v>
+        <v>12311</v>
       </c>
       <c r="G16" s="9">
-        <v>1959</v>
+        <v>1975</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>106</v>
@@ -1704,7 +1707,7 @@
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>21504</v>
+        <v>21705</v>
       </c>
       <c r="L16" s="10" t="s">
         <v>107</v>
@@ -1716,7 +1719,7 @@
         <v>108</v>
       </c>
       <c r="O16" s="9">
-        <v>107991</v>
+        <v>108814</v>
       </c>
       <c r="P16" s="10" t="s">
         <v>109</v>
@@ -1733,13 +1736,13 @@
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55634</v>
+        <v>55720</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>112</v>
       </c>
       <c r="F17" s="9">
-        <v>12085</v>
+        <v>12108</v>
       </c>
       <c r="G17" s="9">
         <v>1187</v>
@@ -1754,7 +1757,7 @@
         <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18790</v>
+        <v>18793</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>114</v>
@@ -1766,7 +1769,7 @@
         <v>115</v>
       </c>
       <c r="O17" s="9">
-        <v>67719</v>
+        <v>67828</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>116</v>
@@ -1783,13 +1786,13 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>72242</v>
+        <v>72561</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>119</v>
       </c>
       <c r="F18" s="9">
-        <v>12457</v>
+        <v>12521</v>
       </c>
       <c r="G18" s="9">
         <v>2405</v>
@@ -1798,13 +1801,13 @@
         <v>120</v>
       </c>
       <c r="I18" s="9">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J18" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22862</v>
+        <v>22899</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>121</v>
@@ -1816,7 +1819,7 @@
         <v>122</v>
       </c>
       <c r="O18" s="9">
-        <v>84699</v>
+        <v>85082</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>123</v>
@@ -1833,13 +1836,13 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33818</v>
+        <v>33869</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>126</v>
       </c>
       <c r="F19" s="9">
-        <v>7283</v>
+        <v>7296</v>
       </c>
       <c r="G19" s="9">
         <v>347</v>
@@ -1854,7 +1857,7 @@
         <v>108</v>
       </c>
       <c r="K19" s="9">
-        <v>7331</v>
+        <v>7333</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>128</v>
@@ -1866,7 +1869,7 @@
         <v>55</v>
       </c>
       <c r="O19" s="9">
-        <v>41101</v>
+        <v>41165</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>129</v>
@@ -1883,28 +1886,28 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>132202</v>
+        <v>133385</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>132</v>
       </c>
       <c r="F20" s="9">
-        <v>36698</v>
+        <v>37018</v>
       </c>
       <c r="G20" s="9">
-        <v>2345</v>
+        <v>2366</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>133</v>
       </c>
       <c r="I20" s="9">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>83927</v>
+        <v>84532</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>134</v>
@@ -1916,7 +1919,7 @@
         <v>135</v>
       </c>
       <c r="O20" s="9">
-        <v>168900</v>
+        <v>170403</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>136</v>
@@ -1933,16 +1936,16 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>33399</v>
+        <v>33606</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>139</v>
       </c>
       <c r="F21" s="9">
-        <v>4869</v>
+        <v>4911</v>
       </c>
       <c r="G21" s="9">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>140</v>
@@ -1954,7 +1957,7 @@
         <v>108</v>
       </c>
       <c r="K21" s="9">
-        <v>11456</v>
+        <v>11528</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>141</v>
@@ -1966,7 +1969,7 @@
         <v>81</v>
       </c>
       <c r="O21" s="9">
-        <v>38268</v>
+        <v>38517</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>142</v>
@@ -1983,28 +1986,28 @@
         <v>2730932</v>
       </c>
       <c r="D22" s="12">
-        <v>1753600</v>
+        <v>1765950</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>309054</v>
+        <v>311247</v>
       </c>
       <c r="G22" s="12">
-        <v>48214</v>
+        <v>48446</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1400</v>
+        <v>1406</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>566466</v>
+        <v>570050</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2016,7 +2019,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2062654</v>
+        <v>2077197</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2143,28 +2146,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6194987</v>
+        <v>6239391</v>
       </c>
       <c r="D6" s="6">
-        <v>106452</v>
+        <v>107069</v>
       </c>
       <c r="E6" s="6">
-        <v>67110</v>
+        <v>67592</v>
       </c>
       <c r="F6" s="6">
-        <v>335546</v>
+        <v>337683</v>
       </c>
       <c r="G6" s="6">
-        <v>54444</v>
+        <v>54828</v>
       </c>
       <c r="H6" s="6">
-        <v>9212</v>
+        <v>9259</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6301439</v>
+        <v>6346460</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2175,28 +2178,28 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>245076</v>
+        <v>245287</v>
       </c>
       <c r="D7" s="9">
-        <v>2876</v>
+        <v>2878</v>
       </c>
       <c r="E7" s="9">
-        <v>2092</v>
+        <v>2095</v>
       </c>
       <c r="F7" s="9">
-        <v>12992</v>
+        <v>12997</v>
       </c>
       <c r="G7" s="9">
         <v>303</v>
       </c>
       <c r="H7" s="9">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="I7" s="9">
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>247952</v>
+        <v>248165</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2207,19 +2210,19 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>431346</v>
+        <v>434703</v>
       </c>
       <c r="D8" s="9">
-        <v>5718</v>
+        <v>5746</v>
       </c>
       <c r="E8" s="9">
-        <v>4245</v>
+        <v>4277</v>
       </c>
       <c r="F8" s="9">
-        <v>33081</v>
+        <v>33311</v>
       </c>
       <c r="G8" s="9">
-        <v>3920</v>
+        <v>3947</v>
       </c>
       <c r="H8" s="9">
         <v>562</v>
@@ -2228,7 +2231,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>437064</v>
+        <v>440449</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2239,28 +2242,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>739502</v>
+        <v>745920</v>
       </c>
       <c r="D9" s="9">
-        <v>12865</v>
+        <v>12973</v>
       </c>
       <c r="E9" s="9">
-        <v>8411</v>
+        <v>8494</v>
       </c>
       <c r="F9" s="9">
-        <v>36804</v>
+        <v>37099</v>
       </c>
       <c r="G9" s="9">
-        <v>4511</v>
+        <v>4561</v>
       </c>
       <c r="H9" s="9">
-        <v>985</v>
+        <v>991</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>752367</v>
+        <v>758893</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2271,28 +2274,28 @@
         <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>767296</v>
+        <v>772890</v>
       </c>
       <c r="D10" s="9">
-        <v>14921</v>
+        <v>15024</v>
       </c>
       <c r="E10" s="9">
-        <v>9030</v>
+        <v>9093</v>
       </c>
       <c r="F10" s="9">
-        <v>38013</v>
+        <v>38280</v>
       </c>
       <c r="G10" s="9">
-        <v>19043</v>
+        <v>19193</v>
       </c>
       <c r="H10" s="9">
-        <v>1051</v>
+        <v>1059</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>782217</v>
+        <v>787914</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2303,28 +2306,28 @@
         <v>71</v>
       </c>
       <c r="C11" s="9">
-        <v>976402</v>
+        <v>983607</v>
       </c>
       <c r="D11" s="9">
-        <v>19857</v>
+        <v>19961</v>
       </c>
       <c r="E11" s="9">
-        <v>11723</v>
+        <v>11806</v>
       </c>
       <c r="F11" s="9">
-        <v>44125</v>
+        <v>44380</v>
       </c>
       <c r="G11" s="9">
-        <v>8030</v>
+        <v>8084</v>
       </c>
       <c r="H11" s="9">
-        <v>1695</v>
+        <v>1708</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>996259</v>
+        <v>1003568</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2335,28 +2338,28 @@
         <v>78</v>
       </c>
       <c r="C12" s="9">
-        <v>473023</v>
+        <v>476494</v>
       </c>
       <c r="D12" s="9">
-        <v>6074</v>
+        <v>6105</v>
       </c>
       <c r="E12" s="9">
-        <v>5706</v>
+        <v>5741</v>
       </c>
       <c r="F12" s="9">
-        <v>27137</v>
+        <v>27330</v>
       </c>
       <c r="G12" s="9">
-        <v>1931</v>
+        <v>1945</v>
       </c>
       <c r="H12" s="9">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>479097</v>
+        <v>482599</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2367,19 +2370,19 @@
         <v>85</v>
       </c>
       <c r="C13" s="9">
-        <v>336267</v>
+        <v>339355</v>
       </c>
       <c r="D13" s="9">
-        <v>4275</v>
+        <v>4296</v>
       </c>
       <c r="E13" s="9">
-        <v>3807</v>
+        <v>3851</v>
       </c>
       <c r="F13" s="9">
-        <v>24240</v>
+        <v>24441</v>
       </c>
       <c r="G13" s="9">
-        <v>1331</v>
+        <v>1338</v>
       </c>
       <c r="H13" s="9">
         <v>458</v>
@@ -2388,7 +2391,7 @@
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>340542</v>
+        <v>343651</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2399,28 +2402,28 @@
         <v>91</v>
       </c>
       <c r="C14" s="9">
-        <v>277214</v>
+        <v>280324</v>
       </c>
       <c r="D14" s="9">
-        <v>7956</v>
+        <v>8037</v>
       </c>
       <c r="E14" s="9">
-        <v>3079</v>
+        <v>3105</v>
       </c>
       <c r="F14" s="9">
-        <v>18878</v>
+        <v>19103</v>
       </c>
       <c r="G14" s="9">
-        <v>1878</v>
+        <v>1892</v>
       </c>
       <c r="H14" s="9">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>285170</v>
+        <v>288361</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2431,28 +2434,28 @@
         <v>97</v>
       </c>
       <c r="C15" s="9">
-        <v>385702</v>
+        <v>387822</v>
       </c>
       <c r="D15" s="9">
-        <v>7528</v>
+        <v>7559</v>
       </c>
       <c r="E15" s="9">
-        <v>6312</v>
+        <v>6346</v>
       </c>
       <c r="F15" s="9">
-        <v>26218</v>
+        <v>26327</v>
       </c>
       <c r="G15" s="9">
-        <v>3776</v>
+        <v>3787</v>
       </c>
       <c r="H15" s="9">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>393230</v>
+        <v>395381</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2463,28 +2466,28 @@
         <v>104</v>
       </c>
       <c r="C16" s="9">
-        <v>319098</v>
+        <v>321547</v>
       </c>
       <c r="D16" s="9">
-        <v>4629</v>
+        <v>4661</v>
       </c>
       <c r="E16" s="9">
-        <v>2766</v>
+        <v>2780</v>
       </c>
       <c r="F16" s="9">
-        <v>18621</v>
+        <v>18734</v>
       </c>
       <c r="G16" s="9">
-        <v>3732</v>
+        <v>3755</v>
       </c>
       <c r="H16" s="9">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>323727</v>
+        <v>326208</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2495,19 +2498,19 @@
         <v>111</v>
       </c>
       <c r="C17" s="9">
-        <v>196353</v>
+        <v>196683</v>
       </c>
       <c r="D17" s="9">
-        <v>4825</v>
+        <v>4830</v>
       </c>
       <c r="E17" s="9">
-        <v>2175</v>
+        <v>2179</v>
       </c>
       <c r="F17" s="9">
-        <v>10264</v>
+        <v>10274</v>
       </c>
       <c r="G17" s="9">
-        <v>1705</v>
+        <v>1708</v>
       </c>
       <c r="H17" s="9">
         <v>399</v>
@@ -2516,7 +2519,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201178</v>
+        <v>201513</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2527,28 +2530,28 @@
         <v>118</v>
       </c>
       <c r="C18" s="9">
-        <v>244147</v>
+        <v>245315</v>
       </c>
       <c r="D18" s="9">
-        <v>5348</v>
+        <v>5364</v>
       </c>
       <c r="E18" s="9">
-        <v>2603</v>
+        <v>2622</v>
       </c>
       <c r="F18" s="9">
-        <v>13983</v>
+        <v>14062</v>
       </c>
       <c r="G18" s="9">
-        <v>2353</v>
+        <v>2366</v>
       </c>
       <c r="H18" s="9">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>249495</v>
+        <v>250679</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2559,16 +2562,16 @@
         <v>125</v>
       </c>
       <c r="C19" s="9">
-        <v>135612</v>
+        <v>135831</v>
       </c>
       <c r="D19" s="9">
-        <v>1736</v>
+        <v>1740</v>
       </c>
       <c r="E19" s="9">
-        <v>1036</v>
+        <v>1041</v>
       </c>
       <c r="F19" s="9">
-        <v>10342</v>
+        <v>10352</v>
       </c>
       <c r="G19" s="9">
         <v>222</v>
@@ -2580,7 +2583,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>137348</v>
+        <v>137571</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2591,28 +2594,28 @@
         <v>131</v>
       </c>
       <c r="C20" s="9">
-        <v>553297</v>
+        <v>558225</v>
       </c>
       <c r="D20" s="9">
-        <v>6760</v>
+        <v>6804</v>
       </c>
       <c r="E20" s="9">
-        <v>3303</v>
+        <v>3337</v>
       </c>
       <c r="F20" s="9">
-        <v>15912</v>
+        <v>16006</v>
       </c>
       <c r="G20" s="9">
-        <v>973</v>
+        <v>987</v>
       </c>
       <c r="H20" s="9">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>560057</v>
+        <v>565029</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2623,28 +2626,28 @@
         <v>138</v>
       </c>
       <c r="C21" s="9">
-        <v>114652</v>
+        <v>115388</v>
       </c>
       <c r="D21" s="9">
-        <v>1084</v>
+        <v>1091</v>
       </c>
       <c r="E21" s="9">
-        <v>822</v>
+        <v>825</v>
       </c>
       <c r="F21" s="9">
-        <v>4936</v>
+        <v>4987</v>
       </c>
       <c r="G21" s="9">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="H21" s="9">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>115736</v>
+        <v>116479</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2655,28 +2658,28 @@
         <v>144</v>
       </c>
       <c r="C22" s="12">
-        <v>6194987</v>
+        <v>6239391</v>
       </c>
       <c r="D22" s="12">
-        <v>106452</v>
+        <v>107069</v>
       </c>
       <c r="E22" s="12">
-        <v>67110</v>
+        <v>67592</v>
       </c>
       <c r="F22" s="12">
-        <v>335546</v>
+        <v>337683</v>
       </c>
       <c r="G22" s="12">
-        <v>54444</v>
+        <v>54828</v>
       </c>
       <c r="H22" s="12">
-        <v>9212</v>
+        <v>9259</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6301439</v>
+        <v>6346460</v>
       </c>
     </row>
   </sheetData>
@@ -2770,10 +2773,10 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1023</v>
+        <v>1047</v>
       </c>
       <c r="D7" s="6">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>157</v>
@@ -2821,7 +2824,7 @@
         <v>58</v>
       </c>
       <c r="C10" s="9">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D10" s="9">
         <v>4</v>
@@ -2838,7 +2841,7 @@
         <v>65</v>
       </c>
       <c r="C11" s="9">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="D11" s="9">
         <v>2</v>
@@ -2855,10 +2858,10 @@
         <v>71</v>
       </c>
       <c r="C12" s="9">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="D12" s="9">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>162</v>
@@ -2872,7 +2875,7 @@
         <v>78</v>
       </c>
       <c r="C13" s="9">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" s="9">
         <v>2</v>
@@ -2889,13 +2892,13 @@
         <v>85</v>
       </c>
       <c r="C14" s="9">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D14" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2906,7 +2909,7 @@
         <v>91</v>
       </c>
       <c r="C15" s="9">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D15" s="9">
         <v>0</v>
@@ -2923,13 +2926,13 @@
         <v>97</v>
       </c>
       <c r="C16" s="9">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D16" s="9">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2940,13 +2943,13 @@
         <v>104</v>
       </c>
       <c r="C17" s="9">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D17" s="9">
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2957,13 +2960,13 @@
         <v>111</v>
       </c>
       <c r="C18" s="9">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D18" s="9">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2977,10 +2980,10 @@
         <v>70</v>
       </c>
       <c r="D19" s="9">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2991,7 +2994,7 @@
         <v>125</v>
       </c>
       <c r="C20" s="9">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D20" s="9">
         <v>0</v>
@@ -3008,13 +3011,13 @@
         <v>131</v>
       </c>
       <c r="C21" s="9">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D21" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3031,7 +3034,7 @@
         <v>12</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3042,10 +3045,10 @@
         <v>144</v>
       </c>
       <c r="C23" s="12">
-        <v>1023</v>
+        <v>1047</v>
       </c>
       <c r="D23" s="12">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>157</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 20/08/2026  6:44:16,95
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -18,7 +18,7 @@
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 19 Agu 2026, 18.16 | Dicetak: 19 Agu 2026, 20.45</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 20 Agu 2026, 06.16 | Dicetak: 20 Agu 2026, 06.42</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,22 +123,22 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>64,66</t>
-  </si>
-  <si>
-    <t>1,77</t>
+    <t>65,09</t>
+  </si>
+  <si>
+    <t>1,78</t>
   </si>
   <si>
     <t>0,05</t>
   </si>
   <si>
-    <t>20,87</t>
+    <t>20,98</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>76,06</t>
+    <t>76,56</t>
   </si>
   <si>
     <t>1801</t>
@@ -156,94 +156,94 @@
     <t>0,04</t>
   </si>
   <si>
+    <t>18,31</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>91,82</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>67,94</t>
+  </si>
+  <si>
+    <t>0,98</t>
+  </si>
+  <si>
+    <t>16,81</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>82,79</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>59,92</t>
+  </si>
+  <si>
+    <t>1,19</t>
+  </si>
+  <si>
+    <t>19,58</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>72,11</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>66,84</t>
+  </si>
+  <si>
+    <t>1,87</t>
+  </si>
+  <si>
+    <t>18,21</t>
+  </si>
+  <si>
+    <t>75,73</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>66,54</t>
+  </si>
+  <si>
+    <t>2,71</t>
+  </si>
+  <si>
     <t>18,28</t>
   </si>
   <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>91,83</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>67,53</t>
-  </si>
-  <si>
-    <t>0,98</t>
-  </si>
-  <si>
-    <t>16,72</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>82,27</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>59,4</t>
-  </si>
-  <si>
-    <t>1,18</t>
-  </si>
-  <si>
-    <t>19,45</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>71,5</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>66,4</t>
-  </si>
-  <si>
-    <t>1,87</t>
-  </si>
-  <si>
-    <t>18,15</t>
-  </si>
-  <si>
-    <t>75,25</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>66,06</t>
-  </si>
-  <si>
-    <t>2,69</t>
-  </si>
-  <si>
-    <t>18,19</t>
-  </si>
-  <si>
-    <t>0,23</t>
-  </si>
-  <si>
-    <t>74,84</t>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>75,39</t>
   </si>
   <si>
     <t>1806</t>
@@ -252,19 +252,22 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>65,73</t>
-  </si>
-  <si>
-    <t>1,94</t>
+    <t>66,17</t>
+  </si>
+  <si>
+    <t>1,95</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>25,55</t>
-  </si>
-  <si>
-    <t>77,18</t>
+    <t>25,7</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>77,7</t>
   </si>
   <si>
     <t>1807</t>
@@ -273,16 +276,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>66,07</t>
-  </si>
-  <si>
-    <t>1,68</t>
-  </si>
-  <si>
-    <t>18,51</t>
-  </si>
-  <si>
-    <t>77,4</t>
+    <t>66,66</t>
+  </si>
+  <si>
+    <t>1,69</t>
+  </si>
+  <si>
+    <t>18,61</t>
+  </si>
+  <si>
+    <t>78,11</t>
   </si>
   <si>
     <t>1808</t>
@@ -291,16 +294,16 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>58,41</t>
+    <t>59,05</t>
   </si>
   <si>
     <t>2,24</t>
   </si>
   <si>
-    <t>25,58</t>
-  </si>
-  <si>
-    <t>70,01</t>
+    <t>25,85</t>
+  </si>
+  <si>
+    <t>70,76</t>
   </si>
   <si>
     <t>1809</t>
@@ -309,19 +312,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>71,06</t>
-  </si>
-  <si>
-    <t>2,96</t>
-  </si>
-  <si>
-    <t>20,95</t>
+    <t>71,38</t>
+  </si>
+  <si>
+    <t>2,97</t>
+  </si>
+  <si>
+    <t>21,05</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>84,58</t>
+    <t>84,98</t>
   </si>
   <si>
     <t>1810</t>
@@ -330,19 +333,19 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>71,09</t>
-  </si>
-  <si>
-    <t>1,45</t>
-  </si>
-  <si>
-    <t>15,99</t>
+    <t>71,58</t>
+  </si>
+  <si>
+    <t>1,46</t>
+  </si>
+  <si>
+    <t>16,04</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>80,16</t>
+    <t>80,71</t>
   </si>
   <si>
     <t>1811</t>
@@ -351,19 +354,19 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>74,18</t>
+    <t>74,22</t>
   </si>
   <si>
     <t>1,58</t>
   </si>
   <si>
-    <t>25,02</t>
+    <t>25</t>
   </si>
   <si>
     <t>0,16</t>
   </si>
   <si>
-    <t>90,3</t>
+    <t>90,35</t>
   </si>
   <si>
     <t>1812</t>
@@ -372,19 +375,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>73,17</t>
+    <t>73,36</t>
   </si>
   <si>
     <t>2,43</t>
   </si>
   <si>
-    <t>23,09</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>85,79</t>
+    <t>23,12</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>86,03</t>
   </si>
   <si>
     <t>1813</t>
@@ -393,7 +396,7 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>81,08</t>
+    <t>81,19</t>
   </si>
   <si>
     <t>0,83</t>
@@ -402,7 +405,7 @@
     <t>17,55</t>
   </si>
   <si>
-    <t>98,55</t>
+    <t>98,7</t>
   </si>
   <si>
     <t>1871</t>
@@ -411,19 +414,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>47,73</t>
+    <t>48,12</t>
   </si>
   <si>
     <t>0,85</t>
   </si>
   <si>
-    <t>30,25</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>60,97</t>
+    <t>30,42</t>
+  </si>
+  <si>
+    <t>61,46</t>
   </si>
   <si>
     <t>1872</t>
@@ -432,16 +432,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>62,81</t>
-  </si>
-  <si>
-    <t>1,35</t>
-  </si>
-  <si>
-    <t>21,55</t>
-  </si>
-  <si>
-    <t>71,99</t>
+    <t>63,1</t>
+  </si>
+  <si>
+    <t>1,36</t>
+  </si>
+  <si>
+    <t>21,58</t>
+  </si>
+  <si>
+    <t>72,31</t>
   </si>
   <si>
     <t/>
@@ -486,7 +486,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>9,84</t>
+    <t>9,78</t>
   </si>
   <si>
     <t>0</t>
@@ -495,13 +495,13 @@
     <t>4</t>
   </si>
   <si>
-    <t>4,35</t>
-  </si>
-  <si>
-    <t>2,04</t>
-  </si>
-  <si>
-    <t>7,19</t>
+    <t>4,3</t>
+  </si>
+  <si>
+    <t>1,98</t>
+  </si>
+  <si>
+    <t>7,14</t>
   </si>
   <si>
     <t>8</t>
@@ -522,7 +522,7 @@
     <t>22,86</t>
   </si>
   <si>
-    <t>2,44</t>
+    <t>2,42</t>
   </si>
   <si>
     <t>19,67</t>
@@ -1186,40 +1186,40 @@
         <v>2730932</v>
       </c>
       <c r="D6" s="6">
-        <v>1765950</v>
+        <v>1777479</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>311247</v>
+        <v>313219</v>
       </c>
       <c r="G6" s="6">
-        <v>48446</v>
+        <v>48606</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1406</v>
+        <v>1415</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>570050</v>
+        <v>572823</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
       </c>
       <c r="M6" s="6">
-        <v>2868</v>
+        <v>2959</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2077197</v>
+        <v>2090698</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1236,16 +1236,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67254</v>
+        <v>67253</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10936</v>
+        <v>10926</v>
       </c>
       <c r="G7" s="9">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1257,19 +1257,19 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15566</v>
+        <v>15588</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
       </c>
       <c r="M7" s="9">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="N7" s="10" t="s">
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78190</v>
+        <v>78179</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1286,40 +1286,40 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>116805</v>
+        <v>117503</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>25495</v>
+        <v>25691</v>
       </c>
       <c r="G8" s="9">
-        <v>1694</v>
+        <v>1699</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="9">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>28910</v>
+        <v>29070</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
       </c>
       <c r="M8" s="9">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="N8" s="10" t="s">
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>142300</v>
+        <v>143194</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1336,40 +1336,40 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>203601</v>
+        <v>205365</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>41439</v>
+        <v>41783</v>
       </c>
       <c r="G9" s="9">
-        <v>4044</v>
+        <v>4064</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>66669</v>
+        <v>67101</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
       </c>
       <c r="M9" s="9">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="N9" s="10" t="s">
         <v>62</v>
       </c>
       <c r="O9" s="9">
-        <v>245040</v>
+        <v>247148</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>63</v>
@@ -1386,40 +1386,40 @@
         <v>362838</v>
       </c>
       <c r="D10" s="9">
-        <v>240930</v>
+        <v>242529</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="9">
-        <v>32095</v>
+        <v>32263</v>
       </c>
       <c r="G10" s="9">
-        <v>6780</v>
+        <v>6801</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>67</v>
       </c>
       <c r="I10" s="9">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>65856</v>
+        <v>66065</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>68</v>
       </c>
       <c r="M10" s="9">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="N10" s="10" t="s">
         <v>55</v>
       </c>
       <c r="O10" s="9">
-        <v>273025</v>
+        <v>274792</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>69</v>
@@ -1436,40 +1436,40 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>297007</v>
+        <v>299168</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>72</v>
       </c>
       <c r="F11" s="9">
-        <v>39469</v>
+        <v>39753</v>
       </c>
       <c r="G11" s="9">
-        <v>12104</v>
+        <v>12164</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I11" s="9">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>81789</v>
+        <v>82204</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>74</v>
       </c>
       <c r="M11" s="9">
-        <v>1033</v>
+        <v>1062</v>
       </c>
       <c r="N11" s="10" t="s">
         <v>75</v>
       </c>
       <c r="O11" s="9">
-        <v>336476</v>
+        <v>338921</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>76</v>
@@ -1486,16 +1486,16 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>131066</v>
+        <v>131945</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>79</v>
       </c>
       <c r="F12" s="9">
-        <v>22835</v>
+        <v>22978</v>
       </c>
       <c r="G12" s="9">
-        <v>3870</v>
+        <v>3880</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>80</v>
@@ -1507,98 +1507,98 @@
         <v>81</v>
       </c>
       <c r="K12" s="9">
-        <v>50944</v>
+        <v>51235</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>82</v>
       </c>
       <c r="M12" s="9">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="N12" s="10" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="O12" s="9">
-        <v>153901</v>
+        <v>154923</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C13" s="9">
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>96522</v>
+        <v>97390</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F13" s="9">
-        <v>16553</v>
+        <v>16723</v>
       </c>
       <c r="G13" s="9">
-        <v>2456</v>
+        <v>2463</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I13" s="9">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J13" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>27041</v>
+        <v>27195</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="M13" s="9">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="O13" s="9">
-        <v>113075</v>
+        <v>114113</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" s="9">
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>78999</v>
+        <v>79864</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F14" s="9">
-        <v>15693</v>
+        <v>15837</v>
       </c>
       <c r="G14" s="9">
-        <v>3025</v>
+        <v>3035</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I14" s="9">
         <v>33</v>
@@ -1607,98 +1607,98 @@
         <v>81</v>
       </c>
       <c r="K14" s="9">
-        <v>34602</v>
+        <v>34958</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M14" s="9">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="N14" s="10" t="s">
         <v>81</v>
       </c>
       <c r="O14" s="9">
-        <v>94692</v>
+        <v>95701</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C15" s="9">
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>108122</v>
+        <v>108615</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F15" s="9">
-        <v>20567</v>
+        <v>20690</v>
       </c>
       <c r="G15" s="9">
-        <v>4508</v>
+        <v>4520</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I15" s="9">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J15" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>31883</v>
+        <v>32032</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M15" s="9">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="O15" s="9">
-        <v>128689</v>
+        <v>129305</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C16" s="9">
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>96503</v>
+        <v>97168</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F16" s="9">
-        <v>12311</v>
+        <v>12392</v>
       </c>
       <c r="G16" s="9">
-        <v>1975</v>
+        <v>1978</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I16" s="9">
         <v>99</v>
@@ -1707,48 +1707,48 @@
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>21705</v>
+        <v>21768</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="M16" s="9">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O16" s="9">
-        <v>108814</v>
+        <v>109560</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C17" s="9">
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55720</v>
+        <v>55753</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F17" s="9">
-        <v>12108</v>
+        <v>12110</v>
       </c>
       <c r="G17" s="9">
         <v>1187</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I17" s="9">
         <v>80</v>
@@ -1757,48 +1757,48 @@
         <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18793</v>
+        <v>18780</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="M17" s="9">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O17" s="9">
-        <v>67828</v>
+        <v>67863</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C18" s="9">
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>72561</v>
+        <v>72755</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F18" s="9">
-        <v>12521</v>
+        <v>12556</v>
       </c>
       <c r="G18" s="9">
         <v>2405</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I18" s="9">
         <v>49</v>
@@ -1807,98 +1807,98 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22899</v>
+        <v>22926</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M18" s="9">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="N18" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O18" s="9">
-        <v>85082</v>
+        <v>85311</v>
       </c>
       <c r="P18" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C19" s="9">
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33869</v>
+        <v>33914</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F19" s="9">
-        <v>7296</v>
+        <v>7315</v>
       </c>
       <c r="G19" s="9">
         <v>347</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I19" s="9">
         <v>27</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K19" s="9">
-        <v>7333</v>
+        <v>7332</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="M19" s="9">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>55</v>
+        <v>109</v>
       </c>
       <c r="O19" s="9">
-        <v>41165</v>
+        <v>41229</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C20" s="9">
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>133385</v>
+        <v>134497</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F20" s="9">
-        <v>37018</v>
+        <v>37273</v>
       </c>
       <c r="G20" s="9">
-        <v>2366</v>
+        <v>2376</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I20" s="9">
         <v>132</v>
@@ -1907,19 +1907,19 @@
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>84532</v>
+        <v>85023</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M20" s="9">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="N20" s="10" t="s">
-        <v>135</v>
+        <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>170403</v>
+        <v>171770</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>136</v>
@@ -1936,16 +1936,16 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>33606</v>
+        <v>33760</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>139</v>
       </c>
       <c r="F21" s="9">
-        <v>4911</v>
+        <v>4929</v>
       </c>
       <c r="G21" s="9">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>140</v>
@@ -1954,22 +1954,22 @@
         <v>33</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K21" s="9">
-        <v>11528</v>
+        <v>11546</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>141</v>
       </c>
       <c r="M21" s="9">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N21" s="10" t="s">
         <v>81</v>
       </c>
       <c r="O21" s="9">
-        <v>38517</v>
+        <v>38689</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>142</v>
@@ -1986,40 +1986,40 @@
         <v>2730932</v>
       </c>
       <c r="D22" s="12">
-        <v>1765950</v>
+        <v>1777479</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>311247</v>
+        <v>313219</v>
       </c>
       <c r="G22" s="12">
-        <v>48446</v>
+        <v>48606</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1406</v>
+        <v>1415</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>570050</v>
+        <v>572823</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
       </c>
       <c r="M22" s="12">
-        <v>2868</v>
+        <v>2959</v>
       </c>
       <c r="N22" s="13" t="s">
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2077197</v>
+        <v>2090698</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2146,28 +2146,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6239391</v>
+        <v>6280021</v>
       </c>
       <c r="D6" s="6">
-        <v>107069</v>
+        <v>107602</v>
       </c>
       <c r="E6" s="6">
-        <v>67592</v>
+        <v>67994</v>
       </c>
       <c r="F6" s="6">
-        <v>337683</v>
+        <v>339757</v>
       </c>
       <c r="G6" s="6">
-        <v>54828</v>
+        <v>55174</v>
       </c>
       <c r="H6" s="6">
-        <v>9259</v>
+        <v>9292</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6346460</v>
+        <v>6387623</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2178,19 +2178,19 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>245287</v>
+        <v>245186</v>
       </c>
       <c r="D7" s="9">
-        <v>2878</v>
+        <v>2869</v>
       </c>
       <c r="E7" s="9">
-        <v>2095</v>
+        <v>2097</v>
       </c>
       <c r="F7" s="9">
-        <v>12997</v>
+        <v>13007</v>
       </c>
       <c r="G7" s="9">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="H7" s="9">
         <v>394</v>
@@ -2199,7 +2199,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>248165</v>
+        <v>248055</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2210,28 +2210,28 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>434703</v>
+        <v>437320</v>
       </c>
       <c r="D8" s="9">
-        <v>5746</v>
+        <v>5793</v>
       </c>
       <c r="E8" s="9">
-        <v>4277</v>
+        <v>4302</v>
       </c>
       <c r="F8" s="9">
-        <v>33311</v>
+        <v>33519</v>
       </c>
       <c r="G8" s="9">
-        <v>3947</v>
+        <v>3970</v>
       </c>
       <c r="H8" s="9">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="I8" s="9">
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>440449</v>
+        <v>443113</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2242,28 +2242,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>745920</v>
+        <v>752353</v>
       </c>
       <c r="D9" s="9">
-        <v>12973</v>
+        <v>13051</v>
       </c>
       <c r="E9" s="9">
-        <v>8494</v>
+        <v>8562</v>
       </c>
       <c r="F9" s="9">
-        <v>37099</v>
+        <v>37416</v>
       </c>
       <c r="G9" s="9">
-        <v>4561</v>
+        <v>4591</v>
       </c>
       <c r="H9" s="9">
-        <v>991</v>
+        <v>997</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>758893</v>
+        <v>765404</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2274,28 +2274,28 @@
         <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>772890</v>
+        <v>777828</v>
       </c>
       <c r="D10" s="9">
-        <v>15024</v>
+        <v>15081</v>
       </c>
       <c r="E10" s="9">
-        <v>9093</v>
+        <v>9140</v>
       </c>
       <c r="F10" s="9">
-        <v>38280</v>
+        <v>38508</v>
       </c>
       <c r="G10" s="9">
-        <v>19193</v>
+        <v>19342</v>
       </c>
       <c r="H10" s="9">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>787914</v>
+        <v>792909</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2306,28 +2306,28 @@
         <v>71</v>
       </c>
       <c r="C11" s="9">
-        <v>983607</v>
+        <v>990808</v>
       </c>
       <c r="D11" s="9">
-        <v>19961</v>
+        <v>20057</v>
       </c>
       <c r="E11" s="9">
-        <v>11806</v>
+        <v>11884</v>
       </c>
       <c r="F11" s="9">
-        <v>44380</v>
+        <v>44654</v>
       </c>
       <c r="G11" s="9">
-        <v>8084</v>
+        <v>8130</v>
       </c>
       <c r="H11" s="9">
-        <v>1708</v>
+        <v>1720</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1003568</v>
+        <v>1010865</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2338,147 +2338,147 @@
         <v>78</v>
       </c>
       <c r="C12" s="9">
-        <v>476494</v>
+        <v>479714</v>
       </c>
       <c r="D12" s="9">
-        <v>6105</v>
+        <v>6128</v>
       </c>
       <c r="E12" s="9">
-        <v>5741</v>
+        <v>5772</v>
       </c>
       <c r="F12" s="9">
-        <v>27330</v>
+        <v>27489</v>
       </c>
       <c r="G12" s="9">
-        <v>1945</v>
+        <v>1959</v>
       </c>
       <c r="H12" s="9">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>482599</v>
+        <v>485842</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C13" s="9">
-        <v>339355</v>
+        <v>342503</v>
       </c>
       <c r="D13" s="9">
-        <v>4296</v>
+        <v>4325</v>
       </c>
       <c r="E13" s="9">
-        <v>3851</v>
+        <v>3884</v>
       </c>
       <c r="F13" s="9">
-        <v>24441</v>
+        <v>24669</v>
       </c>
       <c r="G13" s="9">
-        <v>1338</v>
+        <v>1351</v>
       </c>
       <c r="H13" s="9">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>343651</v>
+        <v>346828</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" s="9">
-        <v>280324</v>
+        <v>283409</v>
       </c>
       <c r="D14" s="9">
-        <v>8037</v>
+        <v>8128</v>
       </c>
       <c r="E14" s="9">
-        <v>3105</v>
+        <v>3141</v>
       </c>
       <c r="F14" s="9">
-        <v>19103</v>
+        <v>19319</v>
       </c>
       <c r="G14" s="9">
-        <v>1892</v>
+        <v>1905</v>
       </c>
       <c r="H14" s="9">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>288361</v>
+        <v>291537</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C15" s="9">
-        <v>387822</v>
+        <v>389784</v>
       </c>
       <c r="D15" s="9">
-        <v>7559</v>
+        <v>7577</v>
       </c>
       <c r="E15" s="9">
-        <v>6346</v>
+        <v>6375</v>
       </c>
       <c r="F15" s="9">
-        <v>26327</v>
+        <v>26420</v>
       </c>
       <c r="G15" s="9">
-        <v>3787</v>
+        <v>3793</v>
       </c>
       <c r="H15" s="9">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>395381</v>
+        <v>397361</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C16" s="9">
-        <v>321547</v>
+        <v>323768</v>
       </c>
       <c r="D16" s="9">
-        <v>4661</v>
+        <v>4697</v>
       </c>
       <c r="E16" s="9">
-        <v>2780</v>
+        <v>2796</v>
       </c>
       <c r="F16" s="9">
-        <v>18734</v>
+        <v>18865</v>
       </c>
       <c r="G16" s="9">
-        <v>3755</v>
+        <v>3787</v>
       </c>
       <c r="H16" s="9">
         <v>253</v>
@@ -2487,18 +2487,18 @@
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>326208</v>
+        <v>328465</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C17" s="9">
-        <v>196683</v>
+        <v>196796</v>
       </c>
       <c r="D17" s="9">
         <v>4830</v>
@@ -2507,7 +2507,7 @@
         <v>2179</v>
       </c>
       <c r="F17" s="9">
-        <v>10274</v>
+        <v>10278</v>
       </c>
       <c r="G17" s="9">
         <v>1708</v>
@@ -2519,62 +2519,62 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201513</v>
+        <v>201626</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C18" s="9">
-        <v>245315</v>
+        <v>246003</v>
       </c>
       <c r="D18" s="9">
-        <v>5364</v>
+        <v>5383</v>
       </c>
       <c r="E18" s="9">
-        <v>2622</v>
+        <v>2627</v>
       </c>
       <c r="F18" s="9">
-        <v>14062</v>
+        <v>14102</v>
       </c>
       <c r="G18" s="9">
-        <v>2366</v>
+        <v>2370</v>
       </c>
       <c r="H18" s="9">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>250679</v>
+        <v>251386</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C19" s="9">
-        <v>135831</v>
+        <v>136048</v>
       </c>
       <c r="D19" s="9">
-        <v>1740</v>
+        <v>1743</v>
       </c>
       <c r="E19" s="9">
         <v>1041</v>
       </c>
       <c r="F19" s="9">
-        <v>10352</v>
+        <v>10376</v>
       </c>
       <c r="G19" s="9">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H19" s="9">
         <v>234</v>
@@ -2583,39 +2583,39 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>137571</v>
+        <v>137791</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C20" s="9">
-        <v>558225</v>
+        <v>562609</v>
       </c>
       <c r="D20" s="9">
-        <v>6804</v>
+        <v>6847</v>
       </c>
       <c r="E20" s="9">
-        <v>3337</v>
+        <v>3364</v>
       </c>
       <c r="F20" s="9">
-        <v>16006</v>
+        <v>16120</v>
       </c>
       <c r="G20" s="9">
-        <v>987</v>
+        <v>997</v>
       </c>
       <c r="H20" s="9">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>565029</v>
+        <v>569456</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2626,28 +2626,28 @@
         <v>138</v>
       </c>
       <c r="C21" s="9">
-        <v>115388</v>
+        <v>115892</v>
       </c>
       <c r="D21" s="9">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="E21" s="9">
-        <v>825</v>
+        <v>830</v>
       </c>
       <c r="F21" s="9">
-        <v>4987</v>
+        <v>5015</v>
       </c>
       <c r="G21" s="9">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="H21" s="9">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>116479</v>
+        <v>116985</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2658,28 +2658,28 @@
         <v>144</v>
       </c>
       <c r="C22" s="12">
-        <v>6239391</v>
+        <v>6280021</v>
       </c>
       <c r="D22" s="12">
-        <v>107069</v>
+        <v>107602</v>
       </c>
       <c r="E22" s="12">
-        <v>67592</v>
+        <v>67994</v>
       </c>
       <c r="F22" s="12">
-        <v>337683</v>
+        <v>339757</v>
       </c>
       <c r="G22" s="12">
-        <v>54828</v>
+        <v>55174</v>
       </c>
       <c r="H22" s="12">
-        <v>9259</v>
+        <v>9292</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6346460</v>
+        <v>6387623</v>
       </c>
     </row>
   </sheetData>
@@ -2773,7 +2773,7 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1047</v>
+        <v>1053</v>
       </c>
       <c r="D7" s="6">
         <v>103</v>
@@ -2824,7 +2824,7 @@
         <v>58</v>
       </c>
       <c r="C10" s="9">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D10" s="9">
         <v>4</v>
@@ -2841,7 +2841,7 @@
         <v>65</v>
       </c>
       <c r="C11" s="9">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D11" s="9">
         <v>2</v>
@@ -2858,7 +2858,7 @@
         <v>71</v>
       </c>
       <c r="C12" s="9">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
@@ -2886,10 +2886,10 @@
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C14" s="9">
         <v>47</v>
@@ -2903,10 +2903,10 @@
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C15" s="9">
         <v>94</v>
@@ -2920,10 +2920,10 @@
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" s="9">
         <v>154</v>
@@ -2937,10 +2937,10 @@
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C17" s="9">
         <v>40</v>
@@ -2954,10 +2954,10 @@
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C18" s="9">
         <v>28</v>
@@ -2971,10 +2971,10 @@
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C19" s="9">
         <v>70</v>
@@ -2988,10 +2988,10 @@
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C20" s="9">
         <v>15</v>
@@ -3005,13 +3005,13 @@
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C21" s="9">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D21" s="9">
         <v>3</v>
@@ -3045,7 +3045,7 @@
         <v>144</v>
       </c>
       <c r="C23" s="12">
-        <v>1047</v>
+        <v>1053</v>
       </c>
       <c r="D23" s="12">
         <v>103</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 20/08/2026 13:27:19,99
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="170">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 20 Agu 2026, 06.16 | Dicetak: 20 Agu 2026, 06.42</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 20 Agu 2026, 12.16 | Dicetak: 20 Agu 2026, 13.23</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,7 +123,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>65,09</t>
+    <t>65,29</t>
   </si>
   <si>
     <t>1,78</t>
@@ -132,13 +132,13 @@
     <t>0,05</t>
   </si>
   <si>
-    <t>20,98</t>
+    <t>21,03</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>76,56</t>
+    <t>76,79</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>78,99</t>
+    <t>78,96</t>
   </si>
   <si>
     <t>1,13</t>
@@ -156,13 +156,13 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>18,31</t>
+    <t>18,32</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>91,82</t>
+    <t>91,77</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>67,94</t>
+    <t>68,18</t>
   </si>
   <si>
     <t>0,98</t>
   </si>
   <si>
-    <t>16,81</t>
+    <t>16,87</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>82,79</t>
+    <t>83,08</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,19 +192,19 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>59,92</t>
+    <t>60,16</t>
   </si>
   <si>
     <t>1,19</t>
   </si>
   <si>
-    <t>19,58</t>
+    <t>19,64</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>72,11</t>
+    <t>72,39</t>
   </si>
   <si>
     <t>1804</t>
@@ -213,16 +213,16 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>66,84</t>
-  </si>
-  <si>
-    <t>1,87</t>
-  </si>
-  <si>
-    <t>18,21</t>
-  </si>
-  <si>
-    <t>75,73</t>
+    <t>67,06</t>
+  </si>
+  <si>
+    <t>1,88</t>
+  </si>
+  <si>
+    <t>18,25</t>
+  </si>
+  <si>
+    <t>75,97</t>
   </si>
   <si>
     <t>1805</t>
@@ -231,19 +231,19 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>66,54</t>
+    <t>66,77</t>
   </si>
   <si>
     <t>2,71</t>
   </si>
   <si>
-    <t>18,28</t>
+    <t>18,35</t>
   </si>
   <si>
     <t>0,24</t>
   </si>
   <si>
-    <t>75,39</t>
+    <t>75,64</t>
   </si>
   <si>
     <t>1806</t>
@@ -252,7 +252,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>66,17</t>
+    <t>66,4</t>
   </si>
   <si>
     <t>1,95</t>
@@ -261,13 +261,13 @@
     <t>0,02</t>
   </si>
   <si>
-    <t>25,7</t>
+    <t>25,79</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>77,7</t>
+    <t>77,97</t>
   </si>
   <si>
     <t>1807</t>
@@ -276,16 +276,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>66,66</t>
+    <t>67</t>
   </si>
   <si>
     <t>1,69</t>
   </si>
   <si>
-    <t>18,61</t>
-  </si>
-  <si>
-    <t>78,11</t>
+    <t>18,67</t>
+  </si>
+  <si>
+    <t>78,49</t>
   </si>
   <si>
     <t>1808</t>
@@ -294,16 +294,16 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>59,05</t>
+    <t>59,33</t>
   </si>
   <si>
     <t>2,24</t>
   </si>
   <si>
-    <t>25,85</t>
-  </si>
-  <si>
-    <t>70,76</t>
+    <t>25,9</t>
+  </si>
+  <si>
+    <t>71,09</t>
   </si>
   <si>
     <t>1809</t>
@@ -312,19 +312,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>71,38</t>
+    <t>71,53</t>
   </si>
   <si>
     <t>2,97</t>
   </si>
   <si>
-    <t>21,05</t>
+    <t>21,09</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>84,98</t>
+    <t>85,16</t>
   </si>
   <si>
     <t>1810</t>
@@ -333,19 +333,19 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>71,58</t>
+    <t>71,89</t>
   </si>
   <si>
     <t>1,46</t>
   </si>
   <si>
-    <t>16,04</t>
+    <t>16,14</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>80,71</t>
+    <t>81,05</t>
   </si>
   <si>
     <t>1811</t>
@@ -354,19 +354,19 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>74,22</t>
+    <t>74,24</t>
   </si>
   <si>
     <t>1,58</t>
   </si>
   <si>
-    <t>25</t>
+    <t>24,98</t>
   </si>
   <si>
     <t>0,16</t>
   </si>
   <si>
-    <t>90,35</t>
+    <t>90,37</t>
   </si>
   <si>
     <t>1812</t>
@@ -375,19 +375,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>73,36</t>
-  </si>
-  <si>
-    <t>2,43</t>
-  </si>
-  <si>
-    <t>23,12</t>
+    <t>73,45</t>
+  </si>
+  <si>
+    <t>2,42</t>
+  </si>
+  <si>
+    <t>23,13</t>
   </si>
   <si>
     <t>0,25</t>
   </si>
   <si>
-    <t>86,03</t>
+    <t>86,17</t>
   </si>
   <si>
     <t>1813</t>
@@ -396,16 +396,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>81,19</t>
+    <t>81,24</t>
   </si>
   <si>
     <t>0,83</t>
   </si>
   <si>
-    <t>17,55</t>
-  </si>
-  <si>
-    <t>98,7</t>
+    <t>17,54</t>
+  </si>
+  <si>
+    <t>98,76</t>
   </si>
   <si>
     <t>1871</t>
@@ -414,16 +414,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>48,12</t>
+    <t>48,26</t>
   </si>
   <si>
     <t>0,85</t>
   </si>
   <si>
-    <t>30,42</t>
-  </si>
-  <si>
-    <t>61,46</t>
+    <t>30,5</t>
+  </si>
+  <si>
+    <t>61,63</t>
   </si>
   <si>
     <t>1872</t>
@@ -432,16 +432,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>63,1</t>
+    <t>63,26</t>
   </si>
   <si>
     <t>1,36</t>
   </si>
   <si>
-    <t>21,58</t>
-  </si>
-  <si>
-    <t>72,31</t>
+    <t>21,62</t>
+  </si>
+  <si>
+    <t>72,5</t>
   </si>
   <si>
     <t/>
@@ -486,7 +486,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>9,78</t>
+    <t>12,11</t>
   </si>
   <si>
     <t>0</t>
@@ -498,34 +498,31 @@
     <t>4,3</t>
   </si>
   <si>
-    <t>1,98</t>
-  </si>
-  <si>
-    <t>7,14</t>
-  </si>
-  <si>
-    <t>8</t>
+    <t>23,3</t>
+  </si>
+  <si>
+    <t>6,98</t>
+  </si>
+  <si>
+    <t>17,86</t>
   </si>
   <si>
     <t>2,13</t>
   </si>
   <si>
-    <t>26,62</t>
-  </si>
-  <si>
-    <t>2,5</t>
+    <t>26,45</t>
+  </si>
+  <si>
+    <t>2,44</t>
   </si>
   <si>
     <t>28,57</t>
   </si>
   <si>
-    <t>22,86</t>
-  </si>
-  <si>
-    <t>2,42</t>
-  </si>
-  <si>
-    <t>19,67</t>
+    <t>24,29</t>
+  </si>
+  <si>
+    <t>19,35</t>
   </si>
 </sst>
 </file>
@@ -1186,28 +1183,28 @@
         <v>2730932</v>
       </c>
       <c r="D6" s="6">
-        <v>1777479</v>
+        <v>1783068</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>313219</v>
+        <v>314094</v>
       </c>
       <c r="G6" s="6">
-        <v>48606</v>
+        <v>48686</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1415</v>
+        <v>1433</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>572823</v>
+        <v>574377</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1219,7 +1216,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2090698</v>
+        <v>2097162</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1236,16 +1233,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67253</v>
+        <v>67233</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10926</v>
+        <v>10904</v>
       </c>
       <c r="G7" s="9">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1257,7 +1254,7 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15588</v>
+        <v>15600</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1269,7 +1266,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78179</v>
+        <v>78137</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1286,28 +1283,28 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>117503</v>
+        <v>117920</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>25691</v>
+        <v>25771</v>
       </c>
       <c r="G8" s="9">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="9">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>29070</v>
+        <v>29181</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1319,7 +1316,7 @@
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>143194</v>
+        <v>143691</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1336,16 +1333,16 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>205365</v>
+        <v>206189</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>41783</v>
+        <v>41926</v>
       </c>
       <c r="G9" s="9">
-        <v>4064</v>
+        <v>4076</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
@@ -1357,7 +1354,7 @@
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>67101</v>
+        <v>67315</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
@@ -1369,7 +1366,7 @@
         <v>62</v>
       </c>
       <c r="O9" s="9">
-        <v>247148</v>
+        <v>248115</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>63</v>
@@ -1386,28 +1383,28 @@
         <v>362838</v>
       </c>
       <c r="D10" s="9">
-        <v>242529</v>
+        <v>243309</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="9">
-        <v>32263</v>
+        <v>32348</v>
       </c>
       <c r="G10" s="9">
-        <v>6801</v>
+        <v>6811</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>67</v>
       </c>
       <c r="I10" s="9">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>66065</v>
+        <v>66216</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>68</v>
@@ -1419,7 +1416,7 @@
         <v>55</v>
       </c>
       <c r="O10" s="9">
-        <v>274792</v>
+        <v>275657</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>69</v>
@@ -1436,28 +1433,28 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>299168</v>
+        <v>300191</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>72</v>
       </c>
       <c r="F11" s="9">
-        <v>39753</v>
+        <v>39874</v>
       </c>
       <c r="G11" s="9">
-        <v>12164</v>
+        <v>12185</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I11" s="9">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>82204</v>
+        <v>82504</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>74</v>
@@ -1469,7 +1466,7 @@
         <v>75</v>
       </c>
       <c r="O11" s="9">
-        <v>338921</v>
+        <v>340065</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>76</v>
@@ -1486,28 +1483,28 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>131945</v>
+        <v>132395</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>79</v>
       </c>
       <c r="F12" s="9">
-        <v>22978</v>
+        <v>23081</v>
       </c>
       <c r="G12" s="9">
-        <v>3880</v>
+        <v>3883</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>80</v>
       </c>
       <c r="I12" s="9">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J12" s="10" t="s">
         <v>81</v>
       </c>
       <c r="K12" s="9">
-        <v>51235</v>
+        <v>51420</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>82</v>
@@ -1519,7 +1516,7 @@
         <v>83</v>
       </c>
       <c r="O12" s="9">
-        <v>154923</v>
+        <v>155476</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>84</v>
@@ -1536,16 +1533,16 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>97390</v>
+        <v>97885</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>87</v>
       </c>
       <c r="F13" s="9">
-        <v>16723</v>
+        <v>16780</v>
       </c>
       <c r="G13" s="9">
-        <v>2463</v>
+        <v>2472</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>88</v>
@@ -1557,7 +1554,7 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>27195</v>
+        <v>27282</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>89</v>
@@ -1569,7 +1566,7 @@
         <v>83</v>
       </c>
       <c r="O13" s="9">
-        <v>114113</v>
+        <v>114665</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>90</v>
@@ -1586,16 +1583,16 @@
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>79864</v>
+        <v>80251</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>93</v>
       </c>
       <c r="F14" s="9">
-        <v>15837</v>
+        <v>15898</v>
       </c>
       <c r="G14" s="9">
-        <v>3035</v>
+        <v>3036</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>94</v>
@@ -1607,7 +1604,7 @@
         <v>81</v>
       </c>
       <c r="K14" s="9">
-        <v>34958</v>
+        <v>35028</v>
       </c>
       <c r="L14" s="10" t="s">
         <v>95</v>
@@ -1619,7 +1616,7 @@
         <v>81</v>
       </c>
       <c r="O14" s="9">
-        <v>95701</v>
+        <v>96149</v>
       </c>
       <c r="P14" s="10" t="s">
         <v>96</v>
@@ -1636,16 +1633,16 @@
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>108615</v>
+        <v>108839</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>99</v>
       </c>
       <c r="F15" s="9">
-        <v>20690</v>
+        <v>20738</v>
       </c>
       <c r="G15" s="9">
-        <v>4520</v>
+        <v>4523</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>100</v>
@@ -1657,7 +1654,7 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>32032</v>
+        <v>32093</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>101</v>
@@ -1669,7 +1666,7 @@
         <v>102</v>
       </c>
       <c r="O15" s="9">
-        <v>129305</v>
+        <v>129577</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>103</v>
@@ -1686,16 +1683,16 @@
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>97168</v>
+        <v>97589</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>106</v>
       </c>
       <c r="F16" s="9">
-        <v>12392</v>
+        <v>12435</v>
       </c>
       <c r="G16" s="9">
-        <v>1978</v>
+        <v>1983</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>107</v>
@@ -1707,7 +1704,7 @@
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>21768</v>
+        <v>21902</v>
       </c>
       <c r="L16" s="10" t="s">
         <v>108</v>
@@ -1719,7 +1716,7 @@
         <v>109</v>
       </c>
       <c r="O16" s="9">
-        <v>109560</v>
+        <v>110024</v>
       </c>
       <c r="P16" s="10" t="s">
         <v>110</v>
@@ -1736,7 +1733,7 @@
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55753</v>
+        <v>55768</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>113</v>
@@ -1757,7 +1754,7 @@
         <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18780</v>
+        <v>18767</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>115</v>
@@ -1769,7 +1766,7 @@
         <v>116</v>
       </c>
       <c r="O17" s="9">
-        <v>67863</v>
+        <v>67878</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>117</v>
@@ -1786,16 +1783,16 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>72755</v>
+        <v>72844</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>120</v>
       </c>
       <c r="F18" s="9">
-        <v>12556</v>
+        <v>12608</v>
       </c>
       <c r="G18" s="9">
-        <v>2405</v>
+        <v>2404</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>121</v>
@@ -1807,7 +1804,7 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22926</v>
+        <v>22935</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>122</v>
@@ -1819,7 +1816,7 @@
         <v>123</v>
       </c>
       <c r="O18" s="9">
-        <v>85311</v>
+        <v>85452</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>124</v>
@@ -1836,16 +1833,16 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33914</v>
+        <v>33934</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>127</v>
       </c>
       <c r="F19" s="9">
-        <v>7315</v>
+        <v>7319</v>
       </c>
       <c r="G19" s="9">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>128</v>
@@ -1857,7 +1854,7 @@
         <v>109</v>
       </c>
       <c r="K19" s="9">
-        <v>7332</v>
+        <v>7327</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>129</v>
@@ -1869,7 +1866,7 @@
         <v>109</v>
       </c>
       <c r="O19" s="9">
-        <v>41229</v>
+        <v>41253</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>130</v>
@@ -1886,28 +1883,28 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>134497</v>
+        <v>134872</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>133</v>
       </c>
       <c r="F20" s="9">
-        <v>37273</v>
+        <v>37358</v>
       </c>
       <c r="G20" s="9">
-        <v>2376</v>
+        <v>2386</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>134</v>
       </c>
       <c r="I20" s="9">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>85023</v>
+        <v>85241</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>135</v>
@@ -1919,7 +1916,7 @@
         <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>171770</v>
+        <v>172230</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>136</v>
@@ -1936,16 +1933,16 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>33760</v>
+        <v>33849</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>139</v>
       </c>
       <c r="F21" s="9">
-        <v>4929</v>
+        <v>4944</v>
       </c>
       <c r="G21" s="9">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>140</v>
@@ -1957,7 +1954,7 @@
         <v>109</v>
       </c>
       <c r="K21" s="9">
-        <v>11546</v>
+        <v>11566</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>141</v>
@@ -1969,7 +1966,7 @@
         <v>81</v>
       </c>
       <c r="O21" s="9">
-        <v>38689</v>
+        <v>38793</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>142</v>
@@ -1986,28 +1983,28 @@
         <v>2730932</v>
       </c>
       <c r="D22" s="12">
-        <v>1777479</v>
+        <v>1783068</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>313219</v>
+        <v>314094</v>
       </c>
       <c r="G22" s="12">
-        <v>48606</v>
+        <v>48686</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1415</v>
+        <v>1433</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>572823</v>
+        <v>574377</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2019,7 +2016,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2090698</v>
+        <v>2097162</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2146,28 +2143,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6280021</v>
+        <v>6299653</v>
       </c>
       <c r="D6" s="6">
-        <v>107602</v>
+        <v>107834</v>
       </c>
       <c r="E6" s="6">
-        <v>67994</v>
+        <v>68219</v>
       </c>
       <c r="F6" s="6">
-        <v>339757</v>
+        <v>340756</v>
       </c>
       <c r="G6" s="6">
-        <v>55174</v>
+        <v>55345</v>
       </c>
       <c r="H6" s="6">
-        <v>9292</v>
+        <v>9307</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6387623</v>
+        <v>6407487</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2178,16 +2175,16 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>245186</v>
+        <v>245022</v>
       </c>
       <c r="D7" s="9">
-        <v>2869</v>
+        <v>2867</v>
       </c>
       <c r="E7" s="9">
         <v>2097</v>
       </c>
       <c r="F7" s="9">
-        <v>13007</v>
+        <v>12987</v>
       </c>
       <c r="G7" s="9">
         <v>305</v>
@@ -2199,7 +2196,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>248055</v>
+        <v>247889</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2210,19 +2207,19 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>437320</v>
+        <v>438790</v>
       </c>
       <c r="D8" s="9">
-        <v>5793</v>
+        <v>5805</v>
       </c>
       <c r="E8" s="9">
-        <v>4302</v>
+        <v>4318</v>
       </c>
       <c r="F8" s="9">
-        <v>33519</v>
+        <v>33620</v>
       </c>
       <c r="G8" s="9">
-        <v>3970</v>
+        <v>3987</v>
       </c>
       <c r="H8" s="9">
         <v>564</v>
@@ -2231,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>443113</v>
+        <v>444595</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2242,28 +2239,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>752353</v>
+        <v>755417</v>
       </c>
       <c r="D9" s="9">
-        <v>13051</v>
+        <v>13091</v>
       </c>
       <c r="E9" s="9">
-        <v>8562</v>
+        <v>8605</v>
       </c>
       <c r="F9" s="9">
-        <v>37416</v>
+        <v>37566</v>
       </c>
       <c r="G9" s="9">
-        <v>4591</v>
+        <v>4614</v>
       </c>
       <c r="H9" s="9">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>765404</v>
+        <v>768508</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2274,28 +2271,28 @@
         <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>777828</v>
+        <v>780317</v>
       </c>
       <c r="D10" s="9">
-        <v>15081</v>
+        <v>15114</v>
       </c>
       <c r="E10" s="9">
-        <v>9140</v>
+        <v>9169</v>
       </c>
       <c r="F10" s="9">
-        <v>38508</v>
+        <v>38618</v>
       </c>
       <c r="G10" s="9">
-        <v>19342</v>
+        <v>19401</v>
       </c>
       <c r="H10" s="9">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>792909</v>
+        <v>795431</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2306,28 +2303,28 @@
         <v>71</v>
       </c>
       <c r="C11" s="9">
-        <v>990808</v>
+        <v>994141</v>
       </c>
       <c r="D11" s="9">
-        <v>20057</v>
+        <v>20109</v>
       </c>
       <c r="E11" s="9">
-        <v>11884</v>
+        <v>11929</v>
       </c>
       <c r="F11" s="9">
-        <v>44654</v>
+        <v>44833</v>
       </c>
       <c r="G11" s="9">
-        <v>8130</v>
+        <v>8163</v>
       </c>
       <c r="H11" s="9">
-        <v>1720</v>
+        <v>1727</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1010865</v>
+        <v>1014250</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2338,28 +2335,28 @@
         <v>78</v>
       </c>
       <c r="C12" s="9">
-        <v>479714</v>
+        <v>481529</v>
       </c>
       <c r="D12" s="9">
-        <v>6128</v>
+        <v>6135</v>
       </c>
       <c r="E12" s="9">
-        <v>5772</v>
+        <v>5793</v>
       </c>
       <c r="F12" s="9">
-        <v>27489</v>
+        <v>27555</v>
       </c>
       <c r="G12" s="9">
-        <v>1959</v>
+        <v>1966</v>
       </c>
       <c r="H12" s="9">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>485842</v>
+        <v>487664</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2370,28 +2367,28 @@
         <v>86</v>
       </c>
       <c r="C13" s="9">
-        <v>342503</v>
+        <v>344179</v>
       </c>
       <c r="D13" s="9">
-        <v>4325</v>
+        <v>4336</v>
       </c>
       <c r="E13" s="9">
-        <v>3884</v>
+        <v>3900</v>
       </c>
       <c r="F13" s="9">
-        <v>24669</v>
+        <v>24769</v>
       </c>
       <c r="G13" s="9">
-        <v>1351</v>
+        <v>1355</v>
       </c>
       <c r="H13" s="9">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>346828</v>
+        <v>348515</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2402,19 +2399,19 @@
         <v>92</v>
       </c>
       <c r="C14" s="9">
-        <v>283409</v>
+        <v>284769</v>
       </c>
       <c r="D14" s="9">
-        <v>8128</v>
+        <v>8150</v>
       </c>
       <c r="E14" s="9">
-        <v>3141</v>
+        <v>3159</v>
       </c>
       <c r="F14" s="9">
-        <v>19319</v>
+        <v>19405</v>
       </c>
       <c r="G14" s="9">
-        <v>1905</v>
+        <v>1910</v>
       </c>
       <c r="H14" s="9">
         <v>340</v>
@@ -2423,7 +2420,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>291537</v>
+        <v>292919</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2434,28 +2431,28 @@
         <v>98</v>
       </c>
       <c r="C15" s="9">
-        <v>389784</v>
+        <v>390603</v>
       </c>
       <c r="D15" s="9">
-        <v>7577</v>
+        <v>7583</v>
       </c>
       <c r="E15" s="9">
-        <v>6375</v>
+        <v>6383</v>
       </c>
       <c r="F15" s="9">
-        <v>26420</v>
+        <v>26469</v>
       </c>
       <c r="G15" s="9">
-        <v>3793</v>
+        <v>3801</v>
       </c>
       <c r="H15" s="9">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>397361</v>
+        <v>398186</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2466,19 +2463,19 @@
         <v>105</v>
       </c>
       <c r="C16" s="9">
-        <v>323768</v>
+        <v>325129</v>
       </c>
       <c r="D16" s="9">
-        <v>4697</v>
+        <v>4710</v>
       </c>
       <c r="E16" s="9">
-        <v>2796</v>
+        <v>2807</v>
       </c>
       <c r="F16" s="9">
-        <v>18865</v>
+        <v>18963</v>
       </c>
       <c r="G16" s="9">
-        <v>3787</v>
+        <v>3795</v>
       </c>
       <c r="H16" s="9">
         <v>253</v>
@@ -2487,7 +2484,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>328465</v>
+        <v>329839</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2498,16 +2495,16 @@
         <v>112</v>
       </c>
       <c r="C17" s="9">
-        <v>196796</v>
+        <v>196837</v>
       </c>
       <c r="D17" s="9">
-        <v>4830</v>
+        <v>4832</v>
       </c>
       <c r="E17" s="9">
         <v>2179</v>
       </c>
       <c r="F17" s="9">
-        <v>10278</v>
+        <v>10281</v>
       </c>
       <c r="G17" s="9">
         <v>1708</v>
@@ -2519,7 +2516,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201626</v>
+        <v>201669</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2530,28 +2527,28 @@
         <v>119</v>
       </c>
       <c r="C18" s="9">
-        <v>246003</v>
+        <v>246413</v>
       </c>
       <c r="D18" s="9">
-        <v>5383</v>
+        <v>5392</v>
       </c>
       <c r="E18" s="9">
-        <v>2627</v>
+        <v>2630</v>
       </c>
       <c r="F18" s="9">
-        <v>14102</v>
+        <v>14136</v>
       </c>
       <c r="G18" s="9">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="H18" s="9">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>251386</v>
+        <v>251805</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2562,16 +2559,16 @@
         <v>126</v>
       </c>
       <c r="C19" s="9">
-        <v>136048</v>
+        <v>136118</v>
       </c>
       <c r="D19" s="9">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="E19" s="9">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="F19" s="9">
-        <v>10376</v>
+        <v>10381</v>
       </c>
       <c r="G19" s="9">
         <v>223</v>
@@ -2583,7 +2580,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>137791</v>
+        <v>137862</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2594,19 +2591,19 @@
         <v>132</v>
       </c>
       <c r="C20" s="9">
-        <v>562609</v>
+        <v>564162</v>
       </c>
       <c r="D20" s="9">
-        <v>6847</v>
+        <v>6868</v>
       </c>
       <c r="E20" s="9">
-        <v>3364</v>
+        <v>3376</v>
       </c>
       <c r="F20" s="9">
-        <v>16120</v>
+        <v>16152</v>
       </c>
       <c r="G20" s="9">
-        <v>997</v>
+        <v>1000</v>
       </c>
       <c r="H20" s="9">
         <v>639</v>
@@ -2615,7 +2612,7 @@
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>569456</v>
+        <v>571030</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2626,28 +2623,28 @@
         <v>138</v>
       </c>
       <c r="C21" s="9">
-        <v>115892</v>
+        <v>116227</v>
       </c>
       <c r="D21" s="9">
-        <v>1093</v>
+        <v>1098</v>
       </c>
       <c r="E21" s="9">
-        <v>830</v>
+        <v>832</v>
       </c>
       <c r="F21" s="9">
-        <v>5015</v>
+        <v>5021</v>
       </c>
       <c r="G21" s="9">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="H21" s="9">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>116985</v>
+        <v>117325</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2658,28 +2655,28 @@
         <v>144</v>
       </c>
       <c r="C22" s="12">
-        <v>6280021</v>
+        <v>6299653</v>
       </c>
       <c r="D22" s="12">
-        <v>107602</v>
+        <v>107834</v>
       </c>
       <c r="E22" s="12">
-        <v>67994</v>
+        <v>68219</v>
       </c>
       <c r="F22" s="12">
-        <v>339757</v>
+        <v>340756</v>
       </c>
       <c r="G22" s="12">
-        <v>55174</v>
+        <v>55345</v>
       </c>
       <c r="H22" s="12">
-        <v>9292</v>
+        <v>9307</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6387623</v>
+        <v>6407487</v>
       </c>
     </row>
   </sheetData>
@@ -2773,10 +2770,10 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1053</v>
+        <v>1065</v>
       </c>
       <c r="D7" s="6">
-        <v>103</v>
+        <v>129</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>157</v>
@@ -2841,10 +2838,10 @@
         <v>65</v>
       </c>
       <c r="C11" s="9">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D11" s="9">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>161</v>
@@ -2858,7 +2855,7 @@
         <v>71</v>
       </c>
       <c r="C12" s="9">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
@@ -2875,10 +2872,10 @@
         <v>78</v>
       </c>
       <c r="C13" s="9">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D13" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>163</v>
@@ -2926,7 +2923,7 @@
         <v>98</v>
       </c>
       <c r="C16" s="9">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D16" s="9">
         <v>41</v>
@@ -2943,7 +2940,7 @@
         <v>105</v>
       </c>
       <c r="C17" s="9">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D17" s="9">
         <v>1</v>
@@ -2980,7 +2977,7 @@
         <v>70</v>
       </c>
       <c r="D19" s="9">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>168</v>
@@ -3017,7 +3014,7 @@
         <v>3</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>169</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3028,13 +3025,13 @@
         <v>138</v>
       </c>
       <c r="C22" s="9">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D22" s="9">
         <v>12</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3045,10 +3042,10 @@
         <v>144</v>
       </c>
       <c r="C23" s="12">
-        <v>1053</v>
+        <v>1065</v>
       </c>
       <c r="D23" s="12">
-        <v>103</v>
+        <v>129</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>157</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 20/08/2026 19:55:56,22
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="171">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 20 Agu 2026, 12.16 | Dicetak: 20 Agu 2026, 13.23</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 20 Agu 2026, 18.16 | Dicetak: 20 Agu 2026, 19.55</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,22 +123,22 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>65,29</t>
-  </si>
-  <si>
-    <t>1,78</t>
+    <t>65,48</t>
+  </si>
+  <si>
+    <t>1,79</t>
   </si>
   <si>
     <t>0,05</t>
   </si>
   <si>
-    <t>21,03</t>
+    <t>21,09</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>76,79</t>
+    <t>77,02</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>78,96</t>
+    <t>79,04</t>
   </si>
   <si>
     <t>1,13</t>
@@ -156,13 +156,13 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>18,32</t>
+    <t>18,35</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>91,77</t>
+    <t>91,82</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>68,18</t>
-  </si>
-  <si>
-    <t>0,98</t>
-  </si>
-  <si>
-    <t>16,87</t>
+    <t>68,36</t>
+  </si>
+  <si>
+    <t>0,99</t>
+  </si>
+  <si>
+    <t>16,93</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>83,08</t>
+    <t>83,29</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,19 +192,19 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>60,16</t>
-  </si>
-  <si>
-    <t>1,19</t>
-  </si>
-  <si>
-    <t>19,64</t>
+    <t>60,39</t>
+  </si>
+  <si>
+    <t>1,2</t>
+  </si>
+  <si>
+    <t>19,71</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>72,39</t>
+    <t>72,67</t>
   </si>
   <si>
     <t>1804</t>
@@ -213,16 +213,16 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>67,06</t>
+    <t>67,3</t>
   </si>
   <si>
     <t>1,88</t>
   </si>
   <si>
-    <t>18,25</t>
-  </si>
-  <si>
-    <t>75,97</t>
+    <t>18,3</t>
+  </si>
+  <si>
+    <t>76,25</t>
   </si>
   <si>
     <t>1805</t>
@@ -231,19 +231,19 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>66,77</t>
-  </si>
-  <si>
-    <t>2,71</t>
-  </si>
-  <si>
-    <t>18,35</t>
+    <t>66,97</t>
+  </si>
+  <si>
+    <t>2,72</t>
+  </si>
+  <si>
+    <t>18,4</t>
   </si>
   <si>
     <t>0,24</t>
   </si>
   <si>
-    <t>75,64</t>
+    <t>75,86</t>
   </si>
   <si>
     <t>1806</t>
@@ -252,7 +252,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>66,4</t>
+    <t>66,55</t>
   </si>
   <si>
     <t>1,95</t>
@@ -261,13 +261,13 @@
     <t>0,02</t>
   </si>
   <si>
-    <t>25,79</t>
+    <t>25,86</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>77,97</t>
+    <t>78,17</t>
   </si>
   <si>
     <t>1807</t>
@@ -276,16 +276,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>67</t>
+    <t>67,21</t>
   </si>
   <si>
     <t>1,69</t>
   </si>
   <si>
-    <t>18,67</t>
-  </si>
-  <si>
-    <t>78,49</t>
+    <t>18,75</t>
+  </si>
+  <si>
+    <t>78,71</t>
   </si>
   <si>
     <t>1808</t>
@@ -294,16 +294,16 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>59,33</t>
-  </si>
-  <si>
-    <t>2,24</t>
-  </si>
-  <si>
-    <t>25,9</t>
-  </si>
-  <si>
-    <t>71,09</t>
+    <t>59,59</t>
+  </si>
+  <si>
+    <t>2,25</t>
+  </si>
+  <si>
+    <t>25,98</t>
+  </si>
+  <si>
+    <t>71,39</t>
   </si>
   <si>
     <t>1809</t>
@@ -312,19 +312,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>71,53</t>
-  </si>
-  <si>
-    <t>2,97</t>
-  </si>
-  <si>
-    <t>21,09</t>
+    <t>71,67</t>
+  </si>
+  <si>
+    <t>2,98</t>
+  </si>
+  <si>
+    <t>21,15</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>85,16</t>
+    <t>85,35</t>
   </si>
   <si>
     <t>1810</t>
@@ -333,19 +333,19 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>71,89</t>
-  </si>
-  <si>
-    <t>1,46</t>
-  </si>
-  <si>
-    <t>16,14</t>
+    <t>72,15</t>
+  </si>
+  <si>
+    <t>1,47</t>
+  </si>
+  <si>
+    <t>16,19</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>81,05</t>
+    <t>81,34</t>
   </si>
   <si>
     <t>1811</t>
@@ -354,7 +354,7 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>74,24</t>
+    <t>74,27</t>
   </si>
   <si>
     <t>1,58</t>
@@ -366,7 +366,7 @@
     <t>0,16</t>
   </si>
   <si>
-    <t>90,37</t>
+    <t>90,4</t>
   </si>
   <si>
     <t>1812</t>
@@ -375,19 +375,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>73,45</t>
-  </si>
-  <si>
-    <t>2,42</t>
-  </si>
-  <si>
-    <t>23,13</t>
+    <t>73,53</t>
+  </si>
+  <si>
+    <t>2,43</t>
+  </si>
+  <si>
+    <t>23,14</t>
   </si>
   <si>
     <t>0,25</t>
   </si>
   <si>
-    <t>86,17</t>
+    <t>86,26</t>
   </si>
   <si>
     <t>1813</t>
@@ -396,7 +396,7 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>81,24</t>
+    <t>81,29</t>
   </si>
   <si>
     <t>0,83</t>
@@ -405,7 +405,7 @@
     <t>17,54</t>
   </si>
   <si>
-    <t>98,76</t>
+    <t>98,91</t>
   </si>
   <si>
     <t>1871</t>
@@ -414,16 +414,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>48,26</t>
-  </si>
-  <si>
-    <t>0,85</t>
-  </si>
-  <si>
-    <t>30,5</t>
-  </si>
-  <si>
-    <t>61,63</t>
+    <t>48,47</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>30,6</t>
+  </si>
+  <si>
+    <t>61,87</t>
   </si>
   <si>
     <t>1872</t>
@@ -432,16 +432,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>63,26</t>
-  </si>
-  <si>
-    <t>1,36</t>
-  </si>
-  <si>
-    <t>21,62</t>
-  </si>
-  <si>
-    <t>72,5</t>
+    <t>63,46</t>
+  </si>
+  <si>
+    <t>1,37</t>
+  </si>
+  <si>
+    <t>21,66</t>
+  </si>
+  <si>
+    <t>72,75</t>
   </si>
   <si>
     <t/>
@@ -486,7 +486,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>12,11</t>
+    <t>12,17</t>
   </si>
   <si>
     <t>0</t>
@@ -495,31 +495,34 @@
     <t>4</t>
   </si>
   <si>
-    <t>4,3</t>
-  </si>
-  <si>
-    <t>23,3</t>
-  </si>
-  <si>
-    <t>6,98</t>
-  </si>
-  <si>
-    <t>17,86</t>
-  </si>
-  <si>
-    <t>2,13</t>
-  </si>
-  <si>
-    <t>26,45</t>
-  </si>
-  <si>
-    <t>2,44</t>
+    <t>4,17</t>
+  </si>
+  <si>
+    <t>23,08</t>
+  </si>
+  <si>
+    <t>6,56</t>
+  </si>
+  <si>
+    <t>17,24</t>
+  </si>
+  <si>
+    <t>2,04</t>
+  </si>
+  <si>
+    <t>26,92</t>
+  </si>
+  <si>
+    <t>4,76</t>
   </si>
   <si>
     <t>28,57</t>
   </si>
   <si>
     <t>24,29</t>
+  </si>
+  <si>
+    <t>3,2</t>
   </si>
   <si>
     <t>19,35</t>
@@ -1183,28 +1186,28 @@
         <v>2730932</v>
       </c>
       <c r="D6" s="6">
-        <v>1783068</v>
+        <v>1788326</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>314094</v>
+        <v>315036</v>
       </c>
       <c r="G6" s="6">
-        <v>48686</v>
+        <v>48805</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1433</v>
+        <v>1436</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>574377</v>
+        <v>576002</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1216,7 +1219,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2097162</v>
+        <v>2103362</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1233,16 +1236,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67233</v>
+        <v>67295</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10904</v>
+        <v>10881</v>
       </c>
       <c r="G7" s="9">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1254,7 +1257,7 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15600</v>
+        <v>15624</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1266,7 +1269,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78137</v>
+        <v>78176</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1283,16 +1286,16 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>117920</v>
+        <v>118227</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>25771</v>
+        <v>25832</v>
       </c>
       <c r="G8" s="9">
-        <v>1700</v>
+        <v>1705</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
@@ -1304,7 +1307,7 @@
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>29181</v>
+        <v>29287</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1316,7 +1319,7 @@
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>143691</v>
+        <v>144059</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1333,28 +1336,28 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>206189</v>
+        <v>206985</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>41926</v>
+        <v>42093</v>
       </c>
       <c r="G9" s="9">
-        <v>4076</v>
+        <v>4096</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>67315</v>
+        <v>67558</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
@@ -1366,7 +1369,7 @@
         <v>62</v>
       </c>
       <c r="O9" s="9">
-        <v>248115</v>
+        <v>249078</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>63</v>
@@ -1383,28 +1386,28 @@
         <v>362838</v>
       </c>
       <c r="D10" s="9">
-        <v>243309</v>
+        <v>244185</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="9">
-        <v>32348</v>
+        <v>32480</v>
       </c>
       <c r="G10" s="9">
-        <v>6811</v>
+        <v>6835</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>67</v>
       </c>
       <c r="I10" s="9">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>66216</v>
+        <v>66390</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>68</v>
@@ -1416,7 +1419,7 @@
         <v>55</v>
       </c>
       <c r="O10" s="9">
-        <v>275657</v>
+        <v>276665</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>69</v>
@@ -1433,28 +1436,28 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>300191</v>
+        <v>301089</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>72</v>
       </c>
       <c r="F11" s="9">
-        <v>39874</v>
+        <v>39978</v>
       </c>
       <c r="G11" s="9">
-        <v>12185</v>
+        <v>12211</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>73</v>
       </c>
       <c r="I11" s="9">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>82504</v>
+        <v>82722</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>74</v>
@@ -1466,7 +1469,7 @@
         <v>75</v>
       </c>
       <c r="O11" s="9">
-        <v>340065</v>
+        <v>341067</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>76</v>
@@ -1483,16 +1486,16 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>132395</v>
+        <v>132696</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>79</v>
       </c>
       <c r="F12" s="9">
-        <v>23081</v>
+        <v>23171</v>
       </c>
       <c r="G12" s="9">
-        <v>3883</v>
+        <v>3886</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>80</v>
@@ -1504,7 +1507,7 @@
         <v>81</v>
       </c>
       <c r="K12" s="9">
-        <v>51420</v>
+        <v>51561</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>82</v>
@@ -1516,7 +1519,7 @@
         <v>83</v>
       </c>
       <c r="O12" s="9">
-        <v>155476</v>
+        <v>155867</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>84</v>
@@ -1533,16 +1536,16 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>97885</v>
+        <v>98184</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>87</v>
       </c>
       <c r="F13" s="9">
-        <v>16780</v>
+        <v>16812</v>
       </c>
       <c r="G13" s="9">
-        <v>2472</v>
+        <v>2476</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>88</v>
@@ -1554,7 +1557,7 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>27282</v>
+        <v>27394</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>89</v>
@@ -1566,7 +1569,7 @@
         <v>83</v>
       </c>
       <c r="O13" s="9">
-        <v>114665</v>
+        <v>114996</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>90</v>
@@ -1583,16 +1586,16 @@
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>80251</v>
+        <v>80593</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>93</v>
       </c>
       <c r="F14" s="9">
-        <v>15898</v>
+        <v>15973</v>
       </c>
       <c r="G14" s="9">
-        <v>3036</v>
+        <v>3045</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>94</v>
@@ -1604,7 +1607,7 @@
         <v>81</v>
       </c>
       <c r="K14" s="9">
-        <v>35028</v>
+        <v>35135</v>
       </c>
       <c r="L14" s="10" t="s">
         <v>95</v>
@@ -1616,7 +1619,7 @@
         <v>81</v>
       </c>
       <c r="O14" s="9">
-        <v>96149</v>
+        <v>96566</v>
       </c>
       <c r="P14" s="10" t="s">
         <v>96</v>
@@ -1633,16 +1636,16 @@
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>108839</v>
+        <v>109051</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>99</v>
       </c>
       <c r="F15" s="9">
-        <v>20738</v>
+        <v>20813</v>
       </c>
       <c r="G15" s="9">
-        <v>4523</v>
+        <v>4533</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>100</v>
@@ -1654,7 +1657,7 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>32093</v>
+        <v>32187</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>101</v>
@@ -1666,7 +1669,7 @@
         <v>102</v>
       </c>
       <c r="O15" s="9">
-        <v>129577</v>
+        <v>129864</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>103</v>
@@ -1683,16 +1686,16 @@
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>97589</v>
+        <v>97933</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>106</v>
       </c>
       <c r="F16" s="9">
-        <v>12435</v>
+        <v>12480</v>
       </c>
       <c r="G16" s="9">
-        <v>1983</v>
+        <v>1989</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>107</v>
@@ -1704,7 +1707,7 @@
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>21902</v>
+        <v>21981</v>
       </c>
       <c r="L16" s="10" t="s">
         <v>108</v>
@@ -1716,7 +1719,7 @@
         <v>109</v>
       </c>
       <c r="O16" s="9">
-        <v>110024</v>
+        <v>110413</v>
       </c>
       <c r="P16" s="10" t="s">
         <v>110</v>
@@ -1733,13 +1736,13 @@
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55768</v>
+        <v>55789</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>113</v>
       </c>
       <c r="F17" s="9">
-        <v>12110</v>
+        <v>12115</v>
       </c>
       <c r="G17" s="9">
         <v>1187</v>
@@ -1754,7 +1757,7 @@
         <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18767</v>
+        <v>18764</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>115</v>
@@ -1766,7 +1769,7 @@
         <v>116</v>
       </c>
       <c r="O17" s="9">
-        <v>67878</v>
+        <v>67904</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>117</v>
@@ -1783,16 +1786,16 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>72844</v>
+        <v>72920</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>120</v>
       </c>
       <c r="F18" s="9">
-        <v>12608</v>
+        <v>12626</v>
       </c>
       <c r="G18" s="9">
-        <v>2404</v>
+        <v>2405</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>121</v>
@@ -1804,7 +1807,7 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22935</v>
+        <v>22952</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>122</v>
@@ -1816,7 +1819,7 @@
         <v>123</v>
       </c>
       <c r="O18" s="9">
-        <v>85452</v>
+        <v>85546</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>124</v>
@@ -1833,13 +1836,13 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33934</v>
+        <v>33957</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>127</v>
       </c>
       <c r="F19" s="9">
-        <v>7319</v>
+        <v>7358</v>
       </c>
       <c r="G19" s="9">
         <v>348</v>
@@ -1854,7 +1857,7 @@
         <v>109</v>
       </c>
       <c r="K19" s="9">
-        <v>7327</v>
+        <v>7325</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>129</v>
@@ -1866,7 +1869,7 @@
         <v>109</v>
       </c>
       <c r="O19" s="9">
-        <v>41253</v>
+        <v>41315</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>130</v>
@@ -1883,16 +1886,16 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>134872</v>
+        <v>135468</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>133</v>
       </c>
       <c r="F20" s="9">
-        <v>37358</v>
+        <v>37455</v>
       </c>
       <c r="G20" s="9">
-        <v>2386</v>
+        <v>2393</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>134</v>
@@ -1904,7 +1907,7 @@
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>85241</v>
+        <v>85530</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>135</v>
@@ -1916,7 +1919,7 @@
         <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>172230</v>
+        <v>172923</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>136</v>
@@ -1933,16 +1936,16 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>33849</v>
+        <v>33954</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>139</v>
       </c>
       <c r="F21" s="9">
-        <v>4944</v>
+        <v>4969</v>
       </c>
       <c r="G21" s="9">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>140</v>
@@ -1954,7 +1957,7 @@
         <v>109</v>
       </c>
       <c r="K21" s="9">
-        <v>11566</v>
+        <v>11592</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>141</v>
@@ -1966,7 +1969,7 @@
         <v>81</v>
       </c>
       <c r="O21" s="9">
-        <v>38793</v>
+        <v>38923</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>142</v>
@@ -1983,28 +1986,28 @@
         <v>2730932</v>
       </c>
       <c r="D22" s="12">
-        <v>1783068</v>
+        <v>1788326</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>314094</v>
+        <v>315036</v>
       </c>
       <c r="G22" s="12">
-        <v>48686</v>
+        <v>48805</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1433</v>
+        <v>1436</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>574377</v>
+        <v>576002</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2016,7 +2019,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2097162</v>
+        <v>2103362</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2143,28 +2146,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6299653</v>
+        <v>6318247</v>
       </c>
       <c r="D6" s="6">
-        <v>107834</v>
+        <v>108035</v>
       </c>
       <c r="E6" s="6">
-        <v>68219</v>
+        <v>68421</v>
       </c>
       <c r="F6" s="6">
-        <v>340756</v>
+        <v>341699</v>
       </c>
       <c r="G6" s="6">
-        <v>55345</v>
+        <v>55532</v>
       </c>
       <c r="H6" s="6">
-        <v>9307</v>
+        <v>9320</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6407487</v>
+        <v>6426282</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2175,16 +2178,16 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>245022</v>
+        <v>245111</v>
       </c>
       <c r="D7" s="9">
-        <v>2867</v>
+        <v>2859</v>
       </c>
       <c r="E7" s="9">
-        <v>2097</v>
+        <v>2095</v>
       </c>
       <c r="F7" s="9">
-        <v>12987</v>
+        <v>12988</v>
       </c>
       <c r="G7" s="9">
         <v>305</v>
@@ -2196,7 +2199,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>247889</v>
+        <v>247970</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2207,19 +2210,19 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>438790</v>
+        <v>439926</v>
       </c>
       <c r="D8" s="9">
-        <v>5805</v>
+        <v>5814</v>
       </c>
       <c r="E8" s="9">
-        <v>4318</v>
+        <v>4326</v>
       </c>
       <c r="F8" s="9">
-        <v>33620</v>
+        <v>33716</v>
       </c>
       <c r="G8" s="9">
-        <v>3987</v>
+        <v>4007</v>
       </c>
       <c r="H8" s="9">
         <v>564</v>
@@ -2228,7 +2231,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>444595</v>
+        <v>445740</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2239,28 +2242,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>755417</v>
+        <v>758395</v>
       </c>
       <c r="D9" s="9">
-        <v>13091</v>
+        <v>13123</v>
       </c>
       <c r="E9" s="9">
-        <v>8605</v>
+        <v>8650</v>
       </c>
       <c r="F9" s="9">
-        <v>37566</v>
+        <v>37720</v>
       </c>
       <c r="G9" s="9">
-        <v>4614</v>
+        <v>4633</v>
       </c>
       <c r="H9" s="9">
-        <v>998</v>
+        <v>1001</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>768508</v>
+        <v>771518</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2271,19 +2274,19 @@
         <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>780317</v>
+        <v>783157</v>
       </c>
       <c r="D10" s="9">
-        <v>15114</v>
+        <v>15136</v>
       </c>
       <c r="E10" s="9">
-        <v>9169</v>
+        <v>9209</v>
       </c>
       <c r="F10" s="9">
-        <v>38618</v>
+        <v>38733</v>
       </c>
       <c r="G10" s="9">
-        <v>19401</v>
+        <v>19486</v>
       </c>
       <c r="H10" s="9">
         <v>1065</v>
@@ -2292,7 +2295,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>795431</v>
+        <v>798293</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2303,28 +2306,28 @@
         <v>71</v>
       </c>
       <c r="C11" s="9">
-        <v>994141</v>
+        <v>997096</v>
       </c>
       <c r="D11" s="9">
-        <v>20109</v>
+        <v>20151</v>
       </c>
       <c r="E11" s="9">
-        <v>11929</v>
+        <v>11966</v>
       </c>
       <c r="F11" s="9">
-        <v>44833</v>
+        <v>44959</v>
       </c>
       <c r="G11" s="9">
-        <v>8163</v>
+        <v>8189</v>
       </c>
       <c r="H11" s="9">
-        <v>1727</v>
+        <v>1730</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1014250</v>
+        <v>1017247</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2335,28 +2338,28 @@
         <v>78</v>
       </c>
       <c r="C12" s="9">
-        <v>481529</v>
+        <v>482748</v>
       </c>
       <c r="D12" s="9">
-        <v>6135</v>
+        <v>6141</v>
       </c>
       <c r="E12" s="9">
-        <v>5793</v>
+        <v>5808</v>
       </c>
       <c r="F12" s="9">
-        <v>27555</v>
+        <v>27636</v>
       </c>
       <c r="G12" s="9">
-        <v>1966</v>
+        <v>1969</v>
       </c>
       <c r="H12" s="9">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>487664</v>
+        <v>488889</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2367,28 +2370,28 @@
         <v>86</v>
       </c>
       <c r="C13" s="9">
-        <v>344179</v>
+        <v>345214</v>
       </c>
       <c r="D13" s="9">
-        <v>4336</v>
+        <v>4344</v>
       </c>
       <c r="E13" s="9">
-        <v>3900</v>
+        <v>3912</v>
       </c>
       <c r="F13" s="9">
-        <v>24769</v>
+        <v>24827</v>
       </c>
       <c r="G13" s="9">
-        <v>1355</v>
+        <v>1357</v>
       </c>
       <c r="H13" s="9">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>348515</v>
+        <v>349558</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2399,28 +2402,28 @@
         <v>92</v>
       </c>
       <c r="C14" s="9">
-        <v>284769</v>
+        <v>286015</v>
       </c>
       <c r="D14" s="9">
-        <v>8150</v>
+        <v>8184</v>
       </c>
       <c r="E14" s="9">
-        <v>3159</v>
+        <v>3164</v>
       </c>
       <c r="F14" s="9">
-        <v>19405</v>
+        <v>19477</v>
       </c>
       <c r="G14" s="9">
-        <v>1910</v>
+        <v>1917</v>
       </c>
       <c r="H14" s="9">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>292919</v>
+        <v>294199</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2431,28 +2434,28 @@
         <v>98</v>
       </c>
       <c r="C15" s="9">
-        <v>390603</v>
+        <v>391457</v>
       </c>
       <c r="D15" s="9">
-        <v>7583</v>
+        <v>7601</v>
       </c>
       <c r="E15" s="9">
-        <v>6383</v>
+        <v>6393</v>
       </c>
       <c r="F15" s="9">
-        <v>26469</v>
+        <v>26529</v>
       </c>
       <c r="G15" s="9">
-        <v>3801</v>
+        <v>3805</v>
       </c>
       <c r="H15" s="9">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>398186</v>
+        <v>399058</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2463,28 +2466,28 @@
         <v>105</v>
       </c>
       <c r="C16" s="9">
-        <v>325129</v>
+        <v>326270</v>
       </c>
       <c r="D16" s="9">
-        <v>4710</v>
+        <v>4729</v>
       </c>
       <c r="E16" s="9">
-        <v>2807</v>
+        <v>2820</v>
       </c>
       <c r="F16" s="9">
-        <v>18963</v>
+        <v>19029</v>
       </c>
       <c r="G16" s="9">
-        <v>3795</v>
+        <v>3809</v>
       </c>
       <c r="H16" s="9">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>329839</v>
+        <v>330999</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2495,7 +2498,7 @@
         <v>112</v>
       </c>
       <c r="C17" s="9">
-        <v>196837</v>
+        <v>196923</v>
       </c>
       <c r="D17" s="9">
         <v>4832</v>
@@ -2516,7 +2519,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201669</v>
+        <v>201755</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2527,19 +2530,19 @@
         <v>119</v>
       </c>
       <c r="C18" s="9">
-        <v>246413</v>
+        <v>246681</v>
       </c>
       <c r="D18" s="9">
-        <v>5392</v>
+        <v>5398</v>
       </c>
       <c r="E18" s="9">
-        <v>2630</v>
+        <v>2632</v>
       </c>
       <c r="F18" s="9">
-        <v>14136</v>
+        <v>14159</v>
       </c>
       <c r="G18" s="9">
-        <v>2373</v>
+        <v>2375</v>
       </c>
       <c r="H18" s="9">
         <v>492</v>
@@ -2548,7 +2551,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>251805</v>
+        <v>252079</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2559,13 +2562,13 @@
         <v>126</v>
       </c>
       <c r="C19" s="9">
-        <v>136118</v>
+        <v>136235</v>
       </c>
       <c r="D19" s="9">
-        <v>1744</v>
+        <v>1745</v>
       </c>
       <c r="E19" s="9">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="F19" s="9">
         <v>10381</v>
@@ -2580,7 +2583,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>137862</v>
+        <v>137980</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2591,28 +2594,28 @@
         <v>132</v>
       </c>
       <c r="C20" s="9">
-        <v>564162</v>
+        <v>566387</v>
       </c>
       <c r="D20" s="9">
-        <v>6868</v>
+        <v>6880</v>
       </c>
       <c r="E20" s="9">
-        <v>3376</v>
+        <v>3389</v>
       </c>
       <c r="F20" s="9">
-        <v>16152</v>
+        <v>16218</v>
       </c>
       <c r="G20" s="9">
-        <v>1000</v>
+        <v>1002</v>
       </c>
       <c r="H20" s="9">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>571030</v>
+        <v>573267</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2623,28 +2626,28 @@
         <v>138</v>
       </c>
       <c r="C21" s="9">
-        <v>116227</v>
+        <v>116632</v>
       </c>
       <c r="D21" s="9">
         <v>1098</v>
       </c>
       <c r="E21" s="9">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="F21" s="9">
-        <v>5021</v>
+        <v>5046</v>
       </c>
       <c r="G21" s="9">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="H21" s="9">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>117325</v>
+        <v>117730</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2655,28 +2658,28 @@
         <v>144</v>
       </c>
       <c r="C22" s="12">
-        <v>6299653</v>
+        <v>6318247</v>
       </c>
       <c r="D22" s="12">
-        <v>107834</v>
+        <v>108035</v>
       </c>
       <c r="E22" s="12">
-        <v>68219</v>
+        <v>68421</v>
       </c>
       <c r="F22" s="12">
-        <v>340756</v>
+        <v>341699</v>
       </c>
       <c r="G22" s="12">
-        <v>55345</v>
+        <v>55532</v>
       </c>
       <c r="H22" s="12">
-        <v>9307</v>
+        <v>9320</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6407487</v>
+        <v>6426282</v>
       </c>
     </row>
   </sheetData>
@@ -2770,10 +2773,10 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1065</v>
+        <v>1085</v>
       </c>
       <c r="D7" s="6">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>157</v>
@@ -2787,7 +2790,7 @@
         <v>43</v>
       </c>
       <c r="C8" s="9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D8" s="9">
         <v>0</v>
@@ -2821,7 +2824,7 @@
         <v>58</v>
       </c>
       <c r="C10" s="9">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D10" s="9">
         <v>4</v>
@@ -2838,7 +2841,7 @@
         <v>65</v>
       </c>
       <c r="C11" s="9">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" s="9">
         <v>24</v>
@@ -2855,7 +2858,7 @@
         <v>71</v>
       </c>
       <c r="C12" s="9">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
@@ -2872,7 +2875,7 @@
         <v>78</v>
       </c>
       <c r="C13" s="9">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13" s="9">
         <v>5</v>
@@ -2889,7 +2892,7 @@
         <v>86</v>
       </c>
       <c r="C14" s="9">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D14" s="9">
         <v>1</v>
@@ -2923,10 +2926,10 @@
         <v>98</v>
       </c>
       <c r="C16" s="9">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D16" s="9">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>165</v>
@@ -2940,10 +2943,10 @@
         <v>105</v>
       </c>
       <c r="C17" s="9">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D17" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>166</v>
@@ -3008,13 +3011,13 @@
         <v>132</v>
       </c>
       <c r="C21" s="9">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D21" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>121</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3031,7 +3034,7 @@
         <v>12</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3042,10 +3045,10 @@
         <v>144</v>
       </c>
       <c r="C23" s="12">
-        <v>1065</v>
+        <v>1085</v>
       </c>
       <c r="D23" s="12">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>157</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 21/08/2026  7:22:13,74
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="172">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 20 Agu 2026, 18.16 | Dicetak: 20 Agu 2026, 19.55</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 21 Agu 2026, 06.16 | Dicetak: 21 Agu 2026, 07.20</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,7 +123,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>65,48</t>
+    <t>65,87</t>
   </si>
   <si>
     <t>1,79</t>
@@ -132,13 +132,13 @@
     <t>0,05</t>
   </si>
   <si>
-    <t>21,09</t>
+    <t>21,19</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>77,02</t>
+    <t>77,47</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>79,04</t>
+    <t>79,2</t>
   </si>
   <si>
     <t>1,13</t>
@@ -156,13 +156,13 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>18,35</t>
+    <t>18,38</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>91,82</t>
+    <t>92,02</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>68,36</t>
+    <t>68,72</t>
   </si>
   <si>
     <t>0,99</t>
   </si>
   <si>
-    <t>16,93</t>
+    <t>17,05</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>83,29</t>
+    <t>83,74</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,19 +192,19 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>60,39</t>
+    <t>60,91</t>
   </si>
   <si>
     <t>1,2</t>
   </si>
   <si>
-    <t>19,71</t>
+    <t>19,86</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>72,67</t>
+    <t>73,29</t>
   </si>
   <si>
     <t>1804</t>
@@ -213,16 +213,19 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>67,3</t>
-  </si>
-  <si>
-    <t>1,88</t>
-  </si>
-  <si>
-    <t>18,3</t>
-  </si>
-  <si>
-    <t>76,25</t>
+    <t>67,74</t>
+  </si>
+  <si>
+    <t>1,89</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>18,37</t>
+  </si>
+  <si>
+    <t>76,75</t>
   </si>
   <si>
     <t>1805</t>
@@ -231,19 +234,19 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>66,97</t>
+    <t>67,38</t>
   </si>
   <si>
     <t>2,72</t>
   </si>
   <si>
-    <t>18,4</t>
+    <t>18,49</t>
   </si>
   <si>
     <t>0,24</t>
   </si>
   <si>
-    <t>75,86</t>
+    <t>76,33</t>
   </si>
   <si>
     <t>1806</t>
@@ -252,7 +255,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>66,55</t>
+    <t>66,83</t>
   </si>
   <si>
     <t>1,95</t>
@@ -261,13 +264,13 @@
     <t>0,02</t>
   </si>
   <si>
-    <t>25,86</t>
+    <t>25,93</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>78,17</t>
+    <t>78,51</t>
   </si>
   <si>
     <t>1807</t>
@@ -276,16 +279,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>67,21</t>
-  </si>
-  <si>
-    <t>1,69</t>
-  </si>
-  <si>
-    <t>18,75</t>
-  </si>
-  <si>
-    <t>78,71</t>
+    <t>67,66</t>
+  </si>
+  <si>
+    <t>1,7</t>
+  </si>
+  <si>
+    <t>18,83</t>
+  </si>
+  <si>
+    <t>79,24</t>
   </si>
   <si>
     <t>1808</t>
@@ -294,16 +297,19 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>59,59</t>
+    <t>60,12</t>
   </si>
   <si>
     <t>2,25</t>
   </si>
   <si>
-    <t>25,98</t>
-  </si>
-  <si>
-    <t>71,39</t>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>26,06</t>
+  </si>
+  <si>
+    <t>72,02</t>
   </si>
   <si>
     <t>1809</t>
@@ -312,19 +318,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>71,67</t>
+    <t>72</t>
   </si>
   <si>
     <t>2,98</t>
   </si>
   <si>
-    <t>21,15</t>
+    <t>21,28</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>85,35</t>
+    <t>85,76</t>
   </si>
   <si>
     <t>1810</t>
@@ -333,19 +339,16 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>72,15</t>
+    <t>72,55</t>
   </si>
   <si>
     <t>1,47</t>
   </si>
   <si>
-    <t>16,19</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>81,34</t>
+    <t>16,27</t>
+  </si>
+  <si>
+    <t>81,81</t>
   </si>
   <si>
     <t>1811</t>
@@ -366,7 +369,7 @@
     <t>0,16</t>
   </si>
   <si>
-    <t>90,4</t>
+    <t>90,42</t>
   </si>
   <si>
     <t>1812</t>
@@ -375,19 +378,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>73,53</t>
-  </si>
-  <si>
-    <t>2,43</t>
-  </si>
-  <si>
-    <t>23,14</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>86,26</t>
+    <t>73,76</t>
+  </si>
+  <si>
+    <t>2,42</t>
+  </si>
+  <si>
+    <t>23,15</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>86,54</t>
   </si>
   <si>
     <t>1813</t>
@@ -396,16 +399,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>81,29</t>
-  </si>
-  <si>
-    <t>0,83</t>
+    <t>81,36</t>
+  </si>
+  <si>
+    <t>0,84</t>
   </si>
   <si>
     <t>17,54</t>
   </si>
   <si>
-    <t>98,91</t>
+    <t>99,01</t>
   </si>
   <si>
     <t>1871</t>
@@ -414,16 +417,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>48,47</t>
+    <t>48,86</t>
   </si>
   <si>
     <t>0,86</t>
   </si>
   <si>
-    <t>30,6</t>
-  </si>
-  <si>
-    <t>61,87</t>
+    <t>30,77</t>
+  </si>
+  <si>
+    <t>62,35</t>
   </si>
   <si>
     <t>1872</t>
@@ -432,16 +435,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>63,46</t>
+    <t>63,71</t>
   </si>
   <si>
     <t>1,37</t>
   </si>
   <si>
-    <t>21,66</t>
-  </si>
-  <si>
-    <t>72,75</t>
+    <t>21,74</t>
+  </si>
+  <si>
+    <t>73,08</t>
   </si>
   <si>
     <t/>
@@ -486,7 +489,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>12,17</t>
+    <t>12,1</t>
   </si>
   <si>
     <t>0</t>
@@ -495,25 +498,25 @@
     <t>4</t>
   </si>
   <si>
-    <t>4,17</t>
-  </si>
-  <si>
-    <t>23,08</t>
-  </si>
-  <si>
-    <t>6,56</t>
-  </si>
-  <si>
-    <t>17,24</t>
-  </si>
-  <si>
-    <t>2,04</t>
-  </si>
-  <si>
-    <t>26,92</t>
-  </si>
-  <si>
-    <t>4,76</t>
+    <t>4,12</t>
+  </si>
+  <si>
+    <t>22,02</t>
+  </si>
+  <si>
+    <t>6,52</t>
+  </si>
+  <si>
+    <t>16,67</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>27,56</t>
+  </si>
+  <si>
+    <t>4,44</t>
   </si>
   <si>
     <t>28,57</t>
@@ -522,7 +525,7 @@
     <t>24,29</t>
   </si>
   <si>
-    <t>3,2</t>
+    <t>3,15</t>
   </si>
   <si>
     <t>19,35</t>
@@ -1183,43 +1186,43 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>2730932</v>
+        <v>2730933</v>
       </c>
       <c r="D6" s="6">
-        <v>1788326</v>
+        <v>1798816</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>315036</v>
+        <v>316902</v>
       </c>
       <c r="G6" s="6">
-        <v>48805</v>
+        <v>48897</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1436</v>
+        <v>1437</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>576002</v>
+        <v>578575</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
       </c>
       <c r="M6" s="6">
-        <v>2959</v>
+        <v>3042</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2103362</v>
+        <v>2115718</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1236,16 +1239,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67295</v>
+        <v>67433</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10881</v>
+        <v>10914</v>
       </c>
       <c r="G7" s="9">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1257,19 +1260,19 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15624</v>
+        <v>15647</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
       </c>
       <c r="M7" s="9">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N7" s="10" t="s">
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78176</v>
+        <v>78347</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1286,16 +1289,16 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>118227</v>
+        <v>118850</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>25832</v>
+        <v>25985</v>
       </c>
       <c r="G8" s="9">
-        <v>1705</v>
+        <v>1711</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
@@ -1307,19 +1310,19 @@
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>29287</v>
+        <v>29489</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
       </c>
       <c r="M8" s="9">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N8" s="10" t="s">
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>144059</v>
+        <v>144835</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1336,40 +1339,40 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>206985</v>
+        <v>208769</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>42093</v>
+        <v>42418</v>
       </c>
       <c r="G9" s="9">
-        <v>4096</v>
+        <v>4113</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>67558</v>
+        <v>68061</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
       </c>
       <c r="M9" s="9">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="N9" s="10" t="s">
         <v>62</v>
       </c>
       <c r="O9" s="9">
-        <v>249078</v>
+        <v>251187</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>63</v>
@@ -1383,172 +1386,172 @@
         <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>362838</v>
+        <v>362839</v>
       </c>
       <c r="D10" s="9">
-        <v>244185</v>
+        <v>245805</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="9">
-        <v>32480</v>
+        <v>32682</v>
       </c>
       <c r="G10" s="9">
-        <v>6835</v>
+        <v>6848</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>67</v>
       </c>
       <c r="I10" s="9">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="K10" s="9">
-        <v>66390</v>
+        <v>66665</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="M10" s="9">
-        <v>259</v>
+        <v>278</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="O10" s="9">
-        <v>276665</v>
+        <v>278487</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C11" s="9">
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>301089</v>
+        <v>302937</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F11" s="9">
-        <v>39978</v>
+        <v>40216</v>
       </c>
       <c r="G11" s="9">
-        <v>12211</v>
+        <v>12233</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I11" s="9">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>82722</v>
+        <v>83130</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M11" s="9">
-        <v>1062</v>
+        <v>1090</v>
       </c>
       <c r="N11" s="10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O11" s="9">
-        <v>341067</v>
+        <v>343153</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C12" s="9">
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>132696</v>
+        <v>133264</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F12" s="9">
-        <v>23171</v>
+        <v>23287</v>
       </c>
       <c r="G12" s="9">
-        <v>3886</v>
+        <v>3889</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I12" s="9">
         <v>49</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K12" s="9">
-        <v>51561</v>
+        <v>51707</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="M12" s="9">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="N12" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O12" s="9">
-        <v>155867</v>
+        <v>156551</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C13" s="9">
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>98184</v>
+        <v>98853</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F13" s="9">
-        <v>16812</v>
+        <v>16912</v>
       </c>
       <c r="G13" s="9">
-        <v>2476</v>
+        <v>2478</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I13" s="9">
         <v>79</v>
@@ -1557,180 +1560,180 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>27394</v>
+        <v>27504</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M13" s="9">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="N13" s="10" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="O13" s="9">
-        <v>114996</v>
+        <v>115765</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C14" s="9">
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>80593</v>
+        <v>81315</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F14" s="9">
-        <v>15973</v>
+        <v>16098</v>
       </c>
       <c r="G14" s="9">
-        <v>3045</v>
+        <v>3050</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I14" s="9">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="K14" s="9">
-        <v>35135</v>
+        <v>35242</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M14" s="9">
         <v>24</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O14" s="9">
-        <v>96566</v>
+        <v>97413</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C15" s="9">
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>109051</v>
+        <v>109555</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F15" s="9">
-        <v>20813</v>
+        <v>20936</v>
       </c>
       <c r="G15" s="9">
-        <v>4533</v>
+        <v>4541</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I15" s="9">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J15" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>32187</v>
+        <v>32382</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="M15" s="9">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="O15" s="9">
-        <v>129864</v>
+        <v>130491</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C16" s="9">
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>97933</v>
+        <v>98478</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F16" s="9">
-        <v>12480</v>
+        <v>12566</v>
       </c>
       <c r="G16" s="9">
-        <v>1989</v>
+        <v>1996</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I16" s="9">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>21981</v>
+        <v>22081</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="M16" s="9">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="O16" s="9">
-        <v>110413</v>
+        <v>111044</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" s="9">
         <v>75115</v>
@@ -1739,16 +1742,16 @@
         <v>55789</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F17" s="9">
-        <v>12115</v>
+        <v>12130</v>
       </c>
       <c r="G17" s="9">
         <v>1187</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I17" s="9">
         <v>80</v>
@@ -1757,48 +1760,48 @@
         <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18764</v>
+        <v>18765</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M17" s="9">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O17" s="9">
-        <v>67904</v>
+        <v>67919</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C18" s="9">
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>72920</v>
+        <v>73151</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F18" s="9">
-        <v>12626</v>
+        <v>12673</v>
       </c>
       <c r="G18" s="9">
-        <v>2405</v>
+        <v>2404</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I18" s="9">
         <v>49</v>
@@ -1807,98 +1810,98 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22952</v>
+        <v>22956</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="M18" s="9">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="N18" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O18" s="9">
-        <v>85546</v>
+        <v>85824</v>
       </c>
       <c r="P18" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C19" s="9">
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33957</v>
+        <v>33986</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F19" s="9">
-        <v>7358</v>
+        <v>7372</v>
       </c>
       <c r="G19" s="9">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I19" s="9">
         <v>27</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="K19" s="9">
         <v>7325</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="M19" s="9">
         <v>27</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="O19" s="9">
-        <v>41315</v>
+        <v>41358</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C20" s="9">
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>135468</v>
+        <v>136541</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F20" s="9">
-        <v>37455</v>
+        <v>37700</v>
       </c>
       <c r="G20" s="9">
-        <v>2393</v>
+        <v>2401</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I20" s="9">
         <v>136</v>
@@ -1907,119 +1910,119 @@
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>85530</v>
+        <v>85990</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M20" s="9">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="N20" s="10" t="s">
         <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>172923</v>
+        <v>174241</v>
       </c>
       <c r="P20" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C21" s="9">
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>33954</v>
+        <v>34090</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F21" s="9">
-        <v>4969</v>
+        <v>5013</v>
       </c>
       <c r="G21" s="9">
         <v>732</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I21" s="9">
         <v>33</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="K21" s="9">
-        <v>11592</v>
+        <v>11631</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M21" s="9">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O21" s="9">
-        <v>38923</v>
+        <v>39103</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C22" s="12">
-        <v>2730932</v>
+        <v>2730933</v>
       </c>
       <c r="D22" s="12">
-        <v>1788326</v>
+        <v>1798816</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>315036</v>
+        <v>316902</v>
       </c>
       <c r="G22" s="12">
-        <v>48805</v>
+        <v>48897</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1436</v>
+        <v>1437</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>576002</v>
+        <v>578575</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
       </c>
       <c r="M22" s="12">
-        <v>2959</v>
+        <v>3042</v>
       </c>
       <c r="N22" s="13" t="s">
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2103362</v>
+        <v>2115718</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2048,7 +2051,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2082,28 +2085,28 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2146,28 +2149,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6318247</v>
+        <v>6355459</v>
       </c>
       <c r="D6" s="6">
-        <v>108035</v>
+        <v>108505</v>
       </c>
       <c r="E6" s="6">
-        <v>68421</v>
+        <v>68807</v>
       </c>
       <c r="F6" s="6">
-        <v>341699</v>
+        <v>343590</v>
       </c>
       <c r="G6" s="6">
-        <v>55532</v>
+        <v>55877</v>
       </c>
       <c r="H6" s="6">
-        <v>9320</v>
+        <v>9346</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6426282</v>
+        <v>6463964</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2178,16 +2181,16 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>245111</v>
+        <v>245643</v>
       </c>
       <c r="D7" s="9">
         <v>2859</v>
       </c>
       <c r="E7" s="9">
-        <v>2095</v>
+        <v>2101</v>
       </c>
       <c r="F7" s="9">
-        <v>12988</v>
+        <v>13025</v>
       </c>
       <c r="G7" s="9">
         <v>305</v>
@@ -2199,7 +2202,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>247970</v>
+        <v>248502</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2210,28 +2213,28 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>439926</v>
+        <v>442315</v>
       </c>
       <c r="D8" s="9">
-        <v>5814</v>
+        <v>5838</v>
       </c>
       <c r="E8" s="9">
-        <v>4326</v>
+        <v>4346</v>
       </c>
       <c r="F8" s="9">
-        <v>33716</v>
+        <v>33917</v>
       </c>
       <c r="G8" s="9">
-        <v>4007</v>
+        <v>4040</v>
       </c>
       <c r="H8" s="9">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="I8" s="9">
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>445740</v>
+        <v>448153</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2242,28 +2245,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>758395</v>
+        <v>764792</v>
       </c>
       <c r="D9" s="9">
-        <v>13123</v>
+        <v>13218</v>
       </c>
       <c r="E9" s="9">
-        <v>8650</v>
+        <v>8718</v>
       </c>
       <c r="F9" s="9">
-        <v>37720</v>
+        <v>38012</v>
       </c>
       <c r="G9" s="9">
-        <v>4633</v>
+        <v>4670</v>
       </c>
       <c r="H9" s="9">
-        <v>1001</v>
+        <v>1005</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>771518</v>
+        <v>778010</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2274,240 +2277,240 @@
         <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>783157</v>
+        <v>788213</v>
       </c>
       <c r="D10" s="9">
-        <v>15136</v>
+        <v>15207</v>
       </c>
       <c r="E10" s="9">
-        <v>9209</v>
+        <v>9277</v>
       </c>
       <c r="F10" s="9">
-        <v>38733</v>
+        <v>38979</v>
       </c>
       <c r="G10" s="9">
-        <v>19486</v>
+        <v>19626</v>
       </c>
       <c r="H10" s="9">
-        <v>1065</v>
+        <v>1067</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>798293</v>
+        <v>803420</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C11" s="9">
-        <v>997096</v>
+        <v>1003298</v>
       </c>
       <c r="D11" s="9">
-        <v>20151</v>
+        <v>20226</v>
       </c>
       <c r="E11" s="9">
-        <v>11966</v>
+        <v>12028</v>
       </c>
       <c r="F11" s="9">
-        <v>44959</v>
+        <v>45203</v>
       </c>
       <c r="G11" s="9">
-        <v>8189</v>
+        <v>8225</v>
       </c>
       <c r="H11" s="9">
-        <v>1730</v>
+        <v>1736</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1017247</v>
+        <v>1023524</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C12" s="9">
-        <v>482748</v>
+        <v>484937</v>
       </c>
       <c r="D12" s="9">
-        <v>6141</v>
+        <v>6152</v>
       </c>
       <c r="E12" s="9">
-        <v>5808</v>
+        <v>5829</v>
       </c>
       <c r="F12" s="9">
-        <v>27636</v>
+        <v>27746</v>
       </c>
       <c r="G12" s="9">
-        <v>1969</v>
+        <v>1981</v>
       </c>
       <c r="H12" s="9">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>488889</v>
+        <v>491089</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C13" s="9">
-        <v>345214</v>
+        <v>347509</v>
       </c>
       <c r="D13" s="9">
-        <v>4344</v>
+        <v>4372</v>
       </c>
       <c r="E13" s="9">
-        <v>3912</v>
+        <v>3940</v>
       </c>
       <c r="F13" s="9">
-        <v>24827</v>
+        <v>25006</v>
       </c>
       <c r="G13" s="9">
-        <v>1357</v>
+        <v>1363</v>
       </c>
       <c r="H13" s="9">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>349558</v>
+        <v>351881</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C14" s="9">
-        <v>286015</v>
+        <v>288570</v>
       </c>
       <c r="D14" s="9">
-        <v>8184</v>
+        <v>8242</v>
       </c>
       <c r="E14" s="9">
-        <v>3164</v>
+        <v>3188</v>
       </c>
       <c r="F14" s="9">
-        <v>19477</v>
+        <v>19629</v>
       </c>
       <c r="G14" s="9">
-        <v>1917</v>
+        <v>1935</v>
       </c>
       <c r="H14" s="9">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>294199</v>
+        <v>296812</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C15" s="9">
-        <v>391457</v>
+        <v>393412</v>
       </c>
       <c r="D15" s="9">
-        <v>7601</v>
+        <v>7620</v>
       </c>
       <c r="E15" s="9">
-        <v>6393</v>
+        <v>6427</v>
       </c>
       <c r="F15" s="9">
-        <v>26529</v>
+        <v>26654</v>
       </c>
       <c r="G15" s="9">
-        <v>3805</v>
+        <v>3820</v>
       </c>
       <c r="H15" s="9">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="I15" s="9">
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>399058</v>
+        <v>401032</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C16" s="9">
-        <v>326270</v>
+        <v>328084</v>
       </c>
       <c r="D16" s="9">
-        <v>4729</v>
+        <v>4752</v>
       </c>
       <c r="E16" s="9">
-        <v>2820</v>
+        <v>2841</v>
       </c>
       <c r="F16" s="9">
-        <v>19029</v>
+        <v>19153</v>
       </c>
       <c r="G16" s="9">
-        <v>3809</v>
+        <v>3840</v>
       </c>
       <c r="H16" s="9">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>330999</v>
+        <v>332836</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" s="9">
-        <v>196923</v>
+        <v>196959</v>
       </c>
       <c r="D17" s="9">
-        <v>4832</v>
+        <v>4833</v>
       </c>
       <c r="E17" s="9">
         <v>2179</v>
       </c>
       <c r="F17" s="9">
-        <v>10281</v>
+        <v>10284</v>
       </c>
       <c r="G17" s="9">
         <v>1708</v>
@@ -2519,30 +2522,30 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201755</v>
+        <v>201792</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C18" s="9">
-        <v>246681</v>
+        <v>247585</v>
       </c>
       <c r="D18" s="9">
-        <v>5398</v>
+        <v>5411</v>
       </c>
       <c r="E18" s="9">
-        <v>2632</v>
+        <v>2637</v>
       </c>
       <c r="F18" s="9">
-        <v>14159</v>
+        <v>14196</v>
       </c>
       <c r="G18" s="9">
-        <v>2375</v>
+        <v>2383</v>
       </c>
       <c r="H18" s="9">
         <v>492</v>
@@ -2551,27 +2554,27 @@
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>252079</v>
+        <v>252996</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C19" s="9">
-        <v>136235</v>
+        <v>136366</v>
       </c>
       <c r="D19" s="9">
         <v>1745</v>
       </c>
       <c r="E19" s="9">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="F19" s="9">
-        <v>10381</v>
+        <v>10386</v>
       </c>
       <c r="G19" s="9">
         <v>223</v>
@@ -2583,103 +2586,103 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>137980</v>
+        <v>138111</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C20" s="9">
-        <v>566387</v>
+        <v>570619</v>
       </c>
       <c r="D20" s="9">
-        <v>6880</v>
+        <v>6922</v>
       </c>
       <c r="E20" s="9">
-        <v>3389</v>
+        <v>3412</v>
       </c>
       <c r="F20" s="9">
-        <v>16218</v>
+        <v>16335</v>
       </c>
       <c r="G20" s="9">
-        <v>1002</v>
+        <v>1010</v>
       </c>
       <c r="H20" s="9">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>573267</v>
+        <v>577541</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C21" s="9">
-        <v>116632</v>
+        <v>117157</v>
       </c>
       <c r="D21" s="9">
-        <v>1098</v>
+        <v>1108</v>
       </c>
       <c r="E21" s="9">
-        <v>834</v>
+        <v>838</v>
       </c>
       <c r="F21" s="9">
-        <v>5046</v>
+        <v>5065</v>
       </c>
       <c r="G21" s="9">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="H21" s="9">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>117730</v>
+        <v>118265</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C22" s="12">
-        <v>6318247</v>
+        <v>6355459</v>
       </c>
       <c r="D22" s="12">
-        <v>108035</v>
+        <v>108505</v>
       </c>
       <c r="E22" s="12">
-        <v>68421</v>
+        <v>68807</v>
       </c>
       <c r="F22" s="12">
-        <v>341699</v>
+        <v>343590</v>
       </c>
       <c r="G22" s="12">
-        <v>55532</v>
+        <v>55877</v>
       </c>
       <c r="H22" s="12">
-        <v>9320</v>
+        <v>9346</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6426282</v>
+        <v>6463964</v>
       </c>
     </row>
   </sheetData>
@@ -2706,7 +2709,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2730,7 +2733,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2739,13 +2742,13 @@
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2773,13 +2776,13 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1085</v>
+        <v>1099</v>
       </c>
       <c r="D7" s="6">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2796,7 +2799,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2813,7 +2816,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2824,13 +2827,13 @@
         <v>58</v>
       </c>
       <c r="C10" s="9">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D10" s="9">
         <v>4</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2841,72 +2844,72 @@
         <v>65</v>
       </c>
       <c r="C11" s="9">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D11" s="9">
         <v>24</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C12" s="9">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C13" s="9">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D13" s="9">
         <v>5</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C14" s="9">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D14" s="9">
         <v>1</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C15" s="9">
         <v>94</v>
@@ -2915,49 +2918,49 @@
         <v>0</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C16" s="9">
         <v>156</v>
       </c>
       <c r="D16" s="9">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C17" s="9">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D17" s="9">
         <v>2</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C18" s="9">
         <v>28</v>
@@ -2966,15 +2969,15 @@
         <v>8</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C19" s="9">
         <v>70</v>
@@ -2983,15 +2986,15 @@
         <v>17</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C20" s="9">
         <v>15</v>
@@ -3000,32 +3003,32 @@
         <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C21" s="9">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D21" s="9">
         <v>4</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C22" s="9">
         <v>62</v>
@@ -3034,24 +3037,24 @@
         <v>12</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C23" s="12">
-        <v>1085</v>
+        <v>1099</v>
       </c>
       <c r="D23" s="12">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 21/08/2026 15:08:29,32
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -18,7 +18,7 @@
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 21 Agu 2026, 06.16 | Dicetak: 21 Agu 2026, 07.20</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 21 Agu 2026, 12.18 | Dicetak: 21 Agu 2026, 15.07</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,7 +123,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>65,87</t>
+    <t>66,05</t>
   </si>
   <si>
     <t>1,79</t>
@@ -132,13 +132,13 @@
     <t>0,05</t>
   </si>
   <si>
-    <t>21,19</t>
+    <t>21,23</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>77,47</t>
+    <t>77,68</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>79,2</t>
+    <t>79,29</t>
   </si>
   <si>
     <t>1,13</t>
@@ -156,13 +156,13 @@
     <t>0,04</t>
   </si>
   <si>
-    <t>18,38</t>
+    <t>18,37</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>92,02</t>
+    <t>92,12</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>68,72</t>
+    <t>68,9</t>
   </si>
   <si>
     <t>0,99</t>
   </si>
   <si>
-    <t>17,05</t>
+    <t>17,1</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>83,74</t>
+    <t>83,99</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,261 +192,261 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>60,91</t>
+    <t>61,16</t>
   </si>
   <si>
     <t>1,2</t>
   </si>
   <si>
-    <t>19,86</t>
+    <t>19,93</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
+    <t>73,59</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>67,95</t>
+  </si>
+  <si>
+    <t>1,89</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>18,43</t>
+  </si>
+  <si>
+    <t>76,99</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>67,56</t>
+  </si>
+  <si>
+    <t>2,73</t>
+  </si>
+  <si>
+    <t>18,53</t>
+  </si>
+  <si>
+    <t>0,24</t>
+  </si>
+  <si>
+    <t>76,53</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>66,99</t>
+  </si>
+  <si>
+    <t>1,95</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>25,96</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>78,7</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>67,9</t>
+  </si>
+  <si>
+    <t>1,7</t>
+  </si>
+  <si>
+    <t>18,84</t>
+  </si>
+  <si>
+    <t>79,53</t>
+  </si>
+  <si>
+    <t>1808</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG</t>
+  </si>
+  <si>
+    <t>60,32</t>
+  </si>
+  <si>
+    <t>2,26</t>
+  </si>
+  <si>
+    <t>26,09</t>
+  </si>
+  <si>
+    <t>0,02</t>
+  </si>
+  <si>
+    <t>72,27</t>
+  </si>
+  <si>
+    <t>1809</t>
+  </si>
+  <si>
+    <t>PESAWARAN</t>
+  </si>
+  <si>
+    <t>72,16</t>
+  </si>
+  <si>
+    <t>2,99</t>
+  </si>
+  <si>
+    <t>21,33</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>85,94</t>
+  </si>
+  <si>
+    <t>1810</t>
+  </si>
+  <si>
+    <t>PRINGSEWU</t>
+  </si>
+  <si>
+    <t>72,75</t>
+  </si>
+  <si>
+    <t>1,47</t>
+  </si>
+  <si>
+    <t>16,32</t>
+  </si>
+  <si>
+    <t>82,04</t>
+  </si>
+  <si>
+    <t>1811</t>
+  </si>
+  <si>
+    <t>MESUJI</t>
+  </si>
+  <si>
+    <t>74,28</t>
+  </si>
+  <si>
+    <t>1,58</t>
+  </si>
+  <si>
+    <t>24,98</t>
+  </si>
+  <si>
+    <t>0,16</t>
+  </si>
+  <si>
+    <t>90,45</t>
+  </si>
+  <si>
+    <t>1812</t>
+  </si>
+  <si>
+    <t>TULANG BAWANG BARAT</t>
+  </si>
+  <si>
+    <t>73,85</t>
+  </si>
+  <si>
+    <t>2,43</t>
+  </si>
+  <si>
+    <t>23,16</t>
+  </si>
+  <si>
+    <t>0,26</t>
+  </si>
+  <si>
+    <t>86,65</t>
+  </si>
+  <si>
+    <t>1813</t>
+  </si>
+  <si>
+    <t>PESISIR BARAT</t>
+  </si>
+  <si>
+    <t>81,42</t>
+  </si>
+  <si>
+    <t>0,84</t>
+  </si>
+  <si>
+    <t>17,53</t>
+  </si>
+  <si>
+    <t>99,08</t>
+  </si>
+  <si>
+    <t>1871</t>
+  </si>
+  <si>
+    <t>BANDAR LAMPUNG</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>0,86</t>
+  </si>
+  <si>
+    <t>30,83</t>
+  </si>
+  <si>
+    <t>62,51</t>
+  </si>
+  <si>
+    <t>1872</t>
+  </si>
+  <si>
+    <t>METRO</t>
+  </si>
+  <si>
+    <t>63,88</t>
+  </si>
+  <si>
+    <t>1,38</t>
+  </si>
+  <si>
+    <t>21,76</t>
+  </si>
+  <si>
     <t>73,29</t>
   </si>
   <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>67,74</t>
-  </si>
-  <si>
-    <t>1,89</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>18,37</t>
-  </si>
-  <si>
-    <t>76,75</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>67,38</t>
-  </si>
-  <si>
-    <t>2,72</t>
-  </si>
-  <si>
-    <t>18,49</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>76,33</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>66,83</t>
-  </si>
-  <si>
-    <t>1,95</t>
-  </si>
-  <si>
-    <t>0,02</t>
-  </si>
-  <si>
-    <t>25,93</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>78,51</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>67,66</t>
-  </si>
-  <si>
-    <t>1,7</t>
-  </si>
-  <si>
-    <t>18,83</t>
-  </si>
-  <si>
-    <t>79,24</t>
-  </si>
-  <si>
-    <t>1808</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG</t>
-  </si>
-  <si>
-    <t>60,12</t>
-  </si>
-  <si>
-    <t>2,25</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>26,06</t>
-  </si>
-  <si>
-    <t>72,02</t>
-  </si>
-  <si>
-    <t>1809</t>
-  </si>
-  <si>
-    <t>PESAWARAN</t>
-  </si>
-  <si>
-    <t>72</t>
-  </si>
-  <si>
-    <t>2,98</t>
-  </si>
-  <si>
-    <t>21,28</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>85,76</t>
-  </si>
-  <si>
-    <t>1810</t>
-  </si>
-  <si>
-    <t>PRINGSEWU</t>
-  </si>
-  <si>
-    <t>72,55</t>
-  </si>
-  <si>
-    <t>1,47</t>
-  </si>
-  <si>
-    <t>16,27</t>
-  </si>
-  <si>
-    <t>81,81</t>
-  </si>
-  <si>
-    <t>1811</t>
-  </si>
-  <si>
-    <t>MESUJI</t>
-  </si>
-  <si>
-    <t>74,27</t>
-  </si>
-  <si>
-    <t>1,58</t>
-  </si>
-  <si>
-    <t>24,98</t>
-  </si>
-  <si>
-    <t>0,16</t>
-  </si>
-  <si>
-    <t>90,42</t>
-  </si>
-  <si>
-    <t>1812</t>
-  </si>
-  <si>
-    <t>TULANG BAWANG BARAT</t>
-  </si>
-  <si>
-    <t>73,76</t>
-  </si>
-  <si>
-    <t>2,42</t>
-  </si>
-  <si>
-    <t>23,15</t>
-  </si>
-  <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>86,54</t>
-  </si>
-  <si>
-    <t>1813</t>
-  </si>
-  <si>
-    <t>PESISIR BARAT</t>
-  </si>
-  <si>
-    <t>81,36</t>
-  </si>
-  <si>
-    <t>0,84</t>
-  </si>
-  <si>
-    <t>17,54</t>
-  </si>
-  <si>
-    <t>99,01</t>
-  </si>
-  <si>
-    <t>1871</t>
-  </si>
-  <si>
-    <t>BANDAR LAMPUNG</t>
-  </si>
-  <si>
-    <t>48,86</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>30,77</t>
-  </si>
-  <si>
-    <t>62,35</t>
-  </si>
-  <si>
-    <t>1872</t>
-  </si>
-  <si>
-    <t>METRO</t>
-  </si>
-  <si>
-    <t>63,71</t>
-  </si>
-  <si>
-    <t>1,37</t>
-  </si>
-  <si>
-    <t>21,74</t>
-  </si>
-  <si>
-    <t>73,08</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -489,7 +489,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>12,1</t>
+    <t>13,32</t>
   </si>
   <si>
     <t>0</t>
@@ -498,37 +498,37 @@
     <t>4</t>
   </si>
   <si>
-    <t>4,12</t>
-  </si>
-  <si>
-    <t>22,02</t>
-  </si>
-  <si>
-    <t>6,52</t>
-  </si>
-  <si>
-    <t>16,67</t>
+    <t>4,04</t>
+  </si>
+  <si>
+    <t>21,43</t>
+  </si>
+  <si>
+    <t>6,45</t>
+  </si>
+  <si>
+    <t>15,63</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
-    <t>27,56</t>
-  </si>
-  <si>
-    <t>4,44</t>
+    <t>27,74</t>
+  </si>
+  <si>
+    <t>4,35</t>
   </si>
   <si>
     <t>28,57</t>
   </si>
   <si>
-    <t>24,29</t>
-  </si>
-  <si>
-    <t>3,15</t>
-  </si>
-  <si>
-    <t>19,35</t>
+    <t>30,99</t>
+  </si>
+  <si>
+    <t>3,94</t>
+  </si>
+  <si>
+    <t>32,81</t>
   </si>
 </sst>
 </file>
@@ -1189,28 +1189,28 @@
         <v>2730933</v>
       </c>
       <c r="D6" s="6">
-        <v>1798816</v>
+        <v>1803657</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>316902</v>
+        <v>317825</v>
       </c>
       <c r="G6" s="6">
-        <v>48897</v>
+        <v>48963</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1437</v>
+        <v>1440</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>578575</v>
+        <v>579739</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1222,7 +1222,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2115718</v>
+        <v>2121482</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1239,16 +1239,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67433</v>
+        <v>67514</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10914</v>
+        <v>10918</v>
       </c>
       <c r="G7" s="9">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1260,7 +1260,7 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15647</v>
+        <v>15637</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1272,7 +1272,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78347</v>
+        <v>78432</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1289,16 +1289,16 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>118850</v>
+        <v>119174</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>25985</v>
+        <v>26084</v>
       </c>
       <c r="G8" s="9">
-        <v>1711</v>
+        <v>1714</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
@@ -1310,7 +1310,7 @@
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>29489</v>
+        <v>29580</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1322,7 +1322,7 @@
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>144835</v>
+        <v>145258</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1339,28 +1339,28 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>208769</v>
+        <v>209613</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>42418</v>
+        <v>42590</v>
       </c>
       <c r="G9" s="9">
-        <v>4113</v>
+        <v>4120</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>68061</v>
+        <v>68295</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
@@ -1372,7 +1372,7 @@
         <v>62</v>
       </c>
       <c r="O9" s="9">
-        <v>251187</v>
+        <v>252203</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>63</v>
@@ -1389,16 +1389,16 @@
         <v>362839</v>
       </c>
       <c r="D10" s="9">
-        <v>245805</v>
+        <v>246559</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="9">
-        <v>32682</v>
+        <v>32781</v>
       </c>
       <c r="G10" s="9">
-        <v>6848</v>
+        <v>6854</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>67</v>
@@ -1410,7 +1410,7 @@
         <v>68</v>
       </c>
       <c r="K10" s="9">
-        <v>66665</v>
+        <v>66875</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>69</v>
@@ -1422,7 +1422,7 @@
         <v>48</v>
       </c>
       <c r="O10" s="9">
-        <v>278487</v>
+        <v>279340</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>70</v>
@@ -1439,28 +1439,28 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>302937</v>
+        <v>303745</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>73</v>
       </c>
       <c r="F11" s="9">
-        <v>40216</v>
+        <v>40328</v>
       </c>
       <c r="G11" s="9">
-        <v>12233</v>
+        <v>12252</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>74</v>
       </c>
       <c r="I11" s="9">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>83130</v>
+        <v>83306</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>75</v>
@@ -1472,7 +1472,7 @@
         <v>76</v>
       </c>
       <c r="O11" s="9">
-        <v>343153</v>
+        <v>344073</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>77</v>
@@ -1489,28 +1489,28 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>133264</v>
+        <v>133569</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>80</v>
       </c>
       <c r="F12" s="9">
-        <v>23287</v>
+        <v>23362</v>
       </c>
       <c r="G12" s="9">
-        <v>3889</v>
+        <v>3890</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>81</v>
       </c>
       <c r="I12" s="9">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J12" s="10" t="s">
         <v>82</v>
       </c>
       <c r="K12" s="9">
-        <v>51707</v>
+        <v>51760</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>83</v>
@@ -1522,7 +1522,7 @@
         <v>84</v>
       </c>
       <c r="O12" s="9">
-        <v>156551</v>
+        <v>156931</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>85</v>
@@ -1539,16 +1539,16 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>98853</v>
+        <v>99198</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>88</v>
       </c>
       <c r="F13" s="9">
-        <v>16912</v>
+        <v>16984</v>
       </c>
       <c r="G13" s="9">
-        <v>2478</v>
+        <v>2488</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>89</v>
@@ -1560,7 +1560,7 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>27504</v>
+        <v>27528</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>90</v>
@@ -1572,7 +1572,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="9">
-        <v>115765</v>
+        <v>116182</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>91</v>
@@ -1589,16 +1589,16 @@
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>81315</v>
+        <v>81589</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>94</v>
       </c>
       <c r="F14" s="9">
-        <v>16098</v>
+        <v>16166</v>
       </c>
       <c r="G14" s="9">
-        <v>3050</v>
+        <v>3052</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>95</v>
@@ -1607,22 +1607,22 @@
         <v>34</v>
       </c>
       <c r="J14" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="K14" s="9">
+        <v>35288</v>
+      </c>
+      <c r="L14" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="K14" s="9">
-        <v>35242</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="M14" s="9">
         <v>24</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="O14" s="9">
-        <v>97413</v>
+        <v>97755</v>
       </c>
       <c r="P14" s="10" t="s">
         <v>98</v>
@@ -1639,16 +1639,16 @@
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>109555</v>
+        <v>109792</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>101</v>
       </c>
       <c r="F15" s="9">
-        <v>20936</v>
+        <v>20978</v>
       </c>
       <c r="G15" s="9">
-        <v>4541</v>
+        <v>4546</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>102</v>
@@ -1660,7 +1660,7 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>32382</v>
+        <v>32459</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>103</v>
@@ -1672,7 +1672,7 @@
         <v>104</v>
       </c>
       <c r="O15" s="9">
-        <v>130491</v>
+        <v>130770</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>105</v>
@@ -1689,16 +1689,16 @@
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>98478</v>
+        <v>98755</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>108</v>
       </c>
       <c r="F16" s="9">
-        <v>12566</v>
+        <v>12608</v>
       </c>
       <c r="G16" s="9">
-        <v>1996</v>
+        <v>2000</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>109</v>
@@ -1710,7 +1710,7 @@
         <v>55</v>
       </c>
       <c r="K16" s="9">
-        <v>22081</v>
+        <v>22159</v>
       </c>
       <c r="L16" s="10" t="s">
         <v>110</v>
@@ -1722,7 +1722,7 @@
         <v>68</v>
       </c>
       <c r="O16" s="9">
-        <v>111044</v>
+        <v>111363</v>
       </c>
       <c r="P16" s="10" t="s">
         <v>111</v>
@@ -1739,16 +1739,16 @@
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55789</v>
+        <v>55793</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>114</v>
       </c>
       <c r="F17" s="9">
-        <v>12130</v>
+        <v>12145</v>
       </c>
       <c r="G17" s="9">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="H17" s="10" t="s">
         <v>115</v>
@@ -1760,7 +1760,7 @@
         <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18765</v>
+        <v>18766</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>116</v>
@@ -1772,7 +1772,7 @@
         <v>117</v>
       </c>
       <c r="O17" s="9">
-        <v>67919</v>
+        <v>67938</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>118</v>
@@ -1789,16 +1789,16 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>73151</v>
+        <v>73232</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>121</v>
       </c>
       <c r="F18" s="9">
-        <v>12673</v>
+        <v>12697</v>
       </c>
       <c r="G18" s="9">
-        <v>2404</v>
+        <v>2406</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>122</v>
@@ -1810,7 +1810,7 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22956</v>
+        <v>22971</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>123</v>
@@ -1822,7 +1822,7 @@
         <v>124</v>
       </c>
       <c r="O18" s="9">
-        <v>85824</v>
+        <v>85929</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>125</v>
@@ -1839,16 +1839,16 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>33986</v>
+        <v>34011</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F19" s="9">
-        <v>7372</v>
+        <v>7375</v>
       </c>
       <c r="G19" s="9">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>129</v>
@@ -1860,7 +1860,7 @@
         <v>68</v>
       </c>
       <c r="K19" s="9">
-        <v>7325</v>
+        <v>7321</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>130</v>
@@ -1872,7 +1872,7 @@
         <v>68</v>
       </c>
       <c r="O19" s="9">
-        <v>41358</v>
+        <v>41386</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>131</v>
@@ -1889,16 +1889,16 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>136541</v>
+        <v>136933</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>134</v>
       </c>
       <c r="F20" s="9">
-        <v>37700</v>
+        <v>37776</v>
       </c>
       <c r="G20" s="9">
-        <v>2401</v>
+        <v>2403</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>135</v>
@@ -1910,7 +1910,7 @@
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>85990</v>
+        <v>86151</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>136</v>
@@ -1922,7 +1922,7 @@
         <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>174241</v>
+        <v>174709</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>137</v>
@@ -1939,28 +1939,28 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>34090</v>
+        <v>34180</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>140</v>
       </c>
       <c r="F21" s="9">
-        <v>5013</v>
+        <v>5033</v>
       </c>
       <c r="G21" s="9">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>141</v>
       </c>
       <c r="I21" s="9">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J21" s="10" t="s">
         <v>68</v>
       </c>
       <c r="K21" s="9">
-        <v>11631</v>
+        <v>11643</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>142</v>
@@ -1969,10 +1969,10 @@
         <v>11</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="O21" s="9">
-        <v>39103</v>
+        <v>39213</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>143</v>
@@ -1989,28 +1989,28 @@
         <v>2730933</v>
       </c>
       <c r="D22" s="12">
-        <v>1798816</v>
+        <v>1803657</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>316902</v>
+        <v>317825</v>
       </c>
       <c r="G22" s="12">
-        <v>48897</v>
+        <v>48963</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1437</v>
+        <v>1440</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>578575</v>
+        <v>579739</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2022,7 +2022,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2115718</v>
+        <v>2121482</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2149,28 +2149,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6355459</v>
+        <v>6373215</v>
       </c>
       <c r="D6" s="6">
-        <v>108505</v>
+        <v>108720</v>
       </c>
       <c r="E6" s="6">
-        <v>68807</v>
+        <v>68968</v>
       </c>
       <c r="F6" s="6">
-        <v>343590</v>
+        <v>344440</v>
       </c>
       <c r="G6" s="6">
-        <v>55877</v>
+        <v>56036</v>
       </c>
       <c r="H6" s="6">
-        <v>9346</v>
+        <v>9355</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6463964</v>
+        <v>6481935</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2181,19 +2181,19 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>245643</v>
+        <v>245919</v>
       </c>
       <c r="D7" s="9">
         <v>2859</v>
       </c>
       <c r="E7" s="9">
-        <v>2101</v>
+        <v>2108</v>
       </c>
       <c r="F7" s="9">
-        <v>13025</v>
+        <v>13012</v>
       </c>
       <c r="G7" s="9">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H7" s="9">
         <v>394</v>
@@ -2202,7 +2202,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>248502</v>
+        <v>248778</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2213,19 +2213,19 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>442315</v>
+        <v>443634</v>
       </c>
       <c r="D8" s="9">
-        <v>5838</v>
+        <v>5854</v>
       </c>
       <c r="E8" s="9">
-        <v>4346</v>
+        <v>4361</v>
       </c>
       <c r="F8" s="9">
-        <v>33917</v>
+        <v>34025</v>
       </c>
       <c r="G8" s="9">
-        <v>4040</v>
+        <v>4051</v>
       </c>
       <c r="H8" s="9">
         <v>563</v>
@@ -2234,7 +2234,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>448153</v>
+        <v>449488</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2245,28 +2245,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>764792</v>
+        <v>768022</v>
       </c>
       <c r="D9" s="9">
-        <v>13218</v>
+        <v>13269</v>
       </c>
       <c r="E9" s="9">
-        <v>8718</v>
+        <v>8742</v>
       </c>
       <c r="F9" s="9">
-        <v>38012</v>
+        <v>38148</v>
       </c>
       <c r="G9" s="9">
-        <v>4670</v>
+        <v>4692</v>
       </c>
       <c r="H9" s="9">
-        <v>1005</v>
+        <v>1009</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>778010</v>
+        <v>781291</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2277,19 +2277,19 @@
         <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>788213</v>
+        <v>790626</v>
       </c>
       <c r="D10" s="9">
-        <v>15207</v>
+        <v>15230</v>
       </c>
       <c r="E10" s="9">
-        <v>9277</v>
+        <v>9309</v>
       </c>
       <c r="F10" s="9">
-        <v>38979</v>
+        <v>39102</v>
       </c>
       <c r="G10" s="9">
-        <v>19626</v>
+        <v>19698</v>
       </c>
       <c r="H10" s="9">
         <v>1067</v>
@@ -2298,7 +2298,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>803420</v>
+        <v>805856</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2309,28 +2309,28 @@
         <v>72</v>
       </c>
       <c r="C11" s="9">
-        <v>1003298</v>
+        <v>1006032</v>
       </c>
       <c r="D11" s="9">
-        <v>20226</v>
+        <v>20251</v>
       </c>
       <c r="E11" s="9">
-        <v>12028</v>
+        <v>12059</v>
       </c>
       <c r="F11" s="9">
-        <v>45203</v>
+        <v>45325</v>
       </c>
       <c r="G11" s="9">
-        <v>8225</v>
+        <v>8238</v>
       </c>
       <c r="H11" s="9">
-        <v>1736</v>
+        <v>1738</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1023524</v>
+        <v>1026283</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2341,19 +2341,19 @@
         <v>79</v>
       </c>
       <c r="C12" s="9">
-        <v>484937</v>
+        <v>486156</v>
       </c>
       <c r="D12" s="9">
-        <v>6152</v>
+        <v>6161</v>
       </c>
       <c r="E12" s="9">
-        <v>5829</v>
+        <v>5838</v>
       </c>
       <c r="F12" s="9">
-        <v>27746</v>
+        <v>27800</v>
       </c>
       <c r="G12" s="9">
-        <v>1981</v>
+        <v>1984</v>
       </c>
       <c r="H12" s="9">
         <v>507</v>
@@ -2362,7 +2362,7 @@
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>491089</v>
+        <v>492317</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2373,28 +2373,28 @@
         <v>87</v>
       </c>
       <c r="C13" s="9">
-        <v>347509</v>
+        <v>348798</v>
       </c>
       <c r="D13" s="9">
-        <v>4372</v>
+        <v>4386</v>
       </c>
       <c r="E13" s="9">
-        <v>3940</v>
+        <v>3953</v>
       </c>
       <c r="F13" s="9">
-        <v>25006</v>
+        <v>25095</v>
       </c>
       <c r="G13" s="9">
-        <v>1363</v>
+        <v>1370</v>
       </c>
       <c r="H13" s="9">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>351881</v>
+        <v>353184</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2405,19 +2405,19 @@
         <v>93</v>
       </c>
       <c r="C14" s="9">
-        <v>288570</v>
+        <v>289632</v>
       </c>
       <c r="D14" s="9">
-        <v>8242</v>
+        <v>8275</v>
       </c>
       <c r="E14" s="9">
-        <v>3188</v>
+        <v>3190</v>
       </c>
       <c r="F14" s="9">
-        <v>19629</v>
+        <v>19691</v>
       </c>
       <c r="G14" s="9">
-        <v>1935</v>
+        <v>1939</v>
       </c>
       <c r="H14" s="9">
         <v>344</v>
@@ -2426,7 +2426,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>296812</v>
+        <v>297907</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2437,19 +2437,19 @@
         <v>100</v>
       </c>
       <c r="C15" s="9">
-        <v>393412</v>
+        <v>394274</v>
       </c>
       <c r="D15" s="9">
-        <v>7620</v>
+        <v>7640</v>
       </c>
       <c r="E15" s="9">
-        <v>6427</v>
+        <v>6441</v>
       </c>
       <c r="F15" s="9">
-        <v>26654</v>
+        <v>26708</v>
       </c>
       <c r="G15" s="9">
-        <v>3820</v>
+        <v>3830</v>
       </c>
       <c r="H15" s="9">
         <v>511</v>
@@ -2458,7 +2458,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>401032</v>
+        <v>401914</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2469,19 +2469,19 @@
         <v>107</v>
       </c>
       <c r="C16" s="9">
-        <v>328084</v>
+        <v>329082</v>
       </c>
       <c r="D16" s="9">
-        <v>4752</v>
+        <v>4759</v>
       </c>
       <c r="E16" s="9">
-        <v>2841</v>
+        <v>2844</v>
       </c>
       <c r="F16" s="9">
-        <v>19153</v>
+        <v>19200</v>
       </c>
       <c r="G16" s="9">
-        <v>3840</v>
+        <v>3851</v>
       </c>
       <c r="H16" s="9">
         <v>256</v>
@@ -2490,7 +2490,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>332836</v>
+        <v>333841</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2501,7 +2501,7 @@
         <v>113</v>
       </c>
       <c r="C17" s="9">
-        <v>196959</v>
+        <v>197014</v>
       </c>
       <c r="D17" s="9">
         <v>4833</v>
@@ -2510,7 +2510,7 @@
         <v>2179</v>
       </c>
       <c r="F17" s="9">
-        <v>10284</v>
+        <v>10288</v>
       </c>
       <c r="G17" s="9">
         <v>1708</v>
@@ -2522,7 +2522,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201792</v>
+        <v>201847</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2533,19 +2533,19 @@
         <v>120</v>
       </c>
       <c r="C18" s="9">
-        <v>247585</v>
+        <v>247911</v>
       </c>
       <c r="D18" s="9">
-        <v>5411</v>
+        <v>5415</v>
       </c>
       <c r="E18" s="9">
-        <v>2637</v>
+        <v>2638</v>
       </c>
       <c r="F18" s="9">
-        <v>14196</v>
+        <v>14215</v>
       </c>
       <c r="G18" s="9">
-        <v>2383</v>
+        <v>2384</v>
       </c>
       <c r="H18" s="9">
         <v>492</v>
@@ -2554,7 +2554,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>252996</v>
+        <v>253326</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2565,16 +2565,16 @@
         <v>127</v>
       </c>
       <c r="C19" s="9">
-        <v>136366</v>
+        <v>136462</v>
       </c>
       <c r="D19" s="9">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="E19" s="9">
         <v>1046</v>
       </c>
       <c r="F19" s="9">
-        <v>10386</v>
+        <v>10394</v>
       </c>
       <c r="G19" s="9">
         <v>223</v>
@@ -2586,7 +2586,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>138111</v>
+        <v>138208</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2597,28 +2597,28 @@
         <v>133</v>
       </c>
       <c r="C20" s="9">
-        <v>570619</v>
+        <v>572171</v>
       </c>
       <c r="D20" s="9">
-        <v>6922</v>
+        <v>6932</v>
       </c>
       <c r="E20" s="9">
-        <v>3412</v>
+        <v>3420</v>
       </c>
       <c r="F20" s="9">
-        <v>16335</v>
+        <v>16360</v>
       </c>
       <c r="G20" s="9">
-        <v>1010</v>
+        <v>1012</v>
       </c>
       <c r="H20" s="9">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>577541</v>
+        <v>579103</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2629,28 +2629,28 @@
         <v>139</v>
       </c>
       <c r="C21" s="9">
-        <v>117157</v>
+        <v>117482</v>
       </c>
       <c r="D21" s="9">
-        <v>1108</v>
+        <v>1110</v>
       </c>
       <c r="E21" s="9">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="F21" s="9">
-        <v>5065</v>
+        <v>5077</v>
       </c>
       <c r="G21" s="9">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="H21" s="9">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>118265</v>
+        <v>118592</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2661,28 +2661,28 @@
         <v>145</v>
       </c>
       <c r="C22" s="12">
-        <v>6355459</v>
+        <v>6373215</v>
       </c>
       <c r="D22" s="12">
-        <v>108505</v>
+        <v>108720</v>
       </c>
       <c r="E22" s="12">
-        <v>68807</v>
+        <v>68968</v>
       </c>
       <c r="F22" s="12">
-        <v>343590</v>
+        <v>344440</v>
       </c>
       <c r="G22" s="12">
-        <v>55877</v>
+        <v>56036</v>
       </c>
       <c r="H22" s="12">
-        <v>9346</v>
+        <v>9355</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6463964</v>
+        <v>6481935</v>
       </c>
     </row>
   </sheetData>
@@ -2776,10 +2776,10 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1099</v>
+        <v>1111</v>
       </c>
       <c r="D7" s="6">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>158</v>
@@ -2827,7 +2827,7 @@
         <v>58</v>
       </c>
       <c r="C10" s="9">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D10" s="9">
         <v>4</v>
@@ -2844,7 +2844,7 @@
         <v>65</v>
       </c>
       <c r="C11" s="9">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D11" s="9">
         <v>24</v>
@@ -2861,7 +2861,7 @@
         <v>72</v>
       </c>
       <c r="C12" s="9">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
@@ -2878,7 +2878,7 @@
         <v>79</v>
       </c>
       <c r="C13" s="9">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="9">
         <v>5</v>
@@ -2929,7 +2929,7 @@
         <v>100</v>
       </c>
       <c r="C16" s="9">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D16" s="9">
         <v>43</v>
@@ -2946,7 +2946,7 @@
         <v>107</v>
       </c>
       <c r="C17" s="9">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D17" s="9">
         <v>2</v>
@@ -2980,10 +2980,10 @@
         <v>120</v>
       </c>
       <c r="C19" s="9">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D19" s="9">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>169</v>
@@ -3017,7 +3017,7 @@
         <v>127</v>
       </c>
       <c r="D21" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>170</v>
@@ -3031,10 +3031,10 @@
         <v>139</v>
       </c>
       <c r="C22" s="9">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D22" s="9">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>171</v>
@@ -3048,10 +3048,10 @@
         <v>145</v>
       </c>
       <c r="C23" s="12">
-        <v>1099</v>
+        <v>1111</v>
       </c>
       <c r="D23" s="12">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>158</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 21/08/2026 21:57:07,33
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="173">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 21 Agu 2026, 12.18 | Dicetak: 21 Agu 2026, 15.07</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 21 Agu 2026, 18.23 | Dicetak: 21 Agu 2026, 21.56</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,22 +123,22 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>66,05</t>
-  </si>
-  <si>
-    <t>1,79</t>
+    <t>66,22</t>
+  </si>
+  <si>
+    <t>1,8</t>
   </si>
   <si>
     <t>0,05</t>
   </si>
   <si>
-    <t>21,23</t>
+    <t>21,28</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>77,68</t>
+    <t>77,9</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,7 +147,7 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>79,29</t>
+    <t>79,33</t>
   </si>
   <si>
     <t>1,13</t>
@@ -162,7 +162,7 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>92,12</t>
+    <t>92,16</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,19 +171,19 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>68,9</t>
+    <t>69,13</t>
   </si>
   <si>
     <t>0,99</t>
   </si>
   <si>
-    <t>17,1</t>
+    <t>17,16</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>83,99</t>
+    <t>84,25</t>
   </si>
   <si>
     <t>1803</t>
@@ -192,19 +192,19 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>61,16</t>
-  </si>
-  <si>
-    <t>1,2</t>
-  </si>
-  <si>
-    <t>19,93</t>
+    <t>61,36</t>
+  </si>
+  <si>
+    <t>1,21</t>
+  </si>
+  <si>
+    <t>20,01</t>
   </si>
   <si>
     <t>0,09</t>
   </si>
   <si>
-    <t>73,59</t>
+    <t>73,84</t>
   </si>
   <si>
     <t>1804</t>
@@ -213,7 +213,7 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>67,95</t>
+    <t>68,14</t>
   </si>
   <si>
     <t>1,89</t>
@@ -222,10 +222,10 @@
     <t>0,06</t>
   </si>
   <si>
-    <t>18,43</t>
-  </si>
-  <si>
-    <t>76,99</t>
+    <t>18,46</t>
+  </si>
+  <si>
+    <t>77,21</t>
   </si>
   <si>
     <t>1805</t>
@@ -234,19 +234,19 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>67,56</t>
+    <t>67,77</t>
   </si>
   <si>
     <t>2,73</t>
   </si>
   <si>
-    <t>18,53</t>
+    <t>18,58</t>
   </si>
   <si>
     <t>0,24</t>
   </si>
   <si>
-    <t>76,53</t>
+    <t>76,77</t>
   </si>
   <si>
     <t>1806</t>
@@ -255,7 +255,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>66,99</t>
+    <t>67,15</t>
   </si>
   <si>
     <t>1,95</t>
@@ -264,13 +264,13 @@
     <t>0,03</t>
   </si>
   <si>
-    <t>25,96</t>
+    <t>25,98</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>78,7</t>
+    <t>78,89</t>
   </si>
   <si>
     <t>1807</t>
@@ -279,16 +279,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>67,9</t>
-  </si>
-  <si>
-    <t>1,7</t>
-  </si>
-  <si>
-    <t>18,84</t>
-  </si>
-  <si>
-    <t>79,53</t>
+    <t>68,18</t>
+  </si>
+  <si>
+    <t>1,71</t>
+  </si>
+  <si>
+    <t>18,9</t>
+  </si>
+  <si>
+    <t>79,86</t>
   </si>
   <si>
     <t>1808</t>
@@ -297,19 +297,19 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>60,32</t>
+    <t>60,57</t>
   </si>
   <si>
     <t>2,26</t>
   </si>
   <si>
-    <t>26,09</t>
+    <t>26,17</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>72,27</t>
+    <t>72,57</t>
   </si>
   <si>
     <t>1809</t>
@@ -318,19 +318,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>72,16</t>
+    <t>72,3</t>
   </si>
   <si>
     <t>2,99</t>
   </si>
   <si>
-    <t>21,33</t>
+    <t>21,39</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>85,94</t>
+    <t>86,11</t>
   </si>
   <si>
     <t>1810</t>
@@ -339,16 +339,16 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>72,75</t>
-  </si>
-  <si>
-    <t>1,47</t>
-  </si>
-  <si>
-    <t>16,32</t>
-  </si>
-  <si>
-    <t>82,04</t>
+    <t>72,99</t>
+  </si>
+  <si>
+    <t>1,48</t>
+  </si>
+  <si>
+    <t>16,35</t>
+  </si>
+  <si>
+    <t>82,31</t>
   </si>
   <si>
     <t>1811</t>
@@ -357,7 +357,7 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>74,28</t>
+    <t>74,29</t>
   </si>
   <si>
     <t>1,58</t>
@@ -369,7 +369,7 @@
     <t>0,16</t>
   </si>
   <si>
-    <t>90,45</t>
+    <t>90,46</t>
   </si>
   <si>
     <t>1812</t>
@@ -378,19 +378,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>73,85</t>
+    <t>73,92</t>
   </si>
   <si>
     <t>2,43</t>
   </si>
   <si>
-    <t>23,16</t>
+    <t>23,17</t>
   </si>
   <si>
     <t>0,26</t>
   </si>
   <si>
-    <t>86,65</t>
+    <t>86,73</t>
   </si>
   <si>
     <t>1813</t>
@@ -399,16 +399,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>81,42</t>
+    <t>81,49</t>
   </si>
   <si>
     <t>0,84</t>
   </si>
   <si>
-    <t>17,53</t>
-  </si>
-  <si>
-    <t>99,08</t>
+    <t>17,5</t>
+  </si>
+  <si>
+    <t>99,17</t>
   </si>
   <si>
     <t>1871</t>
@@ -417,16 +417,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>49</t>
+    <t>49,14</t>
   </si>
   <si>
     <t>0,86</t>
   </si>
   <si>
-    <t>30,83</t>
-  </si>
-  <si>
-    <t>62,51</t>
+    <t>30,91</t>
+  </si>
+  <si>
+    <t>62,69</t>
   </si>
   <si>
     <t>1872</t>
@@ -435,16 +435,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>63,88</t>
+    <t>64,04</t>
   </si>
   <si>
     <t>1,38</t>
   </si>
   <si>
-    <t>21,76</t>
-  </si>
-  <si>
-    <t>73,29</t>
+    <t>21,81</t>
+  </si>
+  <si>
+    <t>73,48</t>
   </si>
   <si>
     <t/>
@@ -489,7 +489,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>13,32</t>
+    <t>14,04</t>
   </si>
   <si>
     <t>0</t>
@@ -501,31 +501,34 @@
     <t>4,04</t>
   </si>
   <si>
-    <t>21,43</t>
-  </si>
-  <si>
-    <t>6,45</t>
+    <t>20,51</t>
+  </si>
+  <si>
+    <t>6,38</t>
   </si>
   <si>
     <t>15,63</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>27,74</t>
+    <t>3,85</t>
+  </si>
+  <si>
+    <t>1,08</t>
+  </si>
+  <si>
+    <t>30,52</t>
   </si>
   <si>
     <t>4,35</t>
   </si>
   <si>
-    <t>28,57</t>
-  </si>
-  <si>
-    <t>30,99</t>
-  </si>
-  <si>
-    <t>3,94</t>
+    <t>29,63</t>
+  </si>
+  <si>
+    <t>32,39</t>
+  </si>
+  <si>
+    <t>5,51</t>
   </si>
   <si>
     <t>32,81</t>
@@ -1189,28 +1192,28 @@
         <v>2730933</v>
       </c>
       <c r="D6" s="6">
-        <v>1803657</v>
+        <v>1808552</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>317825</v>
+        <v>318779</v>
       </c>
       <c r="G6" s="6">
-        <v>48963</v>
+        <v>49044</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1440</v>
+        <v>1444</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>579739</v>
+        <v>581061</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1222,7 +1225,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2121482</v>
+        <v>2127331</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1239,13 +1242,13 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67514</v>
+        <v>67546</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10918</v>
+        <v>10927</v>
       </c>
       <c r="G7" s="9">
         <v>966</v>
@@ -1260,7 +1263,7 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15637</v>
+        <v>15645</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1272,7 +1275,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78432</v>
+        <v>78473</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1289,28 +1292,28 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>119174</v>
+        <v>119564</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>26084</v>
+        <v>26157</v>
       </c>
       <c r="G8" s="9">
-        <v>1714</v>
+        <v>1716</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="9">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>29580</v>
+        <v>29682</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1322,7 +1325,7 @@
         <v>55</v>
       </c>
       <c r="O8" s="9">
-        <v>145258</v>
+        <v>145721</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>56</v>
@@ -1339,28 +1342,28 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>209613</v>
+        <v>210292</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="F9" s="9">
-        <v>42590</v>
+        <v>42799</v>
       </c>
       <c r="G9" s="9">
-        <v>4120</v>
+        <v>4137</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="I9" s="9">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>68295</v>
+        <v>68564</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>61</v>
@@ -1372,7 +1375,7 @@
         <v>62</v>
       </c>
       <c r="O9" s="9">
-        <v>252203</v>
+        <v>253091</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>63</v>
@@ -1389,16 +1392,16 @@
         <v>362839</v>
       </c>
       <c r="D10" s="9">
-        <v>246559</v>
+        <v>247252</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="F10" s="9">
-        <v>32781</v>
+        <v>32880</v>
       </c>
       <c r="G10" s="9">
-        <v>6854</v>
+        <v>6859</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>67</v>
@@ -1410,7 +1413,7 @@
         <v>68</v>
       </c>
       <c r="K10" s="9">
-        <v>66875</v>
+        <v>66986</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>69</v>
@@ -1422,7 +1425,7 @@
         <v>48</v>
       </c>
       <c r="O10" s="9">
-        <v>279340</v>
+        <v>280132</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>70</v>
@@ -1439,28 +1442,28 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>303745</v>
+        <v>304677</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>73</v>
       </c>
       <c r="F11" s="9">
-        <v>40328</v>
+        <v>40448</v>
       </c>
       <c r="G11" s="9">
-        <v>12252</v>
+        <v>12270</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>74</v>
       </c>
       <c r="I11" s="9">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>55</v>
       </c>
       <c r="K11" s="9">
-        <v>83306</v>
+        <v>83525</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>75</v>
@@ -1472,7 +1475,7 @@
         <v>76</v>
       </c>
       <c r="O11" s="9">
-        <v>344073</v>
+        <v>345125</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>77</v>
@@ -1489,16 +1492,16 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>133569</v>
+        <v>133886</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>80</v>
       </c>
       <c r="F12" s="9">
-        <v>23362</v>
+        <v>23425</v>
       </c>
       <c r="G12" s="9">
-        <v>3890</v>
+        <v>3892</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>81</v>
@@ -1510,7 +1513,7 @@
         <v>82</v>
       </c>
       <c r="K12" s="9">
-        <v>51760</v>
+        <v>51811</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>83</v>
@@ -1522,7 +1525,7 @@
         <v>84</v>
       </c>
       <c r="O12" s="9">
-        <v>156931</v>
+        <v>157311</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>85</v>
@@ -1539,16 +1542,16 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>99198</v>
+        <v>99606</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>88</v>
       </c>
       <c r="F13" s="9">
-        <v>16984</v>
+        <v>17067</v>
       </c>
       <c r="G13" s="9">
-        <v>2488</v>
+        <v>2493</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>89</v>
@@ -1560,7 +1563,7 @@
         <v>38</v>
       </c>
       <c r="K13" s="9">
-        <v>27528</v>
+        <v>27614</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>90</v>
@@ -1572,7 +1575,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="9">
-        <v>116182</v>
+        <v>116673</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>91</v>
@@ -1589,16 +1592,16 @@
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>81589</v>
+        <v>81921</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>94</v>
       </c>
       <c r="F14" s="9">
-        <v>16166</v>
+        <v>16234</v>
       </c>
       <c r="G14" s="9">
-        <v>3052</v>
+        <v>3060</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>95</v>
@@ -1610,7 +1613,7 @@
         <v>82</v>
       </c>
       <c r="K14" s="9">
-        <v>35288</v>
+        <v>35393</v>
       </c>
       <c r="L14" s="10" t="s">
         <v>96</v>
@@ -1622,7 +1625,7 @@
         <v>97</v>
       </c>
       <c r="O14" s="9">
-        <v>97755</v>
+        <v>98155</v>
       </c>
       <c r="P14" s="10" t="s">
         <v>98</v>
@@ -1639,16 +1642,16 @@
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>109792</v>
+        <v>110004</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>101</v>
       </c>
       <c r="F15" s="9">
-        <v>20978</v>
+        <v>21021</v>
       </c>
       <c r="G15" s="9">
-        <v>4546</v>
+        <v>4553</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>102</v>
@@ -1660,7 +1663,7 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>32459</v>
+        <v>32551</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>103</v>
@@ -1672,7 +1675,7 @@
         <v>104</v>
       </c>
       <c r="O15" s="9">
-        <v>130770</v>
+        <v>131025</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>105</v>
@@ -1689,28 +1692,28 @@
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>98755</v>
+        <v>99071</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>108</v>
       </c>
       <c r="F16" s="9">
-        <v>12608</v>
+        <v>12651</v>
       </c>
       <c r="G16" s="9">
-        <v>2000</v>
+        <v>2004</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>109</v>
       </c>
       <c r="I16" s="9">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="K16" s="9">
-        <v>22159</v>
+        <v>22196</v>
       </c>
       <c r="L16" s="10" t="s">
         <v>110</v>
@@ -1722,7 +1725,7 @@
         <v>68</v>
       </c>
       <c r="O16" s="9">
-        <v>111363</v>
+        <v>111722</v>
       </c>
       <c r="P16" s="10" t="s">
         <v>111</v>
@@ -1739,13 +1742,13 @@
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55793</v>
+        <v>55800</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>114</v>
       </c>
       <c r="F17" s="9">
-        <v>12145</v>
+        <v>12150</v>
       </c>
       <c r="G17" s="9">
         <v>1186</v>
@@ -1760,7 +1763,7 @@
         <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18766</v>
+        <v>18765</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>116</v>
@@ -1772,7 +1775,7 @@
         <v>117</v>
       </c>
       <c r="O17" s="9">
-        <v>67938</v>
+        <v>67950</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>118</v>
@@ -1789,28 +1792,28 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>73232</v>
+        <v>73301</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>121</v>
       </c>
       <c r="F18" s="9">
-        <v>12697</v>
+        <v>12710</v>
       </c>
       <c r="G18" s="9">
-        <v>2406</v>
+        <v>2408</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>122</v>
       </c>
       <c r="I18" s="9">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J18" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22971</v>
+        <v>22975</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>123</v>
@@ -1822,7 +1825,7 @@
         <v>124</v>
       </c>
       <c r="O18" s="9">
-        <v>85929</v>
+        <v>86011</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>125</v>
@@ -1839,13 +1842,13 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>34011</v>
+        <v>34040</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F19" s="9">
-        <v>7375</v>
+        <v>7386</v>
       </c>
       <c r="G19" s="9">
         <v>350</v>
@@ -1860,7 +1863,7 @@
         <v>68</v>
       </c>
       <c r="K19" s="9">
-        <v>7321</v>
+        <v>7312</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>130</v>
@@ -1872,7 +1875,7 @@
         <v>68</v>
       </c>
       <c r="O19" s="9">
-        <v>41386</v>
+        <v>41426</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>131</v>
@@ -1889,28 +1892,28 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>136933</v>
+        <v>137328</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>134</v>
       </c>
       <c r="F20" s="9">
-        <v>37776</v>
+        <v>37873</v>
       </c>
       <c r="G20" s="9">
-        <v>2403</v>
+        <v>2412</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>135</v>
       </c>
       <c r="I20" s="9">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>86151</v>
+        <v>86374</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>136</v>
@@ -1922,7 +1925,7 @@
         <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>174709</v>
+        <v>175201</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>137</v>
@@ -1939,16 +1942,16 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>34180</v>
+        <v>34264</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>140</v>
       </c>
       <c r="F21" s="9">
-        <v>5033</v>
+        <v>5051</v>
       </c>
       <c r="G21" s="9">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>141</v>
@@ -1960,7 +1963,7 @@
         <v>68</v>
       </c>
       <c r="K21" s="9">
-        <v>11643</v>
+        <v>11668</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>142</v>
@@ -1972,7 +1975,7 @@
         <v>97</v>
       </c>
       <c r="O21" s="9">
-        <v>39213</v>
+        <v>39315</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>143</v>
@@ -1989,28 +1992,28 @@
         <v>2730933</v>
       </c>
       <c r="D22" s="12">
-        <v>1803657</v>
+        <v>1808552</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>317825</v>
+        <v>318779</v>
       </c>
       <c r="G22" s="12">
-        <v>48963</v>
+        <v>49044</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1440</v>
+        <v>1444</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>579739</v>
+        <v>581061</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2022,7 +2025,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2121482</v>
+        <v>2127331</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2149,28 +2152,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6373215</v>
+        <v>6390833</v>
       </c>
       <c r="D6" s="6">
-        <v>108720</v>
+        <v>108927</v>
       </c>
       <c r="E6" s="6">
-        <v>68968</v>
+        <v>69158</v>
       </c>
       <c r="F6" s="6">
-        <v>344440</v>
+        <v>345349</v>
       </c>
       <c r="G6" s="6">
-        <v>56036</v>
+        <v>56190</v>
       </c>
       <c r="H6" s="6">
-        <v>9355</v>
+        <v>9374</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6481935</v>
+        <v>6499760</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2181,28 +2184,28 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>245919</v>
+        <v>246024</v>
       </c>
       <c r="D7" s="9">
-        <v>2859</v>
+        <v>2858</v>
       </c>
       <c r="E7" s="9">
-        <v>2108</v>
+        <v>2109</v>
       </c>
       <c r="F7" s="9">
-        <v>13012</v>
+        <v>13015</v>
       </c>
       <c r="G7" s="9">
         <v>304</v>
       </c>
       <c r="H7" s="9">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="I7" s="9">
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>248778</v>
+        <v>248882</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2213,28 +2216,28 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>443634</v>
+        <v>445035</v>
       </c>
       <c r="D8" s="9">
-        <v>5854</v>
+        <v>5873</v>
       </c>
       <c r="E8" s="9">
-        <v>4361</v>
+        <v>4375</v>
       </c>
       <c r="F8" s="9">
-        <v>34025</v>
+        <v>34144</v>
       </c>
       <c r="G8" s="9">
-        <v>4051</v>
+        <v>4063</v>
       </c>
       <c r="H8" s="9">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="I8" s="9">
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>449488</v>
+        <v>450908</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2245,28 +2248,28 @@
         <v>58</v>
       </c>
       <c r="C9" s="9">
-        <v>768022</v>
+        <v>770716</v>
       </c>
       <c r="D9" s="9">
-        <v>13269</v>
+        <v>13317</v>
       </c>
       <c r="E9" s="9">
-        <v>8742</v>
+        <v>8766</v>
       </c>
       <c r="F9" s="9">
-        <v>38148</v>
+        <v>38260</v>
       </c>
       <c r="G9" s="9">
-        <v>4692</v>
+        <v>4703</v>
       </c>
       <c r="H9" s="9">
-        <v>1009</v>
+        <v>1016</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>781291</v>
+        <v>784033</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2277,28 +2280,28 @@
         <v>65</v>
       </c>
       <c r="C10" s="9">
-        <v>790626</v>
+        <v>792878</v>
       </c>
       <c r="D10" s="9">
-        <v>15230</v>
+        <v>15268</v>
       </c>
       <c r="E10" s="9">
-        <v>9309</v>
+        <v>9340</v>
       </c>
       <c r="F10" s="9">
-        <v>39102</v>
+        <v>39216</v>
       </c>
       <c r="G10" s="9">
-        <v>19698</v>
+        <v>19769</v>
       </c>
       <c r="H10" s="9">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>805856</v>
+        <v>808146</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2309,28 +2312,28 @@
         <v>72</v>
       </c>
       <c r="C11" s="9">
-        <v>1006032</v>
+        <v>1009122</v>
       </c>
       <c r="D11" s="9">
-        <v>20251</v>
+        <v>20258</v>
       </c>
       <c r="E11" s="9">
-        <v>12059</v>
+        <v>12093</v>
       </c>
       <c r="F11" s="9">
-        <v>45325</v>
+        <v>45454</v>
       </c>
       <c r="G11" s="9">
-        <v>8238</v>
+        <v>8257</v>
       </c>
       <c r="H11" s="9">
-        <v>1738</v>
+        <v>1740</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1026283</v>
+        <v>1029380</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2341,28 +2344,28 @@
         <v>79</v>
       </c>
       <c r="C12" s="9">
-        <v>486156</v>
+        <v>487338</v>
       </c>
       <c r="D12" s="9">
-        <v>6161</v>
+        <v>6166</v>
       </c>
       <c r="E12" s="9">
-        <v>5838</v>
+        <v>5857</v>
       </c>
       <c r="F12" s="9">
-        <v>27800</v>
+        <v>27857</v>
       </c>
       <c r="G12" s="9">
-        <v>1984</v>
+        <v>1988</v>
       </c>
       <c r="H12" s="9">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>492317</v>
+        <v>493504</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2373,19 +2376,19 @@
         <v>87</v>
       </c>
       <c r="C13" s="9">
-        <v>348798</v>
+        <v>350314</v>
       </c>
       <c r="D13" s="9">
-        <v>4386</v>
+        <v>4397</v>
       </c>
       <c r="E13" s="9">
-        <v>3953</v>
+        <v>3968</v>
       </c>
       <c r="F13" s="9">
-        <v>25095</v>
+        <v>25199</v>
       </c>
       <c r="G13" s="9">
-        <v>1370</v>
+        <v>1379</v>
       </c>
       <c r="H13" s="9">
         <v>465</v>
@@ -2394,7 +2397,7 @@
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>353184</v>
+        <v>354711</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2405,19 +2408,19 @@
         <v>93</v>
       </c>
       <c r="C14" s="9">
-        <v>289632</v>
+        <v>290847</v>
       </c>
       <c r="D14" s="9">
-        <v>8275</v>
+        <v>8304</v>
       </c>
       <c r="E14" s="9">
-        <v>3190</v>
+        <v>3201</v>
       </c>
       <c r="F14" s="9">
-        <v>19691</v>
+        <v>19760</v>
       </c>
       <c r="G14" s="9">
-        <v>1939</v>
+        <v>1946</v>
       </c>
       <c r="H14" s="9">
         <v>344</v>
@@ -2426,7 +2429,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>297907</v>
+        <v>299151</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2437,19 +2440,19 @@
         <v>100</v>
       </c>
       <c r="C15" s="9">
-        <v>394274</v>
+        <v>395045</v>
       </c>
       <c r="D15" s="9">
-        <v>7640</v>
+        <v>7655</v>
       </c>
       <c r="E15" s="9">
-        <v>6441</v>
+        <v>6459</v>
       </c>
       <c r="F15" s="9">
-        <v>26708</v>
+        <v>26757</v>
       </c>
       <c r="G15" s="9">
-        <v>3830</v>
+        <v>3835</v>
       </c>
       <c r="H15" s="9">
         <v>511</v>
@@ -2458,7 +2461,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>401914</v>
+        <v>402700</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2469,28 +2472,28 @@
         <v>107</v>
       </c>
       <c r="C16" s="9">
-        <v>329082</v>
+        <v>330119</v>
       </c>
       <c r="D16" s="9">
-        <v>4759</v>
+        <v>4769</v>
       </c>
       <c r="E16" s="9">
-        <v>2844</v>
+        <v>2850</v>
       </c>
       <c r="F16" s="9">
-        <v>19200</v>
+        <v>19263</v>
       </c>
       <c r="G16" s="9">
-        <v>3851</v>
+        <v>3862</v>
       </c>
       <c r="H16" s="9">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>333841</v>
+        <v>334888</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2501,19 +2504,19 @@
         <v>113</v>
       </c>
       <c r="C17" s="9">
-        <v>197014</v>
+        <v>197053</v>
       </c>
       <c r="D17" s="9">
-        <v>4833</v>
+        <v>4834</v>
       </c>
       <c r="E17" s="9">
         <v>2179</v>
       </c>
       <c r="F17" s="9">
-        <v>10288</v>
+        <v>10289</v>
       </c>
       <c r="G17" s="9">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="H17" s="9">
         <v>399</v>
@@ -2522,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201847</v>
+        <v>201887</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2533,16 +2536,16 @@
         <v>120</v>
       </c>
       <c r="C18" s="9">
-        <v>247911</v>
+        <v>248165</v>
       </c>
       <c r="D18" s="9">
-        <v>5415</v>
+        <v>5418</v>
       </c>
       <c r="E18" s="9">
-        <v>2638</v>
+        <v>2642</v>
       </c>
       <c r="F18" s="9">
-        <v>14215</v>
+        <v>14228</v>
       </c>
       <c r="G18" s="9">
         <v>2384</v>
@@ -2554,7 +2557,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>253326</v>
+        <v>253583</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2565,16 +2568,16 @@
         <v>127</v>
       </c>
       <c r="C19" s="9">
-        <v>136462</v>
+        <v>136569</v>
       </c>
       <c r="D19" s="9">
-        <v>1746</v>
+        <v>1747</v>
       </c>
       <c r="E19" s="9">
         <v>1046</v>
       </c>
       <c r="F19" s="9">
-        <v>10394</v>
+        <v>10406</v>
       </c>
       <c r="G19" s="9">
         <v>223</v>
@@ -2586,7 +2589,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>138208</v>
+        <v>138316</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2597,28 +2600,28 @@
         <v>133</v>
       </c>
       <c r="C20" s="9">
-        <v>572171</v>
+        <v>573826</v>
       </c>
       <c r="D20" s="9">
-        <v>6932</v>
+        <v>6950</v>
       </c>
       <c r="E20" s="9">
-        <v>3420</v>
+        <v>3428</v>
       </c>
       <c r="F20" s="9">
-        <v>16360</v>
+        <v>16408</v>
       </c>
       <c r="G20" s="9">
-        <v>1012</v>
+        <v>1015</v>
       </c>
       <c r="H20" s="9">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>579103</v>
+        <v>580776</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2629,19 +2632,19 @@
         <v>139</v>
       </c>
       <c r="C21" s="9">
-        <v>117482</v>
+        <v>117782</v>
       </c>
       <c r="D21" s="9">
-        <v>1110</v>
+        <v>1113</v>
       </c>
       <c r="E21" s="9">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="F21" s="9">
-        <v>5077</v>
+        <v>5093</v>
       </c>
       <c r="G21" s="9">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="H21" s="9">
         <v>734</v>
@@ -2650,7 +2653,7 @@
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>118592</v>
+        <v>118895</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2661,28 +2664,28 @@
         <v>145</v>
       </c>
       <c r="C22" s="12">
-        <v>6373215</v>
+        <v>6390833</v>
       </c>
       <c r="D22" s="12">
-        <v>108720</v>
+        <v>108927</v>
       </c>
       <c r="E22" s="12">
-        <v>68968</v>
+        <v>69158</v>
       </c>
       <c r="F22" s="12">
-        <v>344440</v>
+        <v>345349</v>
       </c>
       <c r="G22" s="12">
-        <v>56036</v>
+        <v>56190</v>
       </c>
       <c r="H22" s="12">
-        <v>9355</v>
+        <v>9374</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6481935</v>
+        <v>6499760</v>
       </c>
     </row>
   </sheetData>
@@ -2776,10 +2779,10 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1111</v>
+        <v>1118</v>
       </c>
       <c r="D7" s="6">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>158</v>
@@ -2844,7 +2847,7 @@
         <v>65</v>
       </c>
       <c r="C11" s="9">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D11" s="9">
         <v>24</v>
@@ -2861,7 +2864,7 @@
         <v>72</v>
       </c>
       <c r="C12" s="9">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
@@ -2895,10 +2898,10 @@
         <v>87</v>
       </c>
       <c r="C14" s="9">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D14" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>165</v>
@@ -2912,13 +2915,13 @@
         <v>93</v>
       </c>
       <c r="C15" s="9">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D15" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2929,13 +2932,13 @@
         <v>100</v>
       </c>
       <c r="C16" s="9">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D16" s="9">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2952,7 +2955,7 @@
         <v>2</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2963,13 +2966,13 @@
         <v>113</v>
       </c>
       <c r="C18" s="9">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D18" s="9">
         <v>8</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2983,10 +2986,10 @@
         <v>71</v>
       </c>
       <c r="D19" s="9">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2997,7 +3000,7 @@
         <v>127</v>
       </c>
       <c r="C20" s="9">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D20" s="9">
         <v>0</v>
@@ -3017,10 +3020,10 @@
         <v>127</v>
       </c>
       <c r="D21" s="9">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3037,7 +3040,7 @@
         <v>21</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3048,10 +3051,10 @@
         <v>145</v>
       </c>
       <c r="C23" s="12">
-        <v>1111</v>
+        <v>1118</v>
       </c>
       <c r="D23" s="12">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>158</v>

</xml_diff>

<commit_message>
Perbarui data SE2026 22/08/2026  6:44:32,78
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="172">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 21 Agu 2026, 18.23 | Dicetak: 21 Agu 2026, 21.56</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 22 Agu 2026, 06.19 | Dicetak: 22 Agu 2026, 06.43</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,7 +123,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>66,22</t>
+    <t>66,64</t>
   </si>
   <si>
     <t>1,8</t>
@@ -132,13 +132,13 @@
     <t>0,05</t>
   </si>
   <si>
-    <t>21,28</t>
+    <t>21,37</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>77,9</t>
+    <t>78,4</t>
   </si>
   <si>
     <t>1801</t>
@@ -147,22 +147,22 @@
     <t>LAMPUNG BARAT</t>
   </si>
   <si>
-    <t>79,33</t>
-  </si>
-  <si>
-    <t>1,13</t>
+    <t>79,49</t>
+  </si>
+  <si>
+    <t>1,14</t>
   </si>
   <si>
     <t>0,04</t>
   </si>
   <si>
-    <t>18,37</t>
+    <t>18,38</t>
   </si>
   <si>
     <t>0,08</t>
   </si>
   <si>
-    <t>92,16</t>
+    <t>92,35</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,82 +171,82 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>69,13</t>
-  </si>
-  <si>
-    <t>0,99</t>
-  </si>
-  <si>
-    <t>17,16</t>
+    <t>69,53</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>17,26</t>
+  </si>
+  <si>
+    <t>84,77</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>62,01</t>
+  </si>
+  <si>
+    <t>1,21</t>
+  </si>
+  <si>
+    <t>20,13</t>
+  </si>
+  <si>
+    <t>0,09</t>
+  </si>
+  <si>
+    <t>74,61</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>68,54</t>
+  </si>
+  <si>
+    <t>1,9</t>
+  </si>
+  <si>
+    <t>0,06</t>
+  </si>
+  <si>
+    <t>18,53</t>
+  </si>
+  <si>
+    <t>77,66</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>68,25</t>
+  </si>
+  <si>
+    <t>2,74</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>84,25</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>61,36</t>
-  </si>
-  <si>
-    <t>1,21</t>
-  </si>
-  <si>
-    <t>20,01</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>73,84</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>68,14</t>
-  </si>
-  <si>
-    <t>1,89</t>
-  </si>
-  <si>
-    <t>0,06</t>
-  </si>
-  <si>
-    <t>18,46</t>
-  </si>
-  <si>
-    <t>77,21</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>67,77</t>
-  </si>
-  <si>
-    <t>2,73</t>
-  </si>
-  <si>
-    <t>18,58</t>
-  </si>
-  <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>76,77</t>
+    <t>18,68</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>77,31</t>
   </si>
   <si>
     <t>1806</t>
@@ -255,7 +255,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>67,15</t>
+    <t>67,54</t>
   </si>
   <si>
     <t>1,95</t>
@@ -264,13 +264,10 @@
     <t>0,03</t>
   </si>
   <si>
-    <t>25,98</t>
-  </si>
-  <si>
-    <t>0,1</t>
-  </si>
-  <si>
-    <t>78,89</t>
+    <t>26,05</t>
+  </si>
+  <si>
+    <t>79,37</t>
   </si>
   <si>
     <t>1807</t>
@@ -279,16 +276,16 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>68,18</t>
+    <t>68,77</t>
   </si>
   <si>
     <t>1,71</t>
   </si>
   <si>
-    <t>18,9</t>
-  </si>
-  <si>
-    <t>79,86</t>
+    <t>18,97</t>
+  </si>
+  <si>
+    <t>80,57</t>
   </si>
   <si>
     <t>1808</t>
@@ -297,19 +294,19 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>60,57</t>
-  </si>
-  <si>
-    <t>2,26</t>
-  </si>
-  <si>
-    <t>26,17</t>
+    <t>61,04</t>
+  </si>
+  <si>
+    <t>2,27</t>
+  </si>
+  <si>
+    <t>26,25</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>72,57</t>
+    <t>73,15</t>
   </si>
   <si>
     <t>1809</t>
@@ -318,19 +315,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>72,3</t>
-  </si>
-  <si>
-    <t>2,99</t>
-  </si>
-  <si>
-    <t>21,39</t>
-  </si>
-  <si>
-    <t>0,12</t>
-  </si>
-  <si>
-    <t>86,11</t>
+    <t>72,6</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>21,47</t>
+  </si>
+  <si>
+    <t>0,13</t>
+  </si>
+  <si>
+    <t>86,49</t>
   </si>
   <si>
     <t>1810</t>
@@ -339,16 +336,16 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>72,99</t>
-  </si>
-  <si>
-    <t>1,48</t>
-  </si>
-  <si>
-    <t>16,35</t>
-  </si>
-  <si>
-    <t>82,31</t>
+    <t>73,5</t>
+  </si>
+  <si>
+    <t>1,49</t>
+  </si>
+  <si>
+    <t>16,5</t>
+  </si>
+  <si>
+    <t>82,9</t>
   </si>
   <si>
     <t>1811</t>
@@ -357,19 +354,19 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>74,29</t>
+    <t>74,31</t>
   </si>
   <si>
     <t>1,58</t>
   </si>
   <si>
-    <t>24,98</t>
+    <t>24,95</t>
   </si>
   <si>
     <t>0,16</t>
   </si>
   <si>
-    <t>90,46</t>
+    <t>90,5</t>
   </si>
   <si>
     <t>1812</t>
@@ -378,7 +375,7 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>73,92</t>
+    <t>74,02</t>
   </si>
   <si>
     <t>2,43</t>
@@ -387,10 +384,10 @@
     <t>23,17</t>
   </si>
   <si>
-    <t>0,26</t>
-  </si>
-  <si>
-    <t>86,73</t>
+    <t>0,27</t>
+  </si>
+  <si>
+    <t>86,87</t>
   </si>
   <si>
     <t>1813</t>
@@ -399,16 +396,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>81,49</t>
+    <t>81,62</t>
   </si>
   <si>
     <t>0,84</t>
   </si>
   <si>
-    <t>17,5</t>
-  </si>
-  <si>
-    <t>99,17</t>
+    <t>17,47</t>
+  </si>
+  <si>
+    <t>99,41</t>
   </si>
   <si>
     <t>1871</t>
@@ -417,16 +414,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>49,14</t>
-  </si>
-  <si>
-    <t>0,86</t>
-  </si>
-  <si>
-    <t>30,91</t>
-  </si>
-  <si>
-    <t>62,69</t>
+    <t>49,49</t>
+  </si>
+  <si>
+    <t>0,87</t>
+  </si>
+  <si>
+    <t>31,08</t>
+  </si>
+  <si>
+    <t>63,12</t>
   </si>
   <si>
     <t>1872</t>
@@ -435,16 +432,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>64,04</t>
+    <t>64,38</t>
   </si>
   <si>
     <t>1,38</t>
   </si>
   <si>
-    <t>21,81</t>
-  </si>
-  <si>
-    <t>73,48</t>
+    <t>21,96</t>
+  </si>
+  <si>
+    <t>73,89</t>
   </si>
   <si>
     <t/>
@@ -489,7 +486,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>14,04</t>
+    <t>13,99</t>
   </si>
   <si>
     <t>0</t>
@@ -501,10 +498,10 @@
     <t>4,04</t>
   </si>
   <si>
-    <t>20,51</t>
-  </si>
-  <si>
-    <t>6,38</t>
+    <t>20,17</t>
+  </si>
+  <si>
+    <t>6,28</t>
   </si>
   <si>
     <t>15,63</t>
@@ -513,19 +510,19 @@
     <t>3,85</t>
   </si>
   <si>
-    <t>1,08</t>
-  </si>
-  <si>
-    <t>30,52</t>
-  </si>
-  <si>
-    <t>4,35</t>
-  </si>
-  <si>
-    <t>29,63</t>
-  </si>
-  <si>
-    <t>32,39</t>
+    <t>1,06</t>
+  </si>
+  <si>
+    <t>30,32</t>
+  </si>
+  <si>
+    <t>4,17</t>
+  </si>
+  <si>
+    <t>34,78</t>
+  </si>
+  <si>
+    <t>32,86</t>
   </si>
   <si>
     <t>5,51</t>
@@ -1192,40 +1189,40 @@
         <v>2730933</v>
       </c>
       <c r="D6" s="6">
-        <v>1808552</v>
+        <v>1819978</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>318779</v>
+        <v>320950</v>
       </c>
       <c r="G6" s="6">
-        <v>49044</v>
+        <v>49181</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1444</v>
+        <v>1470</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>581061</v>
+        <v>583599</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
       </c>
       <c r="M6" s="6">
-        <v>3042</v>
+        <v>3132</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2127331</v>
+        <v>2140928</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1242,28 +1239,28 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67546</v>
+        <v>67681</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10927</v>
+        <v>10952</v>
       </c>
       <c r="G7" s="9">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
       </c>
       <c r="I7" s="9">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15645</v>
+        <v>15651</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1275,7 +1272,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78473</v>
+        <v>78633</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1292,16 +1289,16 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>119564</v>
+        <v>120254</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>26157</v>
+        <v>26361</v>
       </c>
       <c r="G8" s="9">
-        <v>1716</v>
+        <v>1722</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
@@ -1313,169 +1310,169 @@
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>29682</v>
+        <v>29856</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
       </c>
       <c r="M8" s="9">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="N8" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="O8" s="9">
+        <v>146615</v>
+      </c>
+      <c r="P8" s="10" t="s">
         <v>55</v>
-      </c>
-      <c r="O8" s="9">
-        <v>145721</v>
-      </c>
-      <c r="P8" s="10" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>57</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>58</v>
       </c>
       <c r="C9" s="9">
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>210292</v>
+        <v>212517</v>
       </c>
       <c r="E9" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="9">
+        <v>43192</v>
+      </c>
+      <c r="G9" s="9">
+        <v>4155</v>
+      </c>
+      <c r="H9" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="9">
-        <v>42799</v>
-      </c>
-      <c r="G9" s="9">
-        <v>4137</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>60</v>
-      </c>
       <c r="I9" s="9">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>68564</v>
+        <v>68996</v>
       </c>
       <c r="L9" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="M9" s="9">
+        <v>319</v>
+      </c>
+      <c r="N9" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="M9" s="9">
-        <v>306</v>
-      </c>
-      <c r="N9" s="10" t="s">
+      <c r="O9" s="9">
+        <v>255709</v>
+      </c>
+      <c r="P9" s="10" t="s">
         <v>62</v>
-      </c>
-      <c r="O9" s="9">
-        <v>253091</v>
-      </c>
-      <c r="P9" s="10" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>65</v>
       </c>
       <c r="C10" s="9">
         <v>362839</v>
       </c>
       <c r="D10" s="9">
-        <v>247252</v>
+        <v>248689</v>
       </c>
       <c r="E10" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="9">
+        <v>33091</v>
+      </c>
+      <c r="G10" s="9">
+        <v>6879</v>
+      </c>
+      <c r="H10" s="10" t="s">
         <v>66</v>
-      </c>
-      <c r="F10" s="9">
-        <v>32880</v>
-      </c>
-      <c r="G10" s="9">
-        <v>6859</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>67</v>
       </c>
       <c r="I10" s="9">
         <v>200</v>
       </c>
       <c r="J10" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="9">
+        <v>67249</v>
+      </c>
+      <c r="L10" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="K10" s="9">
-        <v>66986</v>
-      </c>
-      <c r="L10" s="10" t="s">
-        <v>69</v>
-      </c>
       <c r="M10" s="9">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="N10" s="10" t="s">
         <v>48</v>
       </c>
       <c r="O10" s="9">
-        <v>280132</v>
+        <v>281780</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>71</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>72</v>
       </c>
       <c r="C11" s="9">
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>304677</v>
+        <v>306840</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" s="9">
+        <v>40732</v>
+      </c>
+      <c r="G11" s="9">
+        <v>12303</v>
+      </c>
+      <c r="H11" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="9">
-        <v>40448</v>
-      </c>
-      <c r="G11" s="9">
-        <v>12270</v>
-      </c>
-      <c r="H11" s="10" t="s">
+      <c r="I11" s="9">
+        <v>308</v>
+      </c>
+      <c r="J11" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="I11" s="9">
-        <v>307</v>
-      </c>
-      <c r="J11" s="10" t="s">
-        <v>55</v>
-      </c>
       <c r="K11" s="9">
-        <v>83525</v>
+        <v>83993</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>75</v>
       </c>
       <c r="M11" s="9">
-        <v>1090</v>
+        <v>1107</v>
       </c>
       <c r="N11" s="10" t="s">
         <v>76</v>
       </c>
       <c r="O11" s="9">
-        <v>345125</v>
+        <v>347572</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>77</v>
@@ -1492,119 +1489,119 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>133886</v>
+        <v>134663</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>80</v>
       </c>
       <c r="F12" s="9">
-        <v>23425</v>
+        <v>23604</v>
       </c>
       <c r="G12" s="9">
-        <v>3892</v>
+        <v>3890</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>81</v>
       </c>
       <c r="I12" s="9">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="J12" s="10" t="s">
         <v>82</v>
       </c>
       <c r="K12" s="9">
-        <v>51811</v>
+        <v>51945</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>83</v>
       </c>
       <c r="M12" s="9">
-        <v>199</v>
+        <v>217</v>
       </c>
       <c r="N12" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="O12" s="9">
+        <v>158267</v>
+      </c>
+      <c r="P12" s="10" t="s">
         <v>84</v>
-      </c>
-      <c r="O12" s="9">
-        <v>157311</v>
-      </c>
-      <c r="P12" s="10" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>86</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="C13" s="9">
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>99606</v>
+        <v>100471</v>
       </c>
       <c r="E13" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="F13" s="9">
+        <v>17239</v>
+      </c>
+      <c r="G13" s="9">
+        <v>2502</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="F13" s="9">
-        <v>17067</v>
-      </c>
-      <c r="G13" s="9">
-        <v>2493</v>
-      </c>
-      <c r="H13" s="10" t="s">
+      <c r="I13" s="9">
+        <v>81</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="9">
+        <v>27711</v>
+      </c>
+      <c r="L13" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="I13" s="9">
-        <v>79</v>
-      </c>
-      <c r="J13" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="K13" s="9">
-        <v>27614</v>
-      </c>
-      <c r="L13" s="10" t="s">
-        <v>90</v>
-      </c>
       <c r="M13" s="9">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="N13" s="10" t="s">
         <v>40</v>
       </c>
       <c r="O13" s="9">
-        <v>116673</v>
+        <v>117710</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>92</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>93</v>
       </c>
       <c r="C14" s="9">
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>81921</v>
+        <v>82558</v>
       </c>
       <c r="E14" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="F14" s="9">
+        <v>16377</v>
+      </c>
+      <c r="G14" s="9">
+        <v>3066</v>
+      </c>
+      <c r="H14" s="10" t="s">
         <v>94</v>
-      </c>
-      <c r="F14" s="9">
-        <v>16234</v>
-      </c>
-      <c r="G14" s="9">
-        <v>3060</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>95</v>
       </c>
       <c r="I14" s="9">
         <v>34</v>
@@ -1613,148 +1610,148 @@
         <v>82</v>
       </c>
       <c r="K14" s="9">
-        <v>35393</v>
+        <v>35499</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M14" s="9">
         <v>24</v>
       </c>
       <c r="N14" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="O14" s="9">
+        <v>98935</v>
+      </c>
+      <c r="P14" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="O14" s="9">
-        <v>98155</v>
-      </c>
-      <c r="P14" s="10" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>99</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>100</v>
       </c>
       <c r="C15" s="9">
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>110004</v>
+        <v>110466</v>
       </c>
       <c r="E15" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F15" s="9">
+        <v>21128</v>
+      </c>
+      <c r="G15" s="9">
+        <v>4564</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="F15" s="9">
-        <v>21021</v>
-      </c>
-      <c r="G15" s="9">
-        <v>4553</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>102</v>
-      </c>
       <c r="I15" s="9">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J15" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>32551</v>
+        <v>32663</v>
       </c>
       <c r="L15" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="M15" s="9">
+        <v>192</v>
+      </c>
+      <c r="N15" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="M15" s="9">
-        <v>190</v>
-      </c>
-      <c r="N15" s="10" t="s">
+      <c r="O15" s="9">
+        <v>131594</v>
+      </c>
+      <c r="P15" s="10" t="s">
         <v>104</v>
-      </c>
-      <c r="O15" s="9">
-        <v>131025</v>
-      </c>
-      <c r="P15" s="10" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>106</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>107</v>
       </c>
       <c r="C16" s="9">
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>99071</v>
+        <v>99774</v>
       </c>
       <c r="E16" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F16" s="9">
+        <v>12754</v>
+      </c>
+      <c r="G16" s="9">
+        <v>2018</v>
+      </c>
+      <c r="H16" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="F16" s="9">
-        <v>12651</v>
-      </c>
-      <c r="G16" s="9">
-        <v>2004</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>109</v>
-      </c>
       <c r="I16" s="9">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>48</v>
       </c>
       <c r="K16" s="9">
-        <v>22196</v>
+        <v>22403</v>
       </c>
       <c r="L16" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="M16" s="9">
+        <v>89</v>
+      </c>
+      <c r="N16" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="O16" s="9">
+        <v>112528</v>
+      </c>
+      <c r="P16" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="M16" s="9">
-        <v>88</v>
-      </c>
-      <c r="N16" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="O16" s="9">
-        <v>111722</v>
-      </c>
-      <c r="P16" s="10" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>112</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>113</v>
       </c>
       <c r="C17" s="9">
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55800</v>
+        <v>55820</v>
       </c>
       <c r="E17" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="F17" s="9">
+        <v>12162</v>
+      </c>
+      <c r="G17" s="9">
+        <v>1189</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>114</v>
-      </c>
-      <c r="F17" s="9">
-        <v>12150</v>
-      </c>
-      <c r="G17" s="9">
-        <v>1186</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>115</v>
       </c>
       <c r="I17" s="9">
         <v>80</v>
@@ -1763,48 +1760,48 @@
         <v>40</v>
       </c>
       <c r="K17" s="9">
-        <v>18765</v>
+        <v>18742</v>
       </c>
       <c r="L17" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="M17" s="9">
+        <v>120</v>
+      </c>
+      <c r="N17" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="M17" s="9">
-        <v>123</v>
-      </c>
-      <c r="N17" s="10" t="s">
+      <c r="O17" s="9">
+        <v>67982</v>
+      </c>
+      <c r="P17" s="10" t="s">
         <v>117</v>
-      </c>
-      <c r="O17" s="9">
-        <v>67950</v>
-      </c>
-      <c r="P17" s="10" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>119</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>120</v>
       </c>
       <c r="C18" s="9">
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>73301</v>
+        <v>73400</v>
       </c>
       <c r="E18" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F18" s="9">
+        <v>12744</v>
+      </c>
+      <c r="G18" s="9">
+        <v>2411</v>
+      </c>
+      <c r="H18" s="10" t="s">
         <v>121</v>
-      </c>
-      <c r="F18" s="9">
-        <v>12710</v>
-      </c>
-      <c r="G18" s="9">
-        <v>2408</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>122</v>
       </c>
       <c r="I18" s="9">
         <v>50</v>
@@ -1813,219 +1810,219 @@
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22975</v>
+        <v>22979</v>
       </c>
       <c r="L18" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="M18" s="9">
+        <v>263</v>
+      </c>
+      <c r="N18" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="M18" s="9">
-        <v>253</v>
-      </c>
-      <c r="N18" s="10" t="s">
+      <c r="O18" s="9">
+        <v>86144</v>
+      </c>
+      <c r="P18" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="O18" s="9">
-        <v>86011</v>
-      </c>
-      <c r="P18" s="10" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>126</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>127</v>
       </c>
       <c r="C19" s="9">
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>34040</v>
+        <v>34093</v>
       </c>
       <c r="E19" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="F19" s="9">
+        <v>7434</v>
+      </c>
+      <c r="G19" s="9">
+        <v>352</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="F19" s="9">
-        <v>7386</v>
-      </c>
-      <c r="G19" s="9">
-        <v>350</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>129</v>
       </c>
       <c r="I19" s="9">
         <v>27</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K19" s="9">
-        <v>7312</v>
+        <v>7297</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M19" s="9">
         <v>27</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="O19" s="9">
-        <v>41426</v>
+        <v>41527</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="C20" s="9">
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>137328</v>
+        <v>138304</v>
       </c>
       <c r="E20" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="F20" s="9">
+        <v>38095</v>
+      </c>
+      <c r="G20" s="9">
+        <v>2423</v>
+      </c>
+      <c r="H20" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="F20" s="9">
-        <v>37873</v>
-      </c>
-      <c r="G20" s="9">
-        <v>2412</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>135</v>
-      </c>
       <c r="I20" s="9">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>86374</v>
+        <v>86864</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M20" s="9">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="N20" s="10" t="s">
         <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>175201</v>
+        <v>176399</v>
       </c>
       <c r="P20" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>138</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>139</v>
       </c>
       <c r="C21" s="9">
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>34264</v>
+        <v>34448</v>
       </c>
       <c r="E21" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="F21" s="9">
+        <v>5085</v>
+      </c>
+      <c r="G21" s="9">
+        <v>740</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="F21" s="9">
-        <v>5051</v>
-      </c>
-      <c r="G21" s="9">
-        <v>738</v>
-      </c>
-      <c r="H21" s="10" t="s">
+      <c r="I21" s="9">
+        <v>35</v>
+      </c>
+      <c r="J21" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="K21" s="9">
+        <v>11751</v>
+      </c>
+      <c r="L21" s="10" t="s">
         <v>141</v>
-      </c>
-      <c r="I21" s="9">
-        <v>34</v>
-      </c>
-      <c r="J21" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="K21" s="9">
-        <v>11668</v>
-      </c>
-      <c r="L21" s="10" t="s">
-        <v>142</v>
       </c>
       <c r="M21" s="9">
         <v>11</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O21" s="9">
-        <v>39315</v>
+        <v>39533</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>144</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>145</v>
       </c>
       <c r="C22" s="12">
         <v>2730933</v>
       </c>
       <c r="D22" s="12">
-        <v>1808552</v>
+        <v>1819978</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>318779</v>
+        <v>320950</v>
       </c>
       <c r="G22" s="12">
-        <v>49044</v>
+        <v>49181</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1444</v>
+        <v>1470</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>581061</v>
+        <v>583599</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
       </c>
       <c r="M22" s="12">
-        <v>3042</v>
+        <v>3132</v>
       </c>
       <c r="N22" s="13" t="s">
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2127331</v>
+        <v>2140928</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2054,7 +2051,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2088,28 +2085,28 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>147</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>148</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>150</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>151</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2152,28 +2149,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6390833</v>
+        <v>6432265</v>
       </c>
       <c r="D6" s="6">
-        <v>108927</v>
+        <v>109351</v>
       </c>
       <c r="E6" s="6">
-        <v>69158</v>
+        <v>69589</v>
       </c>
       <c r="F6" s="6">
-        <v>345349</v>
+        <v>347478</v>
       </c>
       <c r="G6" s="6">
-        <v>56190</v>
+        <v>56544</v>
       </c>
       <c r="H6" s="6">
-        <v>9374</v>
+        <v>9400</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6499760</v>
+        <v>6541616</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2184,19 +2181,19 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>246024</v>
+        <v>246521</v>
       </c>
       <c r="D7" s="9">
-        <v>2858</v>
+        <v>2868</v>
       </c>
       <c r="E7" s="9">
-        <v>2109</v>
+        <v>2117</v>
       </c>
       <c r="F7" s="9">
-        <v>13015</v>
+        <v>13070</v>
       </c>
       <c r="G7" s="9">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="H7" s="9">
         <v>397</v>
@@ -2205,7 +2202,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>248882</v>
+        <v>249389</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2216,124 +2213,124 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>445035</v>
+        <v>447851</v>
       </c>
       <c r="D8" s="9">
-        <v>5873</v>
+        <v>5903</v>
       </c>
       <c r="E8" s="9">
-        <v>4375</v>
+        <v>4391</v>
       </c>
       <c r="F8" s="9">
-        <v>34144</v>
+        <v>34349</v>
       </c>
       <c r="G8" s="9">
-        <v>4063</v>
+        <v>4089</v>
       </c>
       <c r="H8" s="9">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="I8" s="9">
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>450908</v>
+        <v>453754</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>58</v>
-      </c>
       <c r="C9" s="9">
-        <v>770716</v>
+        <v>778806</v>
       </c>
       <c r="D9" s="9">
-        <v>13317</v>
+        <v>13446</v>
       </c>
       <c r="E9" s="9">
-        <v>8766</v>
+        <v>8860</v>
       </c>
       <c r="F9" s="9">
-        <v>38260</v>
+        <v>38625</v>
       </c>
       <c r="G9" s="9">
-        <v>4703</v>
+        <v>4740</v>
       </c>
       <c r="H9" s="9">
-        <v>1016</v>
+        <v>1022</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>784033</v>
+        <v>792252</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>65</v>
-      </c>
       <c r="C10" s="9">
-        <v>792878</v>
+        <v>797541</v>
       </c>
       <c r="D10" s="9">
-        <v>15268</v>
+        <v>15340</v>
       </c>
       <c r="E10" s="9">
-        <v>9340</v>
+        <v>9398</v>
       </c>
       <c r="F10" s="9">
-        <v>39216</v>
+        <v>39444</v>
       </c>
       <c r="G10" s="9">
-        <v>19769</v>
+        <v>19889</v>
       </c>
       <c r="H10" s="9">
-        <v>1068</v>
+        <v>1072</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>808146</v>
+        <v>812881</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>72</v>
-      </c>
       <c r="C11" s="9">
-        <v>1009122</v>
+        <v>1016322</v>
       </c>
       <c r="D11" s="9">
-        <v>20258</v>
+        <v>20269</v>
       </c>
       <c r="E11" s="9">
-        <v>12093</v>
+        <v>12183</v>
       </c>
       <c r="F11" s="9">
-        <v>45454</v>
+        <v>45756</v>
       </c>
       <c r="G11" s="9">
-        <v>8257</v>
+        <v>8319</v>
       </c>
       <c r="H11" s="9">
-        <v>1740</v>
+        <v>1743</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1029380</v>
+        <v>1036591</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2344,115 +2341,115 @@
         <v>79</v>
       </c>
       <c r="C12" s="9">
-        <v>487338</v>
+        <v>490372</v>
       </c>
       <c r="D12" s="9">
-        <v>6166</v>
+        <v>6183</v>
       </c>
       <c r="E12" s="9">
-        <v>5857</v>
+        <v>5888</v>
       </c>
       <c r="F12" s="9">
-        <v>27857</v>
+        <v>28035</v>
       </c>
       <c r="G12" s="9">
-        <v>1988</v>
+        <v>1995</v>
       </c>
       <c r="H12" s="9">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>493504</v>
+        <v>496555</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>87</v>
-      </c>
       <c r="C13" s="9">
-        <v>350314</v>
+        <v>353471</v>
       </c>
       <c r="D13" s="9">
-        <v>4397</v>
+        <v>4422</v>
       </c>
       <c r="E13" s="9">
-        <v>3968</v>
+        <v>4004</v>
       </c>
       <c r="F13" s="9">
-        <v>25199</v>
+        <v>25432</v>
       </c>
       <c r="G13" s="9">
-        <v>1379</v>
+        <v>1389</v>
       </c>
       <c r="H13" s="9">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>354711</v>
+        <v>357893</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>93</v>
-      </c>
       <c r="C14" s="9">
-        <v>290847</v>
+        <v>293226</v>
       </c>
       <c r="D14" s="9">
-        <v>8304</v>
+        <v>8347</v>
       </c>
       <c r="E14" s="9">
-        <v>3201</v>
+        <v>3222</v>
       </c>
       <c r="F14" s="9">
-        <v>19760</v>
+        <v>19909</v>
       </c>
       <c r="G14" s="9">
-        <v>1946</v>
+        <v>1967</v>
       </c>
       <c r="H14" s="9">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>299151</v>
+        <v>301573</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>100</v>
-      </c>
       <c r="C15" s="9">
-        <v>395045</v>
+        <v>396828</v>
       </c>
       <c r="D15" s="9">
-        <v>7655</v>
+        <v>7674</v>
       </c>
       <c r="E15" s="9">
-        <v>6459</v>
+        <v>6488</v>
       </c>
       <c r="F15" s="9">
-        <v>26757</v>
+        <v>26874</v>
       </c>
       <c r="G15" s="9">
-        <v>3835</v>
+        <v>3853</v>
       </c>
       <c r="H15" s="9">
         <v>511</v>
@@ -2461,62 +2458,62 @@
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>402700</v>
+        <v>404502</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>107</v>
-      </c>
       <c r="C16" s="9">
-        <v>330119</v>
+        <v>332531</v>
       </c>
       <c r="D16" s="9">
-        <v>4769</v>
+        <v>4799</v>
       </c>
       <c r="E16" s="9">
-        <v>2850</v>
+        <v>2876</v>
       </c>
       <c r="F16" s="9">
-        <v>19263</v>
+        <v>19383</v>
       </c>
       <c r="G16" s="9">
-        <v>3862</v>
+        <v>3905</v>
       </c>
       <c r="H16" s="9">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>334888</v>
+        <v>337330</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>113</v>
-      </c>
       <c r="C17" s="9">
-        <v>197053</v>
+        <v>197150</v>
       </c>
       <c r="D17" s="9">
-        <v>4834</v>
+        <v>4833</v>
       </c>
       <c r="E17" s="9">
-        <v>2179</v>
+        <v>2180</v>
       </c>
       <c r="F17" s="9">
-        <v>10289</v>
+        <v>10293</v>
       </c>
       <c r="G17" s="9">
-        <v>1709</v>
+        <v>1708</v>
       </c>
       <c r="H17" s="9">
         <v>399</v>
@@ -2525,59 +2522,59 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201887</v>
+        <v>201983</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>120</v>
-      </c>
       <c r="C18" s="9">
-        <v>248165</v>
+        <v>248565</v>
       </c>
       <c r="D18" s="9">
-        <v>5418</v>
+        <v>5425</v>
       </c>
       <c r="E18" s="9">
-        <v>2642</v>
+        <v>2644</v>
       </c>
       <c r="F18" s="9">
-        <v>14228</v>
+        <v>14246</v>
       </c>
       <c r="G18" s="9">
-        <v>2384</v>
+        <v>2389</v>
       </c>
       <c r="H18" s="9">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>253583</v>
+        <v>253990</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>127</v>
-      </c>
       <c r="C19" s="9">
-        <v>136569</v>
+        <v>136847</v>
       </c>
       <c r="D19" s="9">
-        <v>1747</v>
+        <v>1752</v>
       </c>
       <c r="E19" s="9">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F19" s="9">
-        <v>10406</v>
+        <v>10418</v>
       </c>
       <c r="G19" s="9">
         <v>223</v>
@@ -2589,103 +2586,103 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>138316</v>
+        <v>138599</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>133</v>
-      </c>
       <c r="C20" s="9">
-        <v>573826</v>
+        <v>577795</v>
       </c>
       <c r="D20" s="9">
-        <v>6950</v>
+        <v>6973</v>
       </c>
       <c r="E20" s="9">
-        <v>3428</v>
+        <v>3444</v>
       </c>
       <c r="F20" s="9">
-        <v>16408</v>
+        <v>16511</v>
       </c>
       <c r="G20" s="9">
-        <v>1015</v>
+        <v>1017</v>
       </c>
       <c r="H20" s="9">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>580776</v>
+        <v>584768</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>139</v>
-      </c>
       <c r="C21" s="9">
-        <v>117782</v>
+        <v>118439</v>
       </c>
       <c r="D21" s="9">
-        <v>1113</v>
+        <v>1117</v>
       </c>
       <c r="E21" s="9">
-        <v>845</v>
+        <v>847</v>
       </c>
       <c r="F21" s="9">
-        <v>5093</v>
+        <v>5133</v>
       </c>
       <c r="G21" s="9">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="H21" s="9">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>118895</v>
+        <v>119556</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>145</v>
-      </c>
       <c r="C22" s="12">
-        <v>6390833</v>
+        <v>6432265</v>
       </c>
       <c r="D22" s="12">
-        <v>108927</v>
+        <v>109351</v>
       </c>
       <c r="E22" s="12">
-        <v>69158</v>
+        <v>69589</v>
       </c>
       <c r="F22" s="12">
-        <v>345349</v>
+        <v>347478</v>
       </c>
       <c r="G22" s="12">
-        <v>56190</v>
+        <v>56544</v>
       </c>
       <c r="H22" s="12">
-        <v>9374</v>
+        <v>9400</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6499760</v>
+        <v>6541616</v>
       </c>
     </row>
   </sheetData>
@@ -2712,7 +2709,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2736,7 +2733,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2745,13 +2742,13 @@
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2779,13 +2776,13 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1118</v>
+        <v>1122</v>
       </c>
       <c r="D7" s="6">
         <v>157</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2802,7 +2799,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2819,15 +2816,15 @@
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>57</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>58</v>
       </c>
       <c r="C10" s="9">
         <v>99</v>
@@ -2836,41 +2833,41 @@
         <v>4</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>65</v>
-      </c>
       <c r="C11" s="9">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D11" s="9">
         <v>24</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>72</v>
-      </c>
       <c r="C12" s="9">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2887,15 +2884,15 @@
         <v>5</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>86</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>87</v>
       </c>
       <c r="C14" s="9">
         <v>52</v>
@@ -2904,100 +2901,100 @@
         <v>2</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>93</v>
-      </c>
       <c r="C15" s="9">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D15" s="9">
         <v>1</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>100</v>
-      </c>
       <c r="C16" s="9">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D16" s="9">
         <v>47</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>107</v>
-      </c>
       <c r="C17" s="9">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D17" s="9">
         <v>2</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>113</v>
-      </c>
       <c r="C18" s="9">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D18" s="9">
         <v>8</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B19" s="8" t="s">
-        <v>120</v>
-      </c>
       <c r="C19" s="9">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D19" s="9">
         <v>23</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>126</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>127</v>
       </c>
       <c r="C20" s="9">
         <v>16</v>
@@ -3006,15 +3003,15 @@
         <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>132</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>133</v>
       </c>
       <c r="C21" s="9">
         <v>127</v>
@@ -3023,15 +3020,15 @@
         <v>7</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>138</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>139</v>
       </c>
       <c r="C22" s="9">
         <v>64</v>
@@ -3040,24 +3037,24 @@
         <v>21</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B23" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>145</v>
-      </c>
       <c r="C23" s="12">
-        <v>1118</v>
+        <v>1122</v>
       </c>
       <c r="D23" s="12">
         <v>157</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 23/08/2026  5:37:45,21
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -18,7 +18,7 @@
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 22 Agu 2026, 06.19 | Dicetak: 22 Agu 2026, 06.43</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 22 Agu 2026, 18.16 | Dicetak: 23 Agu 2026, 05.36</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,169 +123,172 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>66,64</t>
-  </si>
-  <si>
-    <t>1,8</t>
+    <t>67,05</t>
+  </si>
+  <si>
+    <t>1,81</t>
   </si>
   <si>
     <t>0,05</t>
   </si>
   <si>
-    <t>21,37</t>
+    <t>21,46</t>
+  </si>
+  <si>
+    <t>0,12</t>
+  </si>
+  <si>
+    <t>78,88</t>
+  </si>
+  <si>
+    <t>1801</t>
+  </si>
+  <si>
+    <t>LAMPUNG BARAT</t>
+  </si>
+  <si>
+    <t>79,62</t>
+  </si>
+  <si>
+    <t>1,14</t>
+  </si>
+  <si>
+    <t>0,04</t>
+  </si>
+  <si>
+    <t>18,48</t>
+  </si>
+  <si>
+    <t>0,08</t>
+  </si>
+  <si>
+    <t>92,51</t>
+  </si>
+  <si>
+    <t>1802</t>
+  </si>
+  <si>
+    <t>TANGGAMUS</t>
+  </si>
+  <si>
+    <t>69,96</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>17,38</t>
+  </si>
+  <si>
+    <t>85,34</t>
+  </si>
+  <si>
+    <t>1803</t>
+  </si>
+  <si>
+    <t>LAMPUNG SELATAN</t>
+  </si>
+  <si>
+    <t>62,61</t>
+  </si>
+  <si>
+    <t>1,22</t>
+  </si>
+  <si>
+    <t>20,26</t>
+  </si>
+  <si>
+    <t>0,1</t>
+  </si>
+  <si>
+    <t>75,34</t>
+  </si>
+  <si>
+    <t>1804</t>
+  </si>
+  <si>
+    <t>LAMPUNG TIMUR</t>
+  </si>
+  <si>
+    <t>68,91</t>
+  </si>
+  <si>
+    <t>1,9</t>
+  </si>
+  <si>
+    <t>18,62</t>
+  </si>
+  <si>
+    <t>78,09</t>
+  </si>
+  <si>
+    <t>1805</t>
+  </si>
+  <si>
+    <t>LAMPUNG TENGAH</t>
+  </si>
+  <si>
+    <t>68,75</t>
+  </si>
+  <si>
+    <t>2,74</t>
+  </si>
+  <si>
+    <t>0,07</t>
+  </si>
+  <si>
+    <t>18,75</t>
+  </si>
+  <si>
+    <t>0,25</t>
+  </si>
+  <si>
+    <t>77,87</t>
+  </si>
+  <si>
+    <t>1806</t>
+  </si>
+  <si>
+    <t>LAMPUNG UTARA</t>
+  </si>
+  <si>
+    <t>67,89</t>
+  </si>
+  <si>
+    <t>1,96</t>
+  </si>
+  <si>
+    <t>0,03</t>
+  </si>
+  <si>
+    <t>26,15</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>78,4</t>
-  </si>
-  <si>
-    <t>1801</t>
-  </si>
-  <si>
-    <t>LAMPUNG BARAT</t>
-  </si>
-  <si>
-    <t>79,49</t>
-  </si>
-  <si>
-    <t>1,14</t>
-  </si>
-  <si>
-    <t>0,04</t>
-  </si>
-  <si>
-    <t>18,38</t>
-  </si>
-  <si>
-    <t>0,08</t>
-  </si>
-  <si>
-    <t>92,35</t>
-  </si>
-  <si>
-    <t>1802</t>
-  </si>
-  <si>
-    <t>TANGGAMUS</t>
-  </si>
-  <si>
-    <t>69,53</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>17,26</t>
-  </si>
-  <si>
-    <t>84,77</t>
-  </si>
-  <si>
-    <t>1803</t>
-  </si>
-  <si>
-    <t>LAMPUNG SELATAN</t>
-  </si>
-  <si>
-    <t>62,01</t>
-  </si>
-  <si>
-    <t>1,21</t>
-  </si>
-  <si>
-    <t>20,13</t>
-  </si>
-  <si>
-    <t>0,09</t>
-  </si>
-  <si>
-    <t>74,61</t>
-  </si>
-  <si>
-    <t>1804</t>
-  </si>
-  <si>
-    <t>LAMPUNG TIMUR</t>
-  </si>
-  <si>
-    <t>68,54</t>
-  </si>
-  <si>
-    <t>1,9</t>
+    <t>79,81</t>
+  </si>
+  <si>
+    <t>1807</t>
+  </si>
+  <si>
+    <t>WAY KANAN</t>
+  </si>
+  <si>
+    <t>69,45</t>
+  </si>
+  <si>
+    <t>1,72</t>
   </si>
   <si>
     <t>0,06</t>
   </si>
   <si>
-    <t>18,53</t>
-  </si>
-  <si>
-    <t>77,66</t>
-  </si>
-  <si>
-    <t>1805</t>
-  </si>
-  <si>
-    <t>LAMPUNG TENGAH</t>
-  </si>
-  <si>
-    <t>68,25</t>
-  </si>
-  <si>
-    <t>2,74</t>
-  </si>
-  <si>
-    <t>0,07</t>
-  </si>
-  <si>
-    <t>18,68</t>
-  </si>
-  <si>
-    <t>0,25</t>
-  </si>
-  <si>
-    <t>77,31</t>
-  </si>
-  <si>
-    <t>1806</t>
-  </si>
-  <si>
-    <t>LAMPUNG UTARA</t>
-  </si>
-  <si>
-    <t>67,54</t>
-  </si>
-  <si>
-    <t>1,95</t>
-  </si>
-  <si>
-    <t>0,03</t>
-  </si>
-  <si>
-    <t>26,05</t>
-  </si>
-  <si>
-    <t>79,37</t>
-  </si>
-  <si>
-    <t>1807</t>
-  </si>
-  <si>
-    <t>WAY KANAN</t>
-  </si>
-  <si>
-    <t>68,77</t>
-  </si>
-  <si>
-    <t>1,71</t>
-  </si>
-  <si>
-    <t>18,97</t>
-  </si>
-  <si>
-    <t>80,57</t>
+    <t>19,02</t>
+  </si>
+  <si>
+    <t>81,39</t>
   </si>
   <si>
     <t>1808</t>
@@ -294,19 +297,19 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>61,04</t>
+    <t>61,55</t>
   </si>
   <si>
     <t>2,27</t>
   </si>
   <si>
-    <t>26,25</t>
+    <t>26,44</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>73,15</t>
+    <t>73,78</t>
   </si>
   <si>
     <t>1809</t>
@@ -315,19 +318,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>72,6</t>
+    <t>72,85</t>
   </si>
   <si>
     <t>3</t>
   </si>
   <si>
-    <t>21,47</t>
+    <t>21,53</t>
   </si>
   <si>
     <t>0,13</t>
   </si>
   <si>
-    <t>86,49</t>
+    <t>86,78</t>
   </si>
   <si>
     <t>1810</t>
@@ -336,16 +339,16 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>73,5</t>
+    <t>73,98</t>
   </si>
   <si>
     <t>1,49</t>
   </si>
   <si>
-    <t>16,5</t>
-  </si>
-  <si>
-    <t>82,9</t>
+    <t>16,59</t>
+  </si>
+  <si>
+    <t>83,44</t>
   </si>
   <si>
     <t>1811</t>
@@ -354,19 +357,19 @@
     <t>MESUJI</t>
   </si>
   <si>
-    <t>74,31</t>
+    <t>74,34</t>
   </si>
   <si>
     <t>1,58</t>
   </si>
   <si>
-    <t>24,95</t>
+    <t>24,92</t>
   </si>
   <si>
     <t>0,16</t>
   </si>
   <si>
-    <t>90,5</t>
+    <t>90,54</t>
   </si>
   <si>
     <t>1812</t>
@@ -375,19 +378,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>74,02</t>
+    <t>74,1</t>
   </si>
   <si>
     <t>2,43</t>
   </si>
   <si>
-    <t>23,17</t>
+    <t>23,16</t>
   </si>
   <si>
     <t>0,27</t>
   </si>
   <si>
-    <t>86,87</t>
+    <t>86,98</t>
   </si>
   <si>
     <t>1813</t>
@@ -396,16 +399,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>81,62</t>
+    <t>81,65</t>
   </si>
   <si>
     <t>0,84</t>
   </si>
   <si>
-    <t>17,47</t>
-  </si>
-  <si>
-    <t>99,41</t>
+    <t>17,46</t>
+  </si>
+  <si>
+    <t>99,5</t>
   </si>
   <si>
     <t>1871</t>
@@ -414,16 +417,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>49,49</t>
+    <t>49,79</t>
   </si>
   <si>
     <t>0,87</t>
   </si>
   <si>
-    <t>31,08</t>
-  </si>
-  <si>
-    <t>63,12</t>
+    <t>31,23</t>
+  </si>
+  <si>
+    <t>63,51</t>
   </si>
   <si>
     <t>1872</t>
@@ -432,16 +435,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>64,38</t>
-  </si>
-  <si>
-    <t>1,38</t>
-  </si>
-  <si>
-    <t>21,96</t>
-  </si>
-  <si>
-    <t>73,89</t>
+    <t>64,66</t>
+  </si>
+  <si>
+    <t>1,39</t>
+  </si>
+  <si>
+    <t>22,2</t>
+  </si>
+  <si>
+    <t>74,28</t>
   </si>
   <si>
     <t/>
@@ -486,7 +489,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>13,99</t>
+    <t>13,82</t>
   </si>
   <si>
     <t>0</t>
@@ -495,37 +498,34 @@
     <t>4</t>
   </si>
   <si>
-    <t>4,04</t>
-  </si>
-  <si>
-    <t>20,17</t>
-  </si>
-  <si>
-    <t>6,28</t>
+    <t>3,92</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>6,15</t>
   </si>
   <si>
     <t>15,63</t>
   </si>
   <si>
-    <t>3,85</t>
-  </si>
-  <si>
-    <t>1,06</t>
+    <t>3,77</t>
+  </si>
+  <si>
+    <t>1,05</t>
   </si>
   <si>
     <t>30,32</t>
   </si>
   <si>
-    <t>4,17</t>
-  </si>
-  <si>
     <t>34,78</t>
   </si>
   <si>
     <t>32,86</t>
   </si>
   <si>
-    <t>5,51</t>
+    <t>5,47</t>
   </si>
   <si>
     <t>32,81</t>
@@ -1189,40 +1189,40 @@
         <v>2730933</v>
       </c>
       <c r="D6" s="6">
-        <v>1819978</v>
+        <v>1830999</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>320950</v>
+        <v>323213</v>
       </c>
       <c r="G6" s="6">
-        <v>49181</v>
+        <v>49324</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1470</v>
+        <v>1481</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>583599</v>
+        <v>586180</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
       </c>
       <c r="M6" s="6">
-        <v>3132</v>
+        <v>3257</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2140928</v>
+        <v>2154212</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1239,16 +1239,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67681</v>
+        <v>67792</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10952</v>
+        <v>10978</v>
       </c>
       <c r="G7" s="9">
-        <v>967</v>
+        <v>969</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1260,19 +1260,19 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15651</v>
+        <v>15733</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
       </c>
       <c r="M7" s="9">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N7" s="10" t="s">
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78633</v>
+        <v>78770</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1289,40 +1289,40 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>120254</v>
+        <v>120998</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>26361</v>
+        <v>26598</v>
       </c>
       <c r="G8" s="9">
-        <v>1722</v>
+        <v>1732</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="9">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>29856</v>
+        <v>30062</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
       </c>
       <c r="M8" s="9">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="N8" s="10" t="s">
         <v>48</v>
       </c>
       <c r="O8" s="9">
-        <v>146615</v>
+        <v>147596</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>55</v>
@@ -1339,16 +1339,16 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>212517</v>
+        <v>214576</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>58</v>
       </c>
       <c r="F9" s="9">
-        <v>43192</v>
+        <v>43624</v>
       </c>
       <c r="G9" s="9">
-        <v>4155</v>
+        <v>4182</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>59</v>
@@ -1360,19 +1360,19 @@
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>68996</v>
+        <v>69433</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>60</v>
       </c>
       <c r="M9" s="9">
-        <v>319</v>
+        <v>333</v>
       </c>
       <c r="N9" s="10" t="s">
         <v>61</v>
       </c>
       <c r="O9" s="9">
-        <v>255709</v>
+        <v>258200</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>62</v>
@@ -1389,140 +1389,140 @@
         <v>362839</v>
       </c>
       <c r="D10" s="9">
-        <v>248689</v>
+        <v>250043</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>65</v>
       </c>
       <c r="F10" s="9">
-        <v>33091</v>
+        <v>33305</v>
       </c>
       <c r="G10" s="9">
-        <v>6879</v>
+        <v>6897</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I10" s="9">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="J10" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="K10" s="9">
+        <v>67547</v>
+      </c>
+      <c r="L10" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="K10" s="9">
-        <v>67249</v>
-      </c>
-      <c r="L10" s="10" t="s">
-        <v>68</v>
-      </c>
       <c r="M10" s="9">
-        <v>286</v>
+        <v>301</v>
       </c>
       <c r="N10" s="10" t="s">
         <v>48</v>
       </c>
       <c r="O10" s="9">
-        <v>281780</v>
+        <v>283348</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>71</v>
       </c>
       <c r="C11" s="9">
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>306840</v>
+        <v>309065</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="9">
+        <v>41014</v>
+      </c>
+      <c r="G11" s="9">
+        <v>12339</v>
+      </c>
+      <c r="H11" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="9">
-        <v>40732</v>
-      </c>
-      <c r="G11" s="9">
-        <v>12303</v>
-      </c>
-      <c r="H11" s="10" t="s">
+      <c r="I11" s="9">
+        <v>315</v>
+      </c>
+      <c r="J11" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="I11" s="9">
-        <v>308</v>
-      </c>
-      <c r="J11" s="10" t="s">
+      <c r="K11" s="9">
+        <v>84296</v>
+      </c>
+      <c r="L11" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="K11" s="9">
-        <v>83993</v>
-      </c>
-      <c r="L11" s="10" t="s">
+      <c r="M11" s="9">
+        <v>1136</v>
+      </c>
+      <c r="N11" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="M11" s="9">
-        <v>1107</v>
-      </c>
-      <c r="N11" s="10" t="s">
+      <c r="O11" s="9">
+        <v>350079</v>
+      </c>
+      <c r="P11" s="10" t="s">
         <v>76</v>
-      </c>
-      <c r="O11" s="9">
-        <v>347572</v>
-      </c>
-      <c r="P11" s="10" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>78</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>79</v>
       </c>
       <c r="C12" s="9">
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>134663</v>
+        <v>135362</v>
       </c>
       <c r="E12" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="9">
+        <v>23771</v>
+      </c>
+      <c r="G12" s="9">
+        <v>3899</v>
+      </c>
+      <c r="H12" s="10" t="s">
         <v>80</v>
-      </c>
-      <c r="F12" s="9">
-        <v>23604</v>
-      </c>
-      <c r="G12" s="9">
-        <v>3890</v>
-      </c>
-      <c r="H12" s="10" t="s">
-        <v>81</v>
       </c>
       <c r="I12" s="9">
         <v>53</v>
       </c>
       <c r="J12" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="K12" s="9">
+        <v>52142</v>
+      </c>
+      <c r="L12" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="K12" s="9">
-        <v>51945</v>
-      </c>
-      <c r="L12" s="10" t="s">
+      <c r="M12" s="9">
+        <v>225</v>
+      </c>
+      <c r="N12" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="M12" s="9">
-        <v>217</v>
-      </c>
-      <c r="N12" s="10" t="s">
-        <v>40</v>
-      </c>
       <c r="O12" s="9">
-        <v>158267</v>
+        <v>159133</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>84</v>
@@ -1539,16 +1539,16 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>100471</v>
+        <v>101458</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>87</v>
       </c>
       <c r="F13" s="9">
-        <v>17239</v>
+        <v>17445</v>
       </c>
       <c r="G13" s="9">
-        <v>2502</v>
+        <v>2512</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>88</v>
@@ -1557,151 +1557,151 @@
         <v>81</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="K13" s="9">
-        <v>27711</v>
+        <v>27784</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M13" s="9">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="N13" s="10" t="s">
         <v>40</v>
       </c>
       <c r="O13" s="9">
-        <v>117710</v>
+        <v>118903</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C14" s="9">
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>82558</v>
+        <v>83252</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F14" s="9">
-        <v>16377</v>
+        <v>16545</v>
       </c>
       <c r="G14" s="9">
-        <v>3066</v>
+        <v>3075</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I14" s="9">
         <v>34</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K14" s="9">
-        <v>35499</v>
+        <v>35759</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M14" s="9">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O14" s="9">
-        <v>98935</v>
+        <v>99797</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C15" s="9">
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>110466</v>
+        <v>110842</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F15" s="9">
-        <v>21128</v>
+        <v>21208</v>
       </c>
       <c r="G15" s="9">
-        <v>4564</v>
+        <v>4569</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I15" s="9">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J15" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>32663</v>
+        <v>32755</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M15" s="9">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O15" s="9">
-        <v>131594</v>
+        <v>132050</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C16" s="9">
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>99774</v>
+        <v>100420</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F16" s="9">
-        <v>12754</v>
+        <v>12839</v>
       </c>
       <c r="G16" s="9">
-        <v>2018</v>
+        <v>2022</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I16" s="9">
         <v>106</v>
@@ -1710,319 +1710,319 @@
         <v>48</v>
       </c>
       <c r="K16" s="9">
-        <v>22403</v>
+        <v>22525</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M16" s="9">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="N16" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="O16" s="9">
-        <v>112528</v>
+        <v>113259</v>
       </c>
       <c r="P16" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" s="9">
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55820</v>
+        <v>55837</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F17" s="9">
-        <v>12162</v>
+        <v>12169</v>
       </c>
       <c r="G17" s="9">
         <v>1189</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I17" s="9">
         <v>80</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="K17" s="9">
-        <v>18742</v>
+        <v>18717</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M17" s="9">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O17" s="9">
-        <v>67982</v>
+        <v>68006</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C18" s="9">
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>73400</v>
+        <v>73488</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F18" s="9">
-        <v>12744</v>
+        <v>12770</v>
       </c>
       <c r="G18" s="9">
-        <v>2411</v>
+        <v>2410</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I18" s="9">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J18" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22979</v>
+        <v>22972</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="M18" s="9">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="N18" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O18" s="9">
-        <v>86144</v>
+        <v>86258</v>
       </c>
       <c r="P18" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C19" s="9">
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>34093</v>
+        <v>34106</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F19" s="9">
-        <v>7434</v>
+        <v>7457</v>
       </c>
       <c r="G19" s="9">
         <v>352</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I19" s="9">
         <v>27</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="K19" s="9">
-        <v>7297</v>
+        <v>7294</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="M19" s="9">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N19" s="10" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="O19" s="9">
-        <v>41527</v>
+        <v>41563</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C20" s="9">
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>138304</v>
+        <v>139165</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F20" s="9">
-        <v>38095</v>
+        <v>38340</v>
       </c>
       <c r="G20" s="9">
-        <v>2423</v>
+        <v>2434</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I20" s="9">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>86864</v>
+        <v>87282</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M20" s="9">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="N20" s="10" t="s">
         <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>176399</v>
+        <v>177505</v>
       </c>
       <c r="P20" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C21" s="9">
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>34448</v>
+        <v>34595</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F21" s="9">
-        <v>5085</v>
+        <v>5150</v>
       </c>
       <c r="G21" s="9">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I21" s="9">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K21" s="9">
-        <v>11751</v>
+        <v>11879</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M21" s="9">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O21" s="9">
-        <v>39533</v>
+        <v>39745</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C22" s="12">
         <v>2730933</v>
       </c>
       <c r="D22" s="12">
-        <v>1819978</v>
+        <v>1830999</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>320950</v>
+        <v>323213</v>
       </c>
       <c r="G22" s="12">
-        <v>49181</v>
+        <v>49324</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1470</v>
+        <v>1481</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>583599</v>
+        <v>586180</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
       </c>
       <c r="M22" s="12">
-        <v>3132</v>
+        <v>3257</v>
       </c>
       <c r="N22" s="13" t="s">
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2140928</v>
+        <v>2154212</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2051,7 +2051,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2085,28 +2085,28 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2149,28 +2149,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6432265</v>
+        <v>6472589</v>
       </c>
       <c r="D6" s="6">
-        <v>109351</v>
+        <v>109785</v>
       </c>
       <c r="E6" s="6">
-        <v>69589</v>
+        <v>70013</v>
       </c>
       <c r="F6" s="6">
-        <v>347478</v>
+        <v>349425</v>
       </c>
       <c r="G6" s="6">
-        <v>56544</v>
+        <v>56862</v>
       </c>
       <c r="H6" s="6">
-        <v>9400</v>
+        <v>9424</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6541616</v>
+        <v>6582374</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2181,28 +2181,28 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>246521</v>
+        <v>246927</v>
       </c>
       <c r="D7" s="9">
-        <v>2868</v>
+        <v>2874</v>
       </c>
       <c r="E7" s="9">
-        <v>2117</v>
+        <v>2120</v>
       </c>
       <c r="F7" s="9">
-        <v>13070</v>
+        <v>13100</v>
       </c>
       <c r="G7" s="9">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H7" s="9">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="I7" s="9">
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>249389</v>
+        <v>249801</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2213,28 +2213,28 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>447851</v>
+        <v>450740</v>
       </c>
       <c r="D8" s="9">
-        <v>5903</v>
+        <v>5951</v>
       </c>
       <c r="E8" s="9">
-        <v>4391</v>
+        <v>4421</v>
       </c>
       <c r="F8" s="9">
-        <v>34349</v>
+        <v>34619</v>
       </c>
       <c r="G8" s="9">
-        <v>4089</v>
+        <v>4121</v>
       </c>
       <c r="H8" s="9">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="I8" s="9">
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>453754</v>
+        <v>456691</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2245,28 +2245,28 @@
         <v>57</v>
       </c>
       <c r="C9" s="9">
-        <v>778806</v>
+        <v>786643</v>
       </c>
       <c r="D9" s="9">
-        <v>13446</v>
+        <v>13557</v>
       </c>
       <c r="E9" s="9">
-        <v>8860</v>
+        <v>8968</v>
       </c>
       <c r="F9" s="9">
-        <v>38625</v>
+        <v>38938</v>
       </c>
       <c r="G9" s="9">
-        <v>4740</v>
+        <v>4779</v>
       </c>
       <c r="H9" s="9">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>792252</v>
+        <v>800200</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2277,83 +2277,83 @@
         <v>64</v>
       </c>
       <c r="C10" s="9">
-        <v>797541</v>
+        <v>802040</v>
       </c>
       <c r="D10" s="9">
-        <v>15340</v>
+        <v>15399</v>
       </c>
       <c r="E10" s="9">
-        <v>9398</v>
+        <v>9464</v>
       </c>
       <c r="F10" s="9">
-        <v>39444</v>
+        <v>39664</v>
       </c>
       <c r="G10" s="9">
-        <v>19889</v>
+        <v>20009</v>
       </c>
       <c r="H10" s="9">
-        <v>1072</v>
+        <v>1075</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>812881</v>
+        <v>817439</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>71</v>
-      </c>
       <c r="C11" s="9">
-        <v>1016322</v>
+        <v>1023793</v>
       </c>
       <c r="D11" s="9">
-        <v>20269</v>
+        <v>20273</v>
       </c>
       <c r="E11" s="9">
-        <v>12183</v>
+        <v>12245</v>
       </c>
       <c r="F11" s="9">
-        <v>45756</v>
+        <v>45982</v>
       </c>
       <c r="G11" s="9">
-        <v>8319</v>
+        <v>8362</v>
       </c>
       <c r="H11" s="9">
-        <v>1743</v>
+        <v>1752</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1036591</v>
+        <v>1044066</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>79</v>
-      </c>
       <c r="C12" s="9">
-        <v>490372</v>
+        <v>493106</v>
       </c>
       <c r="D12" s="9">
-        <v>6183</v>
+        <v>6200</v>
       </c>
       <c r="E12" s="9">
-        <v>5888</v>
+        <v>5913</v>
       </c>
       <c r="F12" s="9">
-        <v>28035</v>
+        <v>28165</v>
       </c>
       <c r="G12" s="9">
-        <v>1995</v>
+        <v>2004</v>
       </c>
       <c r="H12" s="9">
         <v>510</v>
@@ -2362,7 +2362,7 @@
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>496555</v>
+        <v>499306</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2373,83 +2373,83 @@
         <v>86</v>
       </c>
       <c r="C13" s="9">
-        <v>353471</v>
+        <v>357029</v>
       </c>
       <c r="D13" s="9">
-        <v>4422</v>
+        <v>4448</v>
       </c>
       <c r="E13" s="9">
-        <v>4004</v>
+        <v>4040</v>
       </c>
       <c r="F13" s="9">
-        <v>25432</v>
+        <v>25678</v>
       </c>
       <c r="G13" s="9">
-        <v>1389</v>
+        <v>1403</v>
       </c>
       <c r="H13" s="9">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="I13" s="9">
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>357893</v>
+        <v>361477</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C14" s="9">
-        <v>293226</v>
+        <v>295805</v>
       </c>
       <c r="D14" s="9">
-        <v>8347</v>
+        <v>8405</v>
       </c>
       <c r="E14" s="9">
-        <v>3222</v>
+        <v>3240</v>
       </c>
       <c r="F14" s="9">
-        <v>19909</v>
+        <v>20069</v>
       </c>
       <c r="G14" s="9">
-        <v>1967</v>
+        <v>1976</v>
       </c>
       <c r="H14" s="9">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>301573</v>
+        <v>304210</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C15" s="9">
-        <v>396828</v>
+        <v>398268</v>
       </c>
       <c r="D15" s="9">
-        <v>7674</v>
+        <v>7699</v>
       </c>
       <c r="E15" s="9">
-        <v>6488</v>
+        <v>6509</v>
       </c>
       <c r="F15" s="9">
-        <v>26874</v>
+        <v>26952</v>
       </c>
       <c r="G15" s="9">
-        <v>3853</v>
+        <v>3866</v>
       </c>
       <c r="H15" s="9">
         <v>511</v>
@@ -2458,59 +2458,59 @@
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>404502</v>
+        <v>405967</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C16" s="9">
-        <v>332531</v>
+        <v>334707</v>
       </c>
       <c r="D16" s="9">
-        <v>4799</v>
+        <v>4823</v>
       </c>
       <c r="E16" s="9">
-        <v>2876</v>
+        <v>2897</v>
       </c>
       <c r="F16" s="9">
-        <v>19383</v>
+        <v>19524</v>
       </c>
       <c r="G16" s="9">
-        <v>3905</v>
+        <v>3931</v>
       </c>
       <c r="H16" s="9">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>337330</v>
+        <v>339530</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" s="9">
-        <v>197150</v>
+        <v>197220</v>
       </c>
       <c r="D17" s="9">
-        <v>4833</v>
+        <v>4835</v>
       </c>
       <c r="E17" s="9">
-        <v>2180</v>
+        <v>2181</v>
       </c>
       <c r="F17" s="9">
-        <v>10293</v>
+        <v>10295</v>
       </c>
       <c r="G17" s="9">
         <v>1708</v>
@@ -2522,30 +2522,30 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>201983</v>
+        <v>202055</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C18" s="9">
-        <v>248565</v>
+        <v>248889</v>
       </c>
       <c r="D18" s="9">
-        <v>5425</v>
+        <v>5437</v>
       </c>
       <c r="E18" s="9">
-        <v>2644</v>
+        <v>2646</v>
       </c>
       <c r="F18" s="9">
-        <v>14246</v>
+        <v>14252</v>
       </c>
       <c r="G18" s="9">
-        <v>2389</v>
+        <v>2390</v>
       </c>
       <c r="H18" s="9">
         <v>493</v>
@@ -2554,27 +2554,27 @@
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>253990</v>
+        <v>254326</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C19" s="9">
-        <v>136847</v>
+        <v>136929</v>
       </c>
       <c r="D19" s="9">
-        <v>1752</v>
+        <v>1754</v>
       </c>
       <c r="E19" s="9">
         <v>1047</v>
       </c>
       <c r="F19" s="9">
-        <v>10418</v>
+        <v>10419</v>
       </c>
       <c r="G19" s="9">
         <v>223</v>
@@ -2586,103 +2586,103 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>138599</v>
+        <v>138683</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C20" s="9">
-        <v>577795</v>
+        <v>581376</v>
       </c>
       <c r="D20" s="9">
-        <v>6973</v>
+        <v>7009</v>
       </c>
       <c r="E20" s="9">
-        <v>3444</v>
+        <v>3469</v>
       </c>
       <c r="F20" s="9">
-        <v>16511</v>
+        <v>16612</v>
       </c>
       <c r="G20" s="9">
-        <v>1017</v>
+        <v>1023</v>
       </c>
       <c r="H20" s="9">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>584768</v>
+        <v>588385</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C21" s="9">
-        <v>118439</v>
+        <v>119117</v>
       </c>
       <c r="D21" s="9">
-        <v>1117</v>
+        <v>1121</v>
       </c>
       <c r="E21" s="9">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="F21" s="9">
-        <v>5133</v>
+        <v>5156</v>
       </c>
       <c r="G21" s="9">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="H21" s="9">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>119556</v>
+        <v>120238</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C22" s="12">
-        <v>6432265</v>
+        <v>6472589</v>
       </c>
       <c r="D22" s="12">
-        <v>109351</v>
+        <v>109785</v>
       </c>
       <c r="E22" s="12">
-        <v>69589</v>
+        <v>70013</v>
       </c>
       <c r="F22" s="12">
-        <v>347478</v>
+        <v>349425</v>
       </c>
       <c r="G22" s="12">
-        <v>56544</v>
+        <v>56862</v>
       </c>
       <c r="H22" s="12">
-        <v>9400</v>
+        <v>9424</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6541616</v>
+        <v>6582374</v>
       </c>
     </row>
   </sheetData>
@@ -2709,7 +2709,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2733,7 +2733,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2742,13 +2742,13 @@
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2776,13 +2776,13 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1122</v>
+        <v>1136</v>
       </c>
       <c r="D7" s="6">
         <v>157</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2799,7 +2799,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2816,7 +2816,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2827,13 +2827,13 @@
         <v>57</v>
       </c>
       <c r="C10" s="9">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D10" s="9">
         <v>4</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2844,38 +2844,38 @@
         <v>64</v>
       </c>
       <c r="C11" s="9">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D11" s="9">
         <v>24</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>71</v>
-      </c>
       <c r="C12" s="9">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>78</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>79</v>
       </c>
       <c r="C13" s="9">
         <v>32</v>
@@ -2884,7 +2884,7 @@
         <v>5</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2895,38 +2895,38 @@
         <v>86</v>
       </c>
       <c r="C14" s="9">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D14" s="9">
         <v>2</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C15" s="9">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D15" s="9">
         <v>1</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C16" s="9">
         <v>155</v>
@@ -2935,32 +2935,32 @@
         <v>47</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C17" s="9">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D17" s="9">
         <v>2</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C18" s="9">
         <v>23</v>
@@ -2974,10 +2974,10 @@
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C19" s="9">
         <v>70</v>
@@ -2991,30 +2991,30 @@
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C20" s="9">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D20" s="9">
         <v>0</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C21" s="9">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D21" s="9">
         <v>7</v>
@@ -3025,10 +3025,10 @@
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C22" s="9">
         <v>64</v>
@@ -3042,19 +3042,19 @@
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C23" s="12">
-        <v>1122</v>
+        <v>1136</v>
       </c>
       <c r="D23" s="12">
         <v>157</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Perbarui data SE2026 23/08/2026  6:37:40,48
</commit_message>
<xml_diff>
--- a/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
+++ b/data/Export_Progres_Pemutakhiran_Keluarga_Kabupaten_Kota.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="173">
   <si>
     <t>PROGRES PEMUTAKHIRAN KELUARGA - KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 22 Agu 2026, 18.16 | Dicetak: 23 Agu 2026, 05.36</t>
+    <t>Seluruh data sampai Kabupaten / Kota | Sumber: FASIH Pendataan SE 2026 | Diperbarui: 22 Agu 2026, 18.16 | Dicetak: 23 Agu 2026, 06.36</t>
   </si>
   <si>
     <t>Kode</t>
@@ -123,7 +123,7 @@
     <t>LAMPUNG</t>
   </si>
   <si>
-    <t>67,05</t>
+    <t>67,43</t>
   </si>
   <si>
     <t>1,81</t>
@@ -132,13 +132,13 @@
     <t>0,05</t>
   </si>
   <si>
-    <t>21,46</t>
+    <t>21,54</t>
   </si>
   <si>
     <t>0,12</t>
   </si>
   <si>
-    <t>78,88</t>
+    <t>79,34</t>
   </si>
   <si>
     <t>1801</t>
@@ -162,7 +162,7 @@
     <t>0,08</t>
   </si>
   <si>
-    <t>92,51</t>
+    <t>92,52</t>
   </si>
   <si>
     <t>1802</t>
@@ -171,16 +171,16 @@
     <t>TANGGAMUS</t>
   </si>
   <si>
-    <t>69,96</t>
+    <t>70,36</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>17,38</t>
-  </si>
-  <si>
-    <t>85,34</t>
+    <t>17,46</t>
+  </si>
+  <si>
+    <t>85,83</t>
   </si>
   <si>
     <t>1803</t>
@@ -189,19 +189,19 @@
     <t>LAMPUNG SELATAN</t>
   </si>
   <si>
-    <t>62,61</t>
-  </si>
-  <si>
-    <t>1,22</t>
-  </si>
-  <si>
-    <t>20,26</t>
+    <t>63,18</t>
+  </si>
+  <si>
+    <t>1,23</t>
+  </si>
+  <si>
+    <t>20,38</t>
   </si>
   <si>
     <t>0,1</t>
   </si>
   <si>
-    <t>75,34</t>
+    <t>76,02</t>
   </si>
   <si>
     <t>1804</t>
@@ -210,16 +210,16 @@
     <t>LAMPUNG TIMUR</t>
   </si>
   <si>
-    <t>68,91</t>
+    <t>69,24</t>
   </si>
   <si>
     <t>1,9</t>
   </si>
   <si>
-    <t>18,62</t>
-  </si>
-  <si>
-    <t>78,09</t>
+    <t>18,67</t>
+  </si>
+  <si>
+    <t>78,46</t>
   </si>
   <si>
     <t>1805</t>
@@ -228,22 +228,22 @@
     <t>LAMPUNG TENGAH</t>
   </si>
   <si>
-    <t>68,75</t>
-  </si>
-  <si>
-    <t>2,74</t>
+    <t>69,22</t>
+  </si>
+  <si>
+    <t>2,75</t>
   </si>
   <si>
     <t>0,07</t>
   </si>
   <si>
-    <t>18,75</t>
+    <t>18,83</t>
   </si>
   <si>
     <t>0,25</t>
   </si>
   <si>
-    <t>77,87</t>
+    <t>78,4</t>
   </si>
   <si>
     <t>1806</t>
@@ -252,7 +252,7 @@
     <t>LAMPUNG UTARA</t>
   </si>
   <si>
-    <t>67,89</t>
+    <t>68,24</t>
   </si>
   <si>
     <t>1,96</t>
@@ -261,13 +261,13 @@
     <t>0,03</t>
   </si>
   <si>
-    <t>26,15</t>
+    <t>26,2</t>
   </si>
   <si>
     <t>0,11</t>
   </si>
   <si>
-    <t>79,81</t>
+    <t>80,22</t>
   </si>
   <si>
     <t>1807</t>
@@ -276,7 +276,7 @@
     <t>WAY KANAN</t>
   </si>
   <si>
-    <t>69,45</t>
+    <t>70</t>
   </si>
   <si>
     <t>1,72</t>
@@ -285,10 +285,10 @@
     <t>0,06</t>
   </si>
   <si>
-    <t>19,02</t>
-  </si>
-  <si>
-    <t>81,39</t>
+    <t>19,14</t>
+  </si>
+  <si>
+    <t>82,06</t>
   </si>
   <si>
     <t>1808</t>
@@ -297,19 +297,19 @@
     <t>TULANG BAWANG</t>
   </si>
   <si>
-    <t>61,55</t>
-  </si>
-  <si>
-    <t>2,27</t>
-  </si>
-  <si>
-    <t>26,44</t>
+    <t>61,97</t>
+  </si>
+  <si>
+    <t>2,28</t>
+  </si>
+  <si>
+    <t>26,52</t>
   </si>
   <si>
     <t>0,02</t>
   </si>
   <si>
-    <t>73,78</t>
+    <t>74,26</t>
   </si>
   <si>
     <t>1809</t>
@@ -318,19 +318,19 @@
     <t>PESAWARAN</t>
   </si>
   <si>
-    <t>72,85</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>21,53</t>
+    <t>73,08</t>
+  </si>
+  <si>
+    <t>3,01</t>
+  </si>
+  <si>
+    <t>21,61</t>
   </si>
   <si>
     <t>0,13</t>
   </si>
   <si>
-    <t>86,78</t>
+    <t>87,08</t>
   </si>
   <si>
     <t>1810</t>
@@ -339,16 +339,16 @@
     <t>PRINGSEWU</t>
   </si>
   <si>
-    <t>73,98</t>
+    <t>74,53</t>
   </si>
   <si>
     <t>1,49</t>
   </si>
   <si>
-    <t>16,59</t>
-  </si>
-  <si>
-    <t>83,44</t>
+    <t>16,66</t>
+  </si>
+  <si>
+    <t>84,05</t>
   </si>
   <si>
     <t>1811</t>
@@ -363,7 +363,7 @@
     <t>1,58</t>
   </si>
   <si>
-    <t>24,92</t>
+    <t>24,91</t>
   </si>
   <si>
     <t>0,16</t>
@@ -378,19 +378,19 @@
     <t>TULANG BAWANG BARAT</t>
   </si>
   <si>
-    <t>74,1</t>
+    <t>74,33</t>
   </si>
   <si>
     <t>2,43</t>
   </si>
   <si>
-    <t>23,16</t>
+    <t>23,19</t>
   </si>
   <si>
     <t>0,27</t>
   </si>
   <si>
-    <t>86,98</t>
+    <t>87,25</t>
   </si>
   <si>
     <t>1813</t>
@@ -399,16 +399,16 @@
     <t>PESISIR BARAT</t>
   </si>
   <si>
-    <t>81,65</t>
+    <t>81,8</t>
   </si>
   <si>
     <t>0,84</t>
   </si>
   <si>
-    <t>17,46</t>
-  </si>
-  <si>
-    <t>99,5</t>
+    <t>17,39</t>
+  </si>
+  <si>
+    <t>99,78</t>
   </si>
   <si>
     <t>1871</t>
@@ -417,16 +417,16 @@
     <t>BANDAR LAMPUNG</t>
   </si>
   <si>
-    <t>49,79</t>
+    <t>50,11</t>
   </si>
   <si>
     <t>0,87</t>
   </si>
   <si>
-    <t>31,23</t>
-  </si>
-  <si>
-    <t>63,51</t>
+    <t>31,39</t>
+  </si>
+  <si>
+    <t>63,9</t>
   </si>
   <si>
     <t>1872</t>
@@ -435,16 +435,16 @@
     <t>METRO</t>
   </si>
   <si>
-    <t>64,66</t>
+    <t>64,99</t>
   </si>
   <si>
     <t>1,39</t>
   </si>
   <si>
-    <t>22,2</t>
-  </si>
-  <si>
-    <t>74,28</t>
+    <t>22,26</t>
+  </si>
+  <si>
+    <t>74,71</t>
   </si>
   <si>
     <t/>
@@ -489,7 +489,7 @@
     <t>Persentase Bangunan Keluarga Khusus Didata</t>
   </si>
   <si>
-    <t>13,82</t>
+    <t>13,65</t>
   </si>
   <si>
     <t>0</t>
@@ -501,31 +501,34 @@
     <t>3,92</t>
   </si>
   <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>6,15</t>
+    <t>19,67</t>
+  </si>
+  <si>
+    <t>6,09</t>
   </si>
   <si>
     <t>15,63</t>
   </si>
   <si>
-    <t>3,77</t>
-  </si>
-  <si>
-    <t>1,05</t>
+    <t>3,64</t>
+  </si>
+  <si>
+    <t>1,04</t>
   </si>
   <si>
     <t>30,32</t>
   </si>
   <si>
+    <t>3,7</t>
+  </si>
+  <si>
     <t>34,78</t>
   </si>
   <si>
     <t>32,86</t>
   </si>
   <si>
-    <t>5,47</t>
+    <t>5,38</t>
   </si>
   <si>
     <t>32,81</t>
@@ -1189,28 +1192,28 @@
         <v>2730933</v>
       </c>
       <c r="D6" s="6">
-        <v>1830999</v>
+        <v>1841525</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="6">
-        <v>323213</v>
+        <v>325076</v>
       </c>
       <c r="G6" s="6">
-        <v>49324</v>
+        <v>49441</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>37</v>
       </c>
       <c r="I6" s="6">
-        <v>1481</v>
+        <v>1501</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>38</v>
       </c>
       <c r="K6" s="6">
-        <v>586180</v>
+        <v>588333</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>39</v>
@@ -1222,7 +1225,7 @@
         <v>40</v>
       </c>
       <c r="O6" s="6">
-        <v>2154212</v>
+        <v>2166601</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>41</v>
@@ -1239,16 +1242,16 @@
         <v>85145</v>
       </c>
       <c r="D7" s="9">
-        <v>67792</v>
+        <v>67791</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="F7" s="9">
-        <v>10978</v>
+        <v>10988</v>
       </c>
       <c r="G7" s="9">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>45</v>
@@ -1260,7 +1263,7 @@
         <v>46</v>
       </c>
       <c r="K7" s="9">
-        <v>15733</v>
+        <v>15734</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>47</v>
@@ -1272,7 +1275,7 @@
         <v>48</v>
       </c>
       <c r="O7" s="9">
-        <v>78770</v>
+        <v>78779</v>
       </c>
       <c r="P7" s="10" t="s">
         <v>49</v>
@@ -1289,28 +1292,28 @@
         <v>172957</v>
       </c>
       <c r="D8" s="9">
-        <v>120998</v>
+        <v>121693</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>52</v>
       </c>
       <c r="F8" s="9">
-        <v>26598</v>
+        <v>26755</v>
       </c>
       <c r="G8" s="9">
-        <v>1732</v>
+        <v>1737</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="I8" s="9">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J8" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K8" s="9">
-        <v>30062</v>
+        <v>30201</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>54</v>
@@ -1322,7 +1325,7 @@
         <v>48</v>
       </c>
       <c r="O8" s="9">
-        <v>147596</v>
+        <v>148448</v>
       </c>
       <c r="P8" s="10" t="s">
         <v>55</v>
@@ -1339,28 +1342,28 @@
         <v>342734</v>
       </c>
       <c r="D9" s="9">
-        <v>214576</v>
+        <v>216535</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>58</v>
       </c>
       <c r="F9" s="9">
-        <v>43624</v>
+        <v>44010</v>
       </c>
       <c r="G9" s="9">
-        <v>4182</v>
+        <v>4202</v>
       </c>
       <c r="H9" s="10" t="s">
         <v>59</v>
       </c>
       <c r="I9" s="9">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K9" s="9">
-        <v>69433</v>
+        <v>69863</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>60</v>
@@ -1372,7 +1375,7 @@
         <v>61</v>
       </c>
       <c r="O9" s="9">
-        <v>258200</v>
+        <v>260545</v>
       </c>
       <c r="P9" s="10" t="s">
         <v>62</v>
@@ -1389,16 +1392,16 @@
         <v>362839</v>
       </c>
       <c r="D10" s="9">
-        <v>250043</v>
+        <v>251245</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>65</v>
       </c>
       <c r="F10" s="9">
-        <v>33305</v>
+        <v>33456</v>
       </c>
       <c r="G10" s="9">
-        <v>6897</v>
+        <v>6909</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>66</v>
@@ -1410,7 +1413,7 @@
         <v>38</v>
       </c>
       <c r="K10" s="9">
-        <v>67547</v>
+        <v>67724</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>67</v>
@@ -1422,7 +1425,7 @@
         <v>48</v>
       </c>
       <c r="O10" s="9">
-        <v>283348</v>
+        <v>284701</v>
       </c>
       <c r="P10" s="10" t="s">
         <v>68</v>
@@ -1439,28 +1442,28 @@
         <v>449575</v>
       </c>
       <c r="D11" s="9">
-        <v>309065</v>
+        <v>311197</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="9">
-        <v>41014</v>
+        <v>41254</v>
       </c>
       <c r="G11" s="9">
-        <v>12339</v>
+        <v>12379</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>72</v>
       </c>
       <c r="I11" s="9">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>73</v>
       </c>
       <c r="K11" s="9">
-        <v>84296</v>
+        <v>84635</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>74</v>
@@ -1472,7 +1475,7 @@
         <v>75</v>
       </c>
       <c r="O11" s="9">
-        <v>350079</v>
+        <v>352451</v>
       </c>
       <c r="P11" s="10" t="s">
         <v>76</v>
@@ -1489,28 +1492,28 @@
         <v>199396</v>
       </c>
       <c r="D12" s="9">
-        <v>135362</v>
+        <v>136066</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>79</v>
       </c>
       <c r="F12" s="9">
-        <v>23771</v>
+        <v>23895</v>
       </c>
       <c r="G12" s="9">
-        <v>3899</v>
+        <v>3907</v>
       </c>
       <c r="H12" s="10" t="s">
         <v>80</v>
       </c>
       <c r="I12" s="9">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J12" s="10" t="s">
         <v>81</v>
       </c>
       <c r="K12" s="9">
-        <v>52142</v>
+        <v>52239</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>82</v>
@@ -1522,7 +1525,7 @@
         <v>83</v>
       </c>
       <c r="O12" s="9">
-        <v>159133</v>
+        <v>159961</v>
       </c>
       <c r="P12" s="10" t="s">
         <v>84</v>
@@ -1539,28 +1542,28 @@
         <v>146092</v>
       </c>
       <c r="D13" s="9">
-        <v>101458</v>
+        <v>102269</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>87</v>
       </c>
       <c r="F13" s="9">
-        <v>17445</v>
+        <v>17621</v>
       </c>
       <c r="G13" s="9">
-        <v>2512</v>
+        <v>2518</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>88</v>
       </c>
       <c r="I13" s="9">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="J13" s="10" t="s">
         <v>89</v>
       </c>
       <c r="K13" s="9">
-        <v>27784</v>
+        <v>27966</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>90</v>
@@ -1572,7 +1575,7 @@
         <v>40</v>
       </c>
       <c r="O13" s="9">
-        <v>118903</v>
+        <v>119890</v>
       </c>
       <c r="P13" s="10" t="s">
         <v>91</v>
@@ -1589,16 +1592,16 @@
         <v>135256</v>
       </c>
       <c r="D14" s="9">
-        <v>83252</v>
+        <v>83819</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>94</v>
       </c>
       <c r="F14" s="9">
-        <v>16545</v>
+        <v>16626</v>
       </c>
       <c r="G14" s="9">
-        <v>3075</v>
+        <v>3080</v>
       </c>
       <c r="H14" s="10" t="s">
         <v>95</v>
@@ -1610,7 +1613,7 @@
         <v>81</v>
       </c>
       <c r="K14" s="9">
-        <v>35759</v>
+        <v>35873</v>
       </c>
       <c r="L14" s="10" t="s">
         <v>96</v>
@@ -1622,7 +1625,7 @@
         <v>97</v>
       </c>
       <c r="O14" s="9">
-        <v>99797</v>
+        <v>100445</v>
       </c>
       <c r="P14" s="10" t="s">
         <v>98</v>
@@ -1639,16 +1642,16 @@
         <v>152158</v>
       </c>
       <c r="D15" s="9">
-        <v>110842</v>
+        <v>111197</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>101</v>
       </c>
       <c r="F15" s="9">
-        <v>21208</v>
+        <v>21302</v>
       </c>
       <c r="G15" s="9">
-        <v>4569</v>
+        <v>4580</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>102</v>
@@ -1660,7 +1663,7 @@
         <v>46</v>
       </c>
       <c r="K15" s="9">
-        <v>32755</v>
+        <v>32875</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>103</v>
@@ -1672,7 +1675,7 @@
         <v>104</v>
       </c>
       <c r="O15" s="9">
-        <v>132050</v>
+        <v>132499</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>105</v>
@@ -1689,13 +1692,13 @@
         <v>135741</v>
       </c>
       <c r="D16" s="9">
-        <v>100420</v>
+        <v>101161</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>108</v>
       </c>
       <c r="F16" s="9">
-        <v>12839</v>
+        <v>12932</v>
       </c>
       <c r="G16" s="9">
         <v>2022</v>
@@ -1710,7 +1713,7 @@
         <v>48</v>
       </c>
       <c r="K16" s="9">
-        <v>22525</v>
+        <v>22615</v>
       </c>
       <c r="L16" s="10" t="s">
         <v>110</v>
@@ -1722,7 +1725,7 @@
         <v>73</v>
       </c>
       <c r="O16" s="9">
-        <v>113259</v>
+        <v>114093</v>
       </c>
       <c r="P16" s="10" t="s">
         <v>111</v>
@@ -1739,13 +1742,13 @@
         <v>75115</v>
       </c>
       <c r="D17" s="9">
-        <v>55837</v>
+        <v>55839</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>114</v>
       </c>
       <c r="F17" s="9">
-        <v>12169</v>
+        <v>12173</v>
       </c>
       <c r="G17" s="9">
         <v>1189</v>
@@ -1754,13 +1757,13 @@
         <v>115</v>
       </c>
       <c r="I17" s="9">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J17" s="10" t="s">
         <v>83</v>
       </c>
       <c r="K17" s="9">
-        <v>18717</v>
+        <v>18711</v>
       </c>
       <c r="L17" s="10" t="s">
         <v>116</v>
@@ -1772,7 +1775,7 @@
         <v>117</v>
       </c>
       <c r="O17" s="9">
-        <v>68006</v>
+        <v>68012</v>
       </c>
       <c r="P17" s="10" t="s">
         <v>118</v>
@@ -1789,13 +1792,13 @@
         <v>99169</v>
       </c>
       <c r="D18" s="9">
-        <v>73488</v>
+        <v>73710</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>121</v>
       </c>
       <c r="F18" s="9">
-        <v>12770</v>
+        <v>12814</v>
       </c>
       <c r="G18" s="9">
         <v>2410</v>
@@ -1804,13 +1807,13 @@
         <v>122</v>
       </c>
       <c r="I18" s="9">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J18" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K18" s="9">
-        <v>22972</v>
+        <v>22993</v>
       </c>
       <c r="L18" s="10" t="s">
         <v>123</v>
@@ -1822,7 +1825,7 @@
         <v>124</v>
       </c>
       <c r="O18" s="9">
-        <v>86258</v>
+        <v>86524</v>
       </c>
       <c r="P18" s="10" t="s">
         <v>125</v>
@@ -1839,13 +1842,13 @@
         <v>41772</v>
       </c>
       <c r="D19" s="9">
-        <v>34106</v>
+        <v>34168</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>128</v>
       </c>
       <c r="F19" s="9">
-        <v>7457</v>
+        <v>7513</v>
       </c>
       <c r="G19" s="9">
         <v>352</v>
@@ -1860,7 +1863,7 @@
         <v>89</v>
       </c>
       <c r="K19" s="9">
-        <v>7294</v>
+        <v>7264</v>
       </c>
       <c r="L19" s="10" t="s">
         <v>130</v>
@@ -1872,7 +1875,7 @@
         <v>73</v>
       </c>
       <c r="O19" s="9">
-        <v>41563</v>
+        <v>41681</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>131</v>
@@ -1889,28 +1892,28 @@
         <v>279478</v>
       </c>
       <c r="D20" s="9">
-        <v>139165</v>
+        <v>140059</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>134</v>
       </c>
       <c r="F20" s="9">
-        <v>38340</v>
+        <v>38541</v>
       </c>
       <c r="G20" s="9">
-        <v>2434</v>
+        <v>2439</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>135</v>
       </c>
       <c r="I20" s="9">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K20" s="9">
-        <v>87282</v>
+        <v>87730</v>
       </c>
       <c r="L20" s="10" t="s">
         <v>136</v>
@@ -1922,7 +1925,7 @@
         <v>46</v>
       </c>
       <c r="O20" s="9">
-        <v>177505</v>
+        <v>178600</v>
       </c>
       <c r="P20" s="10" t="s">
         <v>137</v>
@@ -1939,16 +1942,16 @@
         <v>53506</v>
       </c>
       <c r="D21" s="9">
-        <v>34595</v>
+        <v>34776</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>140</v>
       </c>
       <c r="F21" s="9">
-        <v>5150</v>
+        <v>5196</v>
       </c>
       <c r="G21" s="9">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>141</v>
@@ -1960,7 +1963,7 @@
         <v>73</v>
       </c>
       <c r="K21" s="9">
-        <v>11879</v>
+        <v>11910</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>142</v>
@@ -1972,7 +1975,7 @@
         <v>97</v>
       </c>
       <c r="O21" s="9">
-        <v>39745</v>
+        <v>39972</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>143</v>
@@ -1989,28 +1992,28 @@
         <v>2730933</v>
       </c>
       <c r="D22" s="12">
-        <v>1830999</v>
+        <v>1841525</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12">
-        <v>323213</v>
+        <v>325076</v>
       </c>
       <c r="G22" s="12">
-        <v>49324</v>
+        <v>49441</v>
       </c>
       <c r="H22" s="13" t="s">
         <v>37</v>
       </c>
       <c r="I22" s="12">
-        <v>1481</v>
+        <v>1501</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>38</v>
       </c>
       <c r="K22" s="12">
-        <v>586180</v>
+        <v>588333</v>
       </c>
       <c r="L22" s="13" t="s">
         <v>39</v>
@@ -2022,7 +2025,7 @@
         <v>40</v>
       </c>
       <c r="O22" s="12">
-        <v>2154212</v>
+        <v>2166601</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>41</v>
@@ -2149,28 +2152,28 @@
         <v>35</v>
       </c>
       <c r="C6" s="6">
-        <v>6472589</v>
+        <v>6510245</v>
       </c>
       <c r="D6" s="6">
-        <v>109785</v>
+        <v>110199</v>
       </c>
       <c r="E6" s="6">
-        <v>70013</v>
+        <v>70512</v>
       </c>
       <c r="F6" s="6">
-        <v>349425</v>
+        <v>351229</v>
       </c>
       <c r="G6" s="6">
-        <v>56862</v>
+        <v>57166</v>
       </c>
       <c r="H6" s="6">
-        <v>9424</v>
+        <v>9448</v>
       </c>
       <c r="I6" s="6">
         <v>0</v>
       </c>
       <c r="J6" s="6">
-        <v>6582374</v>
+        <v>6620444</v>
       </c>
     </row>
     <row r="7" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2181,16 +2184,16 @@
         <v>43</v>
       </c>
       <c r="C7" s="9">
-        <v>246927</v>
+        <v>246950</v>
       </c>
       <c r="D7" s="9">
-        <v>2874</v>
+        <v>2871</v>
       </c>
       <c r="E7" s="9">
-        <v>2120</v>
+        <v>2121</v>
       </c>
       <c r="F7" s="9">
-        <v>13100</v>
+        <v>13105</v>
       </c>
       <c r="G7" s="9">
         <v>308</v>
@@ -2202,7 +2205,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="9">
-        <v>249801</v>
+        <v>249821</v>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2213,19 +2216,19 @@
         <v>51</v>
       </c>
       <c r="C8" s="9">
-        <v>450740</v>
+        <v>453367</v>
       </c>
       <c r="D8" s="9">
-        <v>5951</v>
+        <v>6001</v>
       </c>
       <c r="E8" s="9">
-        <v>4421</v>
+        <v>4443</v>
       </c>
       <c r="F8" s="9">
-        <v>34619</v>
+        <v>34801</v>
       </c>
       <c r="G8" s="9">
-        <v>4121</v>
+        <v>4131</v>
       </c>
       <c r="H8" s="9">
         <v>564</v>
@@ -2234,7 +2237,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="9">
-        <v>456691</v>
+        <v>459368</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2245,28 +2248,28 @@
         <v>57</v>
       </c>
       <c r="C9" s="9">
-        <v>786643</v>
+        <v>793882</v>
       </c>
       <c r="D9" s="9">
-        <v>13557</v>
+        <v>13642</v>
       </c>
       <c r="E9" s="9">
-        <v>8968</v>
+        <v>9056</v>
       </c>
       <c r="F9" s="9">
-        <v>38938</v>
+        <v>39278</v>
       </c>
       <c r="G9" s="9">
-        <v>4779</v>
+        <v>4824</v>
       </c>
       <c r="H9" s="9">
-        <v>1023</v>
+        <v>1026</v>
       </c>
       <c r="I9" s="9">
         <v>0</v>
       </c>
       <c r="J9" s="9">
-        <v>800200</v>
+        <v>807524</v>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2277,28 +2280,28 @@
         <v>64</v>
       </c>
       <c r="C10" s="9">
-        <v>802040</v>
+        <v>805907</v>
       </c>
       <c r="D10" s="9">
-        <v>15399</v>
+        <v>15446</v>
       </c>
       <c r="E10" s="9">
-        <v>9464</v>
+        <v>9504</v>
       </c>
       <c r="F10" s="9">
-        <v>39664</v>
+        <v>39828</v>
       </c>
       <c r="G10" s="9">
-        <v>20009</v>
+        <v>20122</v>
       </c>
       <c r="H10" s="9">
-        <v>1075</v>
+        <v>1081</v>
       </c>
       <c r="I10" s="9">
         <v>0</v>
       </c>
       <c r="J10" s="9">
-        <v>817439</v>
+        <v>821353</v>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2309,28 +2312,28 @@
         <v>70</v>
       </c>
       <c r="C11" s="9">
-        <v>1023793</v>
+        <v>1030804</v>
       </c>
       <c r="D11" s="9">
-        <v>20273</v>
+        <v>20341</v>
       </c>
       <c r="E11" s="9">
-        <v>12245</v>
+        <v>12319</v>
       </c>
       <c r="F11" s="9">
-        <v>45982</v>
+        <v>46238</v>
       </c>
       <c r="G11" s="9">
-        <v>8362</v>
+        <v>8418</v>
       </c>
       <c r="H11" s="9">
-        <v>1752</v>
+        <v>1756</v>
       </c>
       <c r="I11" s="9">
         <v>0</v>
       </c>
       <c r="J11" s="9">
-        <v>1044066</v>
+        <v>1051145</v>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2341,28 +2344,28 @@
         <v>78</v>
       </c>
       <c r="C12" s="9">
-        <v>493106</v>
+        <v>495725</v>
       </c>
       <c r="D12" s="9">
-        <v>6200</v>
+        <v>6210</v>
       </c>
       <c r="E12" s="9">
-        <v>5913</v>
+        <v>5938</v>
       </c>
       <c r="F12" s="9">
-        <v>28165</v>
+        <v>28313</v>
       </c>
       <c r="G12" s="9">
-        <v>2004</v>
+        <v>2007</v>
       </c>
       <c r="H12" s="9">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="I12" s="9">
         <v>0</v>
       </c>
       <c r="J12" s="9">
-        <v>499306</v>
+        <v>501935</v>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2373,19 +2376,19 @@
         <v>86</v>
       </c>
       <c r="C13" s="9">
-        <v>357029</v>
+        <v>360020</v>
       </c>
       <c r="D13" s="9">
-        <v>4448</v>
+        <v>4481</v>
       </c>
       <c r="E13" s="9">
-        <v>4040</v>
+        <v>4065</v>
       </c>
       <c r="F13" s="9">
-        <v>25678</v>
+        <v>25874</v>
       </c>
       <c r="G13" s="9">
-        <v>1403</v>
+        <v>1420</v>
       </c>
       <c r="H13" s="9">
         <v>473</v>
@@ -2394,7 +2397,7 @@
         <v>0</v>
       </c>
       <c r="J13" s="9">
-        <v>361477</v>
+        <v>364501</v>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2405,28 +2408,28 @@
         <v>93</v>
       </c>
       <c r="C14" s="9">
-        <v>295805</v>
+        <v>297769</v>
       </c>
       <c r="D14" s="9">
-        <v>8405</v>
+        <v>8445</v>
       </c>
       <c r="E14" s="9">
-        <v>3240</v>
+        <v>3260</v>
       </c>
       <c r="F14" s="9">
-        <v>20069</v>
+        <v>20178</v>
       </c>
       <c r="G14" s="9">
-        <v>1976</v>
+        <v>1984</v>
       </c>
       <c r="H14" s="9">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="I14" s="9">
         <v>0</v>
       </c>
       <c r="J14" s="9">
-        <v>304210</v>
+        <v>306214</v>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2437,19 +2440,19 @@
         <v>100</v>
       </c>
       <c r="C15" s="9">
-        <v>398268</v>
+        <v>399695</v>
       </c>
       <c r="D15" s="9">
-        <v>7699</v>
+        <v>7712</v>
       </c>
       <c r="E15" s="9">
-        <v>6509</v>
+        <v>6529</v>
       </c>
       <c r="F15" s="9">
-        <v>26952</v>
+        <v>27047</v>
       </c>
       <c r="G15" s="9">
-        <v>3866</v>
+        <v>3878</v>
       </c>
       <c r="H15" s="9">
         <v>511</v>
@@ -2458,7 +2461,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="9">
-        <v>405967</v>
+        <v>407407</v>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2469,28 +2472,28 @@
         <v>107</v>
       </c>
       <c r="C16" s="9">
-        <v>334707</v>
+        <v>337198</v>
       </c>
       <c r="D16" s="9">
-        <v>4823</v>
+        <v>4843</v>
       </c>
       <c r="E16" s="9">
-        <v>2897</v>
+        <v>2926</v>
       </c>
       <c r="F16" s="9">
-        <v>19524</v>
+        <v>19668</v>
       </c>
       <c r="G16" s="9">
-        <v>3931</v>
+        <v>3958</v>
       </c>
       <c r="H16" s="9">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I16" s="9">
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>339530</v>
+        <v>342041</v>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2501,16 +2504,16 @@
         <v>113</v>
       </c>
       <c r="C17" s="9">
-        <v>197220</v>
+        <v>197236</v>
       </c>
       <c r="D17" s="9">
         <v>4835</v>
       </c>
       <c r="E17" s="9">
-        <v>2181</v>
+        <v>2182</v>
       </c>
       <c r="F17" s="9">
-        <v>10295</v>
+        <v>10296</v>
       </c>
       <c r="G17" s="9">
         <v>1708</v>
@@ -2522,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>202055</v>
+        <v>202071</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2533,19 +2536,19 @@
         <v>120</v>
       </c>
       <c r="C18" s="9">
-        <v>248889</v>
+        <v>249559</v>
       </c>
       <c r="D18" s="9">
-        <v>5437</v>
+        <v>5447</v>
       </c>
       <c r="E18" s="9">
-        <v>2646</v>
+        <v>2770</v>
       </c>
       <c r="F18" s="9">
-        <v>14252</v>
+        <v>14292</v>
       </c>
       <c r="G18" s="9">
-        <v>2390</v>
+        <v>2393</v>
       </c>
       <c r="H18" s="9">
         <v>493</v>
@@ -2554,7 +2557,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>254326</v>
+        <v>255006</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2565,16 +2568,16 @@
         <v>127</v>
       </c>
       <c r="C19" s="9">
-        <v>136929</v>
+        <v>137223</v>
       </c>
       <c r="D19" s="9">
         <v>1754</v>
       </c>
       <c r="E19" s="9">
-        <v>1047</v>
+        <v>1051</v>
       </c>
       <c r="F19" s="9">
-        <v>10419</v>
+        <v>10433</v>
       </c>
       <c r="G19" s="9">
         <v>223</v>
@@ -2586,7 +2589,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>138683</v>
+        <v>138977</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2597,28 +2600,28 @@
         <v>133</v>
       </c>
       <c r="C20" s="9">
-        <v>581376</v>
+        <v>585112</v>
       </c>
       <c r="D20" s="9">
-        <v>7009</v>
+        <v>7047</v>
       </c>
       <c r="E20" s="9">
-        <v>3469</v>
+        <v>3489</v>
       </c>
       <c r="F20" s="9">
-        <v>16612</v>
+        <v>16690</v>
       </c>
       <c r="G20" s="9">
-        <v>1023</v>
+        <v>1030</v>
       </c>
       <c r="H20" s="9">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="I20" s="9">
         <v>0</v>
       </c>
       <c r="J20" s="9">
-        <v>588385</v>
+        <v>592159</v>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2629,28 +2632,28 @@
         <v>139</v>
       </c>
       <c r="C21" s="9">
-        <v>119117</v>
+        <v>119798</v>
       </c>
       <c r="D21" s="9">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="E21" s="9">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="F21" s="9">
-        <v>5156</v>
+        <v>5188</v>
       </c>
       <c r="G21" s="9">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="H21" s="9">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="I21" s="9">
         <v>0</v>
       </c>
       <c r="J21" s="9">
-        <v>120238</v>
+        <v>120922</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2661,28 +2664,28 @@
         <v>145</v>
       </c>
       <c r="C22" s="12">
-        <v>6472589</v>
+        <v>6510245</v>
       </c>
       <c r="D22" s="12">
-        <v>109785</v>
+        <v>110199</v>
       </c>
       <c r="E22" s="12">
-        <v>70013</v>
+        <v>70512</v>
       </c>
       <c r="F22" s="12">
-        <v>349425</v>
+        <v>351229</v>
       </c>
       <c r="G22" s="12">
-        <v>56862</v>
+        <v>57166</v>
       </c>
       <c r="H22" s="12">
-        <v>9424</v>
+        <v>9448</v>
       </c>
       <c r="I22" s="12">
         <v>0</v>
       </c>
       <c r="J22" s="12">
-        <v>6582374</v>
+        <v>6620444</v>
       </c>
     </row>
   </sheetData>
@@ -2776,7 +2779,7 @@
         <v>35</v>
       </c>
       <c r="C7" s="6">
-        <v>1136</v>
+        <v>1150</v>
       </c>
       <c r="D7" s="6">
         <v>157</v>
@@ -2844,7 +2847,7 @@
         <v>64</v>
       </c>
       <c r="C11" s="9">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D11" s="9">
         <v>24</v>
@@ -2861,7 +2864,7 @@
         <v>70</v>
       </c>
       <c r="C12" s="9">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D12" s="9">
         <v>12</v>
@@ -2895,7 +2898,7 @@
         <v>86</v>
       </c>
       <c r="C14" s="9">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D14" s="9">
         <v>2</v>
@@ -2912,7 +2915,7 @@
         <v>93</v>
       </c>
       <c r="C15" s="9">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D15" s="9">
         <v>1</v>
@@ -2946,13 +2949,13 @@
         <v>107</v>
       </c>
       <c r="C17" s="9">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D17" s="9">
         <v>2</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2969,7 +2972,7 @@
         <v>8</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2986,7 +2989,7 @@
         <v>23</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2997,7 +3000,7 @@
         <v>127</v>
       </c>
       <c r="C20" s="9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D20" s="9">
         <v>0</v>
@@ -3014,13 +3017,13 @@
         <v>133</v>
       </c>
       <c r="C21" s="9">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D21" s="9">
         <v>7</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3037,7 +3040,7 @@
         <v>21</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3048,7 +3051,7 @@
         <v>145</v>
       </c>
       <c r="C23" s="12">
-        <v>1136</v>
+        <v>1150</v>
       </c>
       <c r="D23" s="12">
         <v>157</v>

</xml_diff>